<commit_message>
Update game data: day 742, cash 1635866.18, 3-day period 248
</commit_message>
<xml_diff>
--- a/data/supply_chain_game.xlsx
+++ b/data/supply_chain_game.xlsx
@@ -10,18 +10,26 @@
     <sheet name="概览" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="三日周期" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="每日数据" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="资金构成" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="运营参数" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="资金构成_旧版" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="运营参数_旧版" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="决策历史" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="排行榜" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="排行榜_旧版" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="快照历史" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="资金构成" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="运营参数" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="排行榜" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$248</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$742</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'资金构成'!$A$1:$C$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'运营参数'!$A$9:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'排行榜'!$A$1:$C$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$249</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$743</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'资金构成_旧版'!$A$1:$C$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'运营参数_旧版'!$A$9:$F$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'排行榜_旧版'!$A$1:$C$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'运营参数'!$A$1:$J$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -547,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D49"/>
+  <dimension ref="A1:D48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -559,14 +567,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Supply Chain Game 运营看板</t>
+          <t>Supply Chain Game 运营看板（最新）</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>按游戏日每 3 天一个周期汇总；图表数据来自游戏官方 plot / standing / cash / history 页面。</t>
+          <t>本页只显示最新状态。历史抓取、每日和三日周期都是追加，不会覆盖已有行。</t>
         </is>
       </c>
     </row>
@@ -579,7 +587,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-05T15:26:02+08:00</t>
+          <t>2026-09-05T15:35:15+08:00</t>
         </is>
       </c>
     </row>
@@ -602,7 +610,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>741</v>
+        <v>742</v>
       </c>
     </row>
     <row r="7">
@@ -612,7 +620,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>719</v>
+        <v>718</v>
       </c>
     </row>
     <row r="8">
@@ -642,7 +650,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>1621232.07</v>
+        <v>1635866.18</v>
       </c>
     </row>
     <row r="11">
@@ -684,7 +692,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>1219600.35</v>
+        <v>1219918.86</v>
       </c>
     </row>
     <row r="15"/>
@@ -778,7 +786,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>337</v>
+        <v>326</v>
       </c>
     </row>
     <row r="25">
@@ -816,7 +824,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="30">
@@ -827,7 +835,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>739–741</t>
+          <t>742–744</t>
         </is>
       </c>
     </row>
@@ -839,7 +847,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否（进行中）</t>
         </is>
       </c>
     </row>
@@ -898,9 +906,6 @@
         <is>
           <t>周期现金变动</t>
         </is>
-      </c>
-      <c r="B37" s="4" t="n">
-        <v>11057.84364954405</v>
       </c>
     </row>
     <row r="38"/>
@@ -962,7 +967,7 @@
         </is>
       </c>
       <c r="B44" s="4" t="n">
-        <v>11057.84364954405</v>
+        <v>11057.8436453836</v>
       </c>
     </row>
     <row r="45"/>
@@ -977,24 +982,753 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>游戏速度约 1 游戏日 / 14 分钟，3 个游戏日约 42 分钟。脚本每 15 分钟刷新一次，并把完整历史重写成 Excel。</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>「三日周期」按游戏日 1–3、4–6 … 切片。Day 730 起为你们接管后的区间。现金序列已按当前现金校准。</t>
+          <t>时间序列请看「快照历史」「每日数据」「三日周期」。每次抓取只追加新行；已完成的历史行不会被改写。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="3">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A48:D48"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A49:D49"/>
   </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>抓取时间</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="inlineStr">
+        <is>
+          <t>游戏日</t>
+        </is>
+      </c>
+      <c r="C1" s="9" t="inlineStr">
+        <is>
+          <t>工厂地区</t>
+        </is>
+      </c>
+      <c r="D1" s="9" t="inlineStr">
+        <is>
+          <t>当前产能</t>
+        </is>
+      </c>
+      <c r="E1" s="9" t="inlineStr">
+        <is>
+          <t>计划产能</t>
+        </is>
+      </c>
+      <c r="F1" s="9" t="inlineStr">
+        <is>
+          <t>工厂运输</t>
+        </is>
+      </c>
+      <c r="G1" s="9" t="inlineStr">
+        <is>
+          <t>订货点</t>
+        </is>
+      </c>
+      <c r="H1" s="9" t="inlineStr">
+        <is>
+          <t>批量</t>
+        </is>
+      </c>
+      <c r="I1" s="9" t="inlineStr">
+        <is>
+          <t>仓库运输</t>
+        </is>
+      </c>
+      <c r="J1" s="9" t="inlineStr">
+        <is>
+          <t>是否运营</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:35:15+08:00</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="n">
+        <v>742</v>
+      </c>
+      <c r="C2" s="11" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="D2" s="21" t="n">
+        <v>20</v>
+      </c>
+      <c r="E2" s="21" t="n">
+        <v>40</v>
+      </c>
+      <c r="F2" s="11" t="inlineStr">
+        <is>
+          <t>truck</t>
+        </is>
+      </c>
+      <c r="G2" s="22" t="n">
+        <v>3600</v>
+      </c>
+      <c r="H2" s="22" t="n">
+        <v>200</v>
+      </c>
+      <c r="I2" s="11" t="inlineStr">
+        <is>
+          <t>truck</t>
+        </is>
+      </c>
+      <c r="J2" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:J2"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>抓取时间</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="inlineStr">
+        <is>
+          <t>游戏日</t>
+        </is>
+      </c>
+      <c r="C1" s="9" t="inlineStr">
+        <is>
+          <t>排名</t>
+        </is>
+      </c>
+      <c r="D1" s="9" t="inlineStr">
+        <is>
+          <t>队伍</t>
+        </is>
+      </c>
+      <c r="E1" s="9" t="inlineStr">
+        <is>
+          <t>现金</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:35:15+08:00</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="n">
+        <v>742</v>
+      </c>
+      <c r="C2" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="11" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="E2" s="14" t="n">
+        <v>2855785.04</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:35:15+08:00</t>
+        </is>
+      </c>
+      <c r="B3" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="C3" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" s="16" t="inlineStr">
+        <is>
+          <t>montesquieu</t>
+        </is>
+      </c>
+      <c r="E3" s="18" t="n">
+        <v>1886819</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:35:15+08:00</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="n">
+        <v>742</v>
+      </c>
+      <c r="C4" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>nicetry</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="n">
+        <v>1886796.78</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:35:15+08:00</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="C5" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>group7</t>
+        </is>
+      </c>
+      <c r="E5" s="18" t="n">
+        <v>1852842.25</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:35:15+08:00</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="n">
+        <v>742</v>
+      </c>
+      <c r="C6" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>group14</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="n">
+        <v>1852725.6</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:35:15+08:00</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="C7" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>group15</t>
+        </is>
+      </c>
+      <c r="E7" s="18" t="n">
+        <v>1852707.95</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:35:15+08:00</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="n">
+        <v>742</v>
+      </c>
+      <c r="C8" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>group8</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="n">
+        <v>1636140.95</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:35:15+08:00</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="C9" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>group2</t>
+        </is>
+      </c>
+      <c r="E9" s="18" t="n">
+        <v>1635868.62</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:35:15+08:00</t>
+        </is>
+      </c>
+      <c r="B10" s="24" t="n">
+        <v>742</v>
+      </c>
+      <c r="C10" s="24" t="n">
+        <v>9</v>
+      </c>
+      <c r="D10" s="25" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="E10" s="26" t="n">
+        <v>1635866.18</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:35:15+08:00</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="C11" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>teamhlly</t>
+        </is>
+      </c>
+      <c r="E11" s="18" t="n">
+        <v>1635726.76</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:35:15+08:00</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="n">
+        <v>742</v>
+      </c>
+      <c r="C12" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>group9</t>
+        </is>
+      </c>
+      <c r="E12" s="14" t="n">
+        <v>1635722.97</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:35:15+08:00</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="C13" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>group25</t>
+        </is>
+      </c>
+      <c r="E13" s="18" t="n">
+        <v>1635714.78</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:35:15+08:00</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="n">
+        <v>742</v>
+      </c>
+      <c r="C14" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>group11</t>
+        </is>
+      </c>
+      <c r="E14" s="14" t="n">
+        <v>1635702.8</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:35:15+08:00</t>
+        </is>
+      </c>
+      <c r="B15" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="C15" s="15" t="n">
+        <v>14</v>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>88888888</t>
+        </is>
+      </c>
+      <c r="E15" s="18" t="n">
+        <v>1635680.73</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:35:15+08:00</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="n">
+        <v>742</v>
+      </c>
+      <c r="C16" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>t24</t>
+        </is>
+      </c>
+      <c r="E16" s="14" t="n">
+        <v>1535665.81</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:35:15+08:00</t>
+        </is>
+      </c>
+      <c r="B17" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="C17" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>tigagroup20</t>
+        </is>
+      </c>
+      <c r="E17" s="18" t="n">
+        <v>1535261.03</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:35:15+08:00</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="n">
+        <v>742</v>
+      </c>
+      <c r="C18" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>666666</t>
+        </is>
+      </c>
+      <c r="E18" s="14" t="n">
+        <v>1485068.63</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:35:15+08:00</t>
+        </is>
+      </c>
+      <c r="B19" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="C19" s="15" t="n">
+        <v>18</v>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>jit</t>
+        </is>
+      </c>
+      <c r="E19" s="18" t="n">
+        <v>1420233.28</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:35:15+08:00</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="n">
+        <v>742</v>
+      </c>
+      <c r="C20" s="10" t="n">
+        <v>19</v>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>deepsleep</t>
+        </is>
+      </c>
+      <c r="E20" s="14" t="n">
+        <v>1405418.28</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:35:15+08:00</t>
+        </is>
+      </c>
+      <c r="B21" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="C21" s="15" t="n">
+        <v>20</v>
+      </c>
+      <c r="D21" s="16" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E21" s="18" t="n">
+        <v>1351291.41</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:35:15+08:00</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="n">
+        <v>742</v>
+      </c>
+      <c r="C22" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="D22" s="11" t="inlineStr">
+        <is>
+          <t>aaachemicalseller</t>
+        </is>
+      </c>
+      <c r="E22" s="14" t="n">
+        <v>1351219.53</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:35:15+08:00</t>
+        </is>
+      </c>
+      <c r="B23" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="C23" s="15" t="n">
+        <v>22</v>
+      </c>
+      <c r="D23" s="16" t="inlineStr">
+        <is>
+          <t>cleveregg</t>
+        </is>
+      </c>
+      <c r="E23" s="18" t="n">
+        <v>1334488.78</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:35:15+08:00</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="n">
+        <v>742</v>
+      </c>
+      <c r="C24" s="10" t="n">
+        <v>23</v>
+      </c>
+      <c r="D24" s="11" t="inlineStr">
+        <is>
+          <t>newgroup18</t>
+        </is>
+      </c>
+      <c r="E24" s="14" t="n">
+        <v>1245480.84</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:35:15+08:00</t>
+        </is>
+      </c>
+      <c r="B25" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="C25" s="15" t="n">
+        <v>24</v>
+      </c>
+      <c r="D25" s="16" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E25" s="18" t="n">
+        <v>1136937.33</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:35:15+08:00</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="n">
+        <v>742</v>
+      </c>
+      <c r="C26" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="D26" s="11" t="inlineStr">
+        <is>
+          <t>group12</t>
+        </is>
+      </c>
+      <c r="E26" s="14" t="n">
+        <v>1134818.79</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:35:15+08:00</t>
+        </is>
+      </c>
+      <c r="B27" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="C27" s="15" t="n">
+        <v>26</v>
+      </c>
+      <c r="D27" s="16" t="inlineStr">
+        <is>
+          <t>vivo50</t>
+        </is>
+      </c>
+      <c r="E27" s="18" t="n">
+        <v>1134292.56</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:35:15+08:00</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="n">
+        <v>742</v>
+      </c>
+      <c r="C28" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="D28" s="11" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="E28" s="14" t="n">
+        <v>854066.39</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1005,7 +1739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S248"/>
+  <dimension ref="A1:S249"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -16687,8 +17421,69 @@
         <v>15950</v>
       </c>
     </row>
+    <row r="249">
+      <c r="A249" s="15" t="n">
+        <v>248</v>
+      </c>
+      <c r="B249" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="C249" s="15" t="n">
+        <v>744</v>
+      </c>
+      <c r="D249" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E249" s="16" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="F249" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G249" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="H249" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I249" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="J249" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K249" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="L249" s="18" t="n">
+        <v>1635866.18</v>
+      </c>
+      <c r="M249" s="18" t="n">
+        <v>1635866.18</v>
+      </c>
+      <c r="N249" s="16" t="n"/>
+      <c r="O249" s="17" t="n">
+        <v>326</v>
+      </c>
+      <c r="P249" s="17" t="n">
+        <v>326</v>
+      </c>
+      <c r="Q249" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="R249" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="S249" s="18" t="n">
+        <v>15950</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S248"/>
+  <autoFilter ref="A1:S249"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -16699,7 +17494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N742"/>
+  <dimension ref="A1:N743"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -50876,8 +51671,54 @@
         <v>2900</v>
       </c>
     </row>
+    <row r="743">
+      <c r="A743" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="B743" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C743" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="D743" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E743" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="F743" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G743" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="H743" s="18" t="n">
+        <v>1635866.18</v>
+      </c>
+      <c r="I743" s="17" t="n">
+        <v>326</v>
+      </c>
+      <c r="J743" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K743" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L743" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M743" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N743" s="18" t="n">
+        <v>15950</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N742"/>
+  <autoFilter ref="A1:N743"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -50888,7 +51729,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -51101,7 +51942,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -51121,7 +51962,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
         <is>
@@ -51196,8 +52036,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
@@ -51205,7 +52043,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="9" t="inlineStr">
         <is>
@@ -51276,7 +52113,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -51399,8 +52236,32 @@
         <v>3600</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="23" t="n">
+        <v>730.66</v>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E5" s="16" t="inlineStr"/>
+      <c r="F5" s="17" t="n">
+        <v>40</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F4"/>
+  <autoFilter ref="A1:F5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -51411,7 +52272,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -51791,4 +52652,539 @@
   <autoFilter ref="A1:C28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:U2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>抓取时间</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="inlineStr">
+        <is>
+          <t>游戏日</t>
+        </is>
+      </c>
+      <c r="C1" s="9" t="inlineStr">
+        <is>
+          <t>现金</t>
+        </is>
+      </c>
+      <c r="D1" s="9" t="inlineStr">
+        <is>
+          <t>排名</t>
+        </is>
+      </c>
+      <c r="E1" s="9" t="inlineStr">
+        <is>
+          <t>队伍数</t>
+        </is>
+      </c>
+      <c r="F1" s="9" t="inlineStr">
+        <is>
+          <t>领先队伍</t>
+        </is>
+      </c>
+      <c r="G1" s="9" t="inlineStr">
+        <is>
+          <t>距第一名差额</t>
+        </is>
+      </c>
+      <c r="H1" s="9" t="inlineStr">
+        <is>
+          <t>当前产能</t>
+        </is>
+      </c>
+      <c r="I1" s="9" t="inlineStr">
+        <is>
+          <t>计划产能</t>
+        </is>
+      </c>
+      <c r="J1" s="9" t="inlineStr">
+        <is>
+          <t>运输方式</t>
+        </is>
+      </c>
+      <c r="K1" s="9" t="inlineStr">
+        <is>
+          <t>订货点</t>
+        </is>
+      </c>
+      <c r="L1" s="9" t="inlineStr">
+        <is>
+          <t>批量</t>
+        </is>
+      </c>
+      <c r="M1" s="9" t="inlineStr">
+        <is>
+          <t>仓库库存</t>
+        </is>
+      </c>
+      <c r="N1" s="9" t="inlineStr">
+        <is>
+          <t>在途</t>
+        </is>
+      </c>
+      <c r="O1" s="9" t="inlineStr">
+        <is>
+          <t>WIP</t>
+        </is>
+      </c>
+      <c r="P1" s="9" t="inlineStr">
+        <is>
+          <t>当前周期</t>
+        </is>
+      </c>
+      <c r="Q1" s="9" t="inlineStr">
+        <is>
+          <t>周期需求</t>
+        </is>
+      </c>
+      <c r="R1" s="9" t="inlineStr">
+        <is>
+          <t>周期缺货</t>
+        </is>
+      </c>
+      <c r="S1" s="9" t="inlineStr">
+        <is>
+          <t>周期交付</t>
+        </is>
+      </c>
+      <c r="T1" s="9" t="inlineStr">
+        <is>
+          <t>周期服务水平</t>
+        </is>
+      </c>
+      <c r="U1" s="9" t="inlineStr">
+        <is>
+          <t>周期现金变动</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:35:15+08:00</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="n">
+        <v>742</v>
+      </c>
+      <c r="C2" s="14" t="n">
+        <v>1635866.18</v>
+      </c>
+      <c r="D2" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="E2" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="F2" s="11" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="G2" s="14" t="n">
+        <v>1219918.86</v>
+      </c>
+      <c r="H2" s="21" t="n">
+        <v>20</v>
+      </c>
+      <c r="I2" s="21" t="n">
+        <v>40</v>
+      </c>
+      <c r="J2" s="11" t="inlineStr">
+        <is>
+          <t>truck</t>
+        </is>
+      </c>
+      <c r="K2" s="22" t="n">
+        <v>3600</v>
+      </c>
+      <c r="L2" s="22" t="n">
+        <v>200</v>
+      </c>
+      <c r="M2" s="12" t="n">
+        <v>326</v>
+      </c>
+      <c r="N2" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="P2" s="10" t="n">
+        <v>248</v>
+      </c>
+      <c r="Q2" s="12" t="n">
+        <v>11</v>
+      </c>
+      <c r="R2" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" s="12" t="n">
+        <v>11</v>
+      </c>
+      <c r="T2" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="U2" s="11" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:U2"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>抓取时间</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="inlineStr">
+        <is>
+          <t>游戏日</t>
+        </is>
+      </c>
+      <c r="C1" s="9" t="inlineStr">
+        <is>
+          <t>项目</t>
+        </is>
+      </c>
+      <c r="D1" s="9" t="inlineStr">
+        <is>
+          <t>金额</t>
+        </is>
+      </c>
+      <c r="E1" s="9" t="inlineStr">
+        <is>
+          <t>类型</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:35:15+08:00</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="n">
+        <v>742</v>
+      </c>
+      <c r="C2" s="11" t="inlineStr">
+        <is>
+          <t>Starting Cash</t>
+        </is>
+      </c>
+      <c r="D2" s="14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E2" s="11" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:35:15+08:00</t>
+        </is>
+      </c>
+      <c r="B3" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="C3" s="16" t="inlineStr">
+        <is>
+          <t>Cash Sources</t>
+        </is>
+      </c>
+      <c r="D3" s="16" t="n"/>
+      <c r="E3" s="16" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:35:15+08:00</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="n">
+        <v>742</v>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>revenues</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="n">
+        <v>18884800</v>
+      </c>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:35:15+08:00</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D5" s="18" t="n">
+        <v>278476.12</v>
+      </c>
+      <c r="E5" s="16" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:35:15+08:00</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="n">
+        <v>742</v>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>Cash Uses</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="n"/>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:35:15+08:00</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>outbound shipping</t>
+        </is>
+      </c>
+      <c r="D7" s="18" t="n">
+        <v>-1953600</v>
+      </c>
+      <c r="E7" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:35:15+08:00</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="n">
+        <v>742</v>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>inbound shipping</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="n">
+        <v>-1350000</v>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:35:15+08:00</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>FGI holding</t>
+        </is>
+      </c>
+      <c r="D9" s="18" t="n">
+        <v>-13207.2</v>
+      </c>
+      <c r="E9" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:35:15+08:00</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="n">
+        <v>742</v>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>add capacity</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="n">
+        <v>-1000000</v>
+      </c>
+      <c r="E10" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:35:15+08:00</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Pipeline inventory holding</t>
+        </is>
+      </c>
+      <c r="D11" s="18" t="n">
+        <v>-25602.74</v>
+      </c>
+      <c r="E11" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:35:15+08:00</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="n">
+        <v>742</v>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>production</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="n">
+        <v>-13685000</v>
+      </c>
+      <c r="E12" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:35:15+08:00</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Cash Balance</t>
+        </is>
+      </c>
+      <c r="D13" s="18" t="n">
+        <v>1635866.18</v>
+      </c>
+      <c r="E13" s="16" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E13"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update game data: day 742, cash 1638466.18, 3-day period 248
</commit_message>
<xml_diff>
--- a/data/supply_chain_game.xlsx
+++ b/data/supply_chain_game.xlsx
@@ -24,12 +24,12 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$743</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'资金构成_旧版'!$A$1:$C$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'运营参数_旧版'!$A$9:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'排行榜_旧版'!$A$1:$C$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$25</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'运营参数'!$A$1:$J$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$55</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -126,7 +126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -188,6 +188,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -587,7 +590,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-05T15:35:15+08:00</t>
+          <t>2026-09-05T15:41:03+08:00</t>
         </is>
       </c>
     </row>
@@ -650,7 +653,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>1635866.18</v>
+        <v>1638466.18</v>
       </c>
     </row>
     <row r="11">
@@ -967,7 +970,7 @@
         </is>
       </c>
       <c r="B44" s="4" t="n">
-        <v>11057.8436453836</v>
+        <v>11075.41867311462</v>
       </c>
     </row>
     <row r="45"/>
@@ -1123,7 +1126,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -1727,8 +1730,575 @@
         <v>854066.39</v>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B29" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="C29" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" s="16" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="E29" s="18" t="n">
+        <v>2858385.04</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="n">
+        <v>742</v>
+      </c>
+      <c r="C30" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D30" s="11" t="inlineStr">
+        <is>
+          <t>montesquieu</t>
+        </is>
+      </c>
+      <c r="E30" s="14" t="n">
+        <v>1889419</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B31" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="C31" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D31" s="16" t="inlineStr">
+        <is>
+          <t>nicetry</t>
+        </is>
+      </c>
+      <c r="E31" s="18" t="n">
+        <v>1889396.78</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B32" s="10" t="n">
+        <v>742</v>
+      </c>
+      <c r="C32" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D32" s="11" t="inlineStr">
+        <is>
+          <t>group7</t>
+        </is>
+      </c>
+      <c r="E32" s="14" t="n">
+        <v>1855442.25</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B33" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="C33" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="D33" s="16" t="inlineStr">
+        <is>
+          <t>group14</t>
+        </is>
+      </c>
+      <c r="E33" s="18" t="n">
+        <v>1855325.6</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B34" s="10" t="n">
+        <v>742</v>
+      </c>
+      <c r="C34" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="D34" s="11" t="inlineStr">
+        <is>
+          <t>group15</t>
+        </is>
+      </c>
+      <c r="E34" s="14" t="n">
+        <v>1855307.95</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B35" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="C35" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="D35" s="16" t="inlineStr">
+        <is>
+          <t>group8</t>
+        </is>
+      </c>
+      <c r="E35" s="18" t="n">
+        <v>1638740.95</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B36" s="10" t="n">
+        <v>742</v>
+      </c>
+      <c r="C36" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="D36" s="11" t="inlineStr">
+        <is>
+          <t>group2</t>
+        </is>
+      </c>
+      <c r="E36" s="14" t="n">
+        <v>1638468.62</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B37" s="24" t="n">
+        <v>742</v>
+      </c>
+      <c r="C37" s="24" t="n">
+        <v>9</v>
+      </c>
+      <c r="D37" s="25" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="E37" s="26" t="n">
+        <v>1638466.18</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B38" s="10" t="n">
+        <v>742</v>
+      </c>
+      <c r="C38" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="D38" s="11" t="inlineStr">
+        <is>
+          <t>teamhlly</t>
+        </is>
+      </c>
+      <c r="E38" s="14" t="n">
+        <v>1638326.76</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B39" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="C39" s="15" t="n">
+        <v>11</v>
+      </c>
+      <c r="D39" s="16" t="inlineStr">
+        <is>
+          <t>group9</t>
+        </is>
+      </c>
+      <c r="E39" s="18" t="n">
+        <v>1638322.97</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B40" s="10" t="n">
+        <v>742</v>
+      </c>
+      <c r="C40" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="D40" s="11" t="inlineStr">
+        <is>
+          <t>group25</t>
+        </is>
+      </c>
+      <c r="E40" s="14" t="n">
+        <v>1638314.78</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B41" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="C41" s="15" t="n">
+        <v>13</v>
+      </c>
+      <c r="D41" s="16" t="inlineStr">
+        <is>
+          <t>group11</t>
+        </is>
+      </c>
+      <c r="E41" s="18" t="n">
+        <v>1638302.8</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B42" s="10" t="n">
+        <v>742</v>
+      </c>
+      <c r="C42" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="D42" s="11" t="inlineStr">
+        <is>
+          <t>88888888</t>
+        </is>
+      </c>
+      <c r="E42" s="14" t="n">
+        <v>1638280.73</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B43" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="C43" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="D43" s="16" t="inlineStr">
+        <is>
+          <t>t24</t>
+        </is>
+      </c>
+      <c r="E43" s="18" t="n">
+        <v>1538265.81</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B44" s="10" t="n">
+        <v>742</v>
+      </c>
+      <c r="C44" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="D44" s="11" t="inlineStr">
+        <is>
+          <t>tigagroup20</t>
+        </is>
+      </c>
+      <c r="E44" s="14" t="n">
+        <v>1537861.03</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B45" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="C45" s="15" t="n">
+        <v>17</v>
+      </c>
+      <c r="D45" s="16" t="inlineStr">
+        <is>
+          <t>666666</t>
+        </is>
+      </c>
+      <c r="E45" s="18" t="n">
+        <v>1487668.63</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B46" s="10" t="n">
+        <v>742</v>
+      </c>
+      <c r="C46" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="D46" s="11" t="inlineStr">
+        <is>
+          <t>jit</t>
+        </is>
+      </c>
+      <c r="E46" s="14" t="n">
+        <v>1422833.28</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B47" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="C47" s="15" t="n">
+        <v>19</v>
+      </c>
+      <c r="D47" s="16" t="inlineStr">
+        <is>
+          <t>deepsleep</t>
+        </is>
+      </c>
+      <c r="E47" s="18" t="n">
+        <v>1408018.28</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B48" s="10" t="n">
+        <v>742</v>
+      </c>
+      <c r="C48" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="D48" s="11" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E48" s="14" t="n">
+        <v>1353891.41</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B49" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="C49" s="15" t="n">
+        <v>21</v>
+      </c>
+      <c r="D49" s="16" t="inlineStr">
+        <is>
+          <t>aaachemicalseller</t>
+        </is>
+      </c>
+      <c r="E49" s="18" t="n">
+        <v>1353819.53</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B50" s="10" t="n">
+        <v>742</v>
+      </c>
+      <c r="C50" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="D50" s="11" t="inlineStr">
+        <is>
+          <t>cleveregg</t>
+        </is>
+      </c>
+      <c r="E50" s="14" t="n">
+        <v>1337088.78</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B51" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="C51" s="15" t="n">
+        <v>23</v>
+      </c>
+      <c r="D51" s="16" t="inlineStr">
+        <is>
+          <t>newgroup18</t>
+        </is>
+      </c>
+      <c r="E51" s="18" t="n">
+        <v>1248080.84</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B52" s="10" t="n">
+        <v>742</v>
+      </c>
+      <c r="C52" s="10" t="n">
+        <v>24</v>
+      </c>
+      <c r="D52" s="11" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E52" s="14" t="n">
+        <v>1139537.33</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B53" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="C53" s="15" t="n">
+        <v>25</v>
+      </c>
+      <c r="D53" s="16" t="inlineStr">
+        <is>
+          <t>group12</t>
+        </is>
+      </c>
+      <c r="E53" s="18" t="n">
+        <v>1137418.79</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B54" s="10" t="n">
+        <v>742</v>
+      </c>
+      <c r="C54" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="D54" s="11" t="inlineStr">
+        <is>
+          <t>vivo50</t>
+        </is>
+      </c>
+      <c r="E54" s="14" t="n">
+        <v>1136892.56</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B55" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="C55" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="D55" s="16" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="E55" s="18" t="n">
+        <v>856666.39</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E28"/>
+  <autoFilter ref="A1:E55"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17460,10 +18030,10 @@
         <v>11</v>
       </c>
       <c r="L249" s="18" t="n">
-        <v>1635866.18</v>
+        <v>1638466.18</v>
       </c>
       <c r="M249" s="18" t="n">
-        <v>1635866.18</v>
+        <v>1638466.18</v>
       </c>
       <c r="N249" s="16" t="n"/>
       <c r="O249" s="17" t="n">
@@ -51696,7 +52266,7 @@
         <v>11</v>
       </c>
       <c r="H743" s="18" t="n">
-        <v>1635866.18</v>
+        <v>1638466.18</v>
       </c>
       <c r="I743" s="17" t="n">
         <v>326</v>
@@ -51729,7 +52299,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -51942,7 +52512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -52113,7 +52683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -52260,8 +52830,32 @@
         <v>40</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="21" t="n">
+        <v>730.66</v>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="inlineStr"/>
+      <c r="F6" s="12" t="n">
+        <v>40</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F5"/>
+  <autoFilter ref="A1:F6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -52272,7 +52866,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -52660,7 +53254,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U2"/>
+  <dimension ref="A1:U3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -52862,8 +53456,77 @@
       </c>
       <c r="U2" s="11" t="n"/>
     </row>
+    <row r="3">
+      <c r="A3" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B3" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="C3" s="18" t="n">
+        <v>1638466.18</v>
+      </c>
+      <c r="D3" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="E3" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="F3" s="16" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="G3" s="18" t="n">
+        <v>1219918.86</v>
+      </c>
+      <c r="H3" s="23" t="n">
+        <v>20</v>
+      </c>
+      <c r="I3" s="23" t="n">
+        <v>40</v>
+      </c>
+      <c r="J3" s="16" t="inlineStr">
+        <is>
+          <t>truck</t>
+        </is>
+      </c>
+      <c r="K3" s="27" t="n">
+        <v>3600</v>
+      </c>
+      <c r="L3" s="27" t="n">
+        <v>200</v>
+      </c>
+      <c r="M3" s="17" t="n">
+        <v>326</v>
+      </c>
+      <c r="N3" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="P3" s="15" t="n">
+        <v>248</v>
+      </c>
+      <c r="Q3" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="R3" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="T3" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="U3" s="16" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U2"/>
+  <autoFilter ref="A1:U3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -52874,7 +53537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -53183,8 +53846,280 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="n">
+        <v>742</v>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>Starting Cash</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E14" s="11" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B15" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>Cash Sources</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="n"/>
+      <c r="E15" s="16" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="n">
+        <v>742</v>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>revenues</t>
+        </is>
+      </c>
+      <c r="D16" s="14" t="n">
+        <v>18887700</v>
+      </c>
+      <c r="E16" s="11" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B17" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D17" s="18" t="n">
+        <v>278476.12</v>
+      </c>
+      <c r="E17" s="16" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="n">
+        <v>742</v>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>Cash Uses</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="n"/>
+      <c r="E18" s="11" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B19" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>outbound shipping</t>
+        </is>
+      </c>
+      <c r="D19" s="18" t="n">
+        <v>-1953900</v>
+      </c>
+      <c r="E19" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="n">
+        <v>742</v>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>inbound shipping</t>
+        </is>
+      </c>
+      <c r="D20" s="14" t="n">
+        <v>-1350000</v>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B21" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="C21" s="16" t="inlineStr">
+        <is>
+          <t>FGI holding</t>
+        </is>
+      </c>
+      <c r="D21" s="18" t="n">
+        <v>-13207.2</v>
+      </c>
+      <c r="E21" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="n">
+        <v>742</v>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>add capacity</t>
+        </is>
+      </c>
+      <c r="D22" s="14" t="n">
+        <v>-1000000</v>
+      </c>
+      <c r="E22" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B23" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="C23" s="16" t="inlineStr">
+        <is>
+          <t>Pipeline inventory holding</t>
+        </is>
+      </c>
+      <c r="D23" s="18" t="n">
+        <v>-25602.74</v>
+      </c>
+      <c r="E23" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="n">
+        <v>742</v>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>production</t>
+        </is>
+      </c>
+      <c r="D24" s="14" t="n">
+        <v>-13685000</v>
+      </c>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B25" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="C25" s="16" t="inlineStr">
+        <is>
+          <t>Cash Balance</t>
+        </is>
+      </c>
+      <c r="D25" s="18" t="n">
+        <v>1638466.18</v>
+      </c>
+      <c r="E25" s="16" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E13"/>
+  <autoFilter ref="A1:E25"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update game data: day 743, cash 898014.63, 3-day period 248
</commit_message>
<xml_diff>
--- a/data/supply_chain_game.xlsx
+++ b/data/supply_chain_game.xlsx
@@ -21,15 +21,15 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$249</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$743</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$744</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'资金构成_旧版'!$A$1:$C$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'运营参数_旧版'!$A$9:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'排行榜_旧版'!$A$1:$C$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'运营参数'!$A$1:$J$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'运营参数'!$A$1:$J$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$82</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -590,7 +590,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-05T15:41:03+08:00</t>
+          <t>2026-09-05T15:56:03+08:00</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>742</v>
+        <v>743</v>
       </c>
     </row>
     <row r="7">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="8">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>1638466.18</v>
+        <v>898014.63</v>
       </c>
     </row>
     <row r="11">
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>9</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>1219918.86</v>
+        <v>1970127.7</v>
       </c>
     </row>
     <row r="15"/>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B19" s="6" t="n">
-        <v>40</v>
+        <v>55</v>
       </c>
     </row>
     <row r="20">
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="25">
@@ -861,7 +861,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="33">
@@ -881,7 +881,7 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="35">
@@ -901,7 +901,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="37">
@@ -909,6 +909,9 @@
         <is>
           <t>周期现金变动</t>
         </is>
+      </c>
+      <c r="B37" s="4" t="n">
+        <v>-754598.2498661376</v>
       </c>
     </row>
     <row r="38"/>
@@ -970,7 +973,7 @@
         </is>
       </c>
       <c r="B44" s="4" t="n">
-        <v>11075.41867311462</v>
+        <v>11171.04507405777</v>
       </c>
     </row>
     <row r="45"/>
@@ -1005,7 +1008,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1114,8 +1117,50 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B3" s="15" t="n">
+        <v>743</v>
+      </c>
+      <c r="C3" s="16" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="D3" s="23" t="n">
+        <v>20</v>
+      </c>
+      <c r="E3" s="23" t="n">
+        <v>55</v>
+      </c>
+      <c r="F3" s="16" t="inlineStr">
+        <is>
+          <t>truck</t>
+        </is>
+      </c>
+      <c r="G3" s="27" t="n">
+        <v>3600</v>
+      </c>
+      <c r="H3" s="27" t="n">
+        <v>200</v>
+      </c>
+      <c r="I3" s="16" t="inlineStr">
+        <is>
+          <t>truck</t>
+        </is>
+      </c>
+      <c r="J3" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J2"/>
+  <autoFilter ref="A1:J3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1126,7 +1171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -2297,8 +2342,575 @@
         <v>856666.39</v>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B56" s="10" t="n">
+        <v>743</v>
+      </c>
+      <c r="C56" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D56" s="11" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="E56" s="14" t="n">
+        <v>2868142.33</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B57" s="15" t="n">
+        <v>743</v>
+      </c>
+      <c r="C57" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D57" s="16" t="inlineStr">
+        <is>
+          <t>nicetry</t>
+        </is>
+      </c>
+      <c r="E57" s="18" t="n">
+        <v>1898901.01</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B58" s="10" t="n">
+        <v>743</v>
+      </c>
+      <c r="C58" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D58" s="11" t="inlineStr">
+        <is>
+          <t>group7</t>
+        </is>
+      </c>
+      <c r="E58" s="14" t="n">
+        <v>1864937.61</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B59" s="15" t="n">
+        <v>743</v>
+      </c>
+      <c r="C59" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D59" s="16" t="inlineStr">
+        <is>
+          <t>group15</t>
+        </is>
+      </c>
+      <c r="E59" s="18" t="n">
+        <v>1864803.28</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B60" s="10" t="n">
+        <v>743</v>
+      </c>
+      <c r="C60" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="D60" s="11" t="inlineStr">
+        <is>
+          <t>montesquieu</t>
+        </is>
+      </c>
+      <c r="E60" s="14" t="n">
+        <v>1682423.24</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B61" s="15" t="n">
+        <v>743</v>
+      </c>
+      <c r="C61" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="D61" s="16" t="inlineStr">
+        <is>
+          <t>group14</t>
+        </is>
+      </c>
+      <c r="E61" s="18" t="n">
+        <v>1648320.94</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B62" s="10" t="n">
+        <v>743</v>
+      </c>
+      <c r="C62" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="D62" s="11" t="inlineStr">
+        <is>
+          <t>t24</t>
+        </is>
+      </c>
+      <c r="E62" s="14" t="n">
+        <v>1547678.34</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B63" s="15" t="n">
+        <v>743</v>
+      </c>
+      <c r="C63" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="D63" s="16" t="inlineStr">
+        <is>
+          <t>jit</t>
+        </is>
+      </c>
+      <c r="E63" s="18" t="n">
+        <v>1432215.67</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B64" s="10" t="n">
+        <v>743</v>
+      </c>
+      <c r="C64" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="D64" s="11" t="inlineStr">
+        <is>
+          <t>group8</t>
+        </is>
+      </c>
+      <c r="E64" s="14" t="n">
+        <v>1431679.72</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B65" s="15" t="n">
+        <v>743</v>
+      </c>
+      <c r="C65" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="D65" s="16" t="inlineStr">
+        <is>
+          <t>group2</t>
+        </is>
+      </c>
+      <c r="E65" s="18" t="n">
+        <v>1431407.32</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B66" s="10" t="n">
+        <v>743</v>
+      </c>
+      <c r="C66" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="D66" s="11" t="inlineStr">
+        <is>
+          <t>teamhlly</t>
+        </is>
+      </c>
+      <c r="E66" s="14" t="n">
+        <v>1431265.42</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B67" s="15" t="n">
+        <v>743</v>
+      </c>
+      <c r="C67" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="D67" s="16" t="inlineStr">
+        <is>
+          <t>group9</t>
+        </is>
+      </c>
+      <c r="E67" s="18" t="n">
+        <v>1431261.64</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B68" s="10" t="n">
+        <v>743</v>
+      </c>
+      <c r="C68" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="D68" s="11" t="inlineStr">
+        <is>
+          <t>group25</t>
+        </is>
+      </c>
+      <c r="E68" s="14" t="n">
+        <v>1431253.44</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B69" s="15" t="n">
+        <v>743</v>
+      </c>
+      <c r="C69" s="15" t="n">
+        <v>14</v>
+      </c>
+      <c r="D69" s="16" t="inlineStr">
+        <is>
+          <t>group11</t>
+        </is>
+      </c>
+      <c r="E69" s="18" t="n">
+        <v>1431241.45</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B70" s="10" t="n">
+        <v>743</v>
+      </c>
+      <c r="C70" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="D70" s="11" t="inlineStr">
+        <is>
+          <t>88888888</t>
+        </is>
+      </c>
+      <c r="E70" s="14" t="n">
+        <v>1431219.38</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B71" s="15" t="n">
+        <v>743</v>
+      </c>
+      <c r="C71" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="D71" s="16" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E71" s="18" t="n">
+        <v>1363255.79</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B72" s="10" t="n">
+        <v>743</v>
+      </c>
+      <c r="C72" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="D72" s="11" t="inlineStr">
+        <is>
+          <t>aaachemicalseller</t>
+        </is>
+      </c>
+      <c r="E72" s="14" t="n">
+        <v>1363183.89</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B73" s="15" t="n">
+        <v>743</v>
+      </c>
+      <c r="C73" s="15" t="n">
+        <v>18</v>
+      </c>
+      <c r="D73" s="16" t="inlineStr">
+        <is>
+          <t>tigagroup20</t>
+        </is>
+      </c>
+      <c r="E73" s="18" t="n">
+        <v>1330773.45</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B74" s="10" t="n">
+        <v>743</v>
+      </c>
+      <c r="C74" s="10" t="n">
+        <v>19</v>
+      </c>
+      <c r="D74" s="11" t="inlineStr">
+        <is>
+          <t>666666</t>
+        </is>
+      </c>
+      <c r="E74" s="14" t="n">
+        <v>1280567.95</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B75" s="15" t="n">
+        <v>743</v>
+      </c>
+      <c r="C75" s="15" t="n">
+        <v>20</v>
+      </c>
+      <c r="D75" s="16" t="inlineStr">
+        <is>
+          <t>newgroup18</t>
+        </is>
+      </c>
+      <c r="E75" s="18" t="n">
+        <v>1257384.71</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B76" s="10" t="n">
+        <v>743</v>
+      </c>
+      <c r="C76" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="D76" s="11" t="inlineStr">
+        <is>
+          <t>deepsleep</t>
+        </is>
+      </c>
+      <c r="E76" s="14" t="n">
+        <v>1220853.37</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B77" s="15" t="n">
+        <v>743</v>
+      </c>
+      <c r="C77" s="15" t="n">
+        <v>22</v>
+      </c>
+      <c r="D77" s="16" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E77" s="18" t="n">
+        <v>1148845.73</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B78" s="10" t="n">
+        <v>743</v>
+      </c>
+      <c r="C78" s="10" t="n">
+        <v>23</v>
+      </c>
+      <c r="D78" s="11" t="inlineStr">
+        <is>
+          <t>group12</t>
+        </is>
+      </c>
+      <c r="E78" s="14" t="n">
+        <v>1146726.64</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B79" s="15" t="n">
+        <v>743</v>
+      </c>
+      <c r="C79" s="15" t="n">
+        <v>24</v>
+      </c>
+      <c r="D79" s="16" t="inlineStr">
+        <is>
+          <t>cleveregg</t>
+        </is>
+      </c>
+      <c r="E79" s="18" t="n">
+        <v>1129948.77</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B80" s="10" t="n">
+        <v>743</v>
+      </c>
+      <c r="C80" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="D80" s="11" t="inlineStr">
+        <is>
+          <t>vivo50</t>
+        </is>
+      </c>
+      <c r="E80" s="14" t="n">
+        <v>929700.27</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B81" s="24" t="n">
+        <v>743</v>
+      </c>
+      <c r="C81" s="24" t="n">
+        <v>26</v>
+      </c>
+      <c r="D81" s="25" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="E81" s="26" t="n">
+        <v>898014.63</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B82" s="10" t="n">
+        <v>743</v>
+      </c>
+      <c r="C82" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="D82" s="11" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="E82" s="14" t="n">
+        <v>865900.92</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E55"/>
+  <autoFilter ref="A1:E82"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -18002,7 +18614,7 @@
         <v>744</v>
       </c>
       <c r="D249" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E249" s="16" t="inlineStr">
         <is>
@@ -18015,32 +18627,34 @@
         </is>
       </c>
       <c r="G249" s="17" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H249" s="17" t="n">
         <v>0</v>
       </c>
       <c r="I249" s="17" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="J249" s="19" t="n">
         <v>1</v>
       </c>
       <c r="K249" s="17" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="L249" s="18" t="n">
-        <v>1638466.18</v>
+        <v>1652612.879866138</v>
       </c>
       <c r="M249" s="18" t="n">
-        <v>1638466.18</v>
-      </c>
-      <c r="N249" s="16" t="n"/>
+        <v>898014.63</v>
+      </c>
+      <c r="N249" s="18" t="n">
+        <v>-754598.2498661376</v>
+      </c>
       <c r="O249" s="17" t="n">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="P249" s="17" t="n">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="Q249" s="17" t="n">
         <v>0</v>
@@ -18049,7 +18663,7 @@
         <v>200</v>
       </c>
       <c r="S249" s="18" t="n">
-        <v>15950</v>
+        <v>18850</v>
       </c>
     </row>
   </sheetData>
@@ -18064,7 +18678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N743"/>
+  <dimension ref="A1:N744"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -52287,8 +52901,54 @@
         <v>15950</v>
       </c>
     </row>
+    <row r="744">
+      <c r="A744" s="10" t="n">
+        <v>743</v>
+      </c>
+      <c r="B744" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C744" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D744" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E744" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="F744" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G744" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="H744" s="14" t="n">
+        <v>898014.63</v>
+      </c>
+      <c r="I744" s="12" t="n">
+        <v>324</v>
+      </c>
+      <c r="J744" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K744" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L744" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M744" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N744" s="14" t="n">
+        <v>2900</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N743"/>
+  <autoFilter ref="A1:N744"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -52683,7 +53343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -52854,8 +53514,56 @@
         <v>40</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="23" t="n">
+        <v>730.66</v>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E7" s="16" t="inlineStr"/>
+      <c r="F7" s="17" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="21" t="n">
+        <v>742.75</v>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr"/>
+      <c r="F8" s="12" t="n">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F6"/>
+  <autoFilter ref="A1:F8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -53254,7 +53962,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U3"/>
+  <dimension ref="A1:U4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -53263,7 +53971,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
@@ -53277,7 +53985,7 @@
     <col width="12" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="12" customWidth="1" min="20" max="20"/>
-    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="20" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -53525,8 +54233,79 @@
       </c>
       <c r="U3" s="16" t="n"/>
     </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="n">
+        <v>743</v>
+      </c>
+      <c r="C4" s="14" t="n">
+        <v>898014.63</v>
+      </c>
+      <c r="D4" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="E4" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="F4" s="11" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="G4" s="14" t="n">
+        <v>1970127.7</v>
+      </c>
+      <c r="H4" s="21" t="n">
+        <v>20</v>
+      </c>
+      <c r="I4" s="21" t="n">
+        <v>55</v>
+      </c>
+      <c r="J4" s="11" t="inlineStr">
+        <is>
+          <t>truck</t>
+        </is>
+      </c>
+      <c r="K4" s="22" t="n">
+        <v>3600</v>
+      </c>
+      <c r="L4" s="22" t="n">
+        <v>200</v>
+      </c>
+      <c r="M4" s="12" t="n">
+        <v>324</v>
+      </c>
+      <c r="N4" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="P4" s="10" t="n">
+        <v>248</v>
+      </c>
+      <c r="Q4" s="12" t="n">
+        <v>13</v>
+      </c>
+      <c r="R4" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" s="12" t="n">
+        <v>13</v>
+      </c>
+      <c r="T4" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="U4" s="14" t="n">
+        <v>-754598.2498661376</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U3"/>
+  <autoFilter ref="A1:U4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -53537,7 +54316,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -54118,8 +54897,280 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="n">
+        <v>743</v>
+      </c>
+      <c r="C26" s="11" t="inlineStr">
+        <is>
+          <t>Starting Cash</t>
+        </is>
+      </c>
+      <c r="D26" s="14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E26" s="11" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B27" s="15" t="n">
+        <v>743</v>
+      </c>
+      <c r="C27" s="16" t="inlineStr">
+        <is>
+          <t>Cash Sources</t>
+        </is>
+      </c>
+      <c r="D27" s="16" t="n"/>
+      <c r="E27" s="16" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="n">
+        <v>743</v>
+      </c>
+      <c r="C28" s="11" t="inlineStr">
+        <is>
+          <t>revenues</t>
+        </is>
+      </c>
+      <c r="D28" s="14" t="n">
+        <v>18897850</v>
+      </c>
+      <c r="E28" s="11" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B29" s="15" t="n">
+        <v>743</v>
+      </c>
+      <c r="C29" s="16" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D29" s="18" t="n">
+        <v>278854.39</v>
+      </c>
+      <c r="E29" s="16" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="n">
+        <v>743</v>
+      </c>
+      <c r="C30" s="11" t="inlineStr">
+        <is>
+          <t>Cash Uses</t>
+        </is>
+      </c>
+      <c r="D30" s="11" t="n"/>
+      <c r="E30" s="11" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B31" s="15" t="n">
+        <v>743</v>
+      </c>
+      <c r="C31" s="16" t="inlineStr">
+        <is>
+          <t>outbound shipping</t>
+        </is>
+      </c>
+      <c r="D31" s="18" t="n">
+        <v>-1954950</v>
+      </c>
+      <c r="E31" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B32" s="10" t="n">
+        <v>743</v>
+      </c>
+      <c r="C32" s="11" t="inlineStr">
+        <is>
+          <t>inbound shipping</t>
+        </is>
+      </c>
+      <c r="D32" s="14" t="n">
+        <v>-1350000</v>
+      </c>
+      <c r="E32" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B33" s="15" t="n">
+        <v>743</v>
+      </c>
+      <c r="C33" s="16" t="inlineStr">
+        <is>
+          <t>FGI holding</t>
+        </is>
+      </c>
+      <c r="D33" s="18" t="n">
+        <v>-13296.16</v>
+      </c>
+      <c r="E33" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B34" s="10" t="n">
+        <v>743</v>
+      </c>
+      <c r="C34" s="11" t="inlineStr">
+        <is>
+          <t>add capacity</t>
+        </is>
+      </c>
+      <c r="D34" s="14" t="n">
+        <v>-1749840.87</v>
+      </c>
+      <c r="E34" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B35" s="15" t="n">
+        <v>743</v>
+      </c>
+      <c r="C35" s="16" t="inlineStr">
+        <is>
+          <t>Pipeline inventory holding</t>
+        </is>
+      </c>
+      <c r="D35" s="18" t="n">
+        <v>-25602.74</v>
+      </c>
+      <c r="E35" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B36" s="10" t="n">
+        <v>743</v>
+      </c>
+      <c r="C36" s="11" t="inlineStr">
+        <is>
+          <t>production</t>
+        </is>
+      </c>
+      <c r="D36" s="14" t="n">
+        <v>-13685000</v>
+      </c>
+      <c r="E36" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B37" s="15" t="n">
+        <v>743</v>
+      </c>
+      <c r="C37" s="16" t="inlineStr">
+        <is>
+          <t>Cash Balance</t>
+        </is>
+      </c>
+      <c r="D37" s="18" t="n">
+        <v>898014.63</v>
+      </c>
+      <c r="E37" s="16" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E25"/>
+  <autoFilter ref="A1:E37"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update game data: day 744, cash 686861.82, 3-day period 248
</commit_message>
<xml_diff>
--- a/data/supply_chain_game.xlsx
+++ b/data/supply_chain_game.xlsx
@@ -21,15 +21,15 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$249</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$744</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$745</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'资金构成_旧版'!$A$1:$C$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'运营参数_旧版'!$A$9:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'排行榜_旧版'!$A$1:$C$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$49</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'运营参数'!$A$1:$J$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$109</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -590,7 +590,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-05T15:56:03+08:00</t>
+          <t>2026-09-05T16:11:03+08:00</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>743</v>
+        <v>744</v>
       </c>
     </row>
     <row r="7">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>717</v>
+        <v>716</v>
       </c>
     </row>
     <row r="8">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>898014.63</v>
+        <v>686861.8199999999</v>
       </c>
     </row>
     <row r="11">
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>1970127.7</v>
+        <v>2187142.21</v>
       </c>
     </row>
     <row r="15"/>
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>324</v>
+        <v>313</v>
       </c>
     </row>
     <row r="25">
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
     </row>
     <row r="26">
@@ -850,7 +850,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>否（进行中）</t>
+          <t>是</t>
         </is>
       </c>
     </row>
@@ -861,7 +861,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>13</v>
+        <v>24</v>
       </c>
     </row>
     <row r="33">
@@ -881,7 +881,7 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>13</v>
+        <v>24</v>
       </c>
     </row>
     <row r="35">
@@ -901,7 +901,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>13</v>
+        <v>24</v>
       </c>
     </row>
     <row r="37">
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="B37" s="4" t="n">
-        <v>-754598.2498661376</v>
+        <v>-949004.3614473605</v>
       </c>
     </row>
     <row r="38"/>
@@ -929,7 +929,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="41">
@@ -940,7 +940,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>739–741</t>
+          <t>742–744</t>
         </is>
       </c>
     </row>
@@ -952,7 +952,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>11.0 / 0.0 / 11.0</t>
+          <t>24.0 / 0.0 / 24.0</t>
         </is>
       </c>
     </row>
@@ -973,7 +973,7 @@
         </is>
       </c>
       <c r="B44" s="4" t="n">
-        <v>11171.04507405777</v>
+        <v>-949004.3614473605</v>
       </c>
     </row>
     <row r="45"/>
@@ -1171,7 +1171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E82"/>
+  <dimension ref="A1:E109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -2909,8 +2909,575 @@
         <v>865900.92</v>
       </c>
     </row>
+    <row r="83">
+      <c r="A83" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B83" s="15" t="n">
+        <v>744</v>
+      </c>
+      <c r="C83" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D83" s="16" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="E83" s="18" t="n">
+        <v>2874004.03</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B84" s="10" t="n">
+        <v>744</v>
+      </c>
+      <c r="C84" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D84" s="11" t="inlineStr">
+        <is>
+          <t>nicetry</t>
+        </is>
+      </c>
+      <c r="E84" s="14" t="n">
+        <v>1904461.35</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B85" s="15" t="n">
+        <v>744</v>
+      </c>
+      <c r="C85" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D85" s="16" t="inlineStr">
+        <is>
+          <t>group7</t>
+        </is>
+      </c>
+      <c r="E85" s="18" t="n">
+        <v>1870537.33</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B86" s="10" t="n">
+        <v>744</v>
+      </c>
+      <c r="C86" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D86" s="11" t="inlineStr">
+        <is>
+          <t>group15</t>
+        </is>
+      </c>
+      <c r="E86" s="14" t="n">
+        <v>1870402.95</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B87" s="15" t="n">
+        <v>744</v>
+      </c>
+      <c r="C87" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="D87" s="16" t="inlineStr">
+        <is>
+          <t>montesquieu</t>
+        </is>
+      </c>
+      <c r="E87" s="18" t="n">
+        <v>1687933.79</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B88" s="10" t="n">
+        <v>744</v>
+      </c>
+      <c r="C88" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="D88" s="11" t="inlineStr">
+        <is>
+          <t>group14</t>
+        </is>
+      </c>
+      <c r="E88" s="14" t="n">
+        <v>1653872.45</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B89" s="15" t="n">
+        <v>744</v>
+      </c>
+      <c r="C89" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="D89" s="16" t="inlineStr">
+        <is>
+          <t>t24</t>
+        </is>
+      </c>
+      <c r="E89" s="18" t="n">
+        <v>1553195.2</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B90" s="10" t="n">
+        <v>744</v>
+      </c>
+      <c r="C90" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="D90" s="11" t="inlineStr">
+        <is>
+          <t>jit</t>
+        </is>
+      </c>
+      <c r="E90" s="14" t="n">
+        <v>1437702.37</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B91" s="15" t="n">
+        <v>744</v>
+      </c>
+      <c r="C91" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="D91" s="16" t="inlineStr">
+        <is>
+          <t>group8</t>
+        </is>
+      </c>
+      <c r="E91" s="18" t="n">
+        <v>1437124.79</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B92" s="10" t="n">
+        <v>744</v>
+      </c>
+      <c r="C92" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="D92" s="11" t="inlineStr">
+        <is>
+          <t>group2</t>
+        </is>
+      </c>
+      <c r="E92" s="14" t="n">
+        <v>1436852.32</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B93" s="15" t="n">
+        <v>744</v>
+      </c>
+      <c r="C93" s="15" t="n">
+        <v>11</v>
+      </c>
+      <c r="D93" s="16" t="inlineStr">
+        <is>
+          <t>teamhlly</t>
+        </is>
+      </c>
+      <c r="E93" s="18" t="n">
+        <v>1436710.38</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B94" s="10" t="n">
+        <v>744</v>
+      </c>
+      <c r="C94" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="D94" s="11" t="inlineStr">
+        <is>
+          <t>group9</t>
+        </is>
+      </c>
+      <c r="E94" s="14" t="n">
+        <v>1436706.59</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B95" s="15" t="n">
+        <v>744</v>
+      </c>
+      <c r="C95" s="15" t="n">
+        <v>13</v>
+      </c>
+      <c r="D95" s="16" t="inlineStr">
+        <is>
+          <t>group25</t>
+        </is>
+      </c>
+      <c r="E95" s="18" t="n">
+        <v>1436698.39</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B96" s="10" t="n">
+        <v>744</v>
+      </c>
+      <c r="C96" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="D96" s="11" t="inlineStr">
+        <is>
+          <t>group11</t>
+        </is>
+      </c>
+      <c r="E96" s="14" t="n">
+        <v>1436686.41</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B97" s="15" t="n">
+        <v>744</v>
+      </c>
+      <c r="C97" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="D97" s="16" t="inlineStr">
+        <is>
+          <t>88888888</t>
+        </is>
+      </c>
+      <c r="E97" s="18" t="n">
+        <v>1436664.33</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B98" s="10" t="n">
+        <v>744</v>
+      </c>
+      <c r="C98" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="D98" s="11" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E98" s="14" t="n">
+        <v>1368724.49</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B99" s="15" t="n">
+        <v>744</v>
+      </c>
+      <c r="C99" s="15" t="n">
+        <v>17</v>
+      </c>
+      <c r="D99" s="16" t="inlineStr">
+        <is>
+          <t>aaachemicalseller</t>
+        </is>
+      </c>
+      <c r="E99" s="18" t="n">
+        <v>1368652.57</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B100" s="10" t="n">
+        <v>744</v>
+      </c>
+      <c r="C100" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="D100" s="11" t="inlineStr">
+        <is>
+          <t>tigagroup20</t>
+        </is>
+      </c>
+      <c r="E100" s="14" t="n">
+        <v>1336192.17</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B101" s="15" t="n">
+        <v>744</v>
+      </c>
+      <c r="C101" s="15" t="n">
+        <v>19</v>
+      </c>
+      <c r="D101" s="16" t="inlineStr">
+        <is>
+          <t>666666</t>
+        </is>
+      </c>
+      <c r="E101" s="18" t="n">
+        <v>1285973.55</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B102" s="10" t="n">
+        <v>744</v>
+      </c>
+      <c r="C102" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="D102" s="11" t="inlineStr">
+        <is>
+          <t>newgroup18</t>
+        </is>
+      </c>
+      <c r="E102" s="14" t="n">
+        <v>1262792.88</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B103" s="15" t="n">
+        <v>744</v>
+      </c>
+      <c r="C103" s="15" t="n">
+        <v>21</v>
+      </c>
+      <c r="D103" s="16" t="inlineStr">
+        <is>
+          <t>deepsleep</t>
+        </is>
+      </c>
+      <c r="E103" s="18" t="n">
+        <v>1226243.16</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B104" s="10" t="n">
+        <v>744</v>
+      </c>
+      <c r="C104" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="D104" s="11" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E104" s="14" t="n">
+        <v>1154258.43</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B105" s="15" t="n">
+        <v>744</v>
+      </c>
+      <c r="C105" s="15" t="n">
+        <v>23</v>
+      </c>
+      <c r="D105" s="16" t="inlineStr">
+        <is>
+          <t>group12</t>
+        </is>
+      </c>
+      <c r="E105" s="18" t="n">
+        <v>1152138.78</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B106" s="10" t="n">
+        <v>744</v>
+      </c>
+      <c r="C106" s="10" t="n">
+        <v>24</v>
+      </c>
+      <c r="D106" s="11" t="inlineStr">
+        <is>
+          <t>cleveregg</t>
+        </is>
+      </c>
+      <c r="E106" s="14" t="n">
+        <v>1135315.04</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B107" s="15" t="n">
+        <v>744</v>
+      </c>
+      <c r="C107" s="15" t="n">
+        <v>25</v>
+      </c>
+      <c r="D107" s="16" t="inlineStr">
+        <is>
+          <t>vivo50</t>
+        </is>
+      </c>
+      <c r="E107" s="18" t="n">
+        <v>935014.24</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B108" s="10" t="n">
+        <v>744</v>
+      </c>
+      <c r="C108" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="D108" s="11" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="E108" s="14" t="n">
+        <v>871239.72</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B109" s="24" t="n">
+        <v>744</v>
+      </c>
+      <c r="C109" s="24" t="n">
+        <v>27</v>
+      </c>
+      <c r="D109" s="25" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="E109" s="26" t="n">
+        <v>686861.8199999999</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E82"/>
+  <autoFilter ref="A1:E109"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -18614,11 +19181,11 @@
         <v>744</v>
       </c>
       <c r="D249" s="15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E249" s="16" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="F249" s="16" t="inlineStr">
@@ -18627,43 +19194,43 @@
         </is>
       </c>
       <c r="G249" s="17" t="n">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="H249" s="17" t="n">
         <v>0</v>
       </c>
       <c r="I249" s="17" t="n">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="J249" s="19" t="n">
         <v>1</v>
       </c>
       <c r="K249" s="17" t="n">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="L249" s="18" t="n">
-        <v>1652612.879866138</v>
+        <v>1635866.18144736</v>
       </c>
       <c r="M249" s="18" t="n">
-        <v>898014.63</v>
+        <v>686861.8199999999</v>
       </c>
       <c r="N249" s="18" t="n">
-        <v>-754598.2498661376</v>
+        <v>-949004.3614473605</v>
       </c>
       <c r="O249" s="17" t="n">
-        <v>324</v>
+        <v>313</v>
       </c>
       <c r="P249" s="17" t="n">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="Q249" s="17" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="R249" s="17" t="n">
         <v>200</v>
       </c>
       <c r="S249" s="18" t="n">
-        <v>18850</v>
+        <v>34800</v>
       </c>
     </row>
   </sheetData>
@@ -18678,7 +19245,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N744"/>
+  <dimension ref="A1:N745"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -52947,8 +53514,54 @@
         <v>2900</v>
       </c>
     </row>
+    <row r="745">
+      <c r="A745" s="15" t="n">
+        <v>744</v>
+      </c>
+      <c r="B745" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C745" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="D745" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E745" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="F745" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G745" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="H745" s="18" t="n">
+        <v>686861.8199999999</v>
+      </c>
+      <c r="I745" s="17" t="n">
+        <v>313</v>
+      </c>
+      <c r="J745" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K745" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="L745" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="M745" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N745" s="18" t="n">
+        <v>15950</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N744"/>
+  <autoFilter ref="A1:N745"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -53343,7 +53956,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -53562,8 +54175,56 @@
         <v>55</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="23" t="n">
+        <v>730.66</v>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E9" s="16" t="inlineStr"/>
+      <c r="F9" s="17" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="21" t="n">
+        <v>742.75</v>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="inlineStr"/>
+      <c r="F10" s="12" t="n">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F8"/>
+  <autoFilter ref="A1:F10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -53962,7 +54623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U4"/>
+  <dimension ref="A1:U5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -53971,7 +54632,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
@@ -54304,8 +54965,79 @@
         <v>-754598.2498661376</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="n">
+        <v>744</v>
+      </c>
+      <c r="C5" s="18" t="n">
+        <v>686861.8199999999</v>
+      </c>
+      <c r="D5" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="E5" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="F5" s="16" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="G5" s="18" t="n">
+        <v>2187142.21</v>
+      </c>
+      <c r="H5" s="23" t="n">
+        <v>20</v>
+      </c>
+      <c r="I5" s="23" t="n">
+        <v>55</v>
+      </c>
+      <c r="J5" s="16" t="inlineStr">
+        <is>
+          <t>truck</t>
+        </is>
+      </c>
+      <c r="K5" s="27" t="n">
+        <v>3600</v>
+      </c>
+      <c r="L5" s="27" t="n">
+        <v>200</v>
+      </c>
+      <c r="M5" s="17" t="n">
+        <v>313</v>
+      </c>
+      <c r="N5" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="O5" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="P5" s="15" t="n">
+        <v>248</v>
+      </c>
+      <c r="Q5" s="17" t="n">
+        <v>24</v>
+      </c>
+      <c r="R5" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" s="17" t="n">
+        <v>24</v>
+      </c>
+      <c r="T5" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="U5" s="18" t="n">
+        <v>-949004.3614473605</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U4"/>
+  <autoFilter ref="A1:U5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -54316,7 +55048,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -55169,8 +55901,280 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B38" s="10" t="n">
+        <v>744</v>
+      </c>
+      <c r="C38" s="11" t="inlineStr">
+        <is>
+          <t>Starting Cash</t>
+        </is>
+      </c>
+      <c r="D38" s="14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E38" s="11" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B39" s="15" t="n">
+        <v>744</v>
+      </c>
+      <c r="C39" s="16" t="inlineStr">
+        <is>
+          <t>Cash Sources</t>
+        </is>
+      </c>
+      <c r="D39" s="16" t="n"/>
+      <c r="E39" s="16" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B40" s="10" t="n">
+        <v>744</v>
+      </c>
+      <c r="C40" s="11" t="inlineStr">
+        <is>
+          <t>revenues</t>
+        </is>
+      </c>
+      <c r="D40" s="14" t="n">
+        <v>18903650</v>
+      </c>
+      <c r="E40" s="11" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B41" s="15" t="n">
+        <v>744</v>
+      </c>
+      <c r="C41" s="16" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D41" s="18" t="n">
+        <v>279088.65</v>
+      </c>
+      <c r="E41" s="16" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B42" s="10" t="n">
+        <v>744</v>
+      </c>
+      <c r="C42" s="11" t="inlineStr">
+        <is>
+          <t>Cash Uses</t>
+        </is>
+      </c>
+      <c r="D42" s="11" t="n"/>
+      <c r="E42" s="11" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B43" s="15" t="n">
+        <v>744</v>
+      </c>
+      <c r="C43" s="16" t="inlineStr">
+        <is>
+          <t>outbound shipping</t>
+        </is>
+      </c>
+      <c r="D43" s="18" t="n">
+        <v>-1955550</v>
+      </c>
+      <c r="E43" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B44" s="10" t="n">
+        <v>744</v>
+      </c>
+      <c r="C44" s="11" t="inlineStr">
+        <is>
+          <t>inbound shipping</t>
+        </is>
+      </c>
+      <c r="D44" s="14" t="n">
+        <v>-1365000</v>
+      </c>
+      <c r="E44" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B45" s="15" t="n">
+        <v>744</v>
+      </c>
+      <c r="C45" s="16" t="inlineStr">
+        <is>
+          <t>FGI holding</t>
+        </is>
+      </c>
+      <c r="D45" s="18" t="n">
+        <v>-13383.22</v>
+      </c>
+      <c r="E45" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B46" s="10" t="n">
+        <v>744</v>
+      </c>
+      <c r="C46" s="11" t="inlineStr">
+        <is>
+          <t>add capacity</t>
+        </is>
+      </c>
+      <c r="D46" s="14" t="n">
+        <v>-1749840.87</v>
+      </c>
+      <c r="E46" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B47" s="15" t="n">
+        <v>744</v>
+      </c>
+      <c r="C47" s="16" t="inlineStr">
+        <is>
+          <t>Pipeline inventory holding</t>
+        </is>
+      </c>
+      <c r="D47" s="18" t="n">
+        <v>-25602.74</v>
+      </c>
+      <c r="E47" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B48" s="10" t="n">
+        <v>744</v>
+      </c>
+      <c r="C48" s="11" t="inlineStr">
+        <is>
+          <t>production</t>
+        </is>
+      </c>
+      <c r="D48" s="14" t="n">
+        <v>-13886500</v>
+      </c>
+      <c r="E48" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B49" s="15" t="n">
+        <v>744</v>
+      </c>
+      <c r="C49" s="16" t="inlineStr">
+        <is>
+          <t>Cash Balance</t>
+        </is>
+      </c>
+      <c r="D49" s="18" t="n">
+        <v>686861.8199999999</v>
+      </c>
+      <c r="E49" s="16" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E37"/>
+  <autoFilter ref="A1:E49"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update game data: day 745, cash 742803.4, 3-day period 249
</commit_message>
<xml_diff>
--- a/data/supply_chain_game.xlsx
+++ b/data/supply_chain_game.xlsx
@@ -20,16 +20,16 @@
     <sheet name="排行榜" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$249</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$745</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$250</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$746</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'资金构成_旧版'!$A$1:$C$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'运营参数_旧版'!$A$9:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'排行榜_旧版'!$A$1:$C$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$61</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'运营参数'!$A$1:$J$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$109</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$136</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -590,7 +590,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-05T16:11:03+08:00</t>
+          <t>2026-09-05T16:26:03+08:00</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>744</v>
+        <v>745</v>
       </c>
     </row>
     <row r="7">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>716</v>
+        <v>715</v>
       </c>
     </row>
     <row r="8">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>686861.8199999999</v>
+        <v>742803.4</v>
       </c>
     </row>
     <row r="11">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>2187142.21</v>
+        <v>2021256.03</v>
       </c>
     </row>
     <row r="15"/>
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>313</v>
+        <v>297</v>
       </c>
     </row>
     <row r="25">
@@ -827,7 +827,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="30">
@@ -838,7 +838,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>742–744</t>
+          <t>745–747</t>
         </is>
       </c>
     </row>
@@ -850,7 +850,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否（进行中）</t>
         </is>
       </c>
     </row>
@@ -861,7 +861,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
     </row>
     <row r="33">
@@ -881,7 +881,7 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
     </row>
     <row r="35">
@@ -901,7 +901,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
     </row>
     <row r="37">
@@ -909,9 +909,6 @@
         <is>
           <t>周期现金变动</t>
         </is>
-      </c>
-      <c r="B37" s="4" t="n">
-        <v>-949004.3614473605</v>
       </c>
     </row>
     <row r="38"/>
@@ -973,7 +970,7 @@
         </is>
       </c>
       <c r="B44" s="4" t="n">
-        <v>-949004.3614473605</v>
+        <v>-996072.1820592751</v>
       </c>
     </row>
     <row r="45"/>
@@ -1171,7 +1168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E109"/>
+  <dimension ref="A1:E136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -3476,8 +3473,575 @@
         <v>686861.8199999999</v>
       </c>
     </row>
+    <row r="110">
+      <c r="A110" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:26:03+08:00</t>
+        </is>
+      </c>
+      <c r="B110" s="10" t="n">
+        <v>745</v>
+      </c>
+      <c r="C110" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D110" s="11" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="E110" s="14" t="n">
+        <v>2764059.43</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:26:03+08:00</t>
+        </is>
+      </c>
+      <c r="B111" s="15" t="n">
+        <v>745</v>
+      </c>
+      <c r="C111" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D111" s="16" t="inlineStr">
+        <is>
+          <t>group15</t>
+        </is>
+      </c>
+      <c r="E111" s="18" t="n">
+        <v>1926708.42</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:26:03+08:00</t>
+        </is>
+      </c>
+      <c r="B112" s="10" t="n">
+        <v>745</v>
+      </c>
+      <c r="C112" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D112" s="11" t="inlineStr">
+        <is>
+          <t>group7</t>
+        </is>
+      </c>
+      <c r="E112" s="14" t="n">
+        <v>1760330.66</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:26:03+08:00</t>
+        </is>
+      </c>
+      <c r="B113" s="15" t="n">
+        <v>745</v>
+      </c>
+      <c r="C113" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D113" s="16" t="inlineStr">
+        <is>
+          <t>nicetry</t>
+        </is>
+      </c>
+      <c r="E113" s="18" t="n">
+        <v>1744220.91</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:26:03+08:00</t>
+        </is>
+      </c>
+      <c r="B114" s="10" t="n">
+        <v>745</v>
+      </c>
+      <c r="C114" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="D114" s="11" t="inlineStr">
+        <is>
+          <t>montesquieu</t>
+        </is>
+      </c>
+      <c r="E114" s="14" t="n">
+        <v>1744136.8</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:26:03+08:00</t>
+        </is>
+      </c>
+      <c r="B115" s="15" t="n">
+        <v>745</v>
+      </c>
+      <c r="C115" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="D115" s="16" t="inlineStr">
+        <is>
+          <t>group14</t>
+        </is>
+      </c>
+      <c r="E115" s="18" t="n">
+        <v>1710121.36</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:26:03+08:00</t>
+        </is>
+      </c>
+      <c r="B116" s="10" t="n">
+        <v>745</v>
+      </c>
+      <c r="C116" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="D116" s="11" t="inlineStr">
+        <is>
+          <t>t24</t>
+        </is>
+      </c>
+      <c r="E116" s="14" t="n">
+        <v>1609417.82</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:26:03+08:00</t>
+        </is>
+      </c>
+      <c r="B117" s="15" t="n">
+        <v>745</v>
+      </c>
+      <c r="C117" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="D117" s="16" t="inlineStr">
+        <is>
+          <t>jit</t>
+        </is>
+      </c>
+      <c r="E117" s="18" t="n">
+        <v>1493894.83</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:26:03+08:00</t>
+        </is>
+      </c>
+      <c r="B118" s="10" t="n">
+        <v>745</v>
+      </c>
+      <c r="C118" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="D118" s="11" t="inlineStr">
+        <is>
+          <t>group8</t>
+        </is>
+      </c>
+      <c r="E118" s="14" t="n">
+        <v>1493262.3</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:26:03+08:00</t>
+        </is>
+      </c>
+      <c r="B119" s="15" t="n">
+        <v>745</v>
+      </c>
+      <c r="C119" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="D119" s="16" t="inlineStr">
+        <is>
+          <t>group2</t>
+        </is>
+      </c>
+      <c r="E119" s="18" t="n">
+        <v>1492989.76</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:26:03+08:00</t>
+        </is>
+      </c>
+      <c r="B120" s="10" t="n">
+        <v>745</v>
+      </c>
+      <c r="C120" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="D120" s="11" t="inlineStr">
+        <is>
+          <t>teamhlly</t>
+        </is>
+      </c>
+      <c r="E120" s="14" t="n">
+        <v>1492847.78</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:26:03+08:00</t>
+        </is>
+      </c>
+      <c r="B121" s="15" t="n">
+        <v>745</v>
+      </c>
+      <c r="C121" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="D121" s="16" t="inlineStr">
+        <is>
+          <t>group9</t>
+        </is>
+      </c>
+      <c r="E121" s="18" t="n">
+        <v>1492844</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:26:03+08:00</t>
+        </is>
+      </c>
+      <c r="B122" s="10" t="n">
+        <v>745</v>
+      </c>
+      <c r="C122" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="D122" s="11" t="inlineStr">
+        <is>
+          <t>group25</t>
+        </is>
+      </c>
+      <c r="E122" s="14" t="n">
+        <v>1492835.79</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:26:03+08:00</t>
+        </is>
+      </c>
+      <c r="B123" s="15" t="n">
+        <v>745</v>
+      </c>
+      <c r="C123" s="15" t="n">
+        <v>14</v>
+      </c>
+      <c r="D123" s="16" t="inlineStr">
+        <is>
+          <t>group11</t>
+        </is>
+      </c>
+      <c r="E123" s="18" t="n">
+        <v>1492823.8</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:26:03+08:00</t>
+        </is>
+      </c>
+      <c r="B124" s="10" t="n">
+        <v>745</v>
+      </c>
+      <c r="C124" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="D124" s="11" t="inlineStr">
+        <is>
+          <t>88888888</t>
+        </is>
+      </c>
+      <c r="E124" s="14" t="n">
+        <v>1492801.72</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:26:03+08:00</t>
+        </is>
+      </c>
+      <c r="B125" s="15" t="n">
+        <v>745</v>
+      </c>
+      <c r="C125" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="D125" s="16" t="inlineStr">
+        <is>
+          <t>tigagroup20</t>
+        </is>
+      </c>
+      <c r="E125" s="18" t="n">
+        <v>1392303.32</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:26:03+08:00</t>
+        </is>
+      </c>
+      <c r="B126" s="10" t="n">
+        <v>745</v>
+      </c>
+      <c r="C126" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="D126" s="11" t="inlineStr">
+        <is>
+          <t>666666</t>
+        </is>
+      </c>
+      <c r="E126" s="14" t="n">
+        <v>1342071.59</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:26:03+08:00</t>
+        </is>
+      </c>
+      <c r="B127" s="15" t="n">
+        <v>745</v>
+      </c>
+      <c r="C127" s="15" t="n">
+        <v>18</v>
+      </c>
+      <c r="D127" s="16" t="inlineStr">
+        <is>
+          <t>newgroup18</t>
+        </is>
+      </c>
+      <c r="E127" s="18" t="n">
+        <v>1318906.78</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:26:03+08:00</t>
+        </is>
+      </c>
+      <c r="B128" s="10" t="n">
+        <v>745</v>
+      </c>
+      <c r="C128" s="10" t="n">
+        <v>19</v>
+      </c>
+      <c r="D128" s="11" t="inlineStr">
+        <is>
+          <t>deepsleep</t>
+        </is>
+      </c>
+      <c r="E128" s="14" t="n">
+        <v>1282331.07</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:26:03+08:00</t>
+        </is>
+      </c>
+      <c r="B129" s="15" t="n">
+        <v>745</v>
+      </c>
+      <c r="C129" s="15" t="n">
+        <v>20</v>
+      </c>
+      <c r="D129" s="16" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E129" s="18" t="n">
+        <v>1210376.87</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:26:03+08:00</t>
+        </is>
+      </c>
+      <c r="B130" s="10" t="n">
+        <v>745</v>
+      </c>
+      <c r="C130" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="D130" s="11" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E130" s="14" t="n">
+        <v>1208398.93</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:26:03+08:00</t>
+        </is>
+      </c>
+      <c r="B131" s="15" t="n">
+        <v>745</v>
+      </c>
+      <c r="C131" s="15" t="n">
+        <v>22</v>
+      </c>
+      <c r="D131" s="16" t="inlineStr">
+        <is>
+          <t>aaachemicalseller</t>
+        </is>
+      </c>
+      <c r="E131" s="18" t="n">
+        <v>1208311.18</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:26:03+08:00</t>
+        </is>
+      </c>
+      <c r="B132" s="10" t="n">
+        <v>745</v>
+      </c>
+      <c r="C132" s="10" t="n">
+        <v>23</v>
+      </c>
+      <c r="D132" s="11" t="inlineStr">
+        <is>
+          <t>group12</t>
+        </is>
+      </c>
+      <c r="E132" s="14" t="n">
+        <v>1208256.66</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:26:03+08:00</t>
+        </is>
+      </c>
+      <c r="B133" s="15" t="n">
+        <v>745</v>
+      </c>
+      <c r="C133" s="15" t="n">
+        <v>24</v>
+      </c>
+      <c r="D133" s="16" t="inlineStr">
+        <is>
+          <t>cleveregg</t>
+        </is>
+      </c>
+      <c r="E133" s="18" t="n">
+        <v>1191373.73</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:26:03+08:00</t>
+        </is>
+      </c>
+      <c r="B134" s="10" t="n">
+        <v>745</v>
+      </c>
+      <c r="C134" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="D134" s="11" t="inlineStr">
+        <is>
+          <t>vivo50</t>
+        </is>
+      </c>
+      <c r="E134" s="14" t="n">
+        <v>991020.63</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:26:03+08:00</t>
+        </is>
+      </c>
+      <c r="B135" s="15" t="n">
+        <v>745</v>
+      </c>
+      <c r="C135" s="15" t="n">
+        <v>26</v>
+      </c>
+      <c r="D135" s="16" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="E135" s="18" t="n">
+        <v>927284.25</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:26:03+08:00</t>
+        </is>
+      </c>
+      <c r="B136" s="24" t="n">
+        <v>745</v>
+      </c>
+      <c r="C136" s="24" t="n">
+        <v>27</v>
+      </c>
+      <c r="D136" s="25" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="E136" s="26" t="n">
+        <v>742803.4</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E109"/>
+  <autoFilter ref="A1:E136"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3488,7 +4052,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S249"/>
+  <dimension ref="A1:S250"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -19233,8 +19797,69 @@
         <v>34800</v>
       </c>
     </row>
+    <row r="250">
+      <c r="A250" s="10" t="n">
+        <v>249</v>
+      </c>
+      <c r="B250" s="10" t="n">
+        <v>745</v>
+      </c>
+      <c r="C250" s="10" t="n">
+        <v>747</v>
+      </c>
+      <c r="D250" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E250" s="11" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="F250" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G250" s="12" t="n">
+        <v>16</v>
+      </c>
+      <c r="H250" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I250" s="12" t="n">
+        <v>16</v>
+      </c>
+      <c r="J250" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K250" s="12" t="n">
+        <v>16</v>
+      </c>
+      <c r="L250" s="14" t="n">
+        <v>742803.4000000001</v>
+      </c>
+      <c r="M250" s="14" t="n">
+        <v>742803.4000000001</v>
+      </c>
+      <c r="N250" s="11" t="n"/>
+      <c r="O250" s="12" t="n">
+        <v>297</v>
+      </c>
+      <c r="P250" s="12" t="n">
+        <v>297</v>
+      </c>
+      <c r="Q250" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="R250" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="S250" s="14" t="n">
+        <v>23200</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S249"/>
+  <autoFilter ref="A1:S250"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -19245,7 +19870,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N745"/>
+  <dimension ref="A1:N746"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -53560,8 +54185,54 @@
         <v>15950</v>
       </c>
     </row>
+    <row r="746">
+      <c r="A746" s="10" t="n">
+        <v>745</v>
+      </c>
+      <c r="B746" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C746" s="12" t="n">
+        <v>16</v>
+      </c>
+      <c r="D746" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E746" s="12" t="n">
+        <v>16</v>
+      </c>
+      <c r="F746" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G746" s="12" t="n">
+        <v>16</v>
+      </c>
+      <c r="H746" s="14" t="n">
+        <v>742803.4000000001</v>
+      </c>
+      <c r="I746" s="12" t="n">
+        <v>297</v>
+      </c>
+      <c r="J746" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K746" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="L746" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="M746" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N746" s="14" t="n">
+        <v>23200</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N745"/>
+  <autoFilter ref="A1:N746"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -53956,7 +54627,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -54223,8 +54894,56 @@
         <v>55</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="23" t="n">
+        <v>730.66</v>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E11" s="16" t="inlineStr"/>
+      <c r="F11" s="17" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="21" t="n">
+        <v>742.75</v>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="inlineStr"/>
+      <c r="F12" s="12" t="n">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F10"/>
+  <autoFilter ref="A1:F12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -54623,7 +55342,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U5"/>
+  <dimension ref="A1:U6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -54632,7 +55351,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
@@ -55036,8 +55755,77 @@
         <v>-949004.3614473605</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:26:03+08:00</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="n">
+        <v>745</v>
+      </c>
+      <c r="C6" s="14" t="n">
+        <v>742803.4</v>
+      </c>
+      <c r="D6" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="E6" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="G6" s="14" t="n">
+        <v>2021256.03</v>
+      </c>
+      <c r="H6" s="21" t="n">
+        <v>20</v>
+      </c>
+      <c r="I6" s="21" t="n">
+        <v>55</v>
+      </c>
+      <c r="J6" s="11" t="inlineStr">
+        <is>
+          <t>truck</t>
+        </is>
+      </c>
+      <c r="K6" s="22" t="n">
+        <v>3600</v>
+      </c>
+      <c r="L6" s="22" t="n">
+        <v>200</v>
+      </c>
+      <c r="M6" s="12" t="n">
+        <v>297</v>
+      </c>
+      <c r="N6" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="O6" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="P6" s="10" t="n">
+        <v>249</v>
+      </c>
+      <c r="Q6" s="12" t="n">
+        <v>16</v>
+      </c>
+      <c r="R6" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" s="12" t="n">
+        <v>16</v>
+      </c>
+      <c r="T6" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="U6" s="11" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U5"/>
+  <autoFilter ref="A1:U6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -55048,7 +55836,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -56173,8 +56961,280 @@
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:26:03+08:00</t>
+        </is>
+      </c>
+      <c r="B50" s="10" t="n">
+        <v>745</v>
+      </c>
+      <c r="C50" s="11" t="inlineStr">
+        <is>
+          <t>Starting Cash</t>
+        </is>
+      </c>
+      <c r="D50" s="14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E50" s="11" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:26:03+08:00</t>
+        </is>
+      </c>
+      <c r="B51" s="15" t="n">
+        <v>745</v>
+      </c>
+      <c r="C51" s="16" t="inlineStr">
+        <is>
+          <t>Cash Sources</t>
+        </is>
+      </c>
+      <c r="D51" s="16" t="n"/>
+      <c r="E51" s="16" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:26:03+08:00</t>
+        </is>
+      </c>
+      <c r="B52" s="10" t="n">
+        <v>745</v>
+      </c>
+      <c r="C52" s="11" t="inlineStr">
+        <is>
+          <t>revenues</t>
+        </is>
+      </c>
+      <c r="D52" s="14" t="n">
+        <v>18966000</v>
+      </c>
+      <c r="E52" s="11" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:26:03+08:00</t>
+        </is>
+      </c>
+      <c r="B53" s="15" t="n">
+        <v>745</v>
+      </c>
+      <c r="C53" s="16" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D53" s="18" t="n">
+        <v>279269.55</v>
+      </c>
+      <c r="E53" s="16" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:26:03+08:00</t>
+        </is>
+      </c>
+      <c r="B54" s="10" t="n">
+        <v>745</v>
+      </c>
+      <c r="C54" s="11" t="inlineStr">
+        <is>
+          <t>Cash Uses</t>
+        </is>
+      </c>
+      <c r="D54" s="11" t="n"/>
+      <c r="E54" s="11" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:26:03+08:00</t>
+        </is>
+      </c>
+      <c r="B55" s="15" t="n">
+        <v>745</v>
+      </c>
+      <c r="C55" s="16" t="inlineStr">
+        <is>
+          <t>outbound shipping</t>
+        </is>
+      </c>
+      <c r="D55" s="18" t="n">
+        <v>-1962000</v>
+      </c>
+      <c r="E55" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:26:03+08:00</t>
+        </is>
+      </c>
+      <c r="B56" s="10" t="n">
+        <v>745</v>
+      </c>
+      <c r="C56" s="11" t="inlineStr">
+        <is>
+          <t>inbound shipping</t>
+        </is>
+      </c>
+      <c r="D56" s="14" t="n">
+        <v>-1365000</v>
+      </c>
+      <c r="E56" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:26:03+08:00</t>
+        </is>
+      </c>
+      <c r="B57" s="15" t="n">
+        <v>745</v>
+      </c>
+      <c r="C57" s="16" t="inlineStr">
+        <is>
+          <t>FGI holding</t>
+        </is>
+      </c>
+      <c r="D57" s="18" t="n">
+        <v>-13467.75</v>
+      </c>
+      <c r="E57" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:26:03+08:00</t>
+        </is>
+      </c>
+      <c r="B58" s="10" t="n">
+        <v>745</v>
+      </c>
+      <c r="C58" s="11" t="inlineStr">
+        <is>
+          <t>add capacity</t>
+        </is>
+      </c>
+      <c r="D58" s="14" t="n">
+        <v>-1749840.87</v>
+      </c>
+      <c r="E58" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:26:03+08:00</t>
+        </is>
+      </c>
+      <c r="B59" s="15" t="n">
+        <v>745</v>
+      </c>
+      <c r="C59" s="16" t="inlineStr">
+        <is>
+          <t>Pipeline inventory holding</t>
+        </is>
+      </c>
+      <c r="D59" s="18" t="n">
+        <v>-25657.53</v>
+      </c>
+      <c r="E59" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:26:03+08:00</t>
+        </is>
+      </c>
+      <c r="B60" s="10" t="n">
+        <v>745</v>
+      </c>
+      <c r="C60" s="11" t="inlineStr">
+        <is>
+          <t>production</t>
+        </is>
+      </c>
+      <c r="D60" s="14" t="n">
+        <v>-13886500</v>
+      </c>
+      <c r="E60" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:26:03+08:00</t>
+        </is>
+      </c>
+      <c r="B61" s="15" t="n">
+        <v>745</v>
+      </c>
+      <c r="C61" s="16" t="inlineStr">
+        <is>
+          <t>Cash Balance</t>
+        </is>
+      </c>
+      <c r="D61" s="18" t="n">
+        <v>742803.4</v>
+      </c>
+      <c r="E61" s="16" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E49"/>
+  <autoFilter ref="A1:E61"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update game data: day 746, cash 748060.4, 3-day period 249
</commit_message>
<xml_diff>
--- a/data/supply_chain_game.xlsx
+++ b/data/supply_chain_game.xlsx
@@ -21,15 +21,15 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$250</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$746</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$747</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'资金构成_旧版'!$A$1:$C$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'运营参数_旧版'!$A$9:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'排行榜_旧版'!$A$1:$C$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$73</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'运营参数'!$A$1:$J$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$136</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$163</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -590,7 +590,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-05T16:26:03+08:00</t>
+          <t>2026-09-05T16:41:02+08:00</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>745</v>
+        <v>746</v>
       </c>
     </row>
     <row r="7">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>715</v>
+        <v>714</v>
       </c>
     </row>
     <row r="8">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>742803.4</v>
+        <v>748060.4</v>
       </c>
     </row>
     <row r="11">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>2021256.03</v>
+        <v>2021838.7</v>
       </c>
     </row>
     <row r="15"/>
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>297</v>
+        <v>270</v>
       </c>
     </row>
     <row r="25">
@@ -861,7 +861,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>16</v>
+        <v>43</v>
       </c>
     </row>
     <row r="33">
@@ -881,7 +881,7 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>16</v>
+        <v>43</v>
       </c>
     </row>
     <row r="35">
@@ -901,7 +901,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>16</v>
+        <v>43</v>
       </c>
     </row>
     <row r="37">
@@ -909,6 +909,9 @@
         <is>
           <t>周期现金变动</t>
         </is>
+      </c>
+      <c r="B37" s="4" t="n">
+        <v>35403.10349342728</v>
       </c>
     </row>
     <row r="38"/>
@@ -970,7 +973,7 @@
         </is>
       </c>
       <c r="B44" s="4" t="n">
-        <v>-996072.1820592751</v>
+        <v>-955647.3602460161</v>
       </c>
     </row>
     <row r="45"/>
@@ -1168,7 +1171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E136"/>
+  <dimension ref="A1:E163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4040,8 +4043,575 @@
         <v>742803.4</v>
       </c>
     </row>
+    <row r="137">
+      <c r="A137" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B137" s="15" t="n">
+        <v>746</v>
+      </c>
+      <c r="C137" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D137" s="16" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="E137" s="18" t="n">
+        <v>2769899.1</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B138" s="10" t="n">
+        <v>746</v>
+      </c>
+      <c r="C138" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D138" s="11" t="inlineStr">
+        <is>
+          <t>group15</t>
+        </is>
+      </c>
+      <c r="E138" s="14" t="n">
+        <v>1932329.4</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B139" s="15" t="n">
+        <v>746</v>
+      </c>
+      <c r="C139" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D139" s="16" t="inlineStr">
+        <is>
+          <t>group7</t>
+        </is>
+      </c>
+      <c r="E139" s="18" t="n">
+        <v>1765908.2</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B140" s="10" t="n">
+        <v>746</v>
+      </c>
+      <c r="C140" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D140" s="11" t="inlineStr">
+        <is>
+          <t>nicetry</t>
+        </is>
+      </c>
+      <c r="E140" s="14" t="n">
+        <v>1749767.49</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B141" s="15" t="n">
+        <v>746</v>
+      </c>
+      <c r="C141" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="D141" s="16" t="inlineStr">
+        <is>
+          <t>montesquieu</t>
+        </is>
+      </c>
+      <c r="E141" s="18" t="n">
+        <v>1749655.31</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B142" s="10" t="n">
+        <v>746</v>
+      </c>
+      <c r="C142" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="D142" s="11" t="inlineStr">
+        <is>
+          <t>group14</t>
+        </is>
+      </c>
+      <c r="E142" s="14" t="n">
+        <v>1715685.78</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B143" s="15" t="n">
+        <v>746</v>
+      </c>
+      <c r="C143" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="D143" s="16" t="inlineStr">
+        <is>
+          <t>t24</t>
+        </is>
+      </c>
+      <c r="E143" s="18" t="n">
+        <v>1614955.94</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B144" s="10" t="n">
+        <v>746</v>
+      </c>
+      <c r="C144" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="D144" s="11" t="inlineStr">
+        <is>
+          <t>jit</t>
+        </is>
+      </c>
+      <c r="E144" s="14" t="n">
+        <v>1499402.78</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B145" s="15" t="n">
+        <v>746</v>
+      </c>
+      <c r="C145" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="D145" s="16" t="inlineStr">
+        <is>
+          <t>group8</t>
+        </is>
+      </c>
+      <c r="E145" s="18" t="n">
+        <v>1498715.29</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B146" s="10" t="n">
+        <v>746</v>
+      </c>
+      <c r="C146" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="D146" s="11" t="inlineStr">
+        <is>
+          <t>group2</t>
+        </is>
+      </c>
+      <c r="E146" s="14" t="n">
+        <v>1498442.68</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B147" s="15" t="n">
+        <v>746</v>
+      </c>
+      <c r="C147" s="15" t="n">
+        <v>11</v>
+      </c>
+      <c r="D147" s="16" t="inlineStr">
+        <is>
+          <t>teamhlly</t>
+        </is>
+      </c>
+      <c r="E147" s="18" t="n">
+        <v>1498300.67</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B148" s="10" t="n">
+        <v>746</v>
+      </c>
+      <c r="C148" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="D148" s="11" t="inlineStr">
+        <is>
+          <t>group9</t>
+        </is>
+      </c>
+      <c r="E148" s="14" t="n">
+        <v>1498296.88</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B149" s="15" t="n">
+        <v>746</v>
+      </c>
+      <c r="C149" s="15" t="n">
+        <v>13</v>
+      </c>
+      <c r="D149" s="16" t="inlineStr">
+        <is>
+          <t>group25</t>
+        </is>
+      </c>
+      <c r="E149" s="18" t="n">
+        <v>1498288.68</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B150" s="10" t="n">
+        <v>746</v>
+      </c>
+      <c r="C150" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="D150" s="11" t="inlineStr">
+        <is>
+          <t>group11</t>
+        </is>
+      </c>
+      <c r="E150" s="14" t="n">
+        <v>1498276.68</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B151" s="15" t="n">
+        <v>746</v>
+      </c>
+      <c r="C151" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="D151" s="16" t="inlineStr">
+        <is>
+          <t>88888888</t>
+        </is>
+      </c>
+      <c r="E151" s="18" t="n">
+        <v>1498254.59</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B152" s="10" t="n">
+        <v>746</v>
+      </c>
+      <c r="C152" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="D152" s="11" t="inlineStr">
+        <is>
+          <t>tigagroup20</t>
+        </is>
+      </c>
+      <c r="E152" s="14" t="n">
+        <v>1397729.95</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B153" s="15" t="n">
+        <v>746</v>
+      </c>
+      <c r="C153" s="15" t="n">
+        <v>17</v>
+      </c>
+      <c r="D153" s="16" t="inlineStr">
+        <is>
+          <t>666666</t>
+        </is>
+      </c>
+      <c r="E153" s="18" t="n">
+        <v>1347485.1</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B154" s="10" t="n">
+        <v>746</v>
+      </c>
+      <c r="C154" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="D154" s="11" t="inlineStr">
+        <is>
+          <t>newgroup18</t>
+        </is>
+      </c>
+      <c r="E154" s="14" t="n">
+        <v>1324336.16</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B155" s="15" t="n">
+        <v>746</v>
+      </c>
+      <c r="C155" s="15" t="n">
+        <v>19</v>
+      </c>
+      <c r="D155" s="16" t="inlineStr">
+        <is>
+          <t>deepsleep</t>
+        </is>
+      </c>
+      <c r="E155" s="18" t="n">
+        <v>1287734.46</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B156" s="10" t="n">
+        <v>746</v>
+      </c>
+      <c r="C156" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="D156" s="11" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E156" s="14" t="n">
+        <v>1213860.37</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B157" s="15" t="n">
+        <v>746</v>
+      </c>
+      <c r="C157" s="15" t="n">
+        <v>21</v>
+      </c>
+      <c r="D157" s="16" t="inlineStr">
+        <is>
+          <t>aaachemicalseller</t>
+        </is>
+      </c>
+      <c r="E157" s="18" t="n">
+        <v>1213744.55</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B158" s="10" t="n">
+        <v>746</v>
+      </c>
+      <c r="C158" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="D158" s="11" t="inlineStr">
+        <is>
+          <t>group12</t>
+        </is>
+      </c>
+      <c r="E158" s="14" t="n">
+        <v>1213690.02</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B159" s="15" t="n">
+        <v>746</v>
+      </c>
+      <c r="C159" s="15" t="n">
+        <v>23</v>
+      </c>
+      <c r="D159" s="16" t="inlineStr">
+        <is>
+          <t>cleveregg</t>
+        </is>
+      </c>
+      <c r="E159" s="18" t="n">
+        <v>1196747.88</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B160" s="10" t="n">
+        <v>746</v>
+      </c>
+      <c r="C160" s="10" t="n">
+        <v>24</v>
+      </c>
+      <c r="D160" s="11" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E160" s="14" t="n">
+        <v>999310.78</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B161" s="15" t="n">
+        <v>746</v>
+      </c>
+      <c r="C161" s="15" t="n">
+        <v>25</v>
+      </c>
+      <c r="D161" s="16" t="inlineStr">
+        <is>
+          <t>vivo50</t>
+        </is>
+      </c>
+      <c r="E161" s="18" t="n">
+        <v>996342.46</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B162" s="10" t="n">
+        <v>746</v>
+      </c>
+      <c r="C162" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="D162" s="11" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="E162" s="14" t="n">
+        <v>932644.23</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B163" s="24" t="n">
+        <v>746</v>
+      </c>
+      <c r="C163" s="24" t="n">
+        <v>27</v>
+      </c>
+      <c r="D163" s="25" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="E163" s="26" t="n">
+        <v>748060.4</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E136"/>
+  <autoFilter ref="A1:E163"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -19808,7 +20378,7 @@
         <v>747</v>
       </c>
       <c r="D250" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E250" s="11" t="inlineStr">
         <is>
@@ -19821,32 +20391,34 @@
         </is>
       </c>
       <c r="G250" s="12" t="n">
-        <v>16</v>
+        <v>43</v>
       </c>
       <c r="H250" s="12" t="n">
         <v>0</v>
       </c>
       <c r="I250" s="12" t="n">
-        <v>16</v>
+        <v>43</v>
       </c>
       <c r="J250" s="19" t="n">
         <v>1</v>
       </c>
       <c r="K250" s="12" t="n">
-        <v>16</v>
+        <v>43</v>
       </c>
       <c r="L250" s="14" t="n">
-        <v>742803.4000000001</v>
+        <v>712657.2965065727</v>
       </c>
       <c r="M250" s="14" t="n">
-        <v>742803.4000000001</v>
-      </c>
-      <c r="N250" s="11" t="n"/>
+        <v>748060.4</v>
+      </c>
+      <c r="N250" s="14" t="n">
+        <v>35403.10349342728</v>
+      </c>
       <c r="O250" s="12" t="n">
-        <v>297</v>
+        <v>270</v>
       </c>
       <c r="P250" s="12" t="n">
-        <v>297</v>
+        <v>283.5</v>
       </c>
       <c r="Q250" s="12" t="n">
         <v>200</v>
@@ -19855,7 +20427,7 @@
         <v>200</v>
       </c>
       <c r="S250" s="14" t="n">
-        <v>23200</v>
+        <v>62350</v>
       </c>
     </row>
   </sheetData>
@@ -19870,7 +20442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N746"/>
+  <dimension ref="A1:N747"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -54231,8 +54803,54 @@
         <v>23200</v>
       </c>
     </row>
+    <row r="747">
+      <c r="A747" s="15" t="n">
+        <v>746</v>
+      </c>
+      <c r="B747" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C747" s="17" t="n">
+        <v>27</v>
+      </c>
+      <c r="D747" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E747" s="17" t="n">
+        <v>27</v>
+      </c>
+      <c r="F747" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G747" s="17" t="n">
+        <v>27</v>
+      </c>
+      <c r="H747" s="18" t="n">
+        <v>748060.4</v>
+      </c>
+      <c r="I747" s="17" t="n">
+        <v>270</v>
+      </c>
+      <c r="J747" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K747" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="L747" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="M747" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N747" s="18" t="n">
+        <v>39150</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N746"/>
+  <autoFilter ref="A1:N747"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -54627,7 +55245,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -54942,8 +55560,56 @@
         <v>55</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="23" t="n">
+        <v>730.66</v>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E13" s="16" t="inlineStr"/>
+      <c r="F13" s="17" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="21" t="n">
+        <v>742.75</v>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E14" s="11" t="inlineStr"/>
+      <c r="F14" s="12" t="n">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F12"/>
+  <autoFilter ref="A1:F14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -55342,7 +56008,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U6"/>
+  <dimension ref="A1:U7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -55824,8 +56490,79 @@
       </c>
       <c r="U6" s="11" t="n"/>
     </row>
+    <row r="7">
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="n">
+        <v>746</v>
+      </c>
+      <c r="C7" s="18" t="n">
+        <v>748060.4</v>
+      </c>
+      <c r="D7" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="E7" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="G7" s="18" t="n">
+        <v>2021838.7</v>
+      </c>
+      <c r="H7" s="23" t="n">
+        <v>20</v>
+      </c>
+      <c r="I7" s="23" t="n">
+        <v>55</v>
+      </c>
+      <c r="J7" s="16" t="inlineStr">
+        <is>
+          <t>truck</t>
+        </is>
+      </c>
+      <c r="K7" s="27" t="n">
+        <v>3600</v>
+      </c>
+      <c r="L7" s="27" t="n">
+        <v>200</v>
+      </c>
+      <c r="M7" s="17" t="n">
+        <v>270</v>
+      </c>
+      <c r="N7" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="O7" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="P7" s="15" t="n">
+        <v>249</v>
+      </c>
+      <c r="Q7" s="17" t="n">
+        <v>43</v>
+      </c>
+      <c r="R7" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" s="17" t="n">
+        <v>43</v>
+      </c>
+      <c r="T7" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="U7" s="18" t="n">
+        <v>35403.10349342728</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U6"/>
+  <autoFilter ref="A1:U7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -55836,7 +56573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:E73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -57233,8 +57970,280 @@
         </is>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B62" s="10" t="n">
+        <v>746</v>
+      </c>
+      <c r="C62" s="11" t="inlineStr">
+        <is>
+          <t>Starting Cash</t>
+        </is>
+      </c>
+      <c r="D62" s="14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E62" s="11" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B63" s="15" t="n">
+        <v>746</v>
+      </c>
+      <c r="C63" s="16" t="inlineStr">
+        <is>
+          <t>Cash Sources</t>
+        </is>
+      </c>
+      <c r="D63" s="16" t="n"/>
+      <c r="E63" s="16" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B64" s="10" t="n">
+        <v>746</v>
+      </c>
+      <c r="C64" s="11" t="inlineStr">
+        <is>
+          <t>revenues</t>
+        </is>
+      </c>
+      <c r="D64" s="14" t="n">
+        <v>18971800</v>
+      </c>
+      <c r="E64" s="11" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B65" s="15" t="n">
+        <v>746</v>
+      </c>
+      <c r="C65" s="16" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D65" s="18" t="n">
+        <v>279458.99</v>
+      </c>
+      <c r="E65" s="16" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B66" s="10" t="n">
+        <v>746</v>
+      </c>
+      <c r="C66" s="11" t="inlineStr">
+        <is>
+          <t>Cash Uses</t>
+        </is>
+      </c>
+      <c r="D66" s="11" t="n"/>
+      <c r="E66" s="11" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B67" s="15" t="n">
+        <v>746</v>
+      </c>
+      <c r="C67" s="16" t="inlineStr">
+        <is>
+          <t>outbound shipping</t>
+        </is>
+      </c>
+      <c r="D67" s="18" t="n">
+        <v>-1962600</v>
+      </c>
+      <c r="E67" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B68" s="10" t="n">
+        <v>746</v>
+      </c>
+      <c r="C68" s="11" t="inlineStr">
+        <is>
+          <t>inbound shipping</t>
+        </is>
+      </c>
+      <c r="D68" s="14" t="n">
+        <v>-1365000</v>
+      </c>
+      <c r="E68" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B69" s="15" t="n">
+        <v>746</v>
+      </c>
+      <c r="C69" s="16" t="inlineStr">
+        <is>
+          <t>FGI holding</t>
+        </is>
+      </c>
+      <c r="D69" s="18" t="n">
+        <v>-13545.39</v>
+      </c>
+      <c r="E69" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B70" s="10" t="n">
+        <v>746</v>
+      </c>
+      <c r="C70" s="11" t="inlineStr">
+        <is>
+          <t>add capacity</t>
+        </is>
+      </c>
+      <c r="D70" s="14" t="n">
+        <v>-1749840.87</v>
+      </c>
+      <c r="E70" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B71" s="15" t="n">
+        <v>746</v>
+      </c>
+      <c r="C71" s="16" t="inlineStr">
+        <is>
+          <t>Pipeline inventory holding</t>
+        </is>
+      </c>
+      <c r="D71" s="18" t="n">
+        <v>-25712.33</v>
+      </c>
+      <c r="E71" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B72" s="10" t="n">
+        <v>746</v>
+      </c>
+      <c r="C72" s="11" t="inlineStr">
+        <is>
+          <t>production</t>
+        </is>
+      </c>
+      <c r="D72" s="14" t="n">
+        <v>-13886500</v>
+      </c>
+      <c r="E72" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B73" s="15" t="n">
+        <v>746</v>
+      </c>
+      <c r="C73" s="16" t="inlineStr">
+        <is>
+          <t>Cash Balance</t>
+        </is>
+      </c>
+      <c r="D73" s="18" t="n">
+        <v>748060.4</v>
+      </c>
+      <c r="E73" s="16" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E61"/>
+  <autoFilter ref="A1:E73"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update game data: day 747, cash 771527.44, 3-day period 249
</commit_message>
<xml_diff>
--- a/data/supply_chain_game.xlsx
+++ b/data/supply_chain_game.xlsx
@@ -21,15 +21,15 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$250</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$747</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$748</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'资金构成_旧版'!$A$1:$C$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'运营参数_旧版'!$A$9:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'排行榜_旧版'!$A$1:$C$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$85</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'运营参数'!$A$1:$J$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$163</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$190</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -590,7 +590,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-05T16:41:02+08:00</t>
+          <t>2026-09-05T16:56:02+08:00</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>746</v>
+        <v>747</v>
       </c>
     </row>
     <row r="7">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>714</v>
+        <v>713</v>
       </c>
     </row>
     <row r="8">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>748060.4</v>
+        <v>771527.4399999999</v>
       </c>
     </row>
     <row r="11">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>2021838.7</v>
+        <v>2022421.52</v>
       </c>
     </row>
     <row r="15"/>
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>270</v>
+        <v>266</v>
       </c>
     </row>
     <row r="25">
@@ -850,7 +850,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>否（进行中）</t>
+          <t>是</t>
         </is>
       </c>
     </row>
@@ -861,7 +861,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="33">
@@ -881,7 +881,7 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="35">
@@ -901,7 +901,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="37">
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="B37" s="4" t="n">
-        <v>35403.10349342728</v>
+        <v>41688.43415010709</v>
       </c>
     </row>
     <row r="38"/>
@@ -929,7 +929,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="41">
@@ -940,7 +940,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>742–744</t>
+          <t>745–747</t>
         </is>
       </c>
     </row>
@@ -952,7 +952,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>24.0 / 0.0 / 24.0</t>
+          <t>47.0 / 0.0 / 47.0</t>
         </is>
       </c>
     </row>
@@ -973,7 +973,7 @@
         </is>
       </c>
       <c r="B44" s="4" t="n">
-        <v>-955647.3602460161</v>
+        <v>41688.43415010709</v>
       </c>
     </row>
     <row r="45"/>
@@ -1171,7 +1171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E163"/>
+  <dimension ref="A1:E190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4610,8 +4610,575 @@
         <v>748060.4</v>
       </c>
     </row>
+    <row r="164">
+      <c r="A164" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B164" s="10" t="n">
+        <v>747</v>
+      </c>
+      <c r="C164" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D164" s="11" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="E164" s="14" t="n">
+        <v>2793948.96</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B165" s="15" t="n">
+        <v>747</v>
+      </c>
+      <c r="C165" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D165" s="16" t="inlineStr">
+        <is>
+          <t>group15</t>
+        </is>
+      </c>
+      <c r="E165" s="18" t="n">
+        <v>1956160.52</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B166" s="10" t="n">
+        <v>747</v>
+      </c>
+      <c r="C166" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D166" s="11" t="inlineStr">
+        <is>
+          <t>group7</t>
+        </is>
+      </c>
+      <c r="E166" s="14" t="n">
+        <v>1789695.85</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B167" s="15" t="n">
+        <v>747</v>
+      </c>
+      <c r="C167" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D167" s="16" t="inlineStr">
+        <is>
+          <t>nicetry</t>
+        </is>
+      </c>
+      <c r="E167" s="18" t="n">
+        <v>1773496.13</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B168" s="10" t="n">
+        <v>747</v>
+      </c>
+      <c r="C168" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="D168" s="11" t="inlineStr">
+        <is>
+          <t>montesquieu</t>
+        </is>
+      </c>
+      <c r="E168" s="14" t="n">
+        <v>1773383.93</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B169" s="15" t="n">
+        <v>747</v>
+      </c>
+      <c r="C169" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="D169" s="16" t="inlineStr">
+        <is>
+          <t>group14</t>
+        </is>
+      </c>
+      <c r="E169" s="18" t="n">
+        <v>1739460.32</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B170" s="10" t="n">
+        <v>747</v>
+      </c>
+      <c r="C170" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="D170" s="11" t="inlineStr">
+        <is>
+          <t>t24</t>
+        </is>
+      </c>
+      <c r="E170" s="14" t="n">
+        <v>1638704.17</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B171" s="15" t="n">
+        <v>747</v>
+      </c>
+      <c r="C171" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="D171" s="16" t="inlineStr">
+        <is>
+          <t>jit</t>
+        </is>
+      </c>
+      <c r="E171" s="18" t="n">
+        <v>1523120.84</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B172" s="10" t="n">
+        <v>747</v>
+      </c>
+      <c r="C172" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="D172" s="11" t="inlineStr">
+        <is>
+          <t>group8</t>
+        </is>
+      </c>
+      <c r="E172" s="14" t="n">
+        <v>1522378.37</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B173" s="15" t="n">
+        <v>747</v>
+      </c>
+      <c r="C173" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="D173" s="16" t="inlineStr">
+        <is>
+          <t>group2</t>
+        </is>
+      </c>
+      <c r="E173" s="18" t="n">
+        <v>1522105.69</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B174" s="10" t="n">
+        <v>747</v>
+      </c>
+      <c r="C174" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="D174" s="11" t="inlineStr">
+        <is>
+          <t>teamhlly</t>
+        </is>
+      </c>
+      <c r="E174" s="14" t="n">
+        <v>1521963.64</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B175" s="15" t="n">
+        <v>747</v>
+      </c>
+      <c r="C175" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="D175" s="16" t="inlineStr">
+        <is>
+          <t>group9</t>
+        </is>
+      </c>
+      <c r="E175" s="18" t="n">
+        <v>1521959.85</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B176" s="10" t="n">
+        <v>747</v>
+      </c>
+      <c r="C176" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="D176" s="11" t="inlineStr">
+        <is>
+          <t>group25</t>
+        </is>
+      </c>
+      <c r="E176" s="14" t="n">
+        <v>1521951.65</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B177" s="15" t="n">
+        <v>747</v>
+      </c>
+      <c r="C177" s="15" t="n">
+        <v>14</v>
+      </c>
+      <c r="D177" s="16" t="inlineStr">
+        <is>
+          <t>group11</t>
+        </is>
+      </c>
+      <c r="E177" s="18" t="n">
+        <v>1521939.65</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B178" s="10" t="n">
+        <v>747</v>
+      </c>
+      <c r="C178" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="D178" s="11" t="inlineStr">
+        <is>
+          <t>88888888</t>
+        </is>
+      </c>
+      <c r="E178" s="14" t="n">
+        <v>1521917.55</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B179" s="15" t="n">
+        <v>747</v>
+      </c>
+      <c r="C179" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="D179" s="16" t="inlineStr">
+        <is>
+          <t>tigagroup20</t>
+        </is>
+      </c>
+      <c r="E179" s="18" t="n">
+        <v>1421366.66</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B180" s="10" t="n">
+        <v>747</v>
+      </c>
+      <c r="C180" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="D180" s="11" t="inlineStr">
+        <is>
+          <t>666666</t>
+        </is>
+      </c>
+      <c r="E180" s="14" t="n">
+        <v>1371108.68</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B181" s="15" t="n">
+        <v>747</v>
+      </c>
+      <c r="C181" s="15" t="n">
+        <v>18</v>
+      </c>
+      <c r="D181" s="16" t="inlineStr">
+        <is>
+          <t>newgroup18</t>
+        </is>
+      </c>
+      <c r="E181" s="18" t="n">
+        <v>1347975.62</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B182" s="10" t="n">
+        <v>747</v>
+      </c>
+      <c r="C182" s="10" t="n">
+        <v>19</v>
+      </c>
+      <c r="D182" s="11" t="inlineStr">
+        <is>
+          <t>deepsleep</t>
+        </is>
+      </c>
+      <c r="E182" s="14" t="n">
+        <v>1311347.92</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B183" s="15" t="n">
+        <v>747</v>
+      </c>
+      <c r="C183" s="15" t="n">
+        <v>20</v>
+      </c>
+      <c r="D183" s="16" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E183" s="18" t="n">
+        <v>1237503.85</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B184" s="10" t="n">
+        <v>747</v>
+      </c>
+      <c r="C184" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="D184" s="11" t="inlineStr">
+        <is>
+          <t>aaachemicalseller</t>
+        </is>
+      </c>
+      <c r="E184" s="14" t="n">
+        <v>1237388.01</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B185" s="15" t="n">
+        <v>747</v>
+      </c>
+      <c r="C185" s="15" t="n">
+        <v>22</v>
+      </c>
+      <c r="D185" s="16" t="inlineStr">
+        <is>
+          <t>group12</t>
+        </is>
+      </c>
+      <c r="E185" s="18" t="n">
+        <v>1237333.46</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B186" s="10" t="n">
+        <v>747</v>
+      </c>
+      <c r="C186" s="10" t="n">
+        <v>23</v>
+      </c>
+      <c r="D186" s="11" t="inlineStr">
+        <is>
+          <t>cleveregg</t>
+        </is>
+      </c>
+      <c r="E186" s="14" t="n">
+        <v>1220332.1</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B187" s="15" t="n">
+        <v>747</v>
+      </c>
+      <c r="C187" s="15" t="n">
+        <v>24</v>
+      </c>
+      <c r="D187" s="16" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E187" s="18" t="n">
+        <v>1022912.25</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B188" s="10" t="n">
+        <v>747</v>
+      </c>
+      <c r="C188" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="D188" s="11" t="inlineStr">
+        <is>
+          <t>vivo50</t>
+        </is>
+      </c>
+      <c r="E188" s="14" t="n">
+        <v>1019874.34</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B189" s="15" t="n">
+        <v>747</v>
+      </c>
+      <c r="C189" s="15" t="n">
+        <v>26</v>
+      </c>
+      <c r="D189" s="16" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="E189" s="18" t="n">
+        <v>956214.27</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B190" s="24" t="n">
+        <v>747</v>
+      </c>
+      <c r="C190" s="24" t="n">
+        <v>27</v>
+      </c>
+      <c r="D190" s="25" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="E190" s="26" t="n">
+        <v>771527.4399999999</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E163"/>
+  <autoFilter ref="A1:E190"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -20378,11 +20945,11 @@
         <v>747</v>
       </c>
       <c r="D250" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E250" s="11" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="F250" s="11" t="inlineStr">
@@ -20391,34 +20958,34 @@
         </is>
       </c>
       <c r="G250" s="12" t="n">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="H250" s="12" t="n">
         <v>0</v>
       </c>
       <c r="I250" s="12" t="n">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="J250" s="19" t="n">
         <v>1</v>
       </c>
       <c r="K250" s="12" t="n">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="L250" s="14" t="n">
-        <v>712657.2965065727</v>
+        <v>729839.0058498929</v>
       </c>
       <c r="M250" s="14" t="n">
-        <v>748060.4</v>
+        <v>771527.4399999999</v>
       </c>
       <c r="N250" s="14" t="n">
-        <v>35403.10349342728</v>
+        <v>41688.43415010709</v>
       </c>
       <c r="O250" s="12" t="n">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="P250" s="12" t="n">
-        <v>283.5</v>
+        <v>277.6666666666667</v>
       </c>
       <c r="Q250" s="12" t="n">
         <v>200</v>
@@ -20427,7 +20994,7 @@
         <v>200</v>
       </c>
       <c r="S250" s="14" t="n">
-        <v>62350</v>
+        <v>68150</v>
       </c>
     </row>
   </sheetData>
@@ -20442,7 +21009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N747"/>
+  <dimension ref="A1:N748"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -54849,8 +55416,54 @@
         <v>39150</v>
       </c>
     </row>
+    <row r="748">
+      <c r="A748" s="10" t="n">
+        <v>747</v>
+      </c>
+      <c r="B748" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C748" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="D748" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E748" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="F748" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G748" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="H748" s="14" t="n">
+        <v>771527.4399999999</v>
+      </c>
+      <c r="I748" s="12" t="n">
+        <v>266</v>
+      </c>
+      <c r="J748" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K748" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="L748" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="M748" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N748" s="14" t="n">
+        <v>5800</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N747"/>
+  <autoFilter ref="A1:N748"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -55245,7 +55858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -55608,8 +56221,56 @@
         <v>55</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="23" t="n">
+        <v>730.66</v>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E15" s="16" t="inlineStr"/>
+      <c r="F15" s="17" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="21" t="n">
+        <v>742.75</v>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E16" s="11" t="inlineStr"/>
+      <c r="F16" s="12" t="n">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F14"/>
+  <autoFilter ref="A1:F16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -56008,7 +56669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U7"/>
+  <dimension ref="A1:U8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -56017,7 +56678,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
@@ -56561,8 +57222,79 @@
         <v>35403.10349342728</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="n">
+        <v>747</v>
+      </c>
+      <c r="C8" s="14" t="n">
+        <v>771527.4399999999</v>
+      </c>
+      <c r="D8" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="E8" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="G8" s="14" t="n">
+        <v>2022421.52</v>
+      </c>
+      <c r="H8" s="21" t="n">
+        <v>20</v>
+      </c>
+      <c r="I8" s="21" t="n">
+        <v>55</v>
+      </c>
+      <c r="J8" s="11" t="inlineStr">
+        <is>
+          <t>truck</t>
+        </is>
+      </c>
+      <c r="K8" s="22" t="n">
+        <v>3600</v>
+      </c>
+      <c r="L8" s="22" t="n">
+        <v>200</v>
+      </c>
+      <c r="M8" s="12" t="n">
+        <v>266</v>
+      </c>
+      <c r="N8" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="O8" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="P8" s="10" t="n">
+        <v>249</v>
+      </c>
+      <c r="Q8" s="12" t="n">
+        <v>47</v>
+      </c>
+      <c r="R8" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" s="12" t="n">
+        <v>47</v>
+      </c>
+      <c r="T8" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="U8" s="14" t="n">
+        <v>41688.43415010709</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U7"/>
+  <autoFilter ref="A1:U8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -56573,7 +57305,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E73"/>
+  <dimension ref="A1:E85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -58242,8 +58974,280 @@
         </is>
       </c>
     </row>
+    <row r="74">
+      <c r="A74" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B74" s="10" t="n">
+        <v>747</v>
+      </c>
+      <c r="C74" s="11" t="inlineStr">
+        <is>
+          <t>Starting Cash</t>
+        </is>
+      </c>
+      <c r="D74" s="14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E74" s="11" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B75" s="15" t="n">
+        <v>747</v>
+      </c>
+      <c r="C75" s="16" t="inlineStr">
+        <is>
+          <t>Cash Sources</t>
+        </is>
+      </c>
+      <c r="D75" s="16" t="n"/>
+      <c r="E75" s="16" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B76" s="10" t="n">
+        <v>747</v>
+      </c>
+      <c r="C76" s="11" t="inlineStr">
+        <is>
+          <t>revenues</t>
+        </is>
+      </c>
+      <c r="D76" s="14" t="n">
+        <v>18997900</v>
+      </c>
+      <c r="E76" s="11" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B77" s="15" t="n">
+        <v>747</v>
+      </c>
+      <c r="C77" s="16" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D77" s="18" t="n">
+        <v>279653.99</v>
+      </c>
+      <c r="E77" s="16" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B78" s="10" t="n">
+        <v>747</v>
+      </c>
+      <c r="C78" s="11" t="inlineStr">
+        <is>
+          <t>Cash Uses</t>
+        </is>
+      </c>
+      <c r="D78" s="11" t="n"/>
+      <c r="E78" s="11" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B79" s="15" t="n">
+        <v>747</v>
+      </c>
+      <c r="C79" s="16" t="inlineStr">
+        <is>
+          <t>outbound shipping</t>
+        </is>
+      </c>
+      <c r="D79" s="18" t="n">
+        <v>-1965300</v>
+      </c>
+      <c r="E79" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B80" s="10" t="n">
+        <v>747</v>
+      </c>
+      <c r="C80" s="11" t="inlineStr">
+        <is>
+          <t>inbound shipping</t>
+        </is>
+      </c>
+      <c r="D80" s="14" t="n">
+        <v>-1365000</v>
+      </c>
+      <c r="E80" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B81" s="15" t="n">
+        <v>747</v>
+      </c>
+      <c r="C81" s="16" t="inlineStr">
+        <is>
+          <t>FGI holding</t>
+        </is>
+      </c>
+      <c r="D81" s="18" t="n">
+        <v>-13618.56</v>
+      </c>
+      <c r="E81" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B82" s="10" t="n">
+        <v>747</v>
+      </c>
+      <c r="C82" s="11" t="inlineStr">
+        <is>
+          <t>add capacity</t>
+        </is>
+      </c>
+      <c r="D82" s="14" t="n">
+        <v>-1749840.87</v>
+      </c>
+      <c r="E82" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B83" s="15" t="n">
+        <v>747</v>
+      </c>
+      <c r="C83" s="16" t="inlineStr">
+        <is>
+          <t>Pipeline inventory holding</t>
+        </is>
+      </c>
+      <c r="D83" s="18" t="n">
+        <v>-25767.12</v>
+      </c>
+      <c r="E83" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B84" s="10" t="n">
+        <v>747</v>
+      </c>
+      <c r="C84" s="11" t="inlineStr">
+        <is>
+          <t>production</t>
+        </is>
+      </c>
+      <c r="D84" s="14" t="n">
+        <v>-13886500</v>
+      </c>
+      <c r="E84" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B85" s="15" t="n">
+        <v>747</v>
+      </c>
+      <c r="C85" s="16" t="inlineStr">
+        <is>
+          <t>Cash Balance</t>
+        </is>
+      </c>
+      <c r="D85" s="18" t="n">
+        <v>771527.4399999999</v>
+      </c>
+      <c r="E85" s="16" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E73"/>
+  <autoFilter ref="A1:E85"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update game data: day 781, cash 761225.01, 3-day period 261
</commit_message>
<xml_diff>
--- a/data/supply_chain_game.xlsx
+++ b/data/supply_chain_game.xlsx
@@ -20,16 +20,16 @@
     <sheet name="排行榜" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$250</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$748</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$262</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$782</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'资金构成_旧版'!$A$1:$C$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'运营参数_旧版'!$A$9:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'排行榜_旧版'!$A$1:$C$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$85</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$97</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'运营参数'!$A$1:$J$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$190</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$217</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -590,7 +590,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-05T16:56:02+08:00</t>
+          <t>2026-09-06T00:41:03+08:00</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>747</v>
+        <v>781</v>
       </c>
     </row>
     <row r="7">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>713</v>
+        <v>679</v>
       </c>
     </row>
     <row r="8">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>771527.4399999999</v>
+        <v>761225.01</v>
       </c>
     </row>
     <row r="11">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>2022421.52</v>
+        <v>2194307.82</v>
       </c>
     </row>
     <row r="15"/>
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>266</v>
+        <v>568</v>
       </c>
     </row>
     <row r="25">
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -827,7 +827,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>249</v>
+        <v>261</v>
       </c>
     </row>
     <row r="30">
@@ -838,7 +838,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>745–747</t>
+          <t>781–783</t>
         </is>
       </c>
     </row>
@@ -850,7 +850,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否（进行中）</t>
         </is>
       </c>
     </row>
@@ -861,7 +861,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>47</v>
+        <v>61</v>
       </c>
     </row>
     <row r="33">
@@ -881,7 +881,7 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>47</v>
+        <v>61</v>
       </c>
     </row>
     <row r="35">
@@ -901,7 +901,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>47</v>
+        <v>61</v>
       </c>
     </row>
     <row r="37">
@@ -909,9 +909,6 @@
         <is>
           <t>周期现金变动</t>
         </is>
-      </c>
-      <c r="B37" s="4" t="n">
-        <v>41688.43415010709</v>
       </c>
     </row>
     <row r="38"/>
@@ -929,7 +926,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>249</v>
+        <v>260</v>
       </c>
     </row>
     <row r="41">
@@ -940,7 +937,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>745–747</t>
+          <t>778–780</t>
         </is>
       </c>
     </row>
@@ -952,7 +949,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>47.0 / 0.0 / 47.0</t>
+          <t>51.0 / 0.0 / 51.0</t>
         </is>
       </c>
     </row>
@@ -973,7 +970,7 @@
         </is>
       </c>
       <c r="B44" s="4" t="n">
-        <v>41688.43415010709</v>
+        <v>55619.29624028411</v>
       </c>
     </row>
     <row r="45"/>
@@ -1171,7 +1168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E190"/>
+  <dimension ref="A1:E217"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5177,8 +5174,575 @@
         <v>771527.4399999999</v>
       </c>
     </row>
+    <row r="191">
+      <c r="A191" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B191" s="15" t="n">
+        <v>781</v>
+      </c>
+      <c r="C191" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D191" s="16" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="E191" s="18" t="n">
+        <v>2955532.83</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B192" s="10" t="n">
+        <v>781</v>
+      </c>
+      <c r="C192" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D192" s="11" t="inlineStr">
+        <is>
+          <t>nicetry</t>
+        </is>
+      </c>
+      <c r="E192" s="14" t="n">
+        <v>1991549.01</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B193" s="15" t="n">
+        <v>781</v>
+      </c>
+      <c r="C193" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D193" s="16" t="inlineStr">
+        <is>
+          <t>group14</t>
+        </is>
+      </c>
+      <c r="E193" s="18" t="n">
+        <v>1958254.87</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B194" s="10" t="n">
+        <v>781</v>
+      </c>
+      <c r="C194" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D194" s="11" t="inlineStr">
+        <is>
+          <t>group7</t>
+        </is>
+      </c>
+      <c r="E194" s="14" t="n">
+        <v>1942324.06</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B195" s="15" t="n">
+        <v>781</v>
+      </c>
+      <c r="C195" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="D195" s="16" t="inlineStr">
+        <is>
+          <t>group15</t>
+        </is>
+      </c>
+      <c r="E195" s="18" t="n">
+        <v>1904195.67</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B196" s="10" t="n">
+        <v>781</v>
+      </c>
+      <c r="C196" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="D196" s="11" t="inlineStr">
+        <is>
+          <t>montesquieu</t>
+        </is>
+      </c>
+      <c r="E196" s="14" t="n">
+        <v>1771720.37</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B197" s="15" t="n">
+        <v>781</v>
+      </c>
+      <c r="C197" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="D197" s="16" t="inlineStr">
+        <is>
+          <t>t24</t>
+        </is>
+      </c>
+      <c r="E197" s="18" t="n">
+        <v>1638154.32</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B198" s="10" t="n">
+        <v>781</v>
+      </c>
+      <c r="C198" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="D198" s="11" t="inlineStr">
+        <is>
+          <t>deepsleep</t>
+        </is>
+      </c>
+      <c r="E198" s="14" t="n">
+        <v>1564461.18</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B199" s="15" t="n">
+        <v>781</v>
+      </c>
+      <c r="C199" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="D199" s="16" t="inlineStr">
+        <is>
+          <t>group8</t>
+        </is>
+      </c>
+      <c r="E199" s="18" t="n">
+        <v>1519616.55</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B200" s="10" t="n">
+        <v>781</v>
+      </c>
+      <c r="C200" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="D200" s="11" t="inlineStr">
+        <is>
+          <t>group9</t>
+        </is>
+      </c>
+      <c r="E200" s="14" t="n">
+        <v>1518890.36</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B201" s="15" t="n">
+        <v>781</v>
+      </c>
+      <c r="C201" s="15" t="n">
+        <v>11</v>
+      </c>
+      <c r="D201" s="16" t="inlineStr">
+        <is>
+          <t>group2</t>
+        </is>
+      </c>
+      <c r="E201" s="18" t="n">
+        <v>1518201.3</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B202" s="10" t="n">
+        <v>781</v>
+      </c>
+      <c r="C202" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="D202" s="11" t="inlineStr">
+        <is>
+          <t>teamhlly</t>
+        </is>
+      </c>
+      <c r="E202" s="14" t="n">
+        <v>1518106.09</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B203" s="15" t="n">
+        <v>781</v>
+      </c>
+      <c r="C203" s="15" t="n">
+        <v>13</v>
+      </c>
+      <c r="D203" s="16" t="inlineStr">
+        <is>
+          <t>group25</t>
+        </is>
+      </c>
+      <c r="E203" s="18" t="n">
+        <v>1518045.88</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B204" s="10" t="n">
+        <v>781</v>
+      </c>
+      <c r="C204" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="D204" s="11" t="inlineStr">
+        <is>
+          <t>group11</t>
+        </is>
+      </c>
+      <c r="E204" s="14" t="n">
+        <v>1518033.78</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B205" s="15" t="n">
+        <v>781</v>
+      </c>
+      <c r="C205" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="D205" s="16" t="inlineStr">
+        <is>
+          <t>88888888</t>
+        </is>
+      </c>
+      <c r="E205" s="18" t="n">
+        <v>1518011.48</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B206" s="10" t="n">
+        <v>781</v>
+      </c>
+      <c r="C206" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="D206" s="11" t="inlineStr">
+        <is>
+          <t>aaachemicalseller</t>
+        </is>
+      </c>
+      <c r="E206" s="14" t="n">
+        <v>1452083.35</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B207" s="15" t="n">
+        <v>781</v>
+      </c>
+      <c r="C207" s="15" t="n">
+        <v>17</v>
+      </c>
+      <c r="D207" s="16" t="inlineStr">
+        <is>
+          <t>group12</t>
+        </is>
+      </c>
+      <c r="E207" s="18" t="n">
+        <v>1450788.24</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B208" s="10" t="n">
+        <v>781</v>
+      </c>
+      <c r="C208" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="D208" s="11" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E208" s="14" t="n">
+        <v>1396539.28</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B209" s="15" t="n">
+        <v>781</v>
+      </c>
+      <c r="C209" s="15" t="n">
+        <v>19</v>
+      </c>
+      <c r="D209" s="16" t="inlineStr">
+        <is>
+          <t>666666</t>
+        </is>
+      </c>
+      <c r="E209" s="18" t="n">
+        <v>1365857.74</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B210" s="10" t="n">
+        <v>781</v>
+      </c>
+      <c r="C210" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="D210" s="11" t="inlineStr">
+        <is>
+          <t>cleveregg</t>
+        </is>
+      </c>
+      <c r="E210" s="14" t="n">
+        <v>1213736.57</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B211" s="15" t="n">
+        <v>781</v>
+      </c>
+      <c r="C211" s="15" t="n">
+        <v>21</v>
+      </c>
+      <c r="D211" s="16" t="inlineStr">
+        <is>
+          <t>tigagroup20</t>
+        </is>
+      </c>
+      <c r="E211" s="18" t="n">
+        <v>1201121.02</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B212" s="10" t="n">
+        <v>781</v>
+      </c>
+      <c r="C212" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="D212" s="11" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="E212" s="14" t="n">
+        <v>1189859.58</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B213" s="15" t="n">
+        <v>781</v>
+      </c>
+      <c r="C213" s="15" t="n">
+        <v>23</v>
+      </c>
+      <c r="D213" s="16" t="inlineStr">
+        <is>
+          <t>jit</t>
+        </is>
+      </c>
+      <c r="E213" s="18" t="n">
+        <v>1054675.19</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B214" s="10" t="n">
+        <v>781</v>
+      </c>
+      <c r="C214" s="10" t="n">
+        <v>24</v>
+      </c>
+      <c r="D214" s="11" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E214" s="14" t="n">
+        <v>1016280.94</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B215" s="15" t="n">
+        <v>781</v>
+      </c>
+      <c r="C215" s="15" t="n">
+        <v>25</v>
+      </c>
+      <c r="D215" s="16" t="inlineStr">
+        <is>
+          <t>vivo50</t>
+        </is>
+      </c>
+      <c r="E215" s="18" t="n">
+        <v>1011539.29</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B216" s="10" t="n">
+        <v>781</v>
+      </c>
+      <c r="C216" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="D216" s="11" t="inlineStr">
+        <is>
+          <t>newgroup18</t>
+        </is>
+      </c>
+      <c r="E216" s="14" t="n">
+        <v>912392.73</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B217" s="24" t="n">
+        <v>781</v>
+      </c>
+      <c r="C217" s="24" t="n">
+        <v>27</v>
+      </c>
+      <c r="D217" s="25" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="E217" s="26" t="n">
+        <v>761225.01</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E190"/>
+  <autoFilter ref="A1:E217"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5189,7 +5753,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S250"/>
+  <dimension ref="A1:S262"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -20997,8 +21561,762 @@
         <v>68150</v>
       </c>
     </row>
+    <row r="251">
+      <c r="A251" s="15" t="n">
+        <v>250</v>
+      </c>
+      <c r="B251" s="15" t="n">
+        <v>748</v>
+      </c>
+      <c r="C251" s="15" t="n">
+        <v>750</v>
+      </c>
+      <c r="D251" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E251" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="F251" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G251" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="H251" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I251" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="J251" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K251" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="L251" s="18" t="n">
+        <v>786376.0733957965</v>
+      </c>
+      <c r="M251" s="18" t="n">
+        <v>828949.2400185141</v>
+      </c>
+      <c r="N251" s="18" t="n">
+        <v>42573.16662271763</v>
+      </c>
+      <c r="O251" s="17" t="n">
+        <v>216</v>
+      </c>
+      <c r="P251" s="17" t="n">
+        <v>234.3333333333333</v>
+      </c>
+      <c r="Q251" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="R251" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="S251" s="18" t="n">
+        <v>72500</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="10" t="n">
+        <v>251</v>
+      </c>
+      <c r="B252" s="10" t="n">
+        <v>751</v>
+      </c>
+      <c r="C252" s="10" t="n">
+        <v>753</v>
+      </c>
+      <c r="D252" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E252" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="F252" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G252" s="12" t="n">
+        <v>42</v>
+      </c>
+      <c r="H252" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I252" s="12" t="n">
+        <v>42</v>
+      </c>
+      <c r="J252" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K252" s="12" t="n">
+        <v>42</v>
+      </c>
+      <c r="L252" s="14" t="n">
+        <v>840975.1632509046</v>
+      </c>
+      <c r="M252" s="14" t="n">
+        <v>884929.4004929601</v>
+      </c>
+      <c r="N252" s="14" t="n">
+        <v>43954.23724205547</v>
+      </c>
+      <c r="O252" s="12" t="n">
+        <v>374</v>
+      </c>
+      <c r="P252" s="12" t="n">
+        <v>390</v>
+      </c>
+      <c r="Q252" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R252" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="S252" s="14" t="n">
+        <v>60900</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="15" t="n">
+        <v>252</v>
+      </c>
+      <c r="B253" s="15" t="n">
+        <v>754</v>
+      </c>
+      <c r="C253" s="15" t="n">
+        <v>756</v>
+      </c>
+      <c r="D253" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E253" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="F253" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G253" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="H253" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I253" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="J253" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K253" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="L253" s="18" t="n">
+        <v>669711.8819978745</v>
+      </c>
+      <c r="M253" s="18" t="n">
+        <v>688299.8741537313</v>
+      </c>
+      <c r="N253" s="18" t="n">
+        <v>18587.9921558568</v>
+      </c>
+      <c r="O253" s="17" t="n">
+        <v>356</v>
+      </c>
+      <c r="P253" s="17" t="n">
+        <v>363</v>
+      </c>
+      <c r="Q253" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="R253" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="S253" s="18" t="n">
+        <v>26100</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="10" t="n">
+        <v>253</v>
+      </c>
+      <c r="B254" s="10" t="n">
+        <v>757</v>
+      </c>
+      <c r="C254" s="10" t="n">
+        <v>759</v>
+      </c>
+      <c r="D254" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E254" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="F254" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G254" s="12" t="n">
+        <v>28</v>
+      </c>
+      <c r="H254" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I254" s="12" t="n">
+        <v>28</v>
+      </c>
+      <c r="J254" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K254" s="12" t="n">
+        <v>28</v>
+      </c>
+      <c r="L254" s="14" t="n">
+        <v>709529.5852397246</v>
+      </c>
+      <c r="M254" s="14" t="n">
+        <v>725503.6338750813</v>
+      </c>
+      <c r="N254" s="14" t="n">
+        <v>15974.04863535671</v>
+      </c>
+      <c r="O254" s="12" t="n">
+        <v>328</v>
+      </c>
+      <c r="P254" s="12" t="n">
+        <v>334.3333333333333</v>
+      </c>
+      <c r="Q254" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="R254" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="S254" s="14" t="n">
+        <v>40600</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="15" t="n">
+        <v>254</v>
+      </c>
+      <c r="B255" s="15" t="n">
+        <v>760</v>
+      </c>
+      <c r="C255" s="15" t="n">
+        <v>762</v>
+      </c>
+      <c r="D255" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E255" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="F255" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G255" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="H255" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I255" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="J255" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K255" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="L255" s="18" t="n">
+        <v>733497.2033009637</v>
+      </c>
+      <c r="M255" s="18" t="n">
+        <v>752146.8973272459</v>
+      </c>
+      <c r="N255" s="18" t="n">
+        <v>18649.69402628217</v>
+      </c>
+      <c r="O255" s="17" t="n">
+        <v>508</v>
+      </c>
+      <c r="P255" s="17" t="n">
+        <v>448</v>
+      </c>
+      <c r="Q255" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="R255" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="S255" s="18" t="n">
+        <v>29000</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="10" t="n">
+        <v>255</v>
+      </c>
+      <c r="B256" s="10" t="n">
+        <v>763</v>
+      </c>
+      <c r="C256" s="10" t="n">
+        <v>765</v>
+      </c>
+      <c r="D256" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E256" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="F256" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G256" s="12" t="n">
+        <v>21</v>
+      </c>
+      <c r="H256" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I256" s="12" t="n">
+        <v>21</v>
+      </c>
+      <c r="J256" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K256" s="12" t="n">
+        <v>21</v>
+      </c>
+      <c r="L256" s="14" t="n">
+        <v>761478.1784536686</v>
+      </c>
+      <c r="M256" s="14" t="n">
+        <v>559395.306044916</v>
+      </c>
+      <c r="N256" s="14" t="n">
+        <v>-202082.8724087526</v>
+      </c>
+      <c r="O256" s="12" t="n">
+        <v>487</v>
+      </c>
+      <c r="P256" s="12" t="n">
+        <v>494.3333333333333</v>
+      </c>
+      <c r="Q256" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="R256" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="S256" s="14" t="n">
+        <v>30450</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="15" t="n">
+        <v>256</v>
+      </c>
+      <c r="B257" s="15" t="n">
+        <v>766</v>
+      </c>
+      <c r="C257" s="15" t="n">
+        <v>768</v>
+      </c>
+      <c r="D257" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E257" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="F257" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G257" s="17" t="n">
+        <v>45</v>
+      </c>
+      <c r="H257" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I257" s="17" t="n">
+        <v>45</v>
+      </c>
+      <c r="J257" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K257" s="17" t="n">
+        <v>45</v>
+      </c>
+      <c r="L257" s="18" t="n">
+        <v>587181.1901554394</v>
+      </c>
+      <c r="M257" s="18" t="n">
+        <v>618930.0192956959</v>
+      </c>
+      <c r="N257" s="18" t="n">
+        <v>31748.82914025651</v>
+      </c>
+      <c r="O257" s="17" t="n">
+        <v>442</v>
+      </c>
+      <c r="P257" s="17" t="n">
+        <v>453</v>
+      </c>
+      <c r="Q257" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="R257" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="S257" s="18" t="n">
+        <v>65250</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="10" t="n">
+        <v>257</v>
+      </c>
+      <c r="B258" s="10" t="n">
+        <v>769</v>
+      </c>
+      <c r="C258" s="10" t="n">
+        <v>771</v>
+      </c>
+      <c r="D258" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E258" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="F258" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G258" s="12" t="n">
+        <v>59</v>
+      </c>
+      <c r="H258" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I258" s="12" t="n">
+        <v>59</v>
+      </c>
+      <c r="J258" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K258" s="12" t="n">
+        <v>59</v>
+      </c>
+      <c r="L258" s="14" t="n">
+        <v>659993.1608755215</v>
+      </c>
+      <c r="M258" s="14" t="n">
+        <v>697113.1051637947</v>
+      </c>
+      <c r="N258" s="14" t="n">
+        <v>37119.94428827323</v>
+      </c>
+      <c r="O258" s="12" t="n">
+        <v>583</v>
+      </c>
+      <c r="P258" s="12" t="n">
+        <v>463</v>
+      </c>
+      <c r="Q258" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R258" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="S258" s="14" t="n">
+        <v>85550</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="15" t="n">
+        <v>258</v>
+      </c>
+      <c r="B259" s="15" t="n">
+        <v>772</v>
+      </c>
+      <c r="C259" s="15" t="n">
+        <v>774</v>
+      </c>
+      <c r="D259" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E259" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="F259" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G259" s="17" t="n">
+        <v>44</v>
+      </c>
+      <c r="H259" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I259" s="17" t="n">
+        <v>44</v>
+      </c>
+      <c r="J259" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K259" s="17" t="n">
+        <v>44</v>
+      </c>
+      <c r="L259" s="18" t="n">
+        <v>699783.0070550918</v>
+      </c>
+      <c r="M259" s="18" t="n">
+        <v>534841.6764577201</v>
+      </c>
+      <c r="N259" s="18" t="n">
+        <v>-164941.3305973717</v>
+      </c>
+      <c r="O259" s="17" t="n">
+        <v>539</v>
+      </c>
+      <c r="P259" s="17" t="n">
+        <v>563</v>
+      </c>
+      <c r="Q259" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="R259" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="S259" s="18" t="n">
+        <v>63800</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="10" t="n">
+        <v>259</v>
+      </c>
+      <c r="B260" s="10" t="n">
+        <v>775</v>
+      </c>
+      <c r="C260" s="10" t="n">
+        <v>777</v>
+      </c>
+      <c r="D260" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E260" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="F260" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G260" s="12" t="n">
+        <v>59</v>
+      </c>
+      <c r="H260" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I260" s="12" t="n">
+        <v>59</v>
+      </c>
+      <c r="J260" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K260" s="12" t="n">
+        <v>59</v>
+      </c>
+      <c r="L260" s="14" t="n">
+        <v>575852.2827446689</v>
+      </c>
+      <c r="M260" s="14" t="n">
+        <v>612872.8374497481</v>
+      </c>
+      <c r="N260" s="14" t="n">
+        <v>37020.55470507918</v>
+      </c>
+      <c r="O260" s="12" t="n">
+        <v>480</v>
+      </c>
+      <c r="P260" s="12" t="n">
+        <v>494.3333333333333</v>
+      </c>
+      <c r="Q260" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="R260" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="S260" s="14" t="n">
+        <v>85550</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="15" t="n">
+        <v>260</v>
+      </c>
+      <c r="B261" s="15" t="n">
+        <v>778</v>
+      </c>
+      <c r="C261" s="15" t="n">
+        <v>780</v>
+      </c>
+      <c r="D261" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E261" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="F261" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G261" s="17" t="n">
+        <v>51</v>
+      </c>
+      <c r="H261" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I261" s="17" t="n">
+        <v>51</v>
+      </c>
+      <c r="J261" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K261" s="17" t="n">
+        <v>51</v>
+      </c>
+      <c r="L261" s="18" t="n">
+        <v>624770.9641976637</v>
+      </c>
+      <c r="M261" s="18" t="n">
+        <v>680390.2604379478</v>
+      </c>
+      <c r="N261" s="18" t="n">
+        <v>55619.29624028411</v>
+      </c>
+      <c r="O261" s="17" t="n">
+        <v>429</v>
+      </c>
+      <c r="P261" s="17" t="n">
+        <v>452</v>
+      </c>
+      <c r="Q261" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="R261" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="S261" s="18" t="n">
+        <v>73950</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="10" t="n">
+        <v>261</v>
+      </c>
+      <c r="B262" s="10" t="n">
+        <v>781</v>
+      </c>
+      <c r="C262" s="10" t="n">
+        <v>783</v>
+      </c>
+      <c r="D262" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E262" s="11" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="F262" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G262" s="12" t="n">
+        <v>61</v>
+      </c>
+      <c r="H262" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I262" s="12" t="n">
+        <v>61</v>
+      </c>
+      <c r="J262" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K262" s="12" t="n">
+        <v>61</v>
+      </c>
+      <c r="L262" s="14" t="n">
+        <v>761225.01</v>
+      </c>
+      <c r="M262" s="14" t="n">
+        <v>761225.01</v>
+      </c>
+      <c r="N262" s="11" t="n"/>
+      <c r="O262" s="12" t="n">
+        <v>568</v>
+      </c>
+      <c r="P262" s="12" t="n">
+        <v>568</v>
+      </c>
+      <c r="Q262" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R262" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="S262" s="14" t="n">
+        <v>88450</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S250"/>
+  <autoFilter ref="A1:S262"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -21009,7 +22327,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N748"/>
+  <dimension ref="A1:N782"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -55462,8 +56780,1572 @@
         <v>5800</v>
       </c>
     </row>
+    <row r="749">
+      <c r="A749" s="15" t="n">
+        <v>748</v>
+      </c>
+      <c r="B749" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C749" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="D749" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E749" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="F749" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G749" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="H749" s="18" t="n">
+        <v>786376.0733957965</v>
+      </c>
+      <c r="I749" s="17" t="n">
+        <v>248</v>
+      </c>
+      <c r="J749" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K749" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="L749" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="M749" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N749" s="18" t="n">
+        <v>26100</v>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" s="10" t="n">
+        <v>749</v>
+      </c>
+      <c r="B750" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C750" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="D750" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E750" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="F750" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G750" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="H750" s="14" t="n">
+        <v>798383.022239556</v>
+      </c>
+      <c r="I750" s="12" t="n">
+        <v>239</v>
+      </c>
+      <c r="J750" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K750" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="L750" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="M750" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N750" s="14" t="n">
+        <v>13050</v>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" s="15" t="n">
+        <v>750</v>
+      </c>
+      <c r="B751" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C751" s="17" t="n">
+        <v>23</v>
+      </c>
+      <c r="D751" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E751" s="17" t="n">
+        <v>23</v>
+      </c>
+      <c r="F751" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G751" s="17" t="n">
+        <v>23</v>
+      </c>
+      <c r="H751" s="18" t="n">
+        <v>828949.2400185141</v>
+      </c>
+      <c r="I751" s="17" t="n">
+        <v>216</v>
+      </c>
+      <c r="J751" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K751" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="L751" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="M751" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N751" s="18" t="n">
+        <v>33350</v>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" s="10" t="n">
+        <v>751</v>
+      </c>
+      <c r="B752" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C752" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="D752" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E752" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="F752" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G752" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="H752" s="14" t="n">
+        <v>840975.1632509046</v>
+      </c>
+      <c r="I752" s="12" t="n">
+        <v>407</v>
+      </c>
+      <c r="J752" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K752" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L752" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M752" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N752" s="14" t="n">
+        <v>13050</v>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" s="15" t="n">
+        <v>752</v>
+      </c>
+      <c r="B753" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C753" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="D753" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E753" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="F753" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G753" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="H753" s="18" t="n">
+        <v>864935.5383473488</v>
+      </c>
+      <c r="I753" s="17" t="n">
+        <v>389</v>
+      </c>
+      <c r="J753" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K753" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L753" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M753" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N753" s="18" t="n">
+        <v>26100</v>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" s="10" t="n">
+        <v>753</v>
+      </c>
+      <c r="B754" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C754" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="D754" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E754" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="F754" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G754" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="H754" s="14" t="n">
+        <v>884929.4004929601</v>
+      </c>
+      <c r="I754" s="12" t="n">
+        <v>374</v>
+      </c>
+      <c r="J754" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K754" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L754" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M754" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N754" s="14" t="n">
+        <v>21750</v>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" s="15" t="n">
+        <v>754</v>
+      </c>
+      <c r="B755" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C755" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="D755" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E755" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="F755" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G755" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="H755" s="18" t="n">
+        <v>669711.8819978745</v>
+      </c>
+      <c r="I755" s="17" t="n">
+        <v>370</v>
+      </c>
+      <c r="J755" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K755" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="L755" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="M755" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N755" s="18" t="n">
+        <v>5800</v>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" s="10" t="n">
+        <v>755</v>
+      </c>
+      <c r="B756" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C756" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="D756" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E756" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="F756" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G756" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="H756" s="14" t="n">
+        <v>679003.5966981715</v>
+      </c>
+      <c r="I756" s="12" t="n">
+        <v>363</v>
+      </c>
+      <c r="J756" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K756" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="L756" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="M756" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N756" s="14" t="n">
+        <v>10150</v>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" s="15" t="n">
+        <v>756</v>
+      </c>
+      <c r="B757" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C757" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="D757" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E757" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="F757" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G757" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="H757" s="18" t="n">
+        <v>688299.8741537313</v>
+      </c>
+      <c r="I757" s="17" t="n">
+        <v>356</v>
+      </c>
+      <c r="J757" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K757" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="L757" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="M757" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N757" s="18" t="n">
+        <v>10150</v>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" s="10" t="n">
+        <v>757</v>
+      </c>
+      <c r="B758" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C758" s="12" t="n">
+        <v>16</v>
+      </c>
+      <c r="D758" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E758" s="12" t="n">
+        <v>16</v>
+      </c>
+      <c r="F758" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G758" s="12" t="n">
+        <v>16</v>
+      </c>
+      <c r="H758" s="14" t="n">
+        <v>709529.5852397246</v>
+      </c>
+      <c r="I758" s="12" t="n">
+        <v>340</v>
+      </c>
+      <c r="J758" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K758" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="L758" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="M758" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N758" s="14" t="n">
+        <v>23200</v>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" s="15" t="n">
+        <v>758</v>
+      </c>
+      <c r="B759" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C759" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="D759" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E759" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="F759" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G759" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="H759" s="18" t="n">
+        <v>716190.0502871802</v>
+      </c>
+      <c r="I759" s="17" t="n">
+        <v>335</v>
+      </c>
+      <c r="J759" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K759" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="L759" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="M759" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N759" s="18" t="n">
+        <v>7250</v>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" s="10" t="n">
+        <v>759</v>
+      </c>
+      <c r="B760" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C760" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="D760" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E760" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="F760" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G760" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="H760" s="14" t="n">
+        <v>725503.6338750813</v>
+      </c>
+      <c r="I760" s="12" t="n">
+        <v>328</v>
+      </c>
+      <c r="J760" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K760" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="L760" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="M760" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N760" s="14" t="n">
+        <v>10150</v>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" s="15" t="n">
+        <v>760</v>
+      </c>
+      <c r="B761" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C761" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="D761" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E761" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="F761" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G761" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="H761" s="18" t="n">
+        <v>733497.2033009637</v>
+      </c>
+      <c r="I761" s="17" t="n">
+        <v>322</v>
+      </c>
+      <c r="J761" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K761" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="L761" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="M761" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N761" s="18" t="n">
+        <v>8700</v>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" s="10" t="n">
+        <v>761</v>
+      </c>
+      <c r="B762" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C762" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="D762" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E762" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="F762" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G762" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="H762" s="14" t="n">
+        <v>744144.6665980516</v>
+      </c>
+      <c r="I762" s="12" t="n">
+        <v>514</v>
+      </c>
+      <c r="J762" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K762" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L762" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M762" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N762" s="14" t="n">
+        <v>11600</v>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" s="15" t="n">
+        <v>762</v>
+      </c>
+      <c r="B763" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C763" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="D763" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E763" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="F763" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G763" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="H763" s="18" t="n">
+        <v>752146.8973272459</v>
+      </c>
+      <c r="I763" s="17" t="n">
+        <v>508</v>
+      </c>
+      <c r="J763" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K763" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L763" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M763" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N763" s="18" t="n">
+        <v>8700</v>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" s="10" t="n">
+        <v>763</v>
+      </c>
+      <c r="B764" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C764" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="D764" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E764" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="F764" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G764" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="H764" s="14" t="n">
+        <v>761478.1784536686</v>
+      </c>
+      <c r="I764" s="12" t="n">
+        <v>501</v>
+      </c>
+      <c r="J764" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K764" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L764" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M764" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N764" s="14" t="n">
+        <v>10150</v>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" s="15" t="n">
+        <v>764</v>
+      </c>
+      <c r="B765" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C765" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="D765" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E765" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="F765" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G765" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="H765" s="18" t="n">
+        <v>548844.5207170692</v>
+      </c>
+      <c r="I765" s="17" t="n">
+        <v>495</v>
+      </c>
+      <c r="J765" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K765" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="L765" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="M765" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N765" s="18" t="n">
+        <v>8700</v>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" s="10" t="n">
+        <v>765</v>
+      </c>
+      <c r="B766" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C766" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="D766" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E766" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="F766" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G766" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="H766" s="14" t="n">
+        <v>559395.306044916</v>
+      </c>
+      <c r="I766" s="12" t="n">
+        <v>487</v>
+      </c>
+      <c r="J766" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K766" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="L766" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="M766" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N766" s="14" t="n">
+        <v>11600</v>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" s="15" t="n">
+        <v>766</v>
+      </c>
+      <c r="B767" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C767" s="17" t="n">
+        <v>21</v>
+      </c>
+      <c r="D767" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E767" s="17" t="n">
+        <v>21</v>
+      </c>
+      <c r="F767" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G767" s="17" t="n">
+        <v>21</v>
+      </c>
+      <c r="H767" s="18" t="n">
+        <v>587181.1901554394</v>
+      </c>
+      <c r="I767" s="17" t="n">
+        <v>466</v>
+      </c>
+      <c r="J767" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K767" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="L767" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="M767" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N767" s="18" t="n">
+        <v>30450</v>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" s="10" t="n">
+        <v>767</v>
+      </c>
+      <c r="B768" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C768" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="D768" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E768" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="F768" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G768" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="H768" s="14" t="n">
+        <v>607027.2713256801</v>
+      </c>
+      <c r="I768" s="12" t="n">
+        <v>451</v>
+      </c>
+      <c r="J768" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K768" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="L768" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="M768" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N768" s="14" t="n">
+        <v>21750</v>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" s="15" t="n">
+        <v>768</v>
+      </c>
+      <c r="B769" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C769" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="D769" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E769" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="F769" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G769" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="H769" s="18" t="n">
+        <v>618930.0192956959</v>
+      </c>
+      <c r="I769" s="17" t="n">
+        <v>442</v>
+      </c>
+      <c r="J769" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K769" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="L769" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="M769" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N769" s="18" t="n">
+        <v>13050</v>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" s="10" t="n">
+        <v>769</v>
+      </c>
+      <c r="B770" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C770" s="12" t="n">
+        <v>31</v>
+      </c>
+      <c r="D770" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E770" s="12" t="n">
+        <v>31</v>
+      </c>
+      <c r="F770" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G770" s="12" t="n">
+        <v>31</v>
+      </c>
+      <c r="H770" s="14" t="n">
+        <v>659993.1608755215</v>
+      </c>
+      <c r="I770" s="12" t="n">
+        <v>411</v>
+      </c>
+      <c r="J770" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K770" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="L770" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="M770" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N770" s="14" t="n">
+        <v>44950</v>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" s="15" t="n">
+        <v>770</v>
+      </c>
+      <c r="B771" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C771" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="D771" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E771" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="F771" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G771" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="H771" s="18" t="n">
+        <v>681198.5195721132</v>
+      </c>
+      <c r="I771" s="17" t="n">
+        <v>395</v>
+      </c>
+      <c r="J771" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K771" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="L771" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="M771" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N771" s="18" t="n">
+        <v>23200</v>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" s="10" t="n">
+        <v>771</v>
+      </c>
+      <c r="B772" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C772" s="12" t="n">
+        <v>12</v>
+      </c>
+      <c r="D772" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E772" s="12" t="n">
+        <v>12</v>
+      </c>
+      <c r="F772" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G772" s="12" t="n">
+        <v>12</v>
+      </c>
+      <c r="H772" s="14" t="n">
+        <v>697113.1051637947</v>
+      </c>
+      <c r="I772" s="12" t="n">
+        <v>583</v>
+      </c>
+      <c r="J772" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K772" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L772" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M772" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N772" s="14" t="n">
+        <v>17400</v>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" s="15" t="n">
+        <v>772</v>
+      </c>
+      <c r="B773" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C773" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="D773" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E773" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="F773" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G773" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="H773" s="18" t="n">
+        <v>699783.0070550918</v>
+      </c>
+      <c r="I773" s="17" t="n">
+        <v>581</v>
+      </c>
+      <c r="J773" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K773" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L773" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M773" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N773" s="18" t="n">
+        <v>2900</v>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" s="10" t="n">
+        <v>773</v>
+      </c>
+      <c r="B774" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C774" s="12" t="n">
+        <v>12</v>
+      </c>
+      <c r="D774" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E774" s="12" t="n">
+        <v>12</v>
+      </c>
+      <c r="F774" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G774" s="12" t="n">
+        <v>12</v>
+      </c>
+      <c r="H774" s="14" t="n">
+        <v>715707.7686852003</v>
+      </c>
+      <c r="I774" s="12" t="n">
+        <v>569</v>
+      </c>
+      <c r="J774" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K774" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L774" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M774" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N774" s="14" t="n">
+        <v>17400</v>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" s="15" t="n">
+        <v>774</v>
+      </c>
+      <c r="B775" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C775" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="D775" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E775" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="F775" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G775" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="H775" s="18" t="n">
+        <v>534841.6764577201</v>
+      </c>
+      <c r="I775" s="17" t="n">
+        <v>539</v>
+      </c>
+      <c r="J775" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K775" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="L775" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="M775" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N775" s="18" t="n">
+        <v>43500</v>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" s="10" t="n">
+        <v>775</v>
+      </c>
+      <c r="B776" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C776" s="12" t="n">
+        <v>31</v>
+      </c>
+      <c r="D776" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E776" s="12" t="n">
+        <v>31</v>
+      </c>
+      <c r="F776" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G776" s="12" t="n">
+        <v>31</v>
+      </c>
+      <c r="H776" s="14" t="n">
+        <v>575852.2827446689</v>
+      </c>
+      <c r="I776" s="12" t="n">
+        <v>508</v>
+      </c>
+      <c r="J776" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K776" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="L776" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="M776" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N776" s="14" t="n">
+        <v>44950</v>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" s="15" t="n">
+        <v>776</v>
+      </c>
+      <c r="B777" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C777" s="17" t="n">
+        <v>13</v>
+      </c>
+      <c r="D777" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E777" s="17" t="n">
+        <v>13</v>
+      </c>
+      <c r="F777" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G777" s="17" t="n">
+        <v>13</v>
+      </c>
+      <c r="H777" s="18" t="n">
+        <v>593032.6193464252</v>
+      </c>
+      <c r="I777" s="17" t="n">
+        <v>495</v>
+      </c>
+      <c r="J777" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K777" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="L777" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="M777" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N777" s="18" t="n">
+        <v>18850</v>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" s="10" t="n">
+        <v>777</v>
+      </c>
+      <c r="B778" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C778" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="D778" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E778" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="F778" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G778" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="H778" s="14" t="n">
+        <v>612872.8374497481</v>
+      </c>
+      <c r="I778" s="12" t="n">
+        <v>480</v>
+      </c>
+      <c r="J778" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K778" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="L778" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="M778" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N778" s="14" t="n">
+        <v>21750</v>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" s="15" t="n">
+        <v>778</v>
+      </c>
+      <c r="B779" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C779" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="D779" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E779" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="F779" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G779" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="H779" s="18" t="n">
+        <v>624770.9641976637</v>
+      </c>
+      <c r="I779" s="17" t="n">
+        <v>471</v>
+      </c>
+      <c r="J779" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K779" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="L779" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="M779" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N779" s="18" t="n">
+        <v>13050</v>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" s="10" t="n">
+        <v>779</v>
+      </c>
+      <c r="B780" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C780" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="D780" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E780" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="F780" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G780" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="H780" s="14" t="n">
+        <v>644625.1744964955</v>
+      </c>
+      <c r="I780" s="12" t="n">
+        <v>456</v>
+      </c>
+      <c r="J780" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K780" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="L780" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="M780" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N780" s="14" t="n">
+        <v>21750</v>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" s="15" t="n">
+        <v>780</v>
+      </c>
+      <c r="B781" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C781" s="17" t="n">
+        <v>27</v>
+      </c>
+      <c r="D781" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E781" s="17" t="n">
+        <v>27</v>
+      </c>
+      <c r="F781" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G781" s="17" t="n">
+        <v>27</v>
+      </c>
+      <c r="H781" s="18" t="n">
+        <v>680390.2604379478</v>
+      </c>
+      <c r="I781" s="17" t="n">
+        <v>429</v>
+      </c>
+      <c r="J781" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K781" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="L781" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="M781" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N781" s="18" t="n">
+        <v>39150</v>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" s="10" t="n">
+        <v>781</v>
+      </c>
+      <c r="B782" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C782" s="12" t="n">
+        <v>61</v>
+      </c>
+      <c r="D782" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E782" s="12" t="n">
+        <v>61</v>
+      </c>
+      <c r="F782" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G782" s="12" t="n">
+        <v>61</v>
+      </c>
+      <c r="H782" s="14" t="n">
+        <v>761225.01</v>
+      </c>
+      <c r="I782" s="12" t="n">
+        <v>568</v>
+      </c>
+      <c r="J782" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K782" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L782" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M782" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N782" s="14" t="n">
+        <v>88450</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N748"/>
+  <autoFilter ref="A1:N782"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -55858,7 +58740,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -56269,8 +59151,56 @@
         <v>55</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="23" t="n">
+        <v>730.66</v>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E17" s="16" t="inlineStr"/>
+      <c r="F17" s="17" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="21" t="n">
+        <v>742.75</v>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="inlineStr"/>
+      <c r="F18" s="12" t="n">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F16"/>
+  <autoFilter ref="A1:F18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -56669,7 +59599,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U8"/>
+  <dimension ref="A1:U9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -56678,7 +59608,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
@@ -57293,8 +60223,77 @@
         <v>41688.43415010709</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="n">
+        <v>781</v>
+      </c>
+      <c r="C9" s="18" t="n">
+        <v>761225.01</v>
+      </c>
+      <c r="D9" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="E9" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="G9" s="18" t="n">
+        <v>2194307.82</v>
+      </c>
+      <c r="H9" s="23" t="n">
+        <v>20</v>
+      </c>
+      <c r="I9" s="23" t="n">
+        <v>55</v>
+      </c>
+      <c r="J9" s="16" t="inlineStr">
+        <is>
+          <t>truck</t>
+        </is>
+      </c>
+      <c r="K9" s="27" t="n">
+        <v>3600</v>
+      </c>
+      <c r="L9" s="27" t="n">
+        <v>200</v>
+      </c>
+      <c r="M9" s="17" t="n">
+        <v>568</v>
+      </c>
+      <c r="N9" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="P9" s="15" t="n">
+        <v>261</v>
+      </c>
+      <c r="Q9" s="17" t="n">
+        <v>61</v>
+      </c>
+      <c r="R9" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="S9" s="17" t="n">
+        <v>61</v>
+      </c>
+      <c r="T9" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="U9" s="16" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U8"/>
+  <autoFilter ref="A1:U9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -57305,7 +60304,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E85"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -59246,8 +62245,280 @@
         </is>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B86" s="10" t="n">
+        <v>781</v>
+      </c>
+      <c r="C86" s="11" t="inlineStr">
+        <is>
+          <t>Starting Cash</t>
+        </is>
+      </c>
+      <c r="D86" s="14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E86" s="11" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B87" s="15" t="n">
+        <v>781</v>
+      </c>
+      <c r="C87" s="16" t="inlineStr">
+        <is>
+          <t>Cash Sources</t>
+        </is>
+      </c>
+      <c r="D87" s="16" t="n"/>
+      <c r="E87" s="16" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B88" s="10" t="n">
+        <v>781</v>
+      </c>
+      <c r="C88" s="11" t="inlineStr">
+        <is>
+          <t>revenues</t>
+        </is>
+      </c>
+      <c r="D88" s="14" t="n">
+        <v>19709850</v>
+      </c>
+      <c r="E88" s="11" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B89" s="15" t="n">
+        <v>781</v>
+      </c>
+      <c r="C89" s="16" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D89" s="18" t="n">
+        <v>285781.53</v>
+      </c>
+      <c r="E89" s="16" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B90" s="10" t="n">
+        <v>781</v>
+      </c>
+      <c r="C90" s="11" t="inlineStr">
+        <is>
+          <t>Cash Uses</t>
+        </is>
+      </c>
+      <c r="D90" s="11" t="n"/>
+      <c r="E90" s="11" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B91" s="15" t="n">
+        <v>781</v>
+      </c>
+      <c r="C91" s="16" t="inlineStr">
+        <is>
+          <t>outbound shipping</t>
+        </is>
+      </c>
+      <c r="D91" s="18" t="n">
+        <v>-2038950</v>
+      </c>
+      <c r="E91" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B92" s="10" t="n">
+        <v>781</v>
+      </c>
+      <c r="C92" s="11" t="inlineStr">
+        <is>
+          <t>inbound shipping</t>
+        </is>
+      </c>
+      <c r="D92" s="14" t="n">
+        <v>-1410000</v>
+      </c>
+      <c r="E92" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B93" s="15" t="n">
+        <v>781</v>
+      </c>
+      <c r="C93" s="16" t="inlineStr">
+        <is>
+          <t>FGI holding</t>
+        </is>
+      </c>
+      <c r="D93" s="18" t="n">
+        <v>-17478.66</v>
+      </c>
+      <c r="E93" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B94" s="10" t="n">
+        <v>781</v>
+      </c>
+      <c r="C94" s="11" t="inlineStr">
+        <is>
+          <t>add capacity</t>
+        </is>
+      </c>
+      <c r="D94" s="14" t="n">
+        <v>-1749840.87</v>
+      </c>
+      <c r="E94" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B95" s="15" t="n">
+        <v>781</v>
+      </c>
+      <c r="C95" s="16" t="inlineStr">
+        <is>
+          <t>Pipeline inventory holding</t>
+        </is>
+      </c>
+      <c r="D95" s="18" t="n">
+        <v>-27136.99</v>
+      </c>
+      <c r="E95" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B96" s="10" t="n">
+        <v>781</v>
+      </c>
+      <c r="C96" s="11" t="inlineStr">
+        <is>
+          <t>production</t>
+        </is>
+      </c>
+      <c r="D96" s="14" t="n">
+        <v>-14491000</v>
+      </c>
+      <c r="E96" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B97" s="15" t="n">
+        <v>781</v>
+      </c>
+      <c r="C97" s="16" t="inlineStr">
+        <is>
+          <t>Cash Balance</t>
+        </is>
+      </c>
+      <c r="D97" s="18" t="n">
+        <v>761225.01</v>
+      </c>
+      <c r="E97" s="16" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E85"/>
+  <autoFilter ref="A1:E97"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update game data: day 782, cash 776869.12, 3-day period 261
</commit_message>
<xml_diff>
--- a/data/supply_chain_game.xlsx
+++ b/data/supply_chain_game.xlsx
@@ -21,15 +21,15 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$262</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$782</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$783</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'资金构成_旧版'!$A$1:$C$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'运营参数_旧版'!$A$9:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'排行榜_旧版'!$A$1:$C$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$97</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$109</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'运营参数'!$A$1:$J$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$217</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$244</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -590,7 +590,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-06T00:41:03+08:00</t>
+          <t>2026-09-06T00:56:03+08:00</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>781</v>
+        <v>782</v>
       </c>
     </row>
     <row r="7">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>679</v>
+        <v>678</v>
       </c>
     </row>
     <row r="8">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>761225.01</v>
+        <v>776869.12</v>
       </c>
     </row>
     <row r="11">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>2194307.82</v>
+        <v>2194976.76</v>
       </c>
     </row>
     <row r="15"/>
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>568</v>
+        <v>553</v>
       </c>
     </row>
     <row r="25">
@@ -861,7 +861,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>61</v>
+        <v>76</v>
       </c>
     </row>
     <row r="33">
@@ -881,7 +881,7 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>61</v>
+        <v>76</v>
       </c>
     </row>
     <row r="35">
@@ -901,7 +901,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>61</v>
+        <v>76</v>
       </c>
     </row>
     <row r="37">
@@ -909,6 +909,9 @@
         <is>
           <t>周期现金变动</t>
         </is>
+      </c>
+      <c r="B37" s="4" t="n">
+        <v>19809.29173992772</v>
       </c>
     </row>
     <row r="38"/>
@@ -970,7 +973,7 @@
         </is>
       </c>
       <c r="B44" s="4" t="n">
-        <v>55619.29624028411</v>
+        <v>55314.9650976595</v>
       </c>
     </row>
     <row r="45"/>
@@ -1168,7 +1171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E217"/>
+  <dimension ref="A1:E244"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5741,8 +5744,575 @@
         <v>761225.01</v>
       </c>
     </row>
+    <row r="218">
+      <c r="A218" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B218" s="10" t="n">
+        <v>782</v>
+      </c>
+      <c r="C218" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D218" s="11" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="E218" s="14" t="n">
+        <v>2971845.88</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B219" s="15" t="n">
+        <v>782</v>
+      </c>
+      <c r="C219" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D219" s="16" t="inlineStr">
+        <is>
+          <t>nicetry</t>
+        </is>
+      </c>
+      <c r="E219" s="18" t="n">
+        <v>2007569.22</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B220" s="10" t="n">
+        <v>782</v>
+      </c>
+      <c r="C220" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D220" s="11" t="inlineStr">
+        <is>
+          <t>group14</t>
+        </is>
+      </c>
+      <c r="E220" s="14" t="n">
+        <v>1974321.18</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B221" s="15" t="n">
+        <v>782</v>
+      </c>
+      <c r="C221" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D221" s="16" t="inlineStr">
+        <is>
+          <t>group7</t>
+        </is>
+      </c>
+      <c r="E221" s="18" t="n">
+        <v>1958372.51</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B222" s="10" t="n">
+        <v>782</v>
+      </c>
+      <c r="C222" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="D222" s="11" t="inlineStr">
+        <is>
+          <t>group15</t>
+        </is>
+      </c>
+      <c r="E222" s="14" t="n">
+        <v>1904638.17</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B223" s="15" t="n">
+        <v>782</v>
+      </c>
+      <c r="C223" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="D223" s="16" t="inlineStr">
+        <is>
+          <t>montesquieu</t>
+        </is>
+      </c>
+      <c r="E223" s="18" t="n">
+        <v>1787628.37</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B224" s="10" t="n">
+        <v>782</v>
+      </c>
+      <c r="C224" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="D224" s="11" t="inlineStr">
+        <is>
+          <t>t24</t>
+        </is>
+      </c>
+      <c r="E224" s="14" t="n">
+        <v>1654082.23</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B225" s="15" t="n">
+        <v>782</v>
+      </c>
+      <c r="C225" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="D225" s="16" t="inlineStr">
+        <is>
+          <t>deepsleep</t>
+        </is>
+      </c>
+      <c r="E225" s="18" t="n">
+        <v>1580386.29</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B226" s="10" t="n">
+        <v>782</v>
+      </c>
+      <c r="C226" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="D226" s="11" t="inlineStr">
+        <is>
+          <t>group8</t>
+        </is>
+      </c>
+      <c r="E226" s="14" t="n">
+        <v>1535458.71</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B227" s="15" t="n">
+        <v>782</v>
+      </c>
+      <c r="C227" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="D227" s="16" t="inlineStr">
+        <is>
+          <t>group9</t>
+        </is>
+      </c>
+      <c r="E227" s="18" t="n">
+        <v>1534732.33</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B228" s="10" t="n">
+        <v>782</v>
+      </c>
+      <c r="C228" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="D228" s="11" t="inlineStr">
+        <is>
+          <t>group2</t>
+        </is>
+      </c>
+      <c r="E228" s="14" t="n">
+        <v>1534043.1</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B229" s="15" t="n">
+        <v>782</v>
+      </c>
+      <c r="C229" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="D229" s="16" t="inlineStr">
+        <is>
+          <t>teamhlly</t>
+        </is>
+      </c>
+      <c r="E229" s="18" t="n">
+        <v>1533947.86</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B230" s="10" t="n">
+        <v>782</v>
+      </c>
+      <c r="C230" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="D230" s="11" t="inlineStr">
+        <is>
+          <t>group25</t>
+        </is>
+      </c>
+      <c r="E230" s="14" t="n">
+        <v>1533887.63</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B231" s="15" t="n">
+        <v>782</v>
+      </c>
+      <c r="C231" s="15" t="n">
+        <v>14</v>
+      </c>
+      <c r="D231" s="16" t="inlineStr">
+        <is>
+          <t>group11</t>
+        </is>
+      </c>
+      <c r="E231" s="18" t="n">
+        <v>1533875.53</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B232" s="10" t="n">
+        <v>782</v>
+      </c>
+      <c r="C232" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="D232" s="11" t="inlineStr">
+        <is>
+          <t>88888888</t>
+        </is>
+      </c>
+      <c r="E232" s="14" t="n">
+        <v>1533853.23</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B233" s="15" t="n">
+        <v>782</v>
+      </c>
+      <c r="C233" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="D233" s="16" t="inlineStr">
+        <is>
+          <t>aaachemicalseller</t>
+        </is>
+      </c>
+      <c r="E233" s="18" t="n">
+        <v>1468017.46</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B234" s="10" t="n">
+        <v>782</v>
+      </c>
+      <c r="C234" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="D234" s="11" t="inlineStr">
+        <is>
+          <t>group12</t>
+        </is>
+      </c>
+      <c r="E234" s="14" t="n">
+        <v>1466722.02</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B235" s="15" t="n">
+        <v>782</v>
+      </c>
+      <c r="C235" s="15" t="n">
+        <v>18</v>
+      </c>
+      <c r="D235" s="16" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E235" s="18" t="n">
+        <v>1426749.21</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B236" s="10" t="n">
+        <v>782</v>
+      </c>
+      <c r="C236" s="10" t="n">
+        <v>19</v>
+      </c>
+      <c r="D236" s="11" t="inlineStr">
+        <is>
+          <t>666666</t>
+        </is>
+      </c>
+      <c r="E236" s="14" t="n">
+        <v>1381659.75</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B237" s="15" t="n">
+        <v>782</v>
+      </c>
+      <c r="C237" s="15" t="n">
+        <v>20</v>
+      </c>
+      <c r="D237" s="16" t="inlineStr">
+        <is>
+          <t>cleveregg</t>
+        </is>
+      </c>
+      <c r="E237" s="18" t="n">
+        <v>1229498.85</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B238" s="10" t="n">
+        <v>782</v>
+      </c>
+      <c r="C238" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="D238" s="11" t="inlineStr">
+        <is>
+          <t>tigagroup20</t>
+        </is>
+      </c>
+      <c r="E238" s="14" t="n">
+        <v>1216880</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B239" s="15" t="n">
+        <v>782</v>
+      </c>
+      <c r="C239" s="15" t="n">
+        <v>22</v>
+      </c>
+      <c r="D239" s="16" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="E239" s="18" t="n">
+        <v>1146752.61</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B240" s="10" t="n">
+        <v>782</v>
+      </c>
+      <c r="C240" s="10" t="n">
+        <v>23</v>
+      </c>
+      <c r="D240" s="11" t="inlineStr">
+        <is>
+          <t>jit</t>
+        </is>
+      </c>
+      <c r="E240" s="14" t="n">
+        <v>1070395.93</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B241" s="15" t="n">
+        <v>782</v>
+      </c>
+      <c r="C241" s="15" t="n">
+        <v>24</v>
+      </c>
+      <c r="D241" s="16" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E241" s="18" t="n">
+        <v>1031991.65</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B242" s="10" t="n">
+        <v>782</v>
+      </c>
+      <c r="C242" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="D242" s="11" t="inlineStr">
+        <is>
+          <t>vivo50</t>
+        </is>
+      </c>
+      <c r="E242" s="14" t="n">
+        <v>1027248.76</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B243" s="15" t="n">
+        <v>782</v>
+      </c>
+      <c r="C243" s="15" t="n">
+        <v>26</v>
+      </c>
+      <c r="D243" s="16" t="inlineStr">
+        <is>
+          <t>newgroup18</t>
+        </is>
+      </c>
+      <c r="E243" s="18" t="n">
+        <v>928098.39</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B244" s="24" t="n">
+        <v>782</v>
+      </c>
+      <c r="C244" s="24" t="n">
+        <v>27</v>
+      </c>
+      <c r="D244" s="25" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="E244" s="26" t="n">
+        <v>776869.12</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E217"/>
+  <autoFilter ref="A1:E244"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -22265,7 +22835,7 @@
         <v>783</v>
       </c>
       <c r="D262" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E262" s="11" t="inlineStr">
         <is>
@@ -22278,32 +22848,34 @@
         </is>
       </c>
       <c r="G262" s="12" t="n">
-        <v>61</v>
+        <v>76</v>
       </c>
       <c r="H262" s="12" t="n">
         <v>0</v>
       </c>
       <c r="I262" s="12" t="n">
-        <v>61</v>
+        <v>76</v>
       </c>
       <c r="J262" s="19" t="n">
         <v>1</v>
       </c>
       <c r="K262" s="12" t="n">
-        <v>61</v>
+        <v>76</v>
       </c>
       <c r="L262" s="14" t="n">
-        <v>761225.01</v>
+        <v>757059.8282600723</v>
       </c>
       <c r="M262" s="14" t="n">
-        <v>761225.01</v>
-      </c>
-      <c r="N262" s="11" t="n"/>
+        <v>776869.12</v>
+      </c>
+      <c r="N262" s="14" t="n">
+        <v>19809.29173992772</v>
+      </c>
       <c r="O262" s="12" t="n">
-        <v>568</v>
+        <v>553</v>
       </c>
       <c r="P262" s="12" t="n">
-        <v>568</v>
+        <v>560.5</v>
       </c>
       <c r="Q262" s="12" t="n">
         <v>0</v>
@@ -22312,7 +22884,7 @@
         <v>200</v>
       </c>
       <c r="S262" s="14" t="n">
-        <v>88450</v>
+        <v>110200</v>
       </c>
     </row>
   </sheetData>
@@ -22327,7 +22899,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N782"/>
+  <dimension ref="A1:N783"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -58344,8 +58916,54 @@
         <v>88450</v>
       </c>
     </row>
+    <row r="783">
+      <c r="A783" s="15" t="n">
+        <v>782</v>
+      </c>
+      <c r="B783" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C783" s="17" t="n">
+        <v>15</v>
+      </c>
+      <c r="D783" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E783" s="17" t="n">
+        <v>15</v>
+      </c>
+      <c r="F783" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G783" s="17" t="n">
+        <v>15</v>
+      </c>
+      <c r="H783" s="18" t="n">
+        <v>776869.12</v>
+      </c>
+      <c r="I783" s="17" t="n">
+        <v>553</v>
+      </c>
+      <c r="J783" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K783" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L783" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M783" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N783" s="18" t="n">
+        <v>21750</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N782"/>
+  <autoFilter ref="A1:N783"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -58740,7 +59358,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -59199,8 +59817,56 @@
         <v>55</v>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="23" t="n">
+        <v>730.66</v>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E19" s="16" t="inlineStr"/>
+      <c r="F19" s="17" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="21" t="n">
+        <v>742.75</v>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr"/>
+      <c r="F20" s="12" t="n">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F18"/>
+  <autoFilter ref="A1:F20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -59599,7 +60265,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U9"/>
+  <dimension ref="A1:U10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -59608,7 +60274,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
@@ -60292,8 +60958,79 @@
       </c>
       <c r="U9" s="16" t="n"/>
     </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="n">
+        <v>782</v>
+      </c>
+      <c r="C10" s="14" t="n">
+        <v>776869.12</v>
+      </c>
+      <c r="D10" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="E10" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="G10" s="14" t="n">
+        <v>2194976.76</v>
+      </c>
+      <c r="H10" s="21" t="n">
+        <v>20</v>
+      </c>
+      <c r="I10" s="21" t="n">
+        <v>55</v>
+      </c>
+      <c r="J10" s="11" t="inlineStr">
+        <is>
+          <t>truck</t>
+        </is>
+      </c>
+      <c r="K10" s="22" t="n">
+        <v>3600</v>
+      </c>
+      <c r="L10" s="22" t="n">
+        <v>200</v>
+      </c>
+      <c r="M10" s="12" t="n">
+        <v>553</v>
+      </c>
+      <c r="N10" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="P10" s="10" t="n">
+        <v>261</v>
+      </c>
+      <c r="Q10" s="12" t="n">
+        <v>76</v>
+      </c>
+      <c r="R10" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S10" s="12" t="n">
+        <v>76</v>
+      </c>
+      <c r="T10" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="U10" s="14" t="n">
+        <v>19809.29173992772</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U9"/>
+  <autoFilter ref="A1:U10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -60304,7 +61041,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E97"/>
+  <dimension ref="A1:E109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -62517,8 +63254,280 @@
         </is>
       </c>
     </row>
+    <row r="98">
+      <c r="A98" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B98" s="10" t="n">
+        <v>782</v>
+      </c>
+      <c r="C98" s="11" t="inlineStr">
+        <is>
+          <t>Starting Cash</t>
+        </is>
+      </c>
+      <c r="D98" s="14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E98" s="11" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B99" s="15" t="n">
+        <v>782</v>
+      </c>
+      <c r="C99" s="16" t="inlineStr">
+        <is>
+          <t>Cash Sources</t>
+        </is>
+      </c>
+      <c r="D99" s="16" t="n"/>
+      <c r="E99" s="16" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B100" s="10" t="n">
+        <v>782</v>
+      </c>
+      <c r="C100" s="11" t="inlineStr">
+        <is>
+          <t>revenues</t>
+        </is>
+      </c>
+      <c r="D100" s="14" t="n">
+        <v>19727250</v>
+      </c>
+      <c r="E100" s="11" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B101" s="15" t="n">
+        <v>782</v>
+      </c>
+      <c r="C101" s="16" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D101" s="18" t="n">
+        <v>285979.17</v>
+      </c>
+      <c r="E101" s="16" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B102" s="10" t="n">
+        <v>782</v>
+      </c>
+      <c r="C102" s="11" t="inlineStr">
+        <is>
+          <t>Cash Uses</t>
+        </is>
+      </c>
+      <c r="D102" s="11" t="n"/>
+      <c r="E102" s="11" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B103" s="15" t="n">
+        <v>782</v>
+      </c>
+      <c r="C103" s="16" t="inlineStr">
+        <is>
+          <t>outbound shipping</t>
+        </is>
+      </c>
+      <c r="D103" s="18" t="n">
+        <v>-2040750</v>
+      </c>
+      <c r="E103" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B104" s="10" t="n">
+        <v>782</v>
+      </c>
+      <c r="C104" s="11" t="inlineStr">
+        <is>
+          <t>inbound shipping</t>
+        </is>
+      </c>
+      <c r="D104" s="14" t="n">
+        <v>-1410000</v>
+      </c>
+      <c r="E104" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B105" s="15" t="n">
+        <v>782</v>
+      </c>
+      <c r="C105" s="16" t="inlineStr">
+        <is>
+          <t>FGI holding</t>
+        </is>
+      </c>
+      <c r="D105" s="18" t="n">
+        <v>-17632.2</v>
+      </c>
+      <c r="E105" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B106" s="10" t="n">
+        <v>782</v>
+      </c>
+      <c r="C106" s="11" t="inlineStr">
+        <is>
+          <t>add capacity</t>
+        </is>
+      </c>
+      <c r="D106" s="14" t="n">
+        <v>-1749840.87</v>
+      </c>
+      <c r="E106" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B107" s="15" t="n">
+        <v>782</v>
+      </c>
+      <c r="C107" s="16" t="inlineStr">
+        <is>
+          <t>Pipeline inventory holding</t>
+        </is>
+      </c>
+      <c r="D107" s="18" t="n">
+        <v>-27136.99</v>
+      </c>
+      <c r="E107" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B108" s="10" t="n">
+        <v>782</v>
+      </c>
+      <c r="C108" s="11" t="inlineStr">
+        <is>
+          <t>production</t>
+        </is>
+      </c>
+      <c r="D108" s="14" t="n">
+        <v>-14491000</v>
+      </c>
+      <c r="E108" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T00:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B109" s="15" t="n">
+        <v>782</v>
+      </c>
+      <c r="C109" s="16" t="inlineStr">
+        <is>
+          <t>Cash Balance</t>
+        </is>
+      </c>
+      <c r="D109" s="18" t="n">
+        <v>776869.12</v>
+      </c>
+      <c r="E109" s="16" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E97"/>
+  <autoFilter ref="A1:E109"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update game data: day 783, cash 791222.75, 3-day period 261
</commit_message>
<xml_diff>
--- a/data/supply_chain_game.xlsx
+++ b/data/supply_chain_game.xlsx
@@ -21,15 +21,15 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$262</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$783</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$784</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'资金构成_旧版'!$A$1:$C$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'运营参数_旧版'!$A$9:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'排行榜_旧版'!$A$1:$C$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$109</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$121</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'运营参数'!$A$1:$J$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$244</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$271</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -590,7 +590,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-06T00:56:03+08:00</t>
+          <t>2026-09-06T01:11:02+08:00</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>782</v>
+        <v>783</v>
       </c>
     </row>
     <row r="7">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="8">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>776869.12</v>
+        <v>791222.75</v>
       </c>
     </row>
     <row r="11">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>2194976.76</v>
+        <v>2195645.89</v>
       </c>
     </row>
     <row r="15"/>
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>553</v>
+        <v>540</v>
       </c>
     </row>
     <row r="25">
@@ -850,7 +850,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>否（进行中）</t>
+          <t>是</t>
         </is>
       </c>
     </row>
@@ -861,7 +861,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>76</v>
+        <v>89</v>
       </c>
     </row>
     <row r="33">
@@ -881,7 +881,7 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>76</v>
+        <v>89</v>
       </c>
     </row>
     <row r="35">
@@ -901,7 +901,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>76</v>
+        <v>89</v>
       </c>
     </row>
     <row r="37">
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="B37" s="4" t="n">
-        <v>19809.29173992772</v>
+        <v>36861.11894596298</v>
       </c>
     </row>
     <row r="38"/>
@@ -929,7 +929,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="41">
@@ -940,7 +940,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>778–780</t>
+          <t>781–783</t>
         </is>
       </c>
     </row>
@@ -952,7 +952,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>51.0 / 0.0 / 51.0</t>
+          <t>89.0 / 0.0 / 89.0</t>
         </is>
       </c>
     </row>
@@ -973,7 +973,7 @@
         </is>
       </c>
       <c r="B44" s="4" t="n">
-        <v>55314.9650976595</v>
+        <v>36861.11894596298</v>
       </c>
     </row>
     <row r="45"/>
@@ -1171,7 +1171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E244"/>
+  <dimension ref="A1:E271"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -6311,8 +6311,575 @@
         <v>776869.12</v>
       </c>
     </row>
+    <row r="245">
+      <c r="A245" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B245" s="15" t="n">
+        <v>783</v>
+      </c>
+      <c r="C245" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D245" s="16" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="E245" s="18" t="n">
+        <v>2986868.64</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B246" s="10" t="n">
+        <v>783</v>
+      </c>
+      <c r="C246" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D246" s="11" t="inlineStr">
+        <is>
+          <t>nicetry</t>
+        </is>
+      </c>
+      <c r="E246" s="14" t="n">
+        <v>2022299.05</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B247" s="15" t="n">
+        <v>783</v>
+      </c>
+      <c r="C247" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D247" s="16" t="inlineStr">
+        <is>
+          <t>group14</t>
+        </is>
+      </c>
+      <c r="E247" s="18" t="n">
+        <v>1989097.12</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B248" s="10" t="n">
+        <v>783</v>
+      </c>
+      <c r="C248" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D248" s="11" t="inlineStr">
+        <is>
+          <t>group7</t>
+        </is>
+      </c>
+      <c r="E248" s="14" t="n">
+        <v>1973130.59</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B249" s="15" t="n">
+        <v>783</v>
+      </c>
+      <c r="C249" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="D249" s="16" t="inlineStr">
+        <is>
+          <t>group15</t>
+        </is>
+      </c>
+      <c r="E249" s="18" t="n">
+        <v>1905080.79</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B250" s="10" t="n">
+        <v>783</v>
+      </c>
+      <c r="C250" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="D250" s="11" t="inlineStr">
+        <is>
+          <t>t24</t>
+        </is>
+      </c>
+      <c r="E250" s="14" t="n">
+        <v>1668719.75</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B251" s="15" t="n">
+        <v>783</v>
+      </c>
+      <c r="C251" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="D251" s="16" t="inlineStr">
+        <is>
+          <t>montesquieu</t>
+        </is>
+      </c>
+      <c r="E251" s="18" t="n">
+        <v>1585745.97</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B252" s="10" t="n">
+        <v>783</v>
+      </c>
+      <c r="C252" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="D252" s="11" t="inlineStr">
+        <is>
+          <t>group8</t>
+        </is>
+      </c>
+      <c r="E252" s="14" t="n">
+        <v>1550010.45</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B253" s="15" t="n">
+        <v>783</v>
+      </c>
+      <c r="C253" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="D253" s="16" t="inlineStr">
+        <is>
+          <t>group9</t>
+        </is>
+      </c>
+      <c r="E253" s="18" t="n">
+        <v>1549283.88</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B254" s="10" t="n">
+        <v>783</v>
+      </c>
+      <c r="C254" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="D254" s="11" t="inlineStr">
+        <is>
+          <t>teamhlly</t>
+        </is>
+      </c>
+      <c r="E254" s="14" t="n">
+        <v>1548499.21</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B255" s="15" t="n">
+        <v>783</v>
+      </c>
+      <c r="C255" s="15" t="n">
+        <v>11</v>
+      </c>
+      <c r="D255" s="16" t="inlineStr">
+        <is>
+          <t>aaachemicalseller</t>
+        </is>
+      </c>
+      <c r="E255" s="18" t="n">
+        <v>1482661.18</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B256" s="10" t="n">
+        <v>783</v>
+      </c>
+      <c r="C256" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="D256" s="11" t="inlineStr">
+        <is>
+          <t>group12</t>
+        </is>
+      </c>
+      <c r="E256" s="14" t="n">
+        <v>1481365.4</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B257" s="15" t="n">
+        <v>783</v>
+      </c>
+      <c r="C257" s="15" t="n">
+        <v>13</v>
+      </c>
+      <c r="D257" s="16" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E257" s="18" t="n">
+        <v>1441373.38</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B258" s="10" t="n">
+        <v>783</v>
+      </c>
+      <c r="C258" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="D258" s="11" t="inlineStr">
+        <is>
+          <t>deepsleep</t>
+        </is>
+      </c>
+      <c r="E258" s="14" t="n">
+        <v>1398517.85</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B259" s="15" t="n">
+        <v>783</v>
+      </c>
+      <c r="C259" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="D259" s="16" t="inlineStr">
+        <is>
+          <t>group2</t>
+        </is>
+      </c>
+      <c r="E259" s="18" t="n">
+        <v>1332094.47</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B260" s="10" t="n">
+        <v>783</v>
+      </c>
+      <c r="C260" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="D260" s="11" t="inlineStr">
+        <is>
+          <t>group25</t>
+        </is>
+      </c>
+      <c r="E260" s="14" t="n">
+        <v>1331938.97</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B261" s="15" t="n">
+        <v>783</v>
+      </c>
+      <c r="C261" s="15" t="n">
+        <v>17</v>
+      </c>
+      <c r="D261" s="16" t="inlineStr">
+        <is>
+          <t>group11</t>
+        </is>
+      </c>
+      <c r="E261" s="18" t="n">
+        <v>1331926.86</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B262" s="10" t="n">
+        <v>783</v>
+      </c>
+      <c r="C262" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="D262" s="11" t="inlineStr">
+        <is>
+          <t>88888888</t>
+        </is>
+      </c>
+      <c r="E262" s="14" t="n">
+        <v>1331904.55</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B263" s="15" t="n">
+        <v>783</v>
+      </c>
+      <c r="C263" s="15" t="n">
+        <v>19</v>
+      </c>
+      <c r="D263" s="16" t="inlineStr">
+        <is>
+          <t>tigagroup20</t>
+        </is>
+      </c>
+      <c r="E263" s="18" t="n">
+        <v>1231348.55</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B264" s="10" t="n">
+        <v>783</v>
+      </c>
+      <c r="C264" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="D264" s="11" t="inlineStr">
+        <is>
+          <t>666666</t>
+        </is>
+      </c>
+      <c r="E264" s="14" t="n">
+        <v>1179671.33</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B265" s="15" t="n">
+        <v>783</v>
+      </c>
+      <c r="C265" s="15" t="n">
+        <v>21</v>
+      </c>
+      <c r="D265" s="16" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="E265" s="18" t="n">
+        <v>1161341.87</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B266" s="10" t="n">
+        <v>783</v>
+      </c>
+      <c r="C266" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="D266" s="11" t="inlineStr">
+        <is>
+          <t>jit</t>
+        </is>
+      </c>
+      <c r="E266" s="14" t="n">
+        <v>1084826.22</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B267" s="15" t="n">
+        <v>783</v>
+      </c>
+      <c r="C267" s="15" t="n">
+        <v>23</v>
+      </c>
+      <c r="D267" s="16" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E267" s="18" t="n">
+        <v>1046411.91</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B268" s="10" t="n">
+        <v>783</v>
+      </c>
+      <c r="C268" s="10" t="n">
+        <v>24</v>
+      </c>
+      <c r="D268" s="11" t="inlineStr">
+        <is>
+          <t>vivo50</t>
+        </is>
+      </c>
+      <c r="E268" s="14" t="n">
+        <v>1041667.78</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B269" s="15" t="n">
+        <v>783</v>
+      </c>
+      <c r="C269" s="15" t="n">
+        <v>25</v>
+      </c>
+      <c r="D269" s="16" t="inlineStr">
+        <is>
+          <t>cleveregg</t>
+        </is>
+      </c>
+      <c r="E269" s="18" t="n">
+        <v>1027470.69</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B270" s="10" t="n">
+        <v>783</v>
+      </c>
+      <c r="C270" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="D270" s="11" t="inlineStr">
+        <is>
+          <t>newgroup18</t>
+        </is>
+      </c>
+      <c r="E270" s="14" t="n">
+        <v>942458.64</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B271" s="24" t="n">
+        <v>783</v>
+      </c>
+      <c r="C271" s="24" t="n">
+        <v>27</v>
+      </c>
+      <c r="D271" s="25" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="E271" s="26" t="n">
+        <v>791222.75</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E244"/>
+  <autoFilter ref="A1:E271"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -22835,11 +23402,11 @@
         <v>783</v>
       </c>
       <c r="D262" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E262" s="11" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="F262" s="11" t="inlineStr">
@@ -22848,34 +23415,34 @@
         </is>
       </c>
       <c r="G262" s="12" t="n">
-        <v>76</v>
+        <v>89</v>
       </c>
       <c r="H262" s="12" t="n">
         <v>0</v>
       </c>
       <c r="I262" s="12" t="n">
-        <v>76</v>
+        <v>89</v>
       </c>
       <c r="J262" s="19" t="n">
         <v>1</v>
       </c>
       <c r="K262" s="12" t="n">
-        <v>76</v>
+        <v>89</v>
       </c>
       <c r="L262" s="14" t="n">
-        <v>757059.8282600723</v>
+        <v>754361.631054037</v>
       </c>
       <c r="M262" s="14" t="n">
-        <v>776869.12</v>
+        <v>791222.75</v>
       </c>
       <c r="N262" s="14" t="n">
-        <v>19809.29173992772</v>
+        <v>36861.11894596298</v>
       </c>
       <c r="O262" s="12" t="n">
-        <v>553</v>
+        <v>540</v>
       </c>
       <c r="P262" s="12" t="n">
-        <v>560.5</v>
+        <v>553.6666666666666</v>
       </c>
       <c r="Q262" s="12" t="n">
         <v>0</v>
@@ -22884,7 +23451,7 @@
         <v>200</v>
       </c>
       <c r="S262" s="14" t="n">
-        <v>110200</v>
+        <v>129050</v>
       </c>
     </row>
   </sheetData>
@@ -22899,7 +23466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N783"/>
+  <dimension ref="A1:N784"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -58962,8 +59529,54 @@
         <v>21750</v>
       </c>
     </row>
+    <row r="784">
+      <c r="A784" s="10" t="n">
+        <v>783</v>
+      </c>
+      <c r="B784" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C784" s="12" t="n">
+        <v>13</v>
+      </c>
+      <c r="D784" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E784" s="12" t="n">
+        <v>13</v>
+      </c>
+      <c r="F784" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G784" s="12" t="n">
+        <v>13</v>
+      </c>
+      <c r="H784" s="14" t="n">
+        <v>791222.75</v>
+      </c>
+      <c r="I784" s="12" t="n">
+        <v>540</v>
+      </c>
+      <c r="J784" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K784" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L784" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M784" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N784" s="14" t="n">
+        <v>18850</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N783"/>
+  <autoFilter ref="A1:N784"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -59358,7 +59971,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -59865,8 +60478,56 @@
         <v>55</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="23" t="n">
+        <v>730.66</v>
+      </c>
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C21" s="16" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D21" s="16" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E21" s="16" t="inlineStr"/>
+      <c r="F21" s="17" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="21" t="n">
+        <v>742.75</v>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D22" s="11" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E22" s="11" t="inlineStr"/>
+      <c r="F22" s="12" t="n">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F20"/>
+  <autoFilter ref="A1:F22"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -60265,7 +60926,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U10"/>
+  <dimension ref="A1:U11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -61029,8 +61690,79 @@
         <v>19809.29173992772</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="n">
+        <v>783</v>
+      </c>
+      <c r="C11" s="18" t="n">
+        <v>791222.75</v>
+      </c>
+      <c r="D11" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="E11" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="G11" s="18" t="n">
+        <v>2195645.89</v>
+      </c>
+      <c r="H11" s="23" t="n">
+        <v>20</v>
+      </c>
+      <c r="I11" s="23" t="n">
+        <v>55</v>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>truck</t>
+        </is>
+      </c>
+      <c r="K11" s="27" t="n">
+        <v>3600</v>
+      </c>
+      <c r="L11" s="27" t="n">
+        <v>200</v>
+      </c>
+      <c r="M11" s="17" t="n">
+        <v>540</v>
+      </c>
+      <c r="N11" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="P11" s="15" t="n">
+        <v>261</v>
+      </c>
+      <c r="Q11" s="17" t="n">
+        <v>89</v>
+      </c>
+      <c r="R11" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="S11" s="17" t="n">
+        <v>89</v>
+      </c>
+      <c r="T11" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="U11" s="18" t="n">
+        <v>36861.11894596298</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U10"/>
+  <autoFilter ref="A1:U11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -61041,7 +61773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E109"/>
+  <dimension ref="A1:E121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -63526,8 +64258,280 @@
         </is>
       </c>
     </row>
+    <row r="110">
+      <c r="A110" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B110" s="10" t="n">
+        <v>783</v>
+      </c>
+      <c r="C110" s="11" t="inlineStr">
+        <is>
+          <t>Starting Cash</t>
+        </is>
+      </c>
+      <c r="D110" s="14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E110" s="11" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B111" s="15" t="n">
+        <v>783</v>
+      </c>
+      <c r="C111" s="16" t="inlineStr">
+        <is>
+          <t>Cash Sources</t>
+        </is>
+      </c>
+      <c r="D111" s="16" t="n"/>
+      <c r="E111" s="16" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B112" s="10" t="n">
+        <v>783</v>
+      </c>
+      <c r="C112" s="11" t="inlineStr">
+        <is>
+          <t>revenues</t>
+        </is>
+      </c>
+      <c r="D112" s="14" t="n">
+        <v>19743200</v>
+      </c>
+      <c r="E112" s="11" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B113" s="15" t="n">
+        <v>783</v>
+      </c>
+      <c r="C113" s="16" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D113" s="18" t="n">
+        <v>286182.09</v>
+      </c>
+      <c r="E113" s="16" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B114" s="10" t="n">
+        <v>783</v>
+      </c>
+      <c r="C114" s="11" t="inlineStr">
+        <is>
+          <t>Cash Uses</t>
+        </is>
+      </c>
+      <c r="D114" s="11" t="n"/>
+      <c r="E114" s="11" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B115" s="15" t="n">
+        <v>783</v>
+      </c>
+      <c r="C115" s="16" t="inlineStr">
+        <is>
+          <t>outbound shipping</t>
+        </is>
+      </c>
+      <c r="D115" s="18" t="n">
+        <v>-2042400</v>
+      </c>
+      <c r="E115" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B116" s="10" t="n">
+        <v>783</v>
+      </c>
+      <c r="C116" s="11" t="inlineStr">
+        <is>
+          <t>inbound shipping</t>
+        </is>
+      </c>
+      <c r="D116" s="14" t="n">
+        <v>-1410000</v>
+      </c>
+      <c r="E116" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B117" s="15" t="n">
+        <v>783</v>
+      </c>
+      <c r="C117" s="16" t="inlineStr">
+        <is>
+          <t>FGI holding</t>
+        </is>
+      </c>
+      <c r="D117" s="18" t="n">
+        <v>-17781.49</v>
+      </c>
+      <c r="E117" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B118" s="10" t="n">
+        <v>783</v>
+      </c>
+      <c r="C118" s="11" t="inlineStr">
+        <is>
+          <t>add capacity</t>
+        </is>
+      </c>
+      <c r="D118" s="14" t="n">
+        <v>-1749840.87</v>
+      </c>
+      <c r="E118" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B119" s="15" t="n">
+        <v>783</v>
+      </c>
+      <c r="C119" s="16" t="inlineStr">
+        <is>
+          <t>Pipeline inventory holding</t>
+        </is>
+      </c>
+      <c r="D119" s="18" t="n">
+        <v>-27136.99</v>
+      </c>
+      <c r="E119" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B120" s="10" t="n">
+        <v>783</v>
+      </c>
+      <c r="C120" s="11" t="inlineStr">
+        <is>
+          <t>production</t>
+        </is>
+      </c>
+      <c r="D120" s="14" t="n">
+        <v>-14491000</v>
+      </c>
+      <c r="E120" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B121" s="15" t="n">
+        <v>783</v>
+      </c>
+      <c r="C121" s="16" t="inlineStr">
+        <is>
+          <t>Cash Balance</t>
+        </is>
+      </c>
+      <c r="D121" s="18" t="n">
+        <v>791222.75</v>
+      </c>
+      <c r="E121" s="16" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E109"/>
+  <autoFilter ref="A1:E121"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update game data: day 784, cash 598181.96, 3-day period 262
</commit_message>
<xml_diff>
--- a/data/supply_chain_game.xlsx
+++ b/data/supply_chain_game.xlsx
@@ -20,16 +20,16 @@
     <sheet name="排行榜" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$262</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$784</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$263</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$785</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'资金构成_旧版'!$A$1:$C$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'运营参数_旧版'!$A$9:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'排行榜_旧版'!$A$1:$C$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$121</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$133</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'运营参数'!$A$1:$J$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$271</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$298</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -590,7 +590,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-06T01:11:02+08:00</t>
+          <t>2026-09-06T01:26:02+08:00</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>783</v>
+        <v>784</v>
       </c>
     </row>
     <row r="7">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>677</v>
+        <v>676</v>
       </c>
     </row>
     <row r="8">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>791222.75</v>
+        <v>598181.96</v>
       </c>
     </row>
     <row r="11">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>2195645.89</v>
+        <v>2412815.2</v>
       </c>
     </row>
     <row r="15"/>
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>540</v>
+        <v>532</v>
       </c>
     </row>
     <row r="25">
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
     </row>
     <row r="26">
@@ -827,7 +827,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="30">
@@ -838,7 +838,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>781–783</t>
+          <t>784–786</t>
         </is>
       </c>
     </row>
@@ -850,7 +850,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否（进行中）</t>
         </is>
       </c>
     </row>
@@ -861,7 +861,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>89</v>
+        <v>8</v>
       </c>
     </row>
     <row r="33">
@@ -881,7 +881,7 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>89</v>
+        <v>8</v>
       </c>
     </row>
     <row r="35">
@@ -901,7 +901,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>89</v>
+        <v>8</v>
       </c>
     </row>
     <row r="37">
@@ -909,9 +909,6 @@
         <is>
           <t>周期现金变动</t>
         </is>
-      </c>
-      <c r="B37" s="4" t="n">
-        <v>36861.11894596298</v>
       </c>
     </row>
     <row r="38"/>
@@ -973,7 +970,7 @@
         </is>
       </c>
       <c r="B44" s="4" t="n">
-        <v>36861.11894596298</v>
+        <v>37812.55512617959</v>
       </c>
     </row>
     <row r="45"/>
@@ -1171,7 +1168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E271"/>
+  <dimension ref="A1:E298"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -6878,8 +6875,575 @@
         <v>791222.75</v>
       </c>
     </row>
+    <row r="272">
+      <c r="A272" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B272" s="10" t="n">
+        <v>784</v>
+      </c>
+      <c r="C272" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D272" s="11" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="E272" s="14" t="n">
+        <v>3010997.16</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B273" s="15" t="n">
+        <v>784</v>
+      </c>
+      <c r="C273" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D273" s="16" t="inlineStr">
+        <is>
+          <t>nicetry</t>
+        </is>
+      </c>
+      <c r="E273" s="18" t="n">
+        <v>2046134.57</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B274" s="10" t="n">
+        <v>784</v>
+      </c>
+      <c r="C274" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D274" s="11" t="inlineStr">
+        <is>
+          <t>group14</t>
+        </is>
+      </c>
+      <c r="E274" s="14" t="n">
+        <v>2012978.76</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B275" s="15" t="n">
+        <v>784</v>
+      </c>
+      <c r="C275" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D275" s="16" t="inlineStr">
+        <is>
+          <t>group7</t>
+        </is>
+      </c>
+      <c r="E275" s="18" t="n">
+        <v>1996994.36</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B276" s="10" t="n">
+        <v>784</v>
+      </c>
+      <c r="C276" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="D276" s="11" t="inlineStr">
+        <is>
+          <t>group15</t>
+        </is>
+      </c>
+      <c r="E276" s="14" t="n">
+        <v>1905523.52</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B277" s="15" t="n">
+        <v>784</v>
+      </c>
+      <c r="C277" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="D277" s="16" t="inlineStr">
+        <is>
+          <t>t24</t>
+        </is>
+      </c>
+      <c r="E277" s="18" t="n">
+        <v>1692462.93</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B278" s="10" t="n">
+        <v>784</v>
+      </c>
+      <c r="C278" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="D278" s="11" t="inlineStr">
+        <is>
+          <t>montesquieu</t>
+        </is>
+      </c>
+      <c r="E278" s="14" t="n">
+        <v>1609371.19</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B279" s="15" t="n">
+        <v>784</v>
+      </c>
+      <c r="C279" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="D279" s="16" t="inlineStr">
+        <is>
+          <t>group8</t>
+        </is>
+      </c>
+      <c r="E279" s="18" t="n">
+        <v>1573667.83</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B280" s="10" t="n">
+        <v>784</v>
+      </c>
+      <c r="C280" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="D280" s="11" t="inlineStr">
+        <is>
+          <t>group9</t>
+        </is>
+      </c>
+      <c r="E280" s="14" t="n">
+        <v>1572941.07</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B281" s="15" t="n">
+        <v>784</v>
+      </c>
+      <c r="C281" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="D281" s="16" t="inlineStr">
+        <is>
+          <t>aaachemicalseller</t>
+        </is>
+      </c>
+      <c r="E281" s="18" t="n">
+        <v>1506410.56</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B282" s="10" t="n">
+        <v>784</v>
+      </c>
+      <c r="C282" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="D282" s="11" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E282" s="14" t="n">
+        <v>1465103.21</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B283" s="15" t="n">
+        <v>784</v>
+      </c>
+      <c r="C283" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="D283" s="16" t="inlineStr">
+        <is>
+          <t>deepsleep</t>
+        </is>
+      </c>
+      <c r="E283" s="18" t="n">
+        <v>1422157.58</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B284" s="10" t="n">
+        <v>784</v>
+      </c>
+      <c r="C284" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="D284" s="11" t="inlineStr">
+        <is>
+          <t>group2</t>
+        </is>
+      </c>
+      <c r="E284" s="14" t="n">
+        <v>1355653.44</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B285" s="15" t="n">
+        <v>784</v>
+      </c>
+      <c r="C285" s="15" t="n">
+        <v>14</v>
+      </c>
+      <c r="D285" s="16" t="inlineStr">
+        <is>
+          <t>teamhlly</t>
+        </is>
+      </c>
+      <c r="E285" s="18" t="n">
+        <v>1355652.71</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B286" s="10" t="n">
+        <v>784</v>
+      </c>
+      <c r="C286" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="D286" s="11" t="inlineStr">
+        <is>
+          <t>group25</t>
+        </is>
+      </c>
+      <c r="E286" s="14" t="n">
+        <v>1355497.9</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B287" s="15" t="n">
+        <v>784</v>
+      </c>
+      <c r="C287" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="D287" s="16" t="inlineStr">
+        <is>
+          <t>group11</t>
+        </is>
+      </c>
+      <c r="E287" s="18" t="n">
+        <v>1355485.79</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B288" s="10" t="n">
+        <v>784</v>
+      </c>
+      <c r="C288" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="D288" s="11" t="inlineStr">
+        <is>
+          <t>88888888</t>
+        </is>
+      </c>
+      <c r="E288" s="14" t="n">
+        <v>1355463.47</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B289" s="15" t="n">
+        <v>784</v>
+      </c>
+      <c r="C289" s="15" t="n">
+        <v>18</v>
+      </c>
+      <c r="D289" s="16" t="inlineStr">
+        <is>
+          <t>group12</t>
+        </is>
+      </c>
+      <c r="E289" s="18" t="n">
+        <v>1288610.96</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B290" s="10" t="n">
+        <v>784</v>
+      </c>
+      <c r="C290" s="10" t="n">
+        <v>19</v>
+      </c>
+      <c r="D290" s="11" t="inlineStr">
+        <is>
+          <t>tigagroup20</t>
+        </is>
+      </c>
+      <c r="E290" s="14" t="n">
+        <v>1254922.71</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B291" s="15" t="n">
+        <v>784</v>
+      </c>
+      <c r="C291" s="15" t="n">
+        <v>20</v>
+      </c>
+      <c r="D291" s="16" t="inlineStr">
+        <is>
+          <t>666666</t>
+        </is>
+      </c>
+      <c r="E291" s="18" t="n">
+        <v>1203190.49</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B292" s="10" t="n">
+        <v>784</v>
+      </c>
+      <c r="C292" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="D292" s="11" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="E292" s="14" t="n">
+        <v>1185021.03</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B293" s="15" t="n">
+        <v>784</v>
+      </c>
+      <c r="C293" s="15" t="n">
+        <v>22</v>
+      </c>
+      <c r="D293" s="16" t="inlineStr">
+        <is>
+          <t>jit</t>
+        </is>
+      </c>
+      <c r="E293" s="18" t="n">
+        <v>1108362.11</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B294" s="10" t="n">
+        <v>784</v>
+      </c>
+      <c r="C294" s="10" t="n">
+        <v>23</v>
+      </c>
+      <c r="D294" s="11" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E294" s="14" t="n">
+        <v>1069937.77</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B295" s="15" t="n">
+        <v>784</v>
+      </c>
+      <c r="C295" s="15" t="n">
+        <v>24</v>
+      </c>
+      <c r="D295" s="16" t="inlineStr">
+        <is>
+          <t>cleveregg</t>
+        </is>
+      </c>
+      <c r="E295" s="18" t="n">
+        <v>1050950.11</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B296" s="10" t="n">
+        <v>784</v>
+      </c>
+      <c r="C296" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="D296" s="11" t="inlineStr">
+        <is>
+          <t>newgroup18</t>
+        </is>
+      </c>
+      <c r="E296" s="14" t="n">
+        <v>965924.48</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B297" s="15" t="n">
+        <v>784</v>
+      </c>
+      <c r="C297" s="15" t="n">
+        <v>26</v>
+      </c>
+      <c r="D297" s="16" t="inlineStr">
+        <is>
+          <t>vivo50</t>
+        </is>
+      </c>
+      <c r="E297" s="18" t="n">
+        <v>848688.92</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B298" s="24" t="n">
+        <v>784</v>
+      </c>
+      <c r="C298" s="24" t="n">
+        <v>27</v>
+      </c>
+      <c r="D298" s="25" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="E298" s="26" t="n">
+        <v>598181.96</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E271"/>
+  <autoFilter ref="A1:E298"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6890,7 +7454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S262"/>
+  <dimension ref="A1:S263"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -23454,8 +24018,69 @@
         <v>129050</v>
       </c>
     </row>
+    <row r="263">
+      <c r="A263" s="15" t="n">
+        <v>262</v>
+      </c>
+      <c r="B263" s="15" t="n">
+        <v>784</v>
+      </c>
+      <c r="C263" s="15" t="n">
+        <v>786</v>
+      </c>
+      <c r="D263" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E263" s="16" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="F263" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G263" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="H263" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I263" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="J263" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K263" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="L263" s="18" t="n">
+        <v>598181.96</v>
+      </c>
+      <c r="M263" s="18" t="n">
+        <v>598181.96</v>
+      </c>
+      <c r="N263" s="16" t="n"/>
+      <c r="O263" s="17" t="n">
+        <v>532</v>
+      </c>
+      <c r="P263" s="17" t="n">
+        <v>532</v>
+      </c>
+      <c r="Q263" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="R263" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="S263" s="18" t="n">
+        <v>11600</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S262"/>
+  <autoFilter ref="A1:S263"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -23466,7 +24091,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N784"/>
+  <dimension ref="A1:N785"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -59575,8 +60200,54 @@
         <v>18850</v>
       </c>
     </row>
+    <row r="785">
+      <c r="A785" s="15" t="n">
+        <v>784</v>
+      </c>
+      <c r="B785" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C785" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="D785" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E785" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="F785" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G785" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="H785" s="18" t="n">
+        <v>598181.96</v>
+      </c>
+      <c r="I785" s="17" t="n">
+        <v>532</v>
+      </c>
+      <c r="J785" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K785" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="L785" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="M785" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N785" s="18" t="n">
+        <v>11600</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N784"/>
+  <autoFilter ref="A1:N785"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -59971,7 +60642,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -60526,8 +61197,56 @@
         <v>55</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="23" t="n">
+        <v>730.66</v>
+      </c>
+      <c r="B23" s="16" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C23" s="16" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D23" s="16" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E23" s="16" t="inlineStr"/>
+      <c r="F23" s="17" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="21" t="n">
+        <v>742.75</v>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D24" s="11" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E24" s="11" t="inlineStr"/>
+      <c r="F24" s="12" t="n">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F22"/>
+  <autoFilter ref="A1:F24"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -60926,7 +61645,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U11"/>
+  <dimension ref="A1:U12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -61761,8 +62480,77 @@
         <v>36861.11894596298</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="n">
+        <v>784</v>
+      </c>
+      <c r="C12" s="14" t="n">
+        <v>598181.96</v>
+      </c>
+      <c r="D12" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="E12" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="F12" s="11" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="G12" s="14" t="n">
+        <v>2412815.2</v>
+      </c>
+      <c r="H12" s="21" t="n">
+        <v>20</v>
+      </c>
+      <c r="I12" s="21" t="n">
+        <v>55</v>
+      </c>
+      <c r="J12" s="11" t="inlineStr">
+        <is>
+          <t>truck</t>
+        </is>
+      </c>
+      <c r="K12" s="22" t="n">
+        <v>3600</v>
+      </c>
+      <c r="L12" s="22" t="n">
+        <v>200</v>
+      </c>
+      <c r="M12" s="12" t="n">
+        <v>532</v>
+      </c>
+      <c r="N12" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="O12" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="P12" s="10" t="n">
+        <v>262</v>
+      </c>
+      <c r="Q12" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="R12" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S12" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="T12" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="U12" s="11" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U11"/>
+  <autoFilter ref="A1:U12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -61773,7 +62561,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E121"/>
+  <dimension ref="A1:E133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -64530,8 +65318,280 @@
         </is>
       </c>
     </row>
+    <row r="122">
+      <c r="A122" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B122" s="10" t="n">
+        <v>784</v>
+      </c>
+      <c r="C122" s="11" t="inlineStr">
+        <is>
+          <t>Starting Cash</t>
+        </is>
+      </c>
+      <c r="D122" s="14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E122" s="11" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B123" s="15" t="n">
+        <v>784</v>
+      </c>
+      <c r="C123" s="16" t="inlineStr">
+        <is>
+          <t>Cash Sources</t>
+        </is>
+      </c>
+      <c r="D123" s="16" t="n"/>
+      <c r="E123" s="16" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B124" s="10" t="n">
+        <v>784</v>
+      </c>
+      <c r="C124" s="11" t="inlineStr">
+        <is>
+          <t>revenues</t>
+        </is>
+      </c>
+      <c r="D124" s="14" t="n">
+        <v>19769300</v>
+      </c>
+      <c r="E124" s="11" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B125" s="15" t="n">
+        <v>784</v>
+      </c>
+      <c r="C125" s="16" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D125" s="18" t="n">
+        <v>286388.11</v>
+      </c>
+      <c r="E125" s="16" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B126" s="10" t="n">
+        <v>784</v>
+      </c>
+      <c r="C126" s="11" t="inlineStr">
+        <is>
+          <t>Cash Uses</t>
+        </is>
+      </c>
+      <c r="D126" s="11" t="n"/>
+      <c r="E126" s="11" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B127" s="15" t="n">
+        <v>784</v>
+      </c>
+      <c r="C127" s="16" t="inlineStr">
+        <is>
+          <t>outbound shipping</t>
+        </is>
+      </c>
+      <c r="D127" s="18" t="n">
+        <v>-2045100</v>
+      </c>
+      <c r="E127" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B128" s="10" t="n">
+        <v>784</v>
+      </c>
+      <c r="C128" s="11" t="inlineStr">
+        <is>
+          <t>inbound shipping</t>
+        </is>
+      </c>
+      <c r="D128" s="14" t="n">
+        <v>-1425000</v>
+      </c>
+      <c r="E128" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B129" s="15" t="n">
+        <v>784</v>
+      </c>
+      <c r="C129" s="16" t="inlineStr">
+        <is>
+          <t>FGI holding</t>
+        </is>
+      </c>
+      <c r="D129" s="18" t="n">
+        <v>-17928.29</v>
+      </c>
+      <c r="E129" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B130" s="10" t="n">
+        <v>784</v>
+      </c>
+      <c r="C130" s="11" t="inlineStr">
+        <is>
+          <t>add capacity</t>
+        </is>
+      </c>
+      <c r="D130" s="14" t="n">
+        <v>-1749840.87</v>
+      </c>
+      <c r="E130" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B131" s="15" t="n">
+        <v>784</v>
+      </c>
+      <c r="C131" s="16" t="inlineStr">
+        <is>
+          <t>Pipeline inventory holding</t>
+        </is>
+      </c>
+      <c r="D131" s="18" t="n">
+        <v>-27136.99</v>
+      </c>
+      <c r="E131" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B132" s="10" t="n">
+        <v>784</v>
+      </c>
+      <c r="C132" s="11" t="inlineStr">
+        <is>
+          <t>production</t>
+        </is>
+      </c>
+      <c r="D132" s="14" t="n">
+        <v>-14692500</v>
+      </c>
+      <c r="E132" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B133" s="15" t="n">
+        <v>784</v>
+      </c>
+      <c r="C133" s="16" t="inlineStr">
+        <is>
+          <t>Cash Balance</t>
+        </is>
+      </c>
+      <c r="D133" s="18" t="n">
+        <v>598181.96</v>
+      </c>
+      <c r="E133" s="16" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E121"/>
+  <autoFilter ref="A1:E133"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update game data: day 785, cash 611139.86, 3-day period 262
</commit_message>
<xml_diff>
--- a/data/supply_chain_game.xlsx
+++ b/data/supply_chain_game.xlsx
@@ -21,15 +21,15 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$263</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$785</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$786</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'资金构成_旧版'!$A$1:$C$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'运营参数_旧版'!$A$9:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'排行榜_旧版'!$A$1:$C$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$133</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$145</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'运营参数'!$A$1:$J$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$298</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$325</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -590,7 +590,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-06T01:26:02+08:00</t>
+          <t>2026-09-06T01:41:02+08:00</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>784</v>
+        <v>785</v>
       </c>
     </row>
     <row r="7">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>676</v>
+        <v>675</v>
       </c>
     </row>
     <row r="8">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>598181.96</v>
+        <v>611139.86</v>
       </c>
     </row>
     <row r="11">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>2412815.2</v>
+        <v>2413596.01</v>
       </c>
     </row>
     <row r="15"/>
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>532</v>
+        <v>514</v>
       </c>
     </row>
     <row r="25">
@@ -861,7 +861,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>8</v>
+        <v>26</v>
       </c>
     </row>
     <row r="33">
@@ -881,7 +881,7 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>8</v>
+        <v>26</v>
       </c>
     </row>
     <row r="35">
@@ -901,7 +901,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>8</v>
+        <v>26</v>
       </c>
     </row>
     <row r="37">
@@ -909,6 +909,9 @@
         <is>
           <t>周期现金变动</t>
         </is>
+      </c>
+      <c r="B37" s="4" t="n">
+        <v>23762.26981817116</v>
       </c>
     </row>
     <row r="38"/>
@@ -970,7 +973,7 @@
         </is>
       </c>
       <c r="B44" s="4" t="n">
-        <v>37812.55512617959</v>
+        <v>37129.58429677982</v>
       </c>
     </row>
     <row r="45"/>
@@ -1168,7 +1171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E298"/>
+  <dimension ref="A1:E325"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -7442,8 +7445,575 @@
         <v>598181.96</v>
       </c>
     </row>
+    <row r="299">
+      <c r="A299" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B299" s="15" t="n">
+        <v>785</v>
+      </c>
+      <c r="C299" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D299" s="16" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="E299" s="18" t="n">
+        <v>3024735.87</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B300" s="10" t="n">
+        <v>785</v>
+      </c>
+      <c r="C300" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D300" s="11" t="inlineStr">
+        <is>
+          <t>nicetry</t>
+        </is>
+      </c>
+      <c r="E300" s="14" t="n">
+        <v>2059580.2</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B301" s="15" t="n">
+        <v>785</v>
+      </c>
+      <c r="C301" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D301" s="16" t="inlineStr">
+        <is>
+          <t>group7</t>
+        </is>
+      </c>
+      <c r="E301" s="18" t="n">
+        <v>2010468.25</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B302" s="10" t="n">
+        <v>785</v>
+      </c>
+      <c r="C302" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D302" s="11" t="inlineStr">
+        <is>
+          <t>group15</t>
+        </is>
+      </c>
+      <c r="E302" s="14" t="n">
+        <v>1922866.37</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B303" s="15" t="n">
+        <v>785</v>
+      </c>
+      <c r="C303" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="D303" s="16" t="inlineStr">
+        <is>
+          <t>group14</t>
+        </is>
+      </c>
+      <c r="E303" s="18" t="n">
+        <v>1809959.29</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B304" s="10" t="n">
+        <v>785</v>
+      </c>
+      <c r="C304" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="D304" s="11" t="inlineStr">
+        <is>
+          <t>t24</t>
+        </is>
+      </c>
+      <c r="E304" s="14" t="n">
+        <v>1705816.19</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B305" s="15" t="n">
+        <v>785</v>
+      </c>
+      <c r="C305" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="D305" s="16" t="inlineStr">
+        <is>
+          <t>montesquieu</t>
+        </is>
+      </c>
+      <c r="E305" s="18" t="n">
+        <v>1622593.17</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B306" s="10" t="n">
+        <v>785</v>
+      </c>
+      <c r="C306" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="D306" s="11" t="inlineStr">
+        <is>
+          <t>group8</t>
+        </is>
+      </c>
+      <c r="E306" s="14" t="n">
+        <v>1586935.28</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B307" s="15" t="n">
+        <v>785</v>
+      </c>
+      <c r="C307" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="D307" s="16" t="inlineStr">
+        <is>
+          <t>group9</t>
+        </is>
+      </c>
+      <c r="E307" s="18" t="n">
+        <v>1586208.33</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B308" s="10" t="n">
+        <v>785</v>
+      </c>
+      <c r="C308" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="D308" s="11" t="inlineStr">
+        <is>
+          <t>aaachemicalseller</t>
+        </is>
+      </c>
+      <c r="E308" s="14" t="n">
+        <v>1519770.03</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B309" s="15" t="n">
+        <v>785</v>
+      </c>
+      <c r="C309" s="15" t="n">
+        <v>11</v>
+      </c>
+      <c r="D309" s="16" t="inlineStr">
+        <is>
+          <t>deepsleep</t>
+        </is>
+      </c>
+      <c r="E309" s="18" t="n">
+        <v>1435407.38</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B310" s="10" t="n">
+        <v>785</v>
+      </c>
+      <c r="C310" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="D310" s="11" t="inlineStr">
+        <is>
+          <t>group2</t>
+        </is>
+      </c>
+      <c r="E310" s="14" t="n">
+        <v>1368809.16</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B311" s="15" t="n">
+        <v>785</v>
+      </c>
+      <c r="C311" s="15" t="n">
+        <v>13</v>
+      </c>
+      <c r="D311" s="16" t="inlineStr">
+        <is>
+          <t>teamhlly</t>
+        </is>
+      </c>
+      <c r="E311" s="18" t="n">
+        <v>1368808.43</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B312" s="10" t="n">
+        <v>785</v>
+      </c>
+      <c r="C312" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="D312" s="11" t="inlineStr">
+        <is>
+          <t>group25</t>
+        </is>
+      </c>
+      <c r="E312" s="14" t="n">
+        <v>1368653.58</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B313" s="15" t="n">
+        <v>785</v>
+      </c>
+      <c r="C313" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="D313" s="16" t="inlineStr">
+        <is>
+          <t>group11</t>
+        </is>
+      </c>
+      <c r="E313" s="18" t="n">
+        <v>1368641.46</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B314" s="10" t="n">
+        <v>785</v>
+      </c>
+      <c r="C314" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="D314" s="11" t="inlineStr">
+        <is>
+          <t>88888888</t>
+        </is>
+      </c>
+      <c r="E314" s="14" t="n">
+        <v>1368619.14</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B315" s="15" t="n">
+        <v>785</v>
+      </c>
+      <c r="C315" s="15" t="n">
+        <v>17</v>
+      </c>
+      <c r="D315" s="16" t="inlineStr">
+        <is>
+          <t>group12</t>
+        </is>
+      </c>
+      <c r="E315" s="18" t="n">
+        <v>1301858.76</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B316" s="10" t="n">
+        <v>785</v>
+      </c>
+      <c r="C316" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="D316" s="11" t="inlineStr">
+        <is>
+          <t>tigagroup20</t>
+        </is>
+      </c>
+      <c r="E316" s="14" t="n">
+        <v>1268106.91</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B317" s="15" t="n">
+        <v>785</v>
+      </c>
+      <c r="C317" s="15" t="n">
+        <v>19</v>
+      </c>
+      <c r="D317" s="16" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E317" s="18" t="n">
+        <v>1261943.13</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B318" s="10" t="n">
+        <v>785</v>
+      </c>
+      <c r="C318" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="D318" s="11" t="inlineStr">
+        <is>
+          <t>666666</t>
+        </is>
+      </c>
+      <c r="E318" s="14" t="n">
+        <v>1216306.39</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B319" s="15" t="n">
+        <v>785</v>
+      </c>
+      <c r="C319" s="15" t="n">
+        <v>21</v>
+      </c>
+      <c r="D319" s="16" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="E319" s="18" t="n">
+        <v>1139310.27</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B320" s="10" t="n">
+        <v>785</v>
+      </c>
+      <c r="C320" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="D320" s="11" t="inlineStr">
+        <is>
+          <t>jit</t>
+        </is>
+      </c>
+      <c r="E320" s="14" t="n">
+        <v>1121508.04</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B321" s="15" t="n">
+        <v>785</v>
+      </c>
+      <c r="C321" s="15" t="n">
+        <v>23</v>
+      </c>
+      <c r="D321" s="16" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E321" s="18" t="n">
+        <v>1083073.67</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B322" s="10" t="n">
+        <v>785</v>
+      </c>
+      <c r="C322" s="10" t="n">
+        <v>24</v>
+      </c>
+      <c r="D322" s="11" t="inlineStr">
+        <is>
+          <t>cleveregg</t>
+        </is>
+      </c>
+      <c r="E322" s="14" t="n">
+        <v>1064026.25</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B323" s="15" t="n">
+        <v>785</v>
+      </c>
+      <c r="C323" s="15" t="n">
+        <v>25</v>
+      </c>
+      <c r="D323" s="16" t="inlineStr">
+        <is>
+          <t>newgroup18</t>
+        </is>
+      </c>
+      <c r="E323" s="18" t="n">
+        <v>979000.33</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B324" s="10" t="n">
+        <v>785</v>
+      </c>
+      <c r="C324" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="D324" s="11" t="inlineStr">
+        <is>
+          <t>vivo50</t>
+        </is>
+      </c>
+      <c r="E324" s="14" t="n">
+        <v>861712.24</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B325" s="24" t="n">
+        <v>785</v>
+      </c>
+      <c r="C325" s="24" t="n">
+        <v>27</v>
+      </c>
+      <c r="D325" s="25" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="E325" s="26" t="n">
+        <v>611139.86</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E298"/>
+  <autoFilter ref="A1:E325"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -24029,7 +24599,7 @@
         <v>786</v>
       </c>
       <c r="D263" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E263" s="16" t="inlineStr">
         <is>
@@ -24042,32 +24612,34 @@
         </is>
       </c>
       <c r="G263" s="17" t="n">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="H263" s="17" t="n">
         <v>0</v>
       </c>
       <c r="I263" s="17" t="n">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="J263" s="19" t="n">
         <v>1</v>
       </c>
       <c r="K263" s="17" t="n">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="L263" s="18" t="n">
-        <v>598181.96</v>
+        <v>587377.5901818288</v>
       </c>
       <c r="M263" s="18" t="n">
-        <v>598181.96</v>
-      </c>
-      <c r="N263" s="16" t="n"/>
+        <v>611139.86</v>
+      </c>
+      <c r="N263" s="18" t="n">
+        <v>23762.26981817116</v>
+      </c>
       <c r="O263" s="17" t="n">
-        <v>532</v>
+        <v>514</v>
       </c>
       <c r="P263" s="17" t="n">
-        <v>532</v>
+        <v>523</v>
       </c>
       <c r="Q263" s="17" t="n">
         <v>200</v>
@@ -24076,7 +24648,7 @@
         <v>200</v>
       </c>
       <c r="S263" s="18" t="n">
-        <v>11600</v>
+        <v>37700</v>
       </c>
     </row>
   </sheetData>
@@ -24091,7 +24663,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N785"/>
+  <dimension ref="A1:N786"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -60246,8 +60818,54 @@
         <v>11600</v>
       </c>
     </row>
+    <row r="786">
+      <c r="A786" s="10" t="n">
+        <v>785</v>
+      </c>
+      <c r="B786" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C786" s="12" t="n">
+        <v>18</v>
+      </c>
+      <c r="D786" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E786" s="12" t="n">
+        <v>18</v>
+      </c>
+      <c r="F786" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G786" s="12" t="n">
+        <v>18</v>
+      </c>
+      <c r="H786" s="14" t="n">
+        <v>611139.86</v>
+      </c>
+      <c r="I786" s="12" t="n">
+        <v>514</v>
+      </c>
+      <c r="J786" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K786" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="L786" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="M786" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N786" s="14" t="n">
+        <v>26100</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N785"/>
+  <autoFilter ref="A1:N786"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -60642,7 +61260,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -61245,8 +61863,56 @@
         <v>55</v>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="23" t="n">
+        <v>730.66</v>
+      </c>
+      <c r="B25" s="16" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C25" s="16" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D25" s="16" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E25" s="16" t="inlineStr"/>
+      <c r="F25" s="17" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="21" t="n">
+        <v>742.75</v>
+      </c>
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C26" s="11" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D26" s="11" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E26" s="11" t="inlineStr"/>
+      <c r="F26" s="12" t="n">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F24"/>
+  <autoFilter ref="A1:F26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -61645,7 +62311,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U12"/>
+  <dimension ref="A1:U13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -61654,7 +62320,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
@@ -62549,8 +63215,79 @@
       </c>
       <c r="U12" s="11" t="n"/>
     </row>
+    <row r="13">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="n">
+        <v>785</v>
+      </c>
+      <c r="C13" s="18" t="n">
+        <v>611139.86</v>
+      </c>
+      <c r="D13" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="E13" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="G13" s="18" t="n">
+        <v>2413596.01</v>
+      </c>
+      <c r="H13" s="23" t="n">
+        <v>20</v>
+      </c>
+      <c r="I13" s="23" t="n">
+        <v>55</v>
+      </c>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t>truck</t>
+        </is>
+      </c>
+      <c r="K13" s="27" t="n">
+        <v>3600</v>
+      </c>
+      <c r="L13" s="27" t="n">
+        <v>200</v>
+      </c>
+      <c r="M13" s="17" t="n">
+        <v>514</v>
+      </c>
+      <c r="N13" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="O13" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="P13" s="15" t="n">
+        <v>262</v>
+      </c>
+      <c r="Q13" s="17" t="n">
+        <v>26</v>
+      </c>
+      <c r="R13" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="S13" s="17" t="n">
+        <v>26</v>
+      </c>
+      <c r="T13" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="U13" s="18" t="n">
+        <v>23762.26981817116</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U12"/>
+  <autoFilter ref="A1:U13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -62561,7 +63298,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E133"/>
+  <dimension ref="A1:E145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -65590,8 +66327,280 @@
         </is>
       </c>
     </row>
+    <row r="134">
+      <c r="A134" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B134" s="10" t="n">
+        <v>785</v>
+      </c>
+      <c r="C134" s="11" t="inlineStr">
+        <is>
+          <t>Starting Cash</t>
+        </is>
+      </c>
+      <c r="D134" s="14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E134" s="11" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B135" s="15" t="n">
+        <v>785</v>
+      </c>
+      <c r="C135" s="16" t="inlineStr">
+        <is>
+          <t>Cash Sources</t>
+        </is>
+      </c>
+      <c r="D135" s="16" t="n"/>
+      <c r="E135" s="16" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B136" s="10" t="n">
+        <v>785</v>
+      </c>
+      <c r="C136" s="11" t="inlineStr">
+        <is>
+          <t>revenues</t>
+        </is>
+      </c>
+      <c r="D136" s="14" t="n">
+        <v>19783800</v>
+      </c>
+      <c r="E136" s="11" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B137" s="15" t="n">
+        <v>785</v>
+      </c>
+      <c r="C137" s="16" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D137" s="18" t="n">
+        <v>286543.13</v>
+      </c>
+      <c r="E137" s="16" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B138" s="10" t="n">
+        <v>785</v>
+      </c>
+      <c r="C138" s="11" t="inlineStr">
+        <is>
+          <t>Cash Uses</t>
+        </is>
+      </c>
+      <c r="D138" s="11" t="n"/>
+      <c r="E138" s="11" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B139" s="15" t="n">
+        <v>785</v>
+      </c>
+      <c r="C139" s="16" t="inlineStr">
+        <is>
+          <t>outbound shipping</t>
+        </is>
+      </c>
+      <c r="D139" s="18" t="n">
+        <v>-2046600</v>
+      </c>
+      <c r="E139" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B140" s="10" t="n">
+        <v>785</v>
+      </c>
+      <c r="C140" s="11" t="inlineStr">
+        <is>
+          <t>inbound shipping</t>
+        </is>
+      </c>
+      <c r="D140" s="14" t="n">
+        <v>-1425000</v>
+      </c>
+      <c r="E140" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B141" s="15" t="n">
+        <v>785</v>
+      </c>
+      <c r="C141" s="16" t="inlineStr">
+        <is>
+          <t>FGI holding</t>
+        </is>
+      </c>
+      <c r="D141" s="18" t="n">
+        <v>-18070.62</v>
+      </c>
+      <c r="E141" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B142" s="10" t="n">
+        <v>785</v>
+      </c>
+      <c r="C142" s="11" t="inlineStr">
+        <is>
+          <t>add capacity</t>
+        </is>
+      </c>
+      <c r="D142" s="14" t="n">
+        <v>-1749840.87</v>
+      </c>
+      <c r="E142" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B143" s="15" t="n">
+        <v>785</v>
+      </c>
+      <c r="C143" s="16" t="inlineStr">
+        <is>
+          <t>Pipeline inventory holding</t>
+        </is>
+      </c>
+      <c r="D143" s="18" t="n">
+        <v>-27191.78</v>
+      </c>
+      <c r="E143" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B144" s="10" t="n">
+        <v>785</v>
+      </c>
+      <c r="C144" s="11" t="inlineStr">
+        <is>
+          <t>production</t>
+        </is>
+      </c>
+      <c r="D144" s="14" t="n">
+        <v>-14692500</v>
+      </c>
+      <c r="E144" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B145" s="15" t="n">
+        <v>785</v>
+      </c>
+      <c r="C145" s="16" t="inlineStr">
+        <is>
+          <t>Cash Balance</t>
+        </is>
+      </c>
+      <c r="D145" s="18" t="n">
+        <v>611139.86</v>
+      </c>
+      <c r="E145" s="16" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E133"/>
+  <autoFilter ref="A1:E145"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update game data: day 786, cash 634504.1, 3-day period 262
</commit_message>
<xml_diff>
--- a/data/supply_chain_game.xlsx
+++ b/data/supply_chain_game.xlsx
@@ -21,15 +21,15 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$263</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$786</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$787</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'资金构成_旧版'!$A$1:$C$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'运营参数_旧版'!$A$9:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'排行榜_旧版'!$A$1:$C$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$145</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$157</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'运营参数'!$A$1:$J$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$325</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$352</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -590,7 +590,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-06T01:41:02+08:00</t>
+          <t>2026-09-06T01:56:04+08:00</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>785</v>
+        <v>786</v>
       </c>
     </row>
     <row r="7">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>675</v>
+        <v>674</v>
       </c>
     </row>
     <row r="8">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>611139.86</v>
+        <v>634504.1</v>
       </c>
     </row>
     <row r="11">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>2413596.01</v>
+        <v>2247877.02</v>
       </c>
     </row>
     <row r="15"/>
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>514</v>
+        <v>506</v>
       </c>
     </row>
     <row r="25">
@@ -850,7 +850,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>否（进行中）</t>
+          <t>是</t>
         </is>
       </c>
     </row>
@@ -861,7 +861,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
     </row>
     <row r="33">
@@ -881,7 +881,7 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
     </row>
     <row r="35">
@@ -901,7 +901,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
     </row>
     <row r="37">
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="B37" s="4" t="n">
-        <v>23762.26981817116</v>
+        <v>35013.40039060952</v>
       </c>
     </row>
     <row r="38"/>
@@ -929,7 +929,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="41">
@@ -940,7 +940,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>781–783</t>
+          <t>784–786</t>
         </is>
       </c>
     </row>
@@ -952,7 +952,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>89.0 / 0.0 / 89.0</t>
+          <t>34.0 / 0.0 / 34.0</t>
         </is>
       </c>
     </row>
@@ -973,7 +973,7 @@
         </is>
       </c>
       <c r="B44" s="4" t="n">
-        <v>37129.58429677982</v>
+        <v>35013.40039060952</v>
       </c>
     </row>
     <row r="45"/>
@@ -1171,7 +1171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E325"/>
+  <dimension ref="A1:E352"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -8012,8 +8012,575 @@
         <v>611139.86</v>
       </c>
     </row>
+    <row r="326">
+      <c r="A326" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:56:04+08:00</t>
+        </is>
+      </c>
+      <c r="B326" s="10" t="n">
+        <v>786</v>
+      </c>
+      <c r="C326" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D326" s="11" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="E326" s="14" t="n">
+        <v>2882381.12</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:56:04+08:00</t>
+        </is>
+      </c>
+      <c r="B327" s="15" t="n">
+        <v>786</v>
+      </c>
+      <c r="C327" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D327" s="16" t="inlineStr">
+        <is>
+          <t>nicetry</t>
+        </is>
+      </c>
+      <c r="E327" s="18" t="n">
+        <v>2083432.3</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:56:04+08:00</t>
+        </is>
+      </c>
+      <c r="B328" s="10" t="n">
+        <v>786</v>
+      </c>
+      <c r="C328" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D328" s="11" t="inlineStr">
+        <is>
+          <t>group15</t>
+        </is>
+      </c>
+      <c r="E328" s="14" t="n">
+        <v>1946712.93</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:56:04+08:00</t>
+        </is>
+      </c>
+      <c r="B329" s="15" t="n">
+        <v>786</v>
+      </c>
+      <c r="C329" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D329" s="16" t="inlineStr">
+        <is>
+          <t>group7</t>
+        </is>
+      </c>
+      <c r="E329" s="18" t="n">
+        <v>1867848.62</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:56:04+08:00</t>
+        </is>
+      </c>
+      <c r="B330" s="10" t="n">
+        <v>786</v>
+      </c>
+      <c r="C330" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="D330" s="11" t="inlineStr">
+        <is>
+          <t>group14</t>
+        </is>
+      </c>
+      <c r="E330" s="14" t="n">
+        <v>1833746.2</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:56:04+08:00</t>
+        </is>
+      </c>
+      <c r="B331" s="15" t="n">
+        <v>786</v>
+      </c>
+      <c r="C331" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="D331" s="16" t="inlineStr">
+        <is>
+          <t>t24</t>
+        </is>
+      </c>
+      <c r="E331" s="18" t="n">
+        <v>1729575.9</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:56:04+08:00</t>
+        </is>
+      </c>
+      <c r="B332" s="10" t="n">
+        <v>786</v>
+      </c>
+      <c r="C332" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="D332" s="11" t="inlineStr">
+        <is>
+          <t>montesquieu</t>
+        </is>
+      </c>
+      <c r="E332" s="14" t="n">
+        <v>1646221.55</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:56:04+08:00</t>
+        </is>
+      </c>
+      <c r="B333" s="15" t="n">
+        <v>786</v>
+      </c>
+      <c r="C333" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="D333" s="16" t="inlineStr">
+        <is>
+          <t>group8</t>
+        </is>
+      </c>
+      <c r="E333" s="18" t="n">
+        <v>1610609.15</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:56:04+08:00</t>
+        </is>
+      </c>
+      <c r="B334" s="10" t="n">
+        <v>786</v>
+      </c>
+      <c r="C334" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="D334" s="11" t="inlineStr">
+        <is>
+          <t>group9</t>
+        </is>
+      </c>
+      <c r="E334" s="14" t="n">
+        <v>1609882.01</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:56:04+08:00</t>
+        </is>
+      </c>
+      <c r="B335" s="15" t="n">
+        <v>786</v>
+      </c>
+      <c r="C335" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="D335" s="16" t="inlineStr">
+        <is>
+          <t>deepsleep</t>
+        </is>
+      </c>
+      <c r="E335" s="18" t="n">
+        <v>1459063.59</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:56:04+08:00</t>
+        </is>
+      </c>
+      <c r="B336" s="10" t="n">
+        <v>786</v>
+      </c>
+      <c r="C336" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="D336" s="11" t="inlineStr">
+        <is>
+          <t>group2</t>
+        </is>
+      </c>
+      <c r="E336" s="14" t="n">
+        <v>1392371.27</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:56:04+08:00</t>
+        </is>
+      </c>
+      <c r="B337" s="15" t="n">
+        <v>786</v>
+      </c>
+      <c r="C337" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="D337" s="16" t="inlineStr">
+        <is>
+          <t>teamhlly</t>
+        </is>
+      </c>
+      <c r="E337" s="18" t="n">
+        <v>1392370.54</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:56:04+08:00</t>
+        </is>
+      </c>
+      <c r="B338" s="10" t="n">
+        <v>786</v>
+      </c>
+      <c r="C338" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="D338" s="11" t="inlineStr">
+        <is>
+          <t>group25</t>
+        </is>
+      </c>
+      <c r="E338" s="14" t="n">
+        <v>1392215.64</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:56:04+08:00</t>
+        </is>
+      </c>
+      <c r="B339" s="15" t="n">
+        <v>786</v>
+      </c>
+      <c r="C339" s="15" t="n">
+        <v>14</v>
+      </c>
+      <c r="D339" s="16" t="inlineStr">
+        <is>
+          <t>group11</t>
+        </is>
+      </c>
+      <c r="E339" s="18" t="n">
+        <v>1392203.52</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:56:04+08:00</t>
+        </is>
+      </c>
+      <c r="B340" s="10" t="n">
+        <v>786</v>
+      </c>
+      <c r="C340" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="D340" s="11" t="inlineStr">
+        <is>
+          <t>88888888</t>
+        </is>
+      </c>
+      <c r="E340" s="14" t="n">
+        <v>1392181.2</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:56:04+08:00</t>
+        </is>
+      </c>
+      <c r="B341" s="15" t="n">
+        <v>786</v>
+      </c>
+      <c r="C341" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="D341" s="16" t="inlineStr">
+        <is>
+          <t>aaachemicalseller</t>
+        </is>
+      </c>
+      <c r="E341" s="18" t="n">
+        <v>1327000.77</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:56:04+08:00</t>
+        </is>
+      </c>
+      <c r="B342" s="10" t="n">
+        <v>786</v>
+      </c>
+      <c r="C342" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="D342" s="11" t="inlineStr">
+        <is>
+          <t>group12</t>
+        </is>
+      </c>
+      <c r="E342" s="14" t="n">
+        <v>1325512.97</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:56:04+08:00</t>
+        </is>
+      </c>
+      <c r="B343" s="15" t="n">
+        <v>786</v>
+      </c>
+      <c r="C343" s="15" t="n">
+        <v>18</v>
+      </c>
+      <c r="D343" s="16" t="inlineStr">
+        <is>
+          <t>tigagroup20</t>
+        </is>
+      </c>
+      <c r="E343" s="18" t="n">
+        <v>1291697.52</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:56:04+08:00</t>
+        </is>
+      </c>
+      <c r="B344" s="10" t="n">
+        <v>786</v>
+      </c>
+      <c r="C344" s="10" t="n">
+        <v>19</v>
+      </c>
+      <c r="D344" s="11" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E344" s="14" t="n">
+        <v>1285578.15</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:56:04+08:00</t>
+        </is>
+      </c>
+      <c r="B345" s="15" t="n">
+        <v>786</v>
+      </c>
+      <c r="C345" s="15" t="n">
+        <v>20</v>
+      </c>
+      <c r="D345" s="16" t="inlineStr">
+        <is>
+          <t>666666</t>
+        </is>
+      </c>
+      <c r="E345" s="18" t="n">
+        <v>1239828.67</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:56:04+08:00</t>
+        </is>
+      </c>
+      <c r="B346" s="10" t="n">
+        <v>786</v>
+      </c>
+      <c r="C346" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="D346" s="11" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="E346" s="14" t="n">
+        <v>1162978.01</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:56:04+08:00</t>
+        </is>
+      </c>
+      <c r="B347" s="15" t="n">
+        <v>786</v>
+      </c>
+      <c r="C347" s="15" t="n">
+        <v>22</v>
+      </c>
+      <c r="D347" s="16" t="inlineStr">
+        <is>
+          <t>jit</t>
+        </is>
+      </c>
+      <c r="E347" s="18" t="n">
+        <v>1145060.36</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:56:04+08:00</t>
+        </is>
+      </c>
+      <c r="B348" s="10" t="n">
+        <v>786</v>
+      </c>
+      <c r="C348" s="10" t="n">
+        <v>23</v>
+      </c>
+      <c r="D348" s="11" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E348" s="14" t="n">
+        <v>1106615.95</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:56:04+08:00</t>
+        </is>
+      </c>
+      <c r="B349" s="15" t="n">
+        <v>786</v>
+      </c>
+      <c r="C349" s="15" t="n">
+        <v>24</v>
+      </c>
+      <c r="D349" s="16" t="inlineStr">
+        <is>
+          <t>cleveregg</t>
+        </is>
+      </c>
+      <c r="E349" s="18" t="n">
+        <v>1087508.76</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:56:04+08:00</t>
+        </is>
+      </c>
+      <c r="B350" s="10" t="n">
+        <v>786</v>
+      </c>
+      <c r="C350" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="D350" s="11" t="inlineStr">
+        <is>
+          <t>newgroup18</t>
+        </is>
+      </c>
+      <c r="E350" s="14" t="n">
+        <v>1002482.56</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:56:04+08:00</t>
+        </is>
+      </c>
+      <c r="B351" s="15" t="n">
+        <v>786</v>
+      </c>
+      <c r="C351" s="15" t="n">
+        <v>26</v>
+      </c>
+      <c r="D351" s="16" t="inlineStr">
+        <is>
+          <t>vivo50</t>
+        </is>
+      </c>
+      <c r="E351" s="18" t="n">
+        <v>885141.92</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:56:04+08:00</t>
+        </is>
+      </c>
+      <c r="B352" s="24" t="n">
+        <v>786</v>
+      </c>
+      <c r="C352" s="24" t="n">
+        <v>27</v>
+      </c>
+      <c r="D352" s="25" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="E352" s="26" t="n">
+        <v>634504.1</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E325"/>
+  <autoFilter ref="A1:E352"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -24599,11 +25166,11 @@
         <v>786</v>
       </c>
       <c r="D263" s="15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E263" s="16" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="F263" s="16" t="inlineStr">
@@ -24612,34 +25179,34 @@
         </is>
       </c>
       <c r="G263" s="17" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="H263" s="17" t="n">
         <v>0</v>
       </c>
       <c r="I263" s="17" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="J263" s="19" t="n">
         <v>1</v>
       </c>
       <c r="K263" s="17" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="L263" s="18" t="n">
-        <v>587377.5901818288</v>
+        <v>599490.6996093905</v>
       </c>
       <c r="M263" s="18" t="n">
-        <v>611139.86</v>
+        <v>634504.1</v>
       </c>
       <c r="N263" s="18" t="n">
-        <v>23762.26981817116</v>
+        <v>35013.40039060952</v>
       </c>
       <c r="O263" s="17" t="n">
-        <v>514</v>
+        <v>506</v>
       </c>
       <c r="P263" s="17" t="n">
-        <v>523</v>
+        <v>517.3333333333334</v>
       </c>
       <c r="Q263" s="17" t="n">
         <v>200</v>
@@ -24648,7 +25215,7 @@
         <v>200</v>
       </c>
       <c r="S263" s="18" t="n">
-        <v>37700</v>
+        <v>49300</v>
       </c>
     </row>
   </sheetData>
@@ -24663,7 +25230,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N786"/>
+  <dimension ref="A1:N787"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -60864,8 +61431,54 @@
         <v>26100</v>
       </c>
     </row>
+    <row r="787">
+      <c r="A787" s="15" t="n">
+        <v>786</v>
+      </c>
+      <c r="B787" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C787" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="D787" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E787" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="F787" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G787" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="H787" s="18" t="n">
+        <v>634504.1</v>
+      </c>
+      <c r="I787" s="17" t="n">
+        <v>506</v>
+      </c>
+      <c r="J787" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K787" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="L787" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="M787" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N787" s="18" t="n">
+        <v>11600</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N786"/>
+  <autoFilter ref="A1:N787"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -61260,7 +61873,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -61911,8 +62524,56 @@
         <v>55</v>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="23" t="n">
+        <v>730.66</v>
+      </c>
+      <c r="B27" s="16" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C27" s="16" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D27" s="16" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E27" s="16" t="inlineStr"/>
+      <c r="F27" s="17" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="21" t="n">
+        <v>742.75</v>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D28" s="11" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E28" s="11" t="inlineStr"/>
+      <c r="F28" s="12" t="n">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F26"/>
+  <autoFilter ref="A1:F28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -62311,7 +62972,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U13"/>
+  <dimension ref="A1:U14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -62320,7 +62981,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
@@ -63286,8 +63947,79 @@
         <v>23762.26981817116</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:56:04+08:00</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="n">
+        <v>786</v>
+      </c>
+      <c r="C14" s="14" t="n">
+        <v>634504.1</v>
+      </c>
+      <c r="D14" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="E14" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="F14" s="11" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="G14" s="14" t="n">
+        <v>2247877.02</v>
+      </c>
+      <c r="H14" s="21" t="n">
+        <v>20</v>
+      </c>
+      <c r="I14" s="21" t="n">
+        <v>55</v>
+      </c>
+      <c r="J14" s="11" t="inlineStr">
+        <is>
+          <t>truck</t>
+        </is>
+      </c>
+      <c r="K14" s="22" t="n">
+        <v>3600</v>
+      </c>
+      <c r="L14" s="22" t="n">
+        <v>200</v>
+      </c>
+      <c r="M14" s="12" t="n">
+        <v>506</v>
+      </c>
+      <c r="N14" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="O14" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="P14" s="10" t="n">
+        <v>262</v>
+      </c>
+      <c r="Q14" s="12" t="n">
+        <v>34</v>
+      </c>
+      <c r="R14" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S14" s="12" t="n">
+        <v>34</v>
+      </c>
+      <c r="T14" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="U14" s="14" t="n">
+        <v>35013.40039060952</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U13"/>
+  <autoFilter ref="A1:U14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -63298,7 +64030,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E145"/>
+  <dimension ref="A1:E157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -66599,8 +67331,280 @@
         </is>
       </c>
     </row>
+    <row r="146">
+      <c r="A146" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:56:04+08:00</t>
+        </is>
+      </c>
+      <c r="B146" s="10" t="n">
+        <v>786</v>
+      </c>
+      <c r="C146" s="11" t="inlineStr">
+        <is>
+          <t>Starting Cash</t>
+        </is>
+      </c>
+      <c r="D146" s="14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E146" s="11" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:56:04+08:00</t>
+        </is>
+      </c>
+      <c r="B147" s="15" t="n">
+        <v>786</v>
+      </c>
+      <c r="C147" s="16" t="inlineStr">
+        <is>
+          <t>Cash Sources</t>
+        </is>
+      </c>
+      <c r="D147" s="16" t="n"/>
+      <c r="E147" s="16" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:56:04+08:00</t>
+        </is>
+      </c>
+      <c r="B148" s="10" t="n">
+        <v>786</v>
+      </c>
+      <c r="C148" s="11" t="inlineStr">
+        <is>
+          <t>revenues</t>
+        </is>
+      </c>
+      <c r="D148" s="14" t="n">
+        <v>19809900</v>
+      </c>
+      <c r="E148" s="11" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:56:04+08:00</t>
+        </is>
+      </c>
+      <c r="B149" s="15" t="n">
+        <v>786</v>
+      </c>
+      <c r="C149" s="16" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D149" s="18" t="n">
+        <v>286701.66</v>
+      </c>
+      <c r="E149" s="16" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:56:04+08:00</t>
+        </is>
+      </c>
+      <c r="B150" s="10" t="n">
+        <v>786</v>
+      </c>
+      <c r="C150" s="11" t="inlineStr">
+        <is>
+          <t>Cash Uses</t>
+        </is>
+      </c>
+      <c r="D150" s="11" t="n"/>
+      <c r="E150" s="11" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:56:04+08:00</t>
+        </is>
+      </c>
+      <c r="B151" s="15" t="n">
+        <v>786</v>
+      </c>
+      <c r="C151" s="16" t="inlineStr">
+        <is>
+          <t>outbound shipping</t>
+        </is>
+      </c>
+      <c r="D151" s="18" t="n">
+        <v>-2049300</v>
+      </c>
+      <c r="E151" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:56:04+08:00</t>
+        </is>
+      </c>
+      <c r="B152" s="10" t="n">
+        <v>786</v>
+      </c>
+      <c r="C152" s="11" t="inlineStr">
+        <is>
+          <t>inbound shipping</t>
+        </is>
+      </c>
+      <c r="D152" s="14" t="n">
+        <v>-1425000</v>
+      </c>
+      <c r="E152" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:56:04+08:00</t>
+        </is>
+      </c>
+      <c r="B153" s="15" t="n">
+        <v>786</v>
+      </c>
+      <c r="C153" s="16" t="inlineStr">
+        <is>
+          <t>FGI holding</t>
+        </is>
+      </c>
+      <c r="D153" s="18" t="n">
+        <v>-18210.12</v>
+      </c>
+      <c r="E153" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:56:04+08:00</t>
+        </is>
+      </c>
+      <c r="B154" s="10" t="n">
+        <v>786</v>
+      </c>
+      <c r="C154" s="11" t="inlineStr">
+        <is>
+          <t>add capacity</t>
+        </is>
+      </c>
+      <c r="D154" s="14" t="n">
+        <v>-1749840.87</v>
+      </c>
+      <c r="E154" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:56:04+08:00</t>
+        </is>
+      </c>
+      <c r="B155" s="15" t="n">
+        <v>786</v>
+      </c>
+      <c r="C155" s="16" t="inlineStr">
+        <is>
+          <t>Pipeline inventory holding</t>
+        </is>
+      </c>
+      <c r="D155" s="18" t="n">
+        <v>-27246.58</v>
+      </c>
+      <c r="E155" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:56:04+08:00</t>
+        </is>
+      </c>
+      <c r="B156" s="10" t="n">
+        <v>786</v>
+      </c>
+      <c r="C156" s="11" t="inlineStr">
+        <is>
+          <t>production</t>
+        </is>
+      </c>
+      <c r="D156" s="14" t="n">
+        <v>-14692500</v>
+      </c>
+      <c r="E156" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T01:56:04+08:00</t>
+        </is>
+      </c>
+      <c r="B157" s="15" t="n">
+        <v>786</v>
+      </c>
+      <c r="C157" s="16" t="inlineStr">
+        <is>
+          <t>Cash Balance</t>
+        </is>
+      </c>
+      <c r="D157" s="18" t="n">
+        <v>634504.1</v>
+      </c>
+      <c r="E157" s="16" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E145"/>
+  <autoFilter ref="A1:E157"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update game data: day 787, cash 674776.43, 3-day period 263
</commit_message>
<xml_diff>
--- a/data/supply_chain_game.xlsx
+++ b/data/supply_chain_game.xlsx
@@ -20,16 +20,16 @@
     <sheet name="排行榜" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$263</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$787</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$264</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$788</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'资金构成_旧版'!$A$1:$C$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'运营参数_旧版'!$A$9:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'排行榜_旧版'!$A$1:$C$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$157</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$169</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'运营参数'!$A$1:$J$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$352</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$379</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -590,7 +590,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-06T01:56:04+08:00</t>
+          <t>2026-09-06T02:11:02+08:00</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>786</v>
+        <v>787</v>
       </c>
     </row>
     <row r="7">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>674</v>
+        <v>673</v>
       </c>
     </row>
     <row r="8">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>634504.1</v>
+        <v>674776.4300000001</v>
       </c>
     </row>
     <row r="11">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>2247877.02</v>
+        <v>2248642.43</v>
       </c>
     </row>
     <row r="15"/>
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>506</v>
+        <v>488</v>
       </c>
     </row>
     <row r="25">
@@ -827,7 +827,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="30">
@@ -838,7 +838,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>784–786</t>
+          <t>787–789</t>
         </is>
       </c>
     </row>
@@ -850,7 +850,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否（进行中）</t>
         </is>
       </c>
     </row>
@@ -861,7 +861,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>34</v>
+        <v>18</v>
       </c>
     </row>
     <row r="33">
@@ -881,7 +881,7 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>34</v>
+        <v>18</v>
       </c>
     </row>
     <row r="35">
@@ -901,7 +901,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>34</v>
+        <v>18</v>
       </c>
     </row>
     <row r="37">
@@ -909,9 +909,6 @@
         <is>
           <t>周期现金变动</t>
         </is>
-      </c>
-      <c r="B37" s="4" t="n">
-        <v>35013.40039060952</v>
       </c>
     </row>
     <row r="38"/>
@@ -973,7 +970,7 @@
         </is>
       </c>
       <c r="B44" s="4" t="n">
-        <v>35013.40039060952</v>
+        <v>35864.06093034125</v>
       </c>
     </row>
     <row r="45"/>
@@ -1171,7 +1168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E352"/>
+  <dimension ref="A1:E379"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -8579,8 +8576,575 @@
         <v>634504.1</v>
       </c>
     </row>
+    <row r="353">
+      <c r="A353" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B353" s="15" t="n">
+        <v>787</v>
+      </c>
+      <c r="C353" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D353" s="16" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="E353" s="18" t="n">
+        <v>2923418.86</v>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B354" s="10" t="n">
+        <v>787</v>
+      </c>
+      <c r="C354" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D354" s="11" t="inlineStr">
+        <is>
+          <t>nicetry</t>
+        </is>
+      </c>
+      <c r="E354" s="14" t="n">
+        <v>2124192.62</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B355" s="15" t="n">
+        <v>787</v>
+      </c>
+      <c r="C355" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D355" s="16" t="inlineStr">
+        <is>
+          <t>group15</t>
+        </is>
+      </c>
+      <c r="E355" s="18" t="n">
+        <v>1987470.15</v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B356" s="10" t="n">
+        <v>787</v>
+      </c>
+      <c r="C356" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D356" s="11" t="inlineStr">
+        <is>
+          <t>group7</t>
+        </is>
+      </c>
+      <c r="E356" s="14" t="n">
+        <v>1908621.41</v>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B357" s="15" t="n">
+        <v>787</v>
+      </c>
+      <c r="C357" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="D357" s="16" t="inlineStr">
+        <is>
+          <t>group14</t>
+        </is>
+      </c>
+      <c r="E357" s="18" t="n">
+        <v>1874441.31</v>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B358" s="10" t="n">
+        <v>787</v>
+      </c>
+      <c r="C358" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="D358" s="11" t="inlineStr">
+        <is>
+          <t>t24</t>
+        </is>
+      </c>
+      <c r="E358" s="14" t="n">
+        <v>1770243.81</v>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B359" s="15" t="n">
+        <v>787</v>
+      </c>
+      <c r="C359" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="D359" s="16" t="inlineStr">
+        <is>
+          <t>montesquieu</t>
+        </is>
+      </c>
+      <c r="E359" s="18" t="n">
+        <v>1686758.1</v>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B360" s="10" t="n">
+        <v>787</v>
+      </c>
+      <c r="C360" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="D360" s="11" t="inlineStr">
+        <is>
+          <t>group8</t>
+        </is>
+      </c>
+      <c r="E360" s="14" t="n">
+        <v>1651191.19</v>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B361" s="15" t="n">
+        <v>787</v>
+      </c>
+      <c r="C361" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="D361" s="16" t="inlineStr">
+        <is>
+          <t>group9</t>
+        </is>
+      </c>
+      <c r="E361" s="18" t="n">
+        <v>1650463.86</v>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B362" s="10" t="n">
+        <v>787</v>
+      </c>
+      <c r="C362" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="D362" s="11" t="inlineStr">
+        <is>
+          <t>deepsleep</t>
+        </is>
+      </c>
+      <c r="E362" s="14" t="n">
+        <v>1499627.98</v>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B363" s="15" t="n">
+        <v>787</v>
+      </c>
+      <c r="C363" s="15" t="n">
+        <v>11</v>
+      </c>
+      <c r="D363" s="16" t="inlineStr">
+        <is>
+          <t>group2</t>
+        </is>
+      </c>
+      <c r="E363" s="18" t="n">
+        <v>1432841.52</v>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B364" s="10" t="n">
+        <v>787</v>
+      </c>
+      <c r="C364" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="D364" s="11" t="inlineStr">
+        <is>
+          <t>teamhlly</t>
+        </is>
+      </c>
+      <c r="E364" s="14" t="n">
+        <v>1432840.79</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B365" s="15" t="n">
+        <v>787</v>
+      </c>
+      <c r="C365" s="15" t="n">
+        <v>13</v>
+      </c>
+      <c r="D365" s="16" t="inlineStr">
+        <is>
+          <t>group25</t>
+        </is>
+      </c>
+      <c r="E365" s="18" t="n">
+        <v>1432685.86</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B366" s="10" t="n">
+        <v>787</v>
+      </c>
+      <c r="C366" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="D366" s="11" t="inlineStr">
+        <is>
+          <t>group11</t>
+        </is>
+      </c>
+      <c r="E366" s="14" t="n">
+        <v>1432673.74</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B367" s="15" t="n">
+        <v>787</v>
+      </c>
+      <c r="C367" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="D367" s="16" t="inlineStr">
+        <is>
+          <t>88888888</t>
+        </is>
+      </c>
+      <c r="E367" s="18" t="n">
+        <v>1432651.41</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B368" s="10" t="n">
+        <v>787</v>
+      </c>
+      <c r="C368" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="D368" s="11" t="inlineStr">
+        <is>
+          <t>aaachemicalseller</t>
+        </is>
+      </c>
+      <c r="E368" s="14" t="n">
+        <v>1367566.46</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B369" s="15" t="n">
+        <v>787</v>
+      </c>
+      <c r="C369" s="15" t="n">
+        <v>17</v>
+      </c>
+      <c r="D369" s="16" t="inlineStr">
+        <is>
+          <t>group12</t>
+        </is>
+      </c>
+      <c r="E369" s="18" t="n">
+        <v>1366075.36</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B370" s="10" t="n">
+        <v>787</v>
+      </c>
+      <c r="C370" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="D370" s="11" t="inlineStr">
+        <is>
+          <t>tigagroup20</t>
+        </is>
+      </c>
+      <c r="E370" s="14" t="n">
+        <v>1332196.27</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B371" s="15" t="n">
+        <v>787</v>
+      </c>
+      <c r="C371" s="15" t="n">
+        <v>19</v>
+      </c>
+      <c r="D371" s="16" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E371" s="18" t="n">
+        <v>1326121.34</v>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B372" s="10" t="n">
+        <v>787</v>
+      </c>
+      <c r="C372" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="D372" s="11" t="inlineStr">
+        <is>
+          <t>666666</t>
+        </is>
+      </c>
+      <c r="E372" s="14" t="n">
+        <v>1280259.09</v>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B373" s="15" t="n">
+        <v>787</v>
+      </c>
+      <c r="C373" s="15" t="n">
+        <v>21</v>
+      </c>
+      <c r="D373" s="16" t="inlineStr">
+        <is>
+          <t>jit</t>
+        </is>
+      </c>
+      <c r="E373" s="18" t="n">
+        <v>1185520.82</v>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B374" s="10" t="n">
+        <v>787</v>
+      </c>
+      <c r="C374" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="D374" s="11" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E374" s="14" t="n">
+        <v>1147066.37</v>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B375" s="15" t="n">
+        <v>787</v>
+      </c>
+      <c r="C375" s="15" t="n">
+        <v>23</v>
+      </c>
+      <c r="D375" s="16" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="E375" s="18" t="n">
+        <v>1144552.74</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B376" s="10" t="n">
+        <v>787</v>
+      </c>
+      <c r="C376" s="10" t="n">
+        <v>24</v>
+      </c>
+      <c r="D376" s="11" t="inlineStr">
+        <is>
+          <t>cleveregg</t>
+        </is>
+      </c>
+      <c r="E376" s="14" t="n">
+        <v>1127899.4</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B377" s="15" t="n">
+        <v>787</v>
+      </c>
+      <c r="C377" s="15" t="n">
+        <v>25</v>
+      </c>
+      <c r="D377" s="16" t="inlineStr">
+        <is>
+          <t>newgroup18</t>
+        </is>
+      </c>
+      <c r="E377" s="18" t="n">
+        <v>1042872.91</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B378" s="10" t="n">
+        <v>787</v>
+      </c>
+      <c r="C378" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="D378" s="11" t="inlineStr">
+        <is>
+          <t>vivo50</t>
+        </is>
+      </c>
+      <c r="E378" s="14" t="n">
+        <v>925479.71</v>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B379" s="24" t="n">
+        <v>787</v>
+      </c>
+      <c r="C379" s="24" t="n">
+        <v>27</v>
+      </c>
+      <c r="D379" s="25" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="E379" s="26" t="n">
+        <v>674776.4300000001</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E352"/>
+  <autoFilter ref="A1:E379"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8591,7 +9155,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S263"/>
+  <dimension ref="A1:S264"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -25218,8 +25782,69 @@
         <v>49300</v>
       </c>
     </row>
+    <row r="264">
+      <c r="A264" s="10" t="n">
+        <v>263</v>
+      </c>
+      <c r="B264" s="10" t="n">
+        <v>787</v>
+      </c>
+      <c r="C264" s="10" t="n">
+        <v>789</v>
+      </c>
+      <c r="D264" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E264" s="11" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="F264" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G264" s="12" t="n">
+        <v>18</v>
+      </c>
+      <c r="H264" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I264" s="12" t="n">
+        <v>18</v>
+      </c>
+      <c r="J264" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K264" s="12" t="n">
+        <v>18</v>
+      </c>
+      <c r="L264" s="14" t="n">
+        <v>674776.4300000001</v>
+      </c>
+      <c r="M264" s="14" t="n">
+        <v>674776.4300000001</v>
+      </c>
+      <c r="N264" s="11" t="n"/>
+      <c r="O264" s="12" t="n">
+        <v>488</v>
+      </c>
+      <c r="P264" s="12" t="n">
+        <v>488</v>
+      </c>
+      <c r="Q264" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="R264" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="S264" s="14" t="n">
+        <v>26100</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S263"/>
+  <autoFilter ref="A1:S264"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -25230,7 +25855,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N787"/>
+  <dimension ref="A1:N788"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -61477,8 +62102,54 @@
         <v>11600</v>
       </c>
     </row>
+    <row r="788">
+      <c r="A788" s="10" t="n">
+        <v>787</v>
+      </c>
+      <c r="B788" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C788" s="12" t="n">
+        <v>18</v>
+      </c>
+      <c r="D788" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E788" s="12" t="n">
+        <v>18</v>
+      </c>
+      <c r="F788" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G788" s="12" t="n">
+        <v>18</v>
+      </c>
+      <c r="H788" s="14" t="n">
+        <v>674776.4300000001</v>
+      </c>
+      <c r="I788" s="12" t="n">
+        <v>488</v>
+      </c>
+      <c r="J788" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K788" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="L788" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="M788" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N788" s="14" t="n">
+        <v>26100</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N787"/>
+  <autoFilter ref="A1:N788"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -61873,7 +62544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -62572,8 +63243,56 @@
         <v>55</v>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="23" t="n">
+        <v>730.66</v>
+      </c>
+      <c r="B29" s="16" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C29" s="16" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D29" s="16" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E29" s="16" t="inlineStr"/>
+      <c r="F29" s="17" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="21" t="n">
+        <v>742.75</v>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D30" s="11" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E30" s="11" t="inlineStr"/>
+      <c r="F30" s="12" t="n">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F28"/>
+  <autoFilter ref="A1:F30"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -62972,7 +63691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U14"/>
+  <dimension ref="A1:U15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -62981,7 +63700,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
@@ -64018,8 +64737,77 @@
         <v>35013.40039060952</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B15" s="15" t="n">
+        <v>787</v>
+      </c>
+      <c r="C15" s="18" t="n">
+        <v>674776.4300000001</v>
+      </c>
+      <c r="D15" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="E15" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="G15" s="18" t="n">
+        <v>2248642.43</v>
+      </c>
+      <c r="H15" s="23" t="n">
+        <v>20</v>
+      </c>
+      <c r="I15" s="23" t="n">
+        <v>55</v>
+      </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>truck</t>
+        </is>
+      </c>
+      <c r="K15" s="27" t="n">
+        <v>3600</v>
+      </c>
+      <c r="L15" s="27" t="n">
+        <v>200</v>
+      </c>
+      <c r="M15" s="17" t="n">
+        <v>488</v>
+      </c>
+      <c r="N15" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="O15" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="P15" s="15" t="n">
+        <v>263</v>
+      </c>
+      <c r="Q15" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="R15" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="S15" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="T15" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="U15" s="16" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U14"/>
+  <autoFilter ref="A1:U15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -64030,7 +64818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E157"/>
+  <dimension ref="A1:E169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -67603,8 +68391,280 @@
         </is>
       </c>
     </row>
+    <row r="158">
+      <c r="A158" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B158" s="10" t="n">
+        <v>787</v>
+      </c>
+      <c r="C158" s="11" t="inlineStr">
+        <is>
+          <t>Starting Cash</t>
+        </is>
+      </c>
+      <c r="D158" s="14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E158" s="11" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B159" s="15" t="n">
+        <v>787</v>
+      </c>
+      <c r="C159" s="16" t="inlineStr">
+        <is>
+          <t>Cash Sources</t>
+        </is>
+      </c>
+      <c r="D159" s="16" t="n"/>
+      <c r="E159" s="16" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B160" s="10" t="n">
+        <v>787</v>
+      </c>
+      <c r="C160" s="11" t="inlineStr">
+        <is>
+          <t>revenues</t>
+        </is>
+      </c>
+      <c r="D160" s="14" t="n">
+        <v>19854850</v>
+      </c>
+      <c r="E160" s="11" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B161" s="15" t="n">
+        <v>787</v>
+      </c>
+      <c r="C161" s="16" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D161" s="18" t="n">
+        <v>286864.67</v>
+      </c>
+      <c r="E161" s="16" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B162" s="10" t="n">
+        <v>787</v>
+      </c>
+      <c r="C162" s="11" t="inlineStr">
+        <is>
+          <t>Cash Uses</t>
+        </is>
+      </c>
+      <c r="D162" s="11" t="n"/>
+      <c r="E162" s="11" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B163" s="15" t="n">
+        <v>787</v>
+      </c>
+      <c r="C163" s="16" t="inlineStr">
+        <is>
+          <t>outbound shipping</t>
+        </is>
+      </c>
+      <c r="D163" s="18" t="n">
+        <v>-2053950</v>
+      </c>
+      <c r="E163" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B164" s="10" t="n">
+        <v>787</v>
+      </c>
+      <c r="C164" s="11" t="inlineStr">
+        <is>
+          <t>inbound shipping</t>
+        </is>
+      </c>
+      <c r="D164" s="14" t="n">
+        <v>-1425000</v>
+      </c>
+      <c r="E164" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B165" s="15" t="n">
+        <v>787</v>
+      </c>
+      <c r="C165" s="16" t="inlineStr">
+        <is>
+          <t>FGI holding</t>
+        </is>
+      </c>
+      <c r="D165" s="18" t="n">
+        <v>-18346</v>
+      </c>
+      <c r="E165" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B166" s="10" t="n">
+        <v>787</v>
+      </c>
+      <c r="C166" s="11" t="inlineStr">
+        <is>
+          <t>add capacity</t>
+        </is>
+      </c>
+      <c r="D166" s="14" t="n">
+        <v>-1749840.87</v>
+      </c>
+      <c r="E166" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B167" s="15" t="n">
+        <v>787</v>
+      </c>
+      <c r="C167" s="16" t="inlineStr">
+        <is>
+          <t>Pipeline inventory holding</t>
+        </is>
+      </c>
+      <c r="D167" s="18" t="n">
+        <v>-27301.37</v>
+      </c>
+      <c r="E167" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B168" s="10" t="n">
+        <v>787</v>
+      </c>
+      <c r="C168" s="11" t="inlineStr">
+        <is>
+          <t>production</t>
+        </is>
+      </c>
+      <c r="D168" s="14" t="n">
+        <v>-14692500</v>
+      </c>
+      <c r="E168" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B169" s="15" t="n">
+        <v>787</v>
+      </c>
+      <c r="C169" s="16" t="inlineStr">
+        <is>
+          <t>Cash Balance</t>
+        </is>
+      </c>
+      <c r="D169" s="18" t="n">
+        <v>674776.4300000001</v>
+      </c>
+      <c r="E169" s="16" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E157"/>
+  <autoFilter ref="A1:E169"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update game data: day 789, cash 726774.18, 3-day period 263
</commit_message>
<xml_diff>
--- a/data/supply_chain_game.xlsx
+++ b/data/supply_chain_game.xlsx
@@ -21,15 +21,15 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$264</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$788</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$790</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'资金构成_旧版'!$A$1:$C$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'运营参数_旧版'!$A$9:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$32</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'排行榜_旧版'!$A$1:$C$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$169</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$181</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'运营参数'!$A$1:$J$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$379</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$406</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -590,7 +590,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-06T02:11:02+08:00</t>
+          <t>2026-09-06T02:26:02+08:00</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>787</v>
+        <v>789</v>
       </c>
     </row>
     <row r="7">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>673</v>
+        <v>671</v>
       </c>
     </row>
     <row r="8">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>674776.4300000001</v>
+        <v>726774.1800000001</v>
       </c>
     </row>
     <row r="11">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>2248642.43</v>
+        <v>2250036.29</v>
       </c>
     </row>
     <row r="15"/>
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>488</v>
+        <v>417</v>
       </c>
     </row>
     <row r="25">
@@ -850,7 +850,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>否（进行中）</t>
+          <t>是</t>
         </is>
       </c>
     </row>
@@ -861,7 +861,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>18</v>
+        <v>89</v>
       </c>
     </row>
     <row r="33">
@@ -881,7 +881,7 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>18</v>
+        <v>89</v>
       </c>
     </row>
     <row r="35">
@@ -901,7 +901,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>18</v>
+        <v>89</v>
       </c>
     </row>
     <row r="37">
@@ -909,6 +909,9 @@
         <is>
           <t>周期现金变动</t>
         </is>
+      </c>
+      <c r="B37" s="4" t="n">
+        <v>92297.74870919751</v>
       </c>
     </row>
     <row r="38"/>
@@ -926,7 +929,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="41">
@@ -937,7 +940,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>784–786</t>
+          <t>787–789</t>
         </is>
       </c>
     </row>
@@ -949,7 +952,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>34.0 / 0.0 / 34.0</t>
+          <t>89.0 / 0.0 / 89.0</t>
         </is>
       </c>
     </row>
@@ -970,7 +973,7 @@
         </is>
       </c>
       <c r="B44" s="4" t="n">
-        <v>35864.06093034125</v>
+        <v>92297.74870919751</v>
       </c>
     </row>
     <row r="45"/>
@@ -1168,7 +1171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E379"/>
+  <dimension ref="A1:E406"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -9143,8 +9146,575 @@
         <v>674776.4300000001</v>
       </c>
     </row>
+    <row r="380">
+      <c r="A380" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B380" s="10" t="n">
+        <v>789</v>
+      </c>
+      <c r="C380" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D380" s="11" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="E380" s="14" t="n">
+        <v>2976810.47</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B381" s="15" t="n">
+        <v>789</v>
+      </c>
+      <c r="C381" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D381" s="16" t="inlineStr">
+        <is>
+          <t>group15</t>
+        </is>
+      </c>
+      <c r="E381" s="18" t="n">
+        <v>2040438.05</v>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B382" s="10" t="n">
+        <v>789</v>
+      </c>
+      <c r="C382" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D382" s="11" t="inlineStr">
+        <is>
+          <t>group7</t>
+        </is>
+      </c>
+      <c r="E382" s="14" t="n">
+        <v>1961482.9</v>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B383" s="15" t="n">
+        <v>789</v>
+      </c>
+      <c r="C383" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D383" s="16" t="inlineStr">
+        <is>
+          <t>nicetry</t>
+        </is>
+      </c>
+      <c r="E383" s="18" t="n">
+        <v>1960558.52</v>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B384" s="10" t="n">
+        <v>789</v>
+      </c>
+      <c r="C384" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="D384" s="11" t="inlineStr">
+        <is>
+          <t>group14</t>
+        </is>
+      </c>
+      <c r="E384" s="14" t="n">
+        <v>1927284.95</v>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B385" s="15" t="n">
+        <v>789</v>
+      </c>
+      <c r="C385" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="D385" s="16" t="inlineStr">
+        <is>
+          <t>t24</t>
+        </is>
+      </c>
+      <c r="E385" s="18" t="n">
+        <v>1823033.02</v>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B386" s="10" t="n">
+        <v>789</v>
+      </c>
+      <c r="C386" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="D386" s="11" t="inlineStr">
+        <is>
+          <t>montesquieu</t>
+        </is>
+      </c>
+      <c r="E386" s="14" t="n">
+        <v>1739284.49</v>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B387" s="15" t="n">
+        <v>789</v>
+      </c>
+      <c r="C387" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="D387" s="16" t="inlineStr">
+        <is>
+          <t>group8</t>
+        </is>
+      </c>
+      <c r="E387" s="18" t="n">
+        <v>1703808.61</v>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B388" s="10" t="n">
+        <v>789</v>
+      </c>
+      <c r="C388" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="D388" s="11" t="inlineStr">
+        <is>
+          <t>group9</t>
+        </is>
+      </c>
+      <c r="E388" s="14" t="n">
+        <v>1703080.9</v>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B389" s="15" t="n">
+        <v>789</v>
+      </c>
+      <c r="C389" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="D389" s="16" t="inlineStr">
+        <is>
+          <t>deepsleep</t>
+        </is>
+      </c>
+      <c r="E389" s="18" t="n">
+        <v>1552210.06</v>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B390" s="10" t="n">
+        <v>789</v>
+      </c>
+      <c r="C390" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="D390" s="11" t="inlineStr">
+        <is>
+          <t>group2</t>
+        </is>
+      </c>
+      <c r="E390" s="14" t="n">
+        <v>1485235.27</v>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B391" s="15" t="n">
+        <v>789</v>
+      </c>
+      <c r="C391" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="D391" s="16" t="inlineStr">
+        <is>
+          <t>teamhlly</t>
+        </is>
+      </c>
+      <c r="E391" s="18" t="n">
+        <v>1485234.54</v>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B392" s="10" t="n">
+        <v>789</v>
+      </c>
+      <c r="C392" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="D392" s="11" t="inlineStr">
+        <is>
+          <t>group25</t>
+        </is>
+      </c>
+      <c r="E392" s="14" t="n">
+        <v>1485079.53</v>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B393" s="15" t="n">
+        <v>789</v>
+      </c>
+      <c r="C393" s="15" t="n">
+        <v>14</v>
+      </c>
+      <c r="D393" s="16" t="inlineStr">
+        <is>
+          <t>group11</t>
+        </is>
+      </c>
+      <c r="E393" s="18" t="n">
+        <v>1485067.4</v>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B394" s="10" t="n">
+        <v>789</v>
+      </c>
+      <c r="C394" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="D394" s="11" t="inlineStr">
+        <is>
+          <t>88888888</t>
+        </is>
+      </c>
+      <c r="E394" s="14" t="n">
+        <v>1485045.06</v>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B395" s="15" t="n">
+        <v>789</v>
+      </c>
+      <c r="C395" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="D395" s="16" t="inlineStr">
+        <is>
+          <t>aaachemicalseller</t>
+        </is>
+      </c>
+      <c r="E395" s="18" t="n">
+        <v>1420145.32</v>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B396" s="10" t="n">
+        <v>789</v>
+      </c>
+      <c r="C396" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="D396" s="11" t="inlineStr">
+        <is>
+          <t>group12</t>
+        </is>
+      </c>
+      <c r="E396" s="14" t="n">
+        <v>1418653.43</v>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B397" s="15" t="n">
+        <v>789</v>
+      </c>
+      <c r="C397" s="15" t="n">
+        <v>18</v>
+      </c>
+      <c r="D397" s="16" t="inlineStr">
+        <is>
+          <t>tigagroup20</t>
+        </is>
+      </c>
+      <c r="E397" s="18" t="n">
+        <v>1384647.05</v>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B398" s="10" t="n">
+        <v>789</v>
+      </c>
+      <c r="C398" s="10" t="n">
+        <v>19</v>
+      </c>
+      <c r="D398" s="11" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E398" s="14" t="n">
+        <v>1378661.01</v>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B399" s="15" t="n">
+        <v>789</v>
+      </c>
+      <c r="C399" s="15" t="n">
+        <v>20</v>
+      </c>
+      <c r="D399" s="16" t="inlineStr">
+        <is>
+          <t>666666</t>
+        </is>
+      </c>
+      <c r="E399" s="18" t="n">
+        <v>1332573.13</v>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B400" s="10" t="n">
+        <v>789</v>
+      </c>
+      <c r="C400" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="D400" s="11" t="inlineStr">
+        <is>
+          <t>jit</t>
+        </is>
+      </c>
+      <c r="E400" s="14" t="n">
+        <v>1237894.98</v>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B401" s="15" t="n">
+        <v>789</v>
+      </c>
+      <c r="C401" s="15" t="n">
+        <v>22</v>
+      </c>
+      <c r="D401" s="16" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E401" s="18" t="n">
+        <v>1199420.44</v>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B402" s="10" t="n">
+        <v>789</v>
+      </c>
+      <c r="C402" s="10" t="n">
+        <v>23</v>
+      </c>
+      <c r="D402" s="11" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="E402" s="14" t="n">
+        <v>1197113.04</v>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B403" s="15" t="n">
+        <v>789</v>
+      </c>
+      <c r="C403" s="15" t="n">
+        <v>24</v>
+      </c>
+      <c r="D403" s="16" t="inlineStr">
+        <is>
+          <t>cleveregg</t>
+        </is>
+      </c>
+      <c r="E403" s="18" t="n">
+        <v>1180133.86</v>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B404" s="10" t="n">
+        <v>789</v>
+      </c>
+      <c r="C404" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="D404" s="11" t="inlineStr">
+        <is>
+          <t>newgroup18</t>
+        </is>
+      </c>
+      <c r="E404" s="14" t="n">
+        <v>1095106.78</v>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B405" s="15" t="n">
+        <v>789</v>
+      </c>
+      <c r="C405" s="15" t="n">
+        <v>26</v>
+      </c>
+      <c r="D405" s="16" t="inlineStr">
+        <is>
+          <t>vivo50</t>
+        </is>
+      </c>
+      <c r="E405" s="18" t="n">
+        <v>977608.42</v>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B406" s="24" t="n">
+        <v>789</v>
+      </c>
+      <c r="C406" s="24" t="n">
+        <v>27</v>
+      </c>
+      <c r="D406" s="25" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="E406" s="26" t="n">
+        <v>726774.1800000001</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E379"/>
+  <autoFilter ref="A1:E406"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -25793,11 +26363,11 @@
         <v>789</v>
       </c>
       <c r="D264" s="10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E264" s="11" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="F264" s="11" t="inlineStr">
@@ -25806,32 +26376,34 @@
         </is>
       </c>
       <c r="G264" s="12" t="n">
-        <v>18</v>
+        <v>89</v>
       </c>
       <c r="H264" s="12" t="n">
         <v>0</v>
       </c>
       <c r="I264" s="12" t="n">
-        <v>18</v>
+        <v>89</v>
       </c>
       <c r="J264" s="19" t="n">
         <v>1</v>
       </c>
       <c r="K264" s="12" t="n">
-        <v>18</v>
+        <v>89</v>
       </c>
       <c r="L264" s="14" t="n">
-        <v>674776.4300000001</v>
+        <v>634476.4312908025</v>
       </c>
       <c r="M264" s="14" t="n">
-        <v>674776.4300000001</v>
-      </c>
-      <c r="N264" s="11" t="n"/>
+        <v>726774.1800000001</v>
+      </c>
+      <c r="N264" s="14" t="n">
+        <v>92297.74870919751</v>
+      </c>
       <c r="O264" s="12" t="n">
-        <v>488</v>
+        <v>417</v>
       </c>
       <c r="P264" s="12" t="n">
-        <v>488</v>
+        <v>454</v>
       </c>
       <c r="Q264" s="12" t="n">
         <v>200</v>
@@ -25840,7 +26412,7 @@
         <v>200</v>
       </c>
       <c r="S264" s="14" t="n">
-        <v>26100</v>
+        <v>129050</v>
       </c>
     </row>
   </sheetData>
@@ -25855,7 +26427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N788"/>
+  <dimension ref="A1:N790"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -62148,8 +62720,100 @@
         <v>26100</v>
       </c>
     </row>
+    <row r="789">
+      <c r="A789" s="15" t="n">
+        <v>788</v>
+      </c>
+      <c r="B789" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C789" s="17" t="n">
+        <v>31</v>
+      </c>
+      <c r="D789" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E789" s="17" t="n">
+        <v>31</v>
+      </c>
+      <c r="F789" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G789" s="17" t="n">
+        <v>31</v>
+      </c>
+      <c r="H789" s="18" t="n">
+        <v>674764.1076772655</v>
+      </c>
+      <c r="I789" s="17" t="n">
+        <v>457</v>
+      </c>
+      <c r="J789" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K789" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="L789" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="M789" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N789" s="18" t="n">
+        <v>44950</v>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" s="10" t="n">
+        <v>789</v>
+      </c>
+      <c r="B790" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C790" s="12" t="n">
+        <v>40</v>
+      </c>
+      <c r="D790" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E790" s="12" t="n">
+        <v>40</v>
+      </c>
+      <c r="F790" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G790" s="12" t="n">
+        <v>40</v>
+      </c>
+      <c r="H790" s="14" t="n">
+        <v>726774.1800000001</v>
+      </c>
+      <c r="I790" s="12" t="n">
+        <v>417</v>
+      </c>
+      <c r="J790" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K790" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="L790" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="M790" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N790" s="14" t="n">
+        <v>58000</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N788"/>
+  <autoFilter ref="A1:N790"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -62544,7 +63208,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -63291,8 +63955,56 @@
         <v>55</v>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" s="23" t="n">
+        <v>730.66</v>
+      </c>
+      <c r="B31" s="16" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C31" s="16" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D31" s="16" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E31" s="16" t="inlineStr"/>
+      <c r="F31" s="17" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="21" t="n">
+        <v>742.75</v>
+      </c>
+      <c r="B32" s="11" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C32" s="11" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D32" s="11" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E32" s="11" t="inlineStr"/>
+      <c r="F32" s="12" t="n">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F30"/>
+  <autoFilter ref="A1:F32"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -63691,7 +64403,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U15"/>
+  <dimension ref="A1:U16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -63700,7 +64412,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
@@ -64806,8 +65518,79 @@
       </c>
       <c r="U15" s="16" t="n"/>
     </row>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="n">
+        <v>789</v>
+      </c>
+      <c r="C16" s="14" t="n">
+        <v>726774.1800000001</v>
+      </c>
+      <c r="D16" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="E16" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="F16" s="11" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="G16" s="14" t="n">
+        <v>2250036.29</v>
+      </c>
+      <c r="H16" s="21" t="n">
+        <v>20</v>
+      </c>
+      <c r="I16" s="21" t="n">
+        <v>55</v>
+      </c>
+      <c r="J16" s="11" t="inlineStr">
+        <is>
+          <t>truck</t>
+        </is>
+      </c>
+      <c r="K16" s="22" t="n">
+        <v>3600</v>
+      </c>
+      <c r="L16" s="22" t="n">
+        <v>200</v>
+      </c>
+      <c r="M16" s="12" t="n">
+        <v>417</v>
+      </c>
+      <c r="N16" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="O16" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="P16" s="10" t="n">
+        <v>263</v>
+      </c>
+      <c r="Q16" s="12" t="n">
+        <v>89</v>
+      </c>
+      <c r="R16" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S16" s="12" t="n">
+        <v>89</v>
+      </c>
+      <c r="T16" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="U16" s="14" t="n">
+        <v>92297.74870919751</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U15"/>
+  <autoFilter ref="A1:U16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -64818,7 +65601,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E169"/>
+  <dimension ref="A1:E181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -68663,8 +69446,280 @@
         </is>
       </c>
     </row>
+    <row r="170">
+      <c r="A170" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B170" s="10" t="n">
+        <v>789</v>
+      </c>
+      <c r="C170" s="11" t="inlineStr">
+        <is>
+          <t>Starting Cash</t>
+        </is>
+      </c>
+      <c r="D170" s="14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E170" s="11" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B171" s="15" t="n">
+        <v>789</v>
+      </c>
+      <c r="C171" s="16" t="inlineStr">
+        <is>
+          <t>Cash Sources</t>
+        </is>
+      </c>
+      <c r="D171" s="16" t="n"/>
+      <c r="E171" s="16" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B172" s="10" t="n">
+        <v>789</v>
+      </c>
+      <c r="C172" s="11" t="inlineStr">
+        <is>
+          <t>revenues</t>
+        </is>
+      </c>
+      <c r="D172" s="14" t="n">
+        <v>19912850</v>
+      </c>
+      <c r="E172" s="11" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B173" s="15" t="n">
+        <v>789</v>
+      </c>
+      <c r="C173" s="16" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D173" s="18" t="n">
+        <v>287220.04</v>
+      </c>
+      <c r="E173" s="16" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B174" s="10" t="n">
+        <v>789</v>
+      </c>
+      <c r="C174" s="11" t="inlineStr">
+        <is>
+          <t>Cash Uses</t>
+        </is>
+      </c>
+      <c r="D174" s="11" t="n"/>
+      <c r="E174" s="11" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B175" s="15" t="n">
+        <v>789</v>
+      </c>
+      <c r="C175" s="16" t="inlineStr">
+        <is>
+          <t>outbound shipping</t>
+        </is>
+      </c>
+      <c r="D175" s="18" t="n">
+        <v>-2059950</v>
+      </c>
+      <c r="E175" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B176" s="10" t="n">
+        <v>789</v>
+      </c>
+      <c r="C176" s="11" t="inlineStr">
+        <is>
+          <t>inbound shipping</t>
+        </is>
+      </c>
+      <c r="D176" s="14" t="n">
+        <v>-1425000</v>
+      </c>
+      <c r="E176" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B177" s="15" t="n">
+        <v>789</v>
+      </c>
+      <c r="C177" s="16" t="inlineStr">
+        <is>
+          <t>FGI holding</t>
+        </is>
+      </c>
+      <c r="D177" s="18" t="n">
+        <v>-18594.04</v>
+      </c>
+      <c r="E177" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B178" s="10" t="n">
+        <v>789</v>
+      </c>
+      <c r="C178" s="11" t="inlineStr">
+        <is>
+          <t>add capacity</t>
+        </is>
+      </c>
+      <c r="D178" s="14" t="n">
+        <v>-1749840.87</v>
+      </c>
+      <c r="E178" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B179" s="15" t="n">
+        <v>789</v>
+      </c>
+      <c r="C179" s="16" t="inlineStr">
+        <is>
+          <t>Pipeline inventory holding</t>
+        </is>
+      </c>
+      <c r="D179" s="18" t="n">
+        <v>-27410.96</v>
+      </c>
+      <c r="E179" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B180" s="10" t="n">
+        <v>789</v>
+      </c>
+      <c r="C180" s="11" t="inlineStr">
+        <is>
+          <t>production</t>
+        </is>
+      </c>
+      <c r="D180" s="14" t="n">
+        <v>-14692500</v>
+      </c>
+      <c r="E180" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B181" s="15" t="n">
+        <v>789</v>
+      </c>
+      <c r="C181" s="16" t="inlineStr">
+        <is>
+          <t>Cash Balance</t>
+        </is>
+      </c>
+      <c r="D181" s="18" t="n">
+        <v>726774.1800000001</v>
+      </c>
+      <c r="E181" s="16" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E169"/>
+  <autoFilter ref="A1:E181"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update game data: day 790, cash 756702.0, 3-day period 264
</commit_message>
<xml_diff>
--- a/data/supply_chain_game.xlsx
+++ b/data/supply_chain_game.xlsx
@@ -20,16 +20,16 @@
     <sheet name="排行榜" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$264</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$790</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$265</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$791</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'资金构成_旧版'!$A$1:$C$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'运营参数_旧版'!$A$9:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'排行榜_旧版'!$A$1:$C$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$181</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$193</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'运营参数'!$A$1:$J$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$406</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$433</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -590,7 +590,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-06T02:26:02+08:00</t>
+          <t>2026-09-06T02:41:02+08:00</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>789</v>
+        <v>790</v>
       </c>
     </row>
     <row r="7">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>671</v>
+        <v>670</v>
       </c>
     </row>
     <row r="8">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>726774.1800000001</v>
+        <v>756702</v>
       </c>
     </row>
     <row r="11">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>2250036.29</v>
+        <v>2250733.49</v>
       </c>
     </row>
     <row r="15"/>
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>417</v>
+        <v>394</v>
       </c>
     </row>
     <row r="25">
@@ -827,7 +827,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="30">
@@ -838,7 +838,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>787–789</t>
+          <t>790–792</t>
         </is>
       </c>
     </row>
@@ -850,7 +850,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否（进行中）</t>
         </is>
       </c>
     </row>
@@ -861,7 +861,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>89</v>
+        <v>23</v>
       </c>
     </row>
     <row r="33">
@@ -881,7 +881,7 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>89</v>
+        <v>23</v>
       </c>
     </row>
     <row r="35">
@@ -901,7 +901,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>89</v>
+        <v>23</v>
       </c>
     </row>
     <row r="37">
@@ -909,9 +909,6 @@
         <is>
           <t>周期现金变动</t>
         </is>
-      </c>
-      <c r="B37" s="4" t="n">
-        <v>92297.74870919751</v>
       </c>
     </row>
     <row r="38"/>
@@ -973,7 +970,7 @@
         </is>
       </c>
       <c r="B44" s="4" t="n">
-        <v>92297.74870919751</v>
+        <v>92297.74807681097</v>
       </c>
     </row>
     <row r="45"/>
@@ -1171,7 +1168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E406"/>
+  <dimension ref="A1:E433"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -9713,8 +9710,575 @@
         <v>726774.1800000001</v>
       </c>
     </row>
+    <row r="407">
+      <c r="A407" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B407" s="15" t="n">
+        <v>790</v>
+      </c>
+      <c r="C407" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D407" s="16" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="E407" s="18" t="n">
+        <v>3007435.49</v>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B408" s="10" t="n">
+        <v>790</v>
+      </c>
+      <c r="C408" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D408" s="11" t="inlineStr">
+        <is>
+          <t>group15</t>
+        </is>
+      </c>
+      <c r="E408" s="14" t="n">
+        <v>2070851.14</v>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B409" s="15" t="n">
+        <v>790</v>
+      </c>
+      <c r="C409" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D409" s="16" t="inlineStr">
+        <is>
+          <t>group7</t>
+        </is>
+      </c>
+      <c r="E409" s="18" t="n">
+        <v>1991842.77</v>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B410" s="10" t="n">
+        <v>790</v>
+      </c>
+      <c r="C410" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D410" s="11" t="inlineStr">
+        <is>
+          <t>nicetry</t>
+        </is>
+      </c>
+      <c r="E410" s="14" t="n">
+        <v>1990863.35</v>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B411" s="15" t="n">
+        <v>790</v>
+      </c>
+      <c r="C411" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="D411" s="16" t="inlineStr">
+        <is>
+          <t>group14</t>
+        </is>
+      </c>
+      <c r="E411" s="18" t="n">
+        <v>1949835.03</v>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B412" s="10" t="n">
+        <v>790</v>
+      </c>
+      <c r="C412" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="D412" s="11" t="inlineStr">
+        <is>
+          <t>montesquieu</t>
+        </is>
+      </c>
+      <c r="E412" s="14" t="n">
+        <v>1769476.74</v>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B413" s="15" t="n">
+        <v>790</v>
+      </c>
+      <c r="C413" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="D413" s="16" t="inlineStr">
+        <is>
+          <t>group8</t>
+        </is>
+      </c>
+      <c r="E413" s="18" t="n">
+        <v>1734046.39</v>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B414" s="10" t="n">
+        <v>790</v>
+      </c>
+      <c r="C414" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="D414" s="11" t="inlineStr">
+        <is>
+          <t>t24</t>
+        </is>
+      </c>
+      <c r="E414" s="14" t="n">
+        <v>1636827.15</v>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B415" s="15" t="n">
+        <v>790</v>
+      </c>
+      <c r="C415" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="D415" s="16" t="inlineStr">
+        <is>
+          <t>deepsleep</t>
+        </is>
+      </c>
+      <c r="E415" s="18" t="n">
+        <v>1582430.17</v>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B416" s="10" t="n">
+        <v>790</v>
+      </c>
+      <c r="C416" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="D416" s="11" t="inlineStr">
+        <is>
+          <t>group9</t>
+        </is>
+      </c>
+      <c r="E416" s="14" t="n">
+        <v>1516742.01</v>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B417" s="15" t="n">
+        <v>790</v>
+      </c>
+      <c r="C417" s="15" t="n">
+        <v>11</v>
+      </c>
+      <c r="D417" s="16" t="inlineStr">
+        <is>
+          <t>group2</t>
+        </is>
+      </c>
+      <c r="E417" s="18" t="n">
+        <v>1515361.18</v>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B418" s="10" t="n">
+        <v>790</v>
+      </c>
+      <c r="C418" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="D418" s="11" t="inlineStr">
+        <is>
+          <t>teamhlly</t>
+        </is>
+      </c>
+      <c r="E418" s="14" t="n">
+        <v>1515360.44</v>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B419" s="15" t="n">
+        <v>790</v>
+      </c>
+      <c r="C419" s="15" t="n">
+        <v>13</v>
+      </c>
+      <c r="D419" s="16" t="inlineStr">
+        <is>
+          <t>group25</t>
+        </is>
+      </c>
+      <c r="E419" s="18" t="n">
+        <v>1515205.39</v>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B420" s="10" t="n">
+        <v>790</v>
+      </c>
+      <c r="C420" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="D420" s="11" t="inlineStr">
+        <is>
+          <t>group11</t>
+        </is>
+      </c>
+      <c r="E420" s="14" t="n">
+        <v>1515193.26</v>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B421" s="15" t="n">
+        <v>790</v>
+      </c>
+      <c r="C421" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="D421" s="16" t="inlineStr">
+        <is>
+          <t>88888888</t>
+        </is>
+      </c>
+      <c r="E421" s="18" t="n">
+        <v>1515170.91</v>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B422" s="10" t="n">
+        <v>790</v>
+      </c>
+      <c r="C422" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="D422" s="11" t="inlineStr">
+        <is>
+          <t>aaachemicalseller</t>
+        </is>
+      </c>
+      <c r="E422" s="14" t="n">
+        <v>1442562.95</v>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B423" s="15" t="n">
+        <v>790</v>
+      </c>
+      <c r="C423" s="15" t="n">
+        <v>17</v>
+      </c>
+      <c r="D423" s="16" t="inlineStr">
+        <is>
+          <t>group12</t>
+        </is>
+      </c>
+      <c r="E423" s="18" t="n">
+        <v>1441070.68</v>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B424" s="10" t="n">
+        <v>790</v>
+      </c>
+      <c r="C424" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="D424" s="11" t="inlineStr">
+        <is>
+          <t>tigagroup20</t>
+        </is>
+      </c>
+      <c r="E424" s="14" t="n">
+        <v>1414801.48</v>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B425" s="15" t="n">
+        <v>790</v>
+      </c>
+      <c r="C425" s="15" t="n">
+        <v>19</v>
+      </c>
+      <c r="D425" s="16" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E425" s="18" t="n">
+        <v>1408859.9</v>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B426" s="10" t="n">
+        <v>790</v>
+      </c>
+      <c r="C426" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="D426" s="11" t="inlineStr">
+        <is>
+          <t>666666</t>
+        </is>
+      </c>
+      <c r="E426" s="14" t="n">
+        <v>1362659.17</v>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B427" s="15" t="n">
+        <v>790</v>
+      </c>
+      <c r="C427" s="15" t="n">
+        <v>21</v>
+      </c>
+      <c r="D427" s="16" t="inlineStr">
+        <is>
+          <t>jit</t>
+        </is>
+      </c>
+      <c r="E427" s="18" t="n">
+        <v>1268011.08</v>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B428" s="10" t="n">
+        <v>790</v>
+      </c>
+      <c r="C428" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="D428" s="11" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E428" s="14" t="n">
+        <v>1229526.49</v>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B429" s="15" t="n">
+        <v>790</v>
+      </c>
+      <c r="C429" s="15" t="n">
+        <v>23</v>
+      </c>
+      <c r="D429" s="16" t="inlineStr">
+        <is>
+          <t>cleveregg</t>
+        </is>
+      </c>
+      <c r="E429" s="18" t="n">
+        <v>1210180.08</v>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B430" s="10" t="n">
+        <v>790</v>
+      </c>
+      <c r="C430" s="10" t="n">
+        <v>24</v>
+      </c>
+      <c r="D430" s="11" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="E430" s="14" t="n">
+        <v>1168314.39</v>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B431" s="15" t="n">
+        <v>790</v>
+      </c>
+      <c r="C431" s="15" t="n">
+        <v>25</v>
+      </c>
+      <c r="D431" s="16" t="inlineStr">
+        <is>
+          <t>newgroup18</t>
+        </is>
+      </c>
+      <c r="E431" s="18" t="n">
+        <v>1125152.72</v>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B432" s="10" t="n">
+        <v>790</v>
+      </c>
+      <c r="C432" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="D432" s="11" t="inlineStr">
+        <is>
+          <t>vivo50</t>
+        </is>
+      </c>
+      <c r="E432" s="14" t="n">
+        <v>1007601.75</v>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B433" s="24" t="n">
+        <v>790</v>
+      </c>
+      <c r="C433" s="24" t="n">
+        <v>27</v>
+      </c>
+      <c r="D433" s="25" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="E433" s="26" t="n">
+        <v>756702</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E406"/>
+  <autoFilter ref="A1:E433"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9725,7 +10289,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S264"/>
+  <dimension ref="A1:S265"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -26415,8 +26979,69 @@
         <v>129050</v>
       </c>
     </row>
+    <row r="265">
+      <c r="A265" s="15" t="n">
+        <v>264</v>
+      </c>
+      <c r="B265" s="15" t="n">
+        <v>790</v>
+      </c>
+      <c r="C265" s="15" t="n">
+        <v>792</v>
+      </c>
+      <c r="D265" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E265" s="16" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="F265" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G265" s="17" t="n">
+        <v>23</v>
+      </c>
+      <c r="H265" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I265" s="17" t="n">
+        <v>23</v>
+      </c>
+      <c r="J265" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K265" s="17" t="n">
+        <v>23</v>
+      </c>
+      <c r="L265" s="18" t="n">
+        <v>756702</v>
+      </c>
+      <c r="M265" s="18" t="n">
+        <v>756702</v>
+      </c>
+      <c r="N265" s="16" t="n"/>
+      <c r="O265" s="17" t="n">
+        <v>394</v>
+      </c>
+      <c r="P265" s="17" t="n">
+        <v>394</v>
+      </c>
+      <c r="Q265" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="R265" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="S265" s="18" t="n">
+        <v>33350</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S264"/>
+  <autoFilter ref="A1:S265"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -26427,7 +27052,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N790"/>
+  <dimension ref="A1:N791"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -62812,8 +63437,54 @@
         <v>58000</v>
       </c>
     </row>
+    <row r="791">
+      <c r="A791" s="15" t="n">
+        <v>790</v>
+      </c>
+      <c r="B791" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C791" s="17" t="n">
+        <v>23</v>
+      </c>
+      <c r="D791" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E791" s="17" t="n">
+        <v>23</v>
+      </c>
+      <c r="F791" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G791" s="17" t="n">
+        <v>23</v>
+      </c>
+      <c r="H791" s="18" t="n">
+        <v>756702</v>
+      </c>
+      <c r="I791" s="17" t="n">
+        <v>394</v>
+      </c>
+      <c r="J791" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K791" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="L791" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="M791" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N791" s="18" t="n">
+        <v>33350</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N790"/>
+  <autoFilter ref="A1:N791"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -63208,7 +63879,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -64003,8 +64674,56 @@
         <v>55</v>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="23" t="n">
+        <v>730.66</v>
+      </c>
+      <c r="B33" s="16" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C33" s="16" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D33" s="16" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E33" s="16" t="inlineStr"/>
+      <c r="F33" s="17" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="21" t="n">
+        <v>742.75</v>
+      </c>
+      <c r="B34" s="11" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D34" s="11" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E34" s="11" t="inlineStr"/>
+      <c r="F34" s="12" t="n">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F32"/>
+  <autoFilter ref="A1:F34"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -64403,7 +65122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U16"/>
+  <dimension ref="A1:U17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -65589,8 +66308,77 @@
         <v>92297.74870919751</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B17" s="15" t="n">
+        <v>790</v>
+      </c>
+      <c r="C17" s="18" t="n">
+        <v>756702</v>
+      </c>
+      <c r="D17" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="E17" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="G17" s="18" t="n">
+        <v>2250733.49</v>
+      </c>
+      <c r="H17" s="23" t="n">
+        <v>20</v>
+      </c>
+      <c r="I17" s="23" t="n">
+        <v>55</v>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>truck</t>
+        </is>
+      </c>
+      <c r="K17" s="27" t="n">
+        <v>3600</v>
+      </c>
+      <c r="L17" s="27" t="n">
+        <v>200</v>
+      </c>
+      <c r="M17" s="17" t="n">
+        <v>394</v>
+      </c>
+      <c r="N17" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="O17" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="P17" s="15" t="n">
+        <v>264</v>
+      </c>
+      <c r="Q17" s="17" t="n">
+        <v>23</v>
+      </c>
+      <c r="R17" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="S17" s="17" t="n">
+        <v>23</v>
+      </c>
+      <c r="T17" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="U17" s="16" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U16"/>
+  <autoFilter ref="A1:U17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -65601,7 +66389,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E181"/>
+  <dimension ref="A1:E193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -69718,8 +70506,280 @@
         </is>
       </c>
     </row>
+    <row r="182">
+      <c r="A182" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B182" s="10" t="n">
+        <v>790</v>
+      </c>
+      <c r="C182" s="11" t="inlineStr">
+        <is>
+          <t>Starting Cash</t>
+        </is>
+      </c>
+      <c r="D182" s="14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E182" s="11" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B183" s="15" t="n">
+        <v>790</v>
+      </c>
+      <c r="C183" s="16" t="inlineStr">
+        <is>
+          <t>Cash Sources</t>
+        </is>
+      </c>
+      <c r="D183" s="16" t="n"/>
+      <c r="E183" s="16" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B184" s="10" t="n">
+        <v>790</v>
+      </c>
+      <c r="C184" s="11" t="inlineStr">
+        <is>
+          <t>revenues</t>
+        </is>
+      </c>
+      <c r="D184" s="14" t="n">
+        <v>19946200</v>
+      </c>
+      <c r="E184" s="11" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B185" s="15" t="n">
+        <v>790</v>
+      </c>
+      <c r="C185" s="16" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D185" s="18" t="n">
+        <v>287413.76</v>
+      </c>
+      <c r="E185" s="16" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B186" s="10" t="n">
+        <v>790</v>
+      </c>
+      <c r="C186" s="11" t="inlineStr">
+        <is>
+          <t>Cash Uses</t>
+        </is>
+      </c>
+      <c r="D186" s="11" t="n"/>
+      <c r="E186" s="11" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B187" s="15" t="n">
+        <v>790</v>
+      </c>
+      <c r="C187" s="16" t="inlineStr">
+        <is>
+          <t>outbound shipping</t>
+        </is>
+      </c>
+      <c r="D187" s="18" t="n">
+        <v>-2063400</v>
+      </c>
+      <c r="E187" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B188" s="10" t="n">
+        <v>790</v>
+      </c>
+      <c r="C188" s="11" t="inlineStr">
+        <is>
+          <t>inbound shipping</t>
+        </is>
+      </c>
+      <c r="D188" s="14" t="n">
+        <v>-1425000</v>
+      </c>
+      <c r="E188" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B189" s="15" t="n">
+        <v>790</v>
+      </c>
+      <c r="C189" s="16" t="inlineStr">
+        <is>
+          <t>FGI holding</t>
+        </is>
+      </c>
+      <c r="D189" s="18" t="n">
+        <v>-18705.13</v>
+      </c>
+      <c r="E189" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B190" s="10" t="n">
+        <v>790</v>
+      </c>
+      <c r="C190" s="11" t="inlineStr">
+        <is>
+          <t>add capacity</t>
+        </is>
+      </c>
+      <c r="D190" s="14" t="n">
+        <v>-1749840.87</v>
+      </c>
+      <c r="E190" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B191" s="15" t="n">
+        <v>790</v>
+      </c>
+      <c r="C191" s="16" t="inlineStr">
+        <is>
+          <t>Pipeline inventory holding</t>
+        </is>
+      </c>
+      <c r="D191" s="18" t="n">
+        <v>-27465.75</v>
+      </c>
+      <c r="E191" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B192" s="10" t="n">
+        <v>790</v>
+      </c>
+      <c r="C192" s="11" t="inlineStr">
+        <is>
+          <t>production</t>
+        </is>
+      </c>
+      <c r="D192" s="14" t="n">
+        <v>-14692500</v>
+      </c>
+      <c r="E192" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B193" s="15" t="n">
+        <v>790</v>
+      </c>
+      <c r="C193" s="16" t="inlineStr">
+        <is>
+          <t>Cash Balance</t>
+        </is>
+      </c>
+      <c r="D193" s="18" t="n">
+        <v>756702</v>
+      </c>
+      <c r="E193" s="16" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E181"/>
+  <autoFilter ref="A1:E193"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update game data: day 791, cash 764538.28, 3-day period 264
</commit_message>
<xml_diff>
--- a/data/supply_chain_game.xlsx
+++ b/data/supply_chain_game.xlsx
@@ -21,15 +21,15 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$265</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$791</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$792</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'资金构成_旧版'!$A$1:$C$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'运营参数_旧版'!$A$9:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'排行榜_旧版'!$A$1:$C$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$193</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$205</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'运营参数'!$A$1:$J$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$433</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$460</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -590,7 +590,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-06T02:41:02+08:00</t>
+          <t>2026-09-06T02:56:02+08:00</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>790</v>
+        <v>791</v>
       </c>
     </row>
     <row r="7">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>670</v>
+        <v>669</v>
       </c>
     </row>
     <row r="8">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>756702</v>
+        <v>764538.28</v>
       </c>
     </row>
     <row r="11">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>2250733.49</v>
+        <v>2251430.88</v>
       </c>
     </row>
     <row r="15"/>
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>394</v>
+        <v>590</v>
       </c>
     </row>
     <row r="25">
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -861,7 +861,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="33">
@@ -881,7 +881,7 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="35">
@@ -901,7 +901,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="37">
@@ -909,6 +909,9 @@
         <is>
           <t>周期现金变动</t>
         </is>
+      </c>
+      <c r="B37" s="4" t="n">
+        <v>5254.146354625002</v>
       </c>
     </row>
     <row r="38"/>
@@ -970,7 +973,7 @@
         </is>
       </c>
       <c r="B44" s="4" t="n">
-        <v>92297.74807681097</v>
+        <v>92612.70048965176</v>
       </c>
     </row>
     <row r="45"/>
@@ -1168,7 +1171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E433"/>
+  <dimension ref="A1:E460"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -10277,8 +10280,575 @@
         <v>756702</v>
       </c>
     </row>
+    <row r="434">
+      <c r="A434" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B434" s="10" t="n">
+        <v>791</v>
+      </c>
+      <c r="C434" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D434" s="11" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="E434" s="14" t="n">
+        <v>3015969.16</v>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B435" s="15" t="n">
+        <v>791</v>
+      </c>
+      <c r="C435" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D435" s="16" t="inlineStr">
+        <is>
+          <t>group15</t>
+        </is>
+      </c>
+      <c r="E435" s="18" t="n">
+        <v>2079126.36</v>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B436" s="10" t="n">
+        <v>791</v>
+      </c>
+      <c r="C436" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D436" s="11" t="inlineStr">
+        <is>
+          <t>group7</t>
+        </is>
+      </c>
+      <c r="E436" s="14" t="n">
+        <v>2000111.21</v>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B437" s="15" t="n">
+        <v>791</v>
+      </c>
+      <c r="C437" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D437" s="16" t="inlineStr">
+        <is>
+          <t>nicetry</t>
+        </is>
+      </c>
+      <c r="E437" s="18" t="n">
+        <v>1999076.74</v>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B438" s="10" t="n">
+        <v>791</v>
+      </c>
+      <c r="C438" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="D438" s="11" t="inlineStr">
+        <is>
+          <t>group14</t>
+        </is>
+      </c>
+      <c r="E438" s="14" t="n">
+        <v>1950289.45</v>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B439" s="15" t="n">
+        <v>791</v>
+      </c>
+      <c r="C439" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="D439" s="16" t="inlineStr">
+        <is>
+          <t>montesquieu</t>
+        </is>
+      </c>
+      <c r="E439" s="18" t="n">
+        <v>1777577.52</v>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B440" s="10" t="n">
+        <v>791</v>
+      </c>
+      <c r="C440" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="D440" s="11" t="inlineStr">
+        <is>
+          <t>t24</t>
+        </is>
+      </c>
+      <c r="E440" s="14" t="n">
+        <v>1644948.08</v>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B441" s="15" t="n">
+        <v>791</v>
+      </c>
+      <c r="C441" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="D441" s="16" t="inlineStr">
+        <is>
+          <t>deepsleep</t>
+        </is>
+      </c>
+      <c r="E441" s="18" t="n">
+        <v>1590558.8</v>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B442" s="10" t="n">
+        <v>791</v>
+      </c>
+      <c r="C442" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="D442" s="11" t="inlineStr">
+        <is>
+          <t>group8</t>
+        </is>
+      </c>
+      <c r="E442" s="14" t="n">
+        <v>1525644.48</v>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B443" s="15" t="n">
+        <v>791</v>
+      </c>
+      <c r="C443" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="D443" s="16" t="inlineStr">
+        <is>
+          <t>group9</t>
+        </is>
+      </c>
+      <c r="E443" s="18" t="n">
+        <v>1524776.77</v>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B444" s="10" t="n">
+        <v>791</v>
+      </c>
+      <c r="C444" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="D444" s="11" t="inlineStr">
+        <is>
+          <t>group2</t>
+        </is>
+      </c>
+      <c r="E444" s="14" t="n">
+        <v>1523395.58</v>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B445" s="15" t="n">
+        <v>791</v>
+      </c>
+      <c r="C445" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="D445" s="16" t="inlineStr">
+        <is>
+          <t>teamhlly</t>
+        </is>
+      </c>
+      <c r="E445" s="18" t="n">
+        <v>1523394.85</v>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B446" s="10" t="n">
+        <v>791</v>
+      </c>
+      <c r="C446" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="D446" s="11" t="inlineStr">
+        <is>
+          <t>group25</t>
+        </is>
+      </c>
+      <c r="E446" s="14" t="n">
+        <v>1523239.76</v>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B447" s="15" t="n">
+        <v>791</v>
+      </c>
+      <c r="C447" s="15" t="n">
+        <v>14</v>
+      </c>
+      <c r="D447" s="16" t="inlineStr">
+        <is>
+          <t>group11</t>
+        </is>
+      </c>
+      <c r="E447" s="18" t="n">
+        <v>1523227.62</v>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B448" s="10" t="n">
+        <v>791</v>
+      </c>
+      <c r="C448" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="D448" s="11" t="inlineStr">
+        <is>
+          <t>88888888</t>
+        </is>
+      </c>
+      <c r="E448" s="14" t="n">
+        <v>1523205.27</v>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B449" s="15" t="n">
+        <v>791</v>
+      </c>
+      <c r="C449" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="D449" s="16" t="inlineStr">
+        <is>
+          <t>group12</t>
+        </is>
+      </c>
+      <c r="E449" s="18" t="n">
+        <v>1451792.35</v>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B450" s="10" t="n">
+        <v>791</v>
+      </c>
+      <c r="C450" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="D450" s="11" t="inlineStr">
+        <is>
+          <t>aaachemicalseller</t>
+        </is>
+      </c>
+      <c r="E450" s="14" t="n">
+        <v>1442884.9</v>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B451" s="15" t="n">
+        <v>791</v>
+      </c>
+      <c r="C451" s="15" t="n">
+        <v>18</v>
+      </c>
+      <c r="D451" s="16" t="inlineStr">
+        <is>
+          <t>tigagroup20</t>
+        </is>
+      </c>
+      <c r="E451" s="18" t="n">
+        <v>1422864.42</v>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B452" s="10" t="n">
+        <v>791</v>
+      </c>
+      <c r="C452" s="10" t="n">
+        <v>19</v>
+      </c>
+      <c r="D452" s="11" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E452" s="14" t="n">
+        <v>1416967.32</v>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B453" s="15" t="n">
+        <v>791</v>
+      </c>
+      <c r="C453" s="15" t="n">
+        <v>20</v>
+      </c>
+      <c r="D453" s="16" t="inlineStr">
+        <is>
+          <t>666666</t>
+        </is>
+      </c>
+      <c r="E453" s="18" t="n">
+        <v>1370653.7</v>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B454" s="10" t="n">
+        <v>791</v>
+      </c>
+      <c r="C454" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="D454" s="11" t="inlineStr">
+        <is>
+          <t>jit</t>
+        </is>
+      </c>
+      <c r="E454" s="14" t="n">
+        <v>1276035.69</v>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B455" s="15" t="n">
+        <v>791</v>
+      </c>
+      <c r="C455" s="15" t="n">
+        <v>22</v>
+      </c>
+      <c r="D455" s="16" t="inlineStr">
+        <is>
+          <t>cleveregg</t>
+        </is>
+      </c>
+      <c r="E455" s="18" t="n">
+        <v>1218134.79</v>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B456" s="10" t="n">
+        <v>791</v>
+      </c>
+      <c r="C456" s="10" t="n">
+        <v>23</v>
+      </c>
+      <c r="D456" s="11" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="E456" s="14" t="n">
+        <v>1176396.33</v>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B457" s="15" t="n">
+        <v>791</v>
+      </c>
+      <c r="C457" s="15" t="n">
+        <v>24</v>
+      </c>
+      <c r="D457" s="16" t="inlineStr">
+        <is>
+          <t>newgroup18</t>
+        </is>
+      </c>
+      <c r="E457" s="18" t="n">
+        <v>1133107.14</v>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B458" s="10" t="n">
+        <v>791</v>
+      </c>
+      <c r="C458" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="D458" s="11" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E458" s="14" t="n">
+        <v>1020992.82</v>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B459" s="15" t="n">
+        <v>791</v>
+      </c>
+      <c r="C459" s="15" t="n">
+        <v>26</v>
+      </c>
+      <c r="D459" s="16" t="inlineStr">
+        <is>
+          <t>vivo50</t>
+        </is>
+      </c>
+      <c r="E459" s="18" t="n">
+        <v>1015503.56</v>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B460" s="24" t="n">
+        <v>791</v>
+      </c>
+      <c r="C460" s="24" t="n">
+        <v>27</v>
+      </c>
+      <c r="D460" s="25" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="E460" s="26" t="n">
+        <v>764538.28</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E433"/>
+  <autoFilter ref="A1:E460"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -26990,7 +27560,7 @@
         <v>792</v>
       </c>
       <c r="D265" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E265" s="16" t="inlineStr">
         <is>
@@ -27003,41 +27573,43 @@
         </is>
       </c>
       <c r="G265" s="17" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="H265" s="17" t="n">
         <v>0</v>
       </c>
       <c r="I265" s="17" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="J265" s="19" t="n">
         <v>1</v>
       </c>
       <c r="K265" s="17" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="L265" s="18" t="n">
-        <v>756702</v>
+        <v>759284.133645375</v>
       </c>
       <c r="M265" s="18" t="n">
-        <v>756702</v>
-      </c>
-      <c r="N265" s="16" t="n"/>
+        <v>764538.28</v>
+      </c>
+      <c r="N265" s="18" t="n">
+        <v>5254.146354625002</v>
+      </c>
       <c r="O265" s="17" t="n">
-        <v>394</v>
+        <v>590</v>
       </c>
       <c r="P265" s="17" t="n">
-        <v>394</v>
+        <v>492</v>
       </c>
       <c r="Q265" s="17" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="R265" s="17" t="n">
         <v>200</v>
       </c>
       <c r="S265" s="18" t="n">
-        <v>33350</v>
+        <v>39150</v>
       </c>
     </row>
   </sheetData>
@@ -27052,7 +27624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N791"/>
+  <dimension ref="A1:N792"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -63483,8 +64055,54 @@
         <v>33350</v>
       </c>
     </row>
+    <row r="792">
+      <c r="A792" s="10" t="n">
+        <v>791</v>
+      </c>
+      <c r="B792" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C792" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="D792" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E792" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="F792" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G792" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="H792" s="14" t="n">
+        <v>764538.28</v>
+      </c>
+      <c r="I792" s="12" t="n">
+        <v>590</v>
+      </c>
+      <c r="J792" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K792" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L792" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M792" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N792" s="14" t="n">
+        <v>5800</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N791"/>
+  <autoFilter ref="A1:N792"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -63879,7 +64497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -64722,8 +65340,56 @@
         <v>55</v>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" s="23" t="n">
+        <v>730.66</v>
+      </c>
+      <c r="B35" s="16" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C35" s="16" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D35" s="16" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E35" s="16" t="inlineStr"/>
+      <c r="F35" s="17" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="21" t="n">
+        <v>742.75</v>
+      </c>
+      <c r="B36" s="11" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C36" s="11" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D36" s="11" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E36" s="11" t="inlineStr"/>
+      <c r="F36" s="12" t="n">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F34"/>
+  <autoFilter ref="A1:F36"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -65122,7 +65788,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U17"/>
+  <dimension ref="A1:U18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -66377,8 +67043,79 @@
       </c>
       <c r="U17" s="16" t="n"/>
     </row>
+    <row r="18">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="n">
+        <v>791</v>
+      </c>
+      <c r="C18" s="14" t="n">
+        <v>764538.28</v>
+      </c>
+      <c r="D18" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="E18" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="F18" s="11" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="G18" s="14" t="n">
+        <v>2251430.88</v>
+      </c>
+      <c r="H18" s="21" t="n">
+        <v>20</v>
+      </c>
+      <c r="I18" s="21" t="n">
+        <v>55</v>
+      </c>
+      <c r="J18" s="11" t="inlineStr">
+        <is>
+          <t>truck</t>
+        </is>
+      </c>
+      <c r="K18" s="22" t="n">
+        <v>3600</v>
+      </c>
+      <c r="L18" s="22" t="n">
+        <v>200</v>
+      </c>
+      <c r="M18" s="12" t="n">
+        <v>590</v>
+      </c>
+      <c r="N18" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="P18" s="10" t="n">
+        <v>264</v>
+      </c>
+      <c r="Q18" s="12" t="n">
+        <v>27</v>
+      </c>
+      <c r="R18" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S18" s="12" t="n">
+        <v>27</v>
+      </c>
+      <c r="T18" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="U18" s="14" t="n">
+        <v>5254.146354625002</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U17"/>
+  <autoFilter ref="A1:U18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -66389,7 +67126,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E193"/>
+  <dimension ref="A1:E205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -70778,8 +71515,280 @@
         </is>
       </c>
     </row>
+    <row r="194">
+      <c r="A194" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B194" s="10" t="n">
+        <v>791</v>
+      </c>
+      <c r="C194" s="11" t="inlineStr">
+        <is>
+          <t>Starting Cash</t>
+        </is>
+      </c>
+      <c r="D194" s="14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E194" s="11" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B195" s="15" t="n">
+        <v>791</v>
+      </c>
+      <c r="C195" s="16" t="inlineStr">
+        <is>
+          <t>Cash Sources</t>
+        </is>
+      </c>
+      <c r="D195" s="16" t="n"/>
+      <c r="E195" s="16" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B196" s="10" t="n">
+        <v>791</v>
+      </c>
+      <c r="C196" s="11" t="inlineStr">
+        <is>
+          <t>revenues</t>
+        </is>
+      </c>
+      <c r="D196" s="14" t="n">
+        <v>19954900</v>
+      </c>
+      <c r="E196" s="11" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B197" s="15" t="n">
+        <v>791</v>
+      </c>
+      <c r="C197" s="16" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D197" s="18" t="n">
+        <v>287612.15</v>
+      </c>
+      <c r="E197" s="16" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B198" s="10" t="n">
+        <v>791</v>
+      </c>
+      <c r="C198" s="11" t="inlineStr">
+        <is>
+          <t>Cash Uses</t>
+        </is>
+      </c>
+      <c r="D198" s="11" t="n"/>
+      <c r="E198" s="11" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B199" s="15" t="n">
+        <v>791</v>
+      </c>
+      <c r="C199" s="16" t="inlineStr">
+        <is>
+          <t>outbound shipping</t>
+        </is>
+      </c>
+      <c r="D199" s="18" t="n">
+        <v>-2064300</v>
+      </c>
+      <c r="E199" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B200" s="10" t="n">
+        <v>791</v>
+      </c>
+      <c r="C200" s="11" t="inlineStr">
+        <is>
+          <t>inbound shipping</t>
+        </is>
+      </c>
+      <c r="D200" s="14" t="n">
+        <v>-1425000</v>
+      </c>
+      <c r="E200" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B201" s="15" t="n">
+        <v>791</v>
+      </c>
+      <c r="C201" s="16" t="inlineStr">
+        <is>
+          <t>FGI holding</t>
+        </is>
+      </c>
+      <c r="D201" s="18" t="n">
+        <v>-18812.45</v>
+      </c>
+      <c r="E201" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B202" s="10" t="n">
+        <v>791</v>
+      </c>
+      <c r="C202" s="11" t="inlineStr">
+        <is>
+          <t>add capacity</t>
+        </is>
+      </c>
+      <c r="D202" s="14" t="n">
+        <v>-1749840.87</v>
+      </c>
+      <c r="E202" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B203" s="15" t="n">
+        <v>791</v>
+      </c>
+      <c r="C203" s="16" t="inlineStr">
+        <is>
+          <t>Pipeline inventory holding</t>
+        </is>
+      </c>
+      <c r="D203" s="18" t="n">
+        <v>-27520.55</v>
+      </c>
+      <c r="E203" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B204" s="10" t="n">
+        <v>791</v>
+      </c>
+      <c r="C204" s="11" t="inlineStr">
+        <is>
+          <t>production</t>
+        </is>
+      </c>
+      <c r="D204" s="14" t="n">
+        <v>-14692500</v>
+      </c>
+      <c r="E204" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T02:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B205" s="15" t="n">
+        <v>791</v>
+      </c>
+      <c r="C205" s="16" t="inlineStr">
+        <is>
+          <t>Cash Balance</t>
+        </is>
+      </c>
+      <c r="D205" s="18" t="n">
+        <v>764538.28</v>
+      </c>
+      <c r="E205" s="16" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E193"/>
+  <autoFilter ref="A1:E205"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update game data: day 792, cash 793180.94, 3-day period 264
</commit_message>
<xml_diff>
--- a/data/supply_chain_game.xlsx
+++ b/data/supply_chain_game.xlsx
@@ -21,15 +21,15 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$265</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$792</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$793</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'资金构成_旧版'!$A$1:$C$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'运营参数_旧版'!$A$9:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$38</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'排行榜_旧版'!$A$1:$C$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$18</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$205</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$217</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'运营参数'!$A$1:$J$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$460</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$487</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -590,7 +590,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-06T02:56:02+08:00</t>
+          <t>2026-09-06T03:11:02+08:00</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>791</v>
+        <v>792</v>
       </c>
     </row>
     <row r="7">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>669</v>
+        <v>668</v>
       </c>
     </row>
     <row r="8">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>764538.28</v>
+        <v>793180.9399999999</v>
       </c>
     </row>
     <row r="11">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>2251430.88</v>
+        <v>2252128.45</v>
       </c>
     </row>
     <row r="15"/>
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>590</v>
+        <v>571</v>
       </c>
     </row>
     <row r="25">
@@ -850,7 +850,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>否（进行中）</t>
+          <t>是</t>
         </is>
       </c>
     </row>
@@ -861,7 +861,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>27</v>
+        <v>46</v>
       </c>
     </row>
     <row r="33">
@@ -881,7 +881,7 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>27</v>
+        <v>46</v>
       </c>
     </row>
     <row r="35">
@@ -901,7 +901,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>27</v>
+        <v>46</v>
       </c>
     </row>
     <row r="37">
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="B37" s="4" t="n">
-        <v>5254.146354625002</v>
+        <v>30226.64187802165</v>
       </c>
     </row>
     <row r="38"/>
@@ -929,7 +929,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="41">
@@ -940,7 +940,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>787–789</t>
+          <t>790–792</t>
         </is>
       </c>
     </row>
@@ -952,7 +952,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>89.0 / 0.0 / 89.0</t>
+          <t>46.0 / 0.0 / 46.0</t>
         </is>
       </c>
     </row>
@@ -973,7 +973,7 @@
         </is>
       </c>
       <c r="B44" s="4" t="n">
-        <v>92612.70048965176</v>
+        <v>30226.64187802165</v>
       </c>
     </row>
     <row r="45"/>
@@ -1171,7 +1171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E460"/>
+  <dimension ref="A1:E487"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -10847,8 +10847,575 @@
         <v>764538.28</v>
       </c>
     </row>
+    <row r="461">
+      <c r="A461" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T03:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B461" s="15" t="n">
+        <v>792</v>
+      </c>
+      <c r="C461" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D461" s="16" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="E461" s="18" t="n">
+        <v>3045309.39</v>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T03:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B462" s="10" t="n">
+        <v>792</v>
+      </c>
+      <c r="C462" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D462" s="11" t="inlineStr">
+        <is>
+          <t>group15</t>
+        </is>
+      </c>
+      <c r="E462" s="14" t="n">
+        <v>2108199.73</v>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T03:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B463" s="15" t="n">
+        <v>792</v>
+      </c>
+      <c r="C463" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D463" s="16" t="inlineStr">
+        <is>
+          <t>group7</t>
+        </is>
+      </c>
+      <c r="E463" s="18" t="n">
+        <v>2029186.13</v>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T03:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B464" s="10" t="n">
+        <v>792</v>
+      </c>
+      <c r="C464" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D464" s="11" t="inlineStr">
+        <is>
+          <t>nicetry</t>
+        </is>
+      </c>
+      <c r="E464" s="14" t="n">
+        <v>2028096.6</v>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T03:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B465" s="15" t="n">
+        <v>792</v>
+      </c>
+      <c r="C465" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="D465" s="16" t="inlineStr">
+        <is>
+          <t>group14</t>
+        </is>
+      </c>
+      <c r="E465" s="18" t="n">
+        <v>1981945.17</v>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T03:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B466" s="10" t="n">
+        <v>792</v>
+      </c>
+      <c r="C466" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="D466" s="11" t="inlineStr">
+        <is>
+          <t>montesquieu</t>
+        </is>
+      </c>
+      <c r="E466" s="14" t="n">
+        <v>1806484.74</v>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T03:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B467" s="15" t="n">
+        <v>792</v>
+      </c>
+      <c r="C467" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="D467" s="16" t="inlineStr">
+        <is>
+          <t>t24</t>
+        </is>
+      </c>
+      <c r="E467" s="18" t="n">
+        <v>1673875.46</v>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T03:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B468" s="10" t="n">
+        <v>792</v>
+      </c>
+      <c r="C468" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="D468" s="11" t="inlineStr">
+        <is>
+          <t>group8</t>
+        </is>
+      </c>
+      <c r="E468" s="14" t="n">
+        <v>1554485.91</v>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T03:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B469" s="15" t="n">
+        <v>792</v>
+      </c>
+      <c r="C469" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="D469" s="16" t="inlineStr">
+        <is>
+          <t>group9</t>
+        </is>
+      </c>
+      <c r="E469" s="18" t="n">
+        <v>1553617.98</v>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T03:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B470" s="10" t="n">
+        <v>792</v>
+      </c>
+      <c r="C470" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="D470" s="11" t="inlineStr">
+        <is>
+          <t>group2</t>
+        </is>
+      </c>
+      <c r="E470" s="14" t="n">
+        <v>1552236.43</v>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T03:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B471" s="15" t="n">
+        <v>792</v>
+      </c>
+      <c r="C471" s="15" t="n">
+        <v>11</v>
+      </c>
+      <c r="D471" s="16" t="inlineStr">
+        <is>
+          <t>teamhlly</t>
+        </is>
+      </c>
+      <c r="E471" s="18" t="n">
+        <v>1552235.7</v>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T03:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B472" s="10" t="n">
+        <v>792</v>
+      </c>
+      <c r="C472" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="D472" s="11" t="inlineStr">
+        <is>
+          <t>group25</t>
+        </is>
+      </c>
+      <c r="E472" s="14" t="n">
+        <v>1552080.56</v>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T03:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B473" s="15" t="n">
+        <v>792</v>
+      </c>
+      <c r="C473" s="15" t="n">
+        <v>13</v>
+      </c>
+      <c r="D473" s="16" t="inlineStr">
+        <is>
+          <t>group11</t>
+        </is>
+      </c>
+      <c r="E473" s="18" t="n">
+        <v>1552068.42</v>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T03:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B474" s="10" t="n">
+        <v>792</v>
+      </c>
+      <c r="C474" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="D474" s="11" t="inlineStr">
+        <is>
+          <t>88888888</t>
+        </is>
+      </c>
+      <c r="E474" s="14" t="n">
+        <v>1552046.06</v>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T03:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B475" s="15" t="n">
+        <v>792</v>
+      </c>
+      <c r="C475" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="D475" s="16" t="inlineStr">
+        <is>
+          <t>group12</t>
+        </is>
+      </c>
+      <c r="E475" s="18" t="n">
+        <v>1480722.99</v>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T03:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B476" s="10" t="n">
+        <v>792</v>
+      </c>
+      <c r="C476" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="D476" s="11" t="inlineStr">
+        <is>
+          <t>tigagroup20</t>
+        </is>
+      </c>
+      <c r="E476" s="14" t="n">
+        <v>1451733.8</v>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T03:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B477" s="15" t="n">
+        <v>792</v>
+      </c>
+      <c r="C477" s="15" t="n">
+        <v>17</v>
+      </c>
+      <c r="D477" s="16" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E477" s="18" t="n">
+        <v>1445881.19</v>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T03:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B478" s="10" t="n">
+        <v>792</v>
+      </c>
+      <c r="C478" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="D478" s="11" t="inlineStr">
+        <is>
+          <t>aaachemicalseller</t>
+        </is>
+      </c>
+      <c r="E478" s="14" t="n">
+        <v>1443206.92</v>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T03:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B479" s="15" t="n">
+        <v>792</v>
+      </c>
+      <c r="C479" s="15" t="n">
+        <v>19</v>
+      </c>
+      <c r="D479" s="16" t="inlineStr">
+        <is>
+          <t>deepsleep</t>
+        </is>
+      </c>
+      <c r="E479" s="18" t="n">
+        <v>1422990.75</v>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T03:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B480" s="10" t="n">
+        <v>792</v>
+      </c>
+      <c r="C480" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="D480" s="11" t="inlineStr">
+        <is>
+          <t>666666</t>
+        </is>
+      </c>
+      <c r="E480" s="14" t="n">
+        <v>1399454.65</v>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T03:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B481" s="15" t="n">
+        <v>792</v>
+      </c>
+      <c r="C481" s="15" t="n">
+        <v>21</v>
+      </c>
+      <c r="D481" s="16" t="inlineStr">
+        <is>
+          <t>jit</t>
+        </is>
+      </c>
+      <c r="E481" s="18" t="n">
+        <v>1304866.72</v>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T03:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B482" s="10" t="n">
+        <v>792</v>
+      </c>
+      <c r="C482" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="D482" s="11" t="inlineStr">
+        <is>
+          <t>cleveregg</t>
+        </is>
+      </c>
+      <c r="E482" s="14" t="n">
+        <v>1246895.91</v>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T03:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B483" s="15" t="n">
+        <v>792</v>
+      </c>
+      <c r="C483" s="15" t="n">
+        <v>23</v>
+      </c>
+      <c r="D483" s="16" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="E483" s="18" t="n">
+        <v>1205283.54</v>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T03:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B484" s="10" t="n">
+        <v>792</v>
+      </c>
+      <c r="C484" s="10" t="n">
+        <v>24</v>
+      </c>
+      <c r="D484" s="11" t="inlineStr">
+        <is>
+          <t>newgroup18</t>
+        </is>
+      </c>
+      <c r="E484" s="14" t="n">
+        <v>1161867.97</v>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T03:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B485" s="15" t="n">
+        <v>792</v>
+      </c>
+      <c r="C485" s="15" t="n">
+        <v>25</v>
+      </c>
+      <c r="D485" s="16" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E485" s="18" t="n">
+        <v>1049702.46</v>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T03:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B486" s="10" t="n">
+        <v>792</v>
+      </c>
+      <c r="C486" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="D486" s="11" t="inlineStr">
+        <is>
+          <t>vivo50</t>
+        </is>
+      </c>
+      <c r="E486" s="14" t="n">
+        <v>1044211.76</v>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-06T03:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B487" s="24" t="n">
+        <v>792</v>
+      </c>
+      <c r="C487" s="24" t="n">
+        <v>27</v>
+      </c>
+      <c r="D487" s="25" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="E487" s="26" t="n">
+        <v>793180.9399999999</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E460"/>
+  <autoFilter ref="A1:E487"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -27560,11 +28127,11 @@
         <v>792</v>
       </c>
       <c r="D265" s="15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E265" s="16" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="F265" s="16" t="inlineStr">
@@ -27573,34 +28140,34 @@
         </is>
       </c>
       <c r="G265" s="17" t="n">
-        <v>27</v>
+        <v>46</v>
       </c>
       <c r="H265" s="17" t="n">
         <v>0</v>
       </c>
       <c r="I265" s="17" t="n">
-        <v>27</v>
+        <v>46</v>
       </c>
       <c r="J265" s="19" t="n">
         <v>1</v>
       </c>
       <c r="K265" s="17" t="n">
-        <v>27</v>
+        <v>46</v>
       </c>
       <c r="L265" s="18" t="n">
-        <v>759284.133645375</v>
+        <v>762954.2981219783</v>
       </c>
       <c r="M265" s="18" t="n">
-        <v>764538.28</v>
+        <v>793180.9399999999</v>
       </c>
       <c r="N265" s="18" t="n">
-        <v>5254.146354625002</v>
+        <v>30226.64187802165</v>
       </c>
       <c r="O265" s="17" t="n">
-        <v>590</v>
+        <v>571</v>
       </c>
       <c r="P265" s="17" t="n">
-        <v>492</v>
+        <v>518.3333333333334</v>
       </c>
       <c r="Q265" s="17" t="n">
         <v>0</v>
@@ -27609,7 +28176,7 @@
         <v>200</v>
       </c>
       <c r="S265" s="18" t="n">
-        <v>39150</v>
+        <v>66700</v>
       </c>
     </row>
   </sheetData>
@@ -27624,7 +28191,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N792"/>
+  <dimension ref="A1:N793"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -64101,8 +64668,54 @@
         <v>5800</v>
       </c>
     </row>
+    <row r="793">
+      <c r="A793" s="15" t="n">
+        <v>792</v>
+      </c>
+      <c r="B793" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C793" s="17" t="n">
+        <v>19</v>
+      </c>
+      <c r="D793" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E793" s="17" t="n">
+        <v>19</v>
+      </c>
+      <c r="F793" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G793" s="17" t="n">
+        <v>19</v>
+      </c>
+      <c r="H793" s="18" t="n">
+        <v>793180.9399999999</v>
+      </c>
+      <c r="I793" s="17" t="n">
+        <v>571</v>
+      </c>
+      <c r="J793" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K793" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L793" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M793" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N793" s="18" t="n">
+        <v>27550</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N792"/>
+  <autoFilter ref="A1:N793"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -64497,7 +65110,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -65388,8 +66001,56 @@
         <v>55</v>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" s="23" t="n">
+        <v>730.66</v>
+      </c>
+      <c r="B37" s="16" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C37" s="16" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D37" s="16" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E37" s="16" t="inlineStr"/>
+      <c r="F37" s="17" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="21" t="n">
+        <v>742.75</v>
+      </c>
+      <c r="B38" s="11" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C38" s="11" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D38" s="11" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E38" s="11" t="inlineStr"/>
+      <c r="F38" s="12" t="n">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F36"/>
+  <autoFilter ref="A1:F38"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -65788,7 +66449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U18"/>
+  <dimension ref="A1:U19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -67114,8 +67775,79 @@
         <v>5254.146354625002</v>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T03:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B19" s="15" t="n">
+        <v>792</v>
+      </c>
+      <c r="C19" s="18" t="n">
+        <v>793180.9399999999</v>
+      </c>
+      <c r="D19" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="E19" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="G19" s="18" t="n">
+        <v>2252128.45</v>
+      </c>
+      <c r="H19" s="23" t="n">
+        <v>20</v>
+      </c>
+      <c r="I19" s="23" t="n">
+        <v>55</v>
+      </c>
+      <c r="J19" s="16" t="inlineStr">
+        <is>
+          <t>truck</t>
+        </is>
+      </c>
+      <c r="K19" s="27" t="n">
+        <v>3600</v>
+      </c>
+      <c r="L19" s="27" t="n">
+        <v>200</v>
+      </c>
+      <c r="M19" s="17" t="n">
+        <v>571</v>
+      </c>
+      <c r="N19" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="P19" s="15" t="n">
+        <v>264</v>
+      </c>
+      <c r="Q19" s="17" t="n">
+        <v>46</v>
+      </c>
+      <c r="R19" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="S19" s="17" t="n">
+        <v>46</v>
+      </c>
+      <c r="T19" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="U19" s="18" t="n">
+        <v>30226.64187802165</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U18"/>
+  <autoFilter ref="A1:U19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -67126,7 +67858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E205"/>
+  <dimension ref="A1:E217"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -71787,8 +72519,280 @@
         </is>
       </c>
     </row>
+    <row r="206">
+      <c r="A206" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T03:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B206" s="10" t="n">
+        <v>792</v>
+      </c>
+      <c r="C206" s="11" t="inlineStr">
+        <is>
+          <t>Starting Cash</t>
+        </is>
+      </c>
+      <c r="D206" s="14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E206" s="11" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T03:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B207" s="15" t="n">
+        <v>792</v>
+      </c>
+      <c r="C207" s="16" t="inlineStr">
+        <is>
+          <t>Cash Sources</t>
+        </is>
+      </c>
+      <c r="D207" s="16" t="n"/>
+      <c r="E207" s="16" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T03:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B208" s="10" t="n">
+        <v>792</v>
+      </c>
+      <c r="C208" s="11" t="inlineStr">
+        <is>
+          <t>revenues</t>
+        </is>
+      </c>
+      <c r="D208" s="14" t="n">
+        <v>19986800</v>
+      </c>
+      <c r="E208" s="11" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T03:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B209" s="15" t="n">
+        <v>792</v>
+      </c>
+      <c r="C209" s="16" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D209" s="18" t="n">
+        <v>287814.08</v>
+      </c>
+      <c r="E209" s="16" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T03:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B210" s="10" t="n">
+        <v>792</v>
+      </c>
+      <c r="C210" s="11" t="inlineStr">
+        <is>
+          <t>Cash Uses</t>
+        </is>
+      </c>
+      <c r="D210" s="11" t="n"/>
+      <c r="E210" s="11" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T03:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B211" s="15" t="n">
+        <v>792</v>
+      </c>
+      <c r="C211" s="16" t="inlineStr">
+        <is>
+          <t>outbound shipping</t>
+        </is>
+      </c>
+      <c r="D211" s="18" t="n">
+        <v>-2067600</v>
+      </c>
+      <c r="E211" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T03:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B212" s="10" t="n">
+        <v>792</v>
+      </c>
+      <c r="C212" s="11" t="inlineStr">
+        <is>
+          <t>inbound shipping</t>
+        </is>
+      </c>
+      <c r="D212" s="14" t="n">
+        <v>-1425000</v>
+      </c>
+      <c r="E212" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T03:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B213" s="15" t="n">
+        <v>792</v>
+      </c>
+      <c r="C213" s="16" t="inlineStr">
+        <is>
+          <t>FGI holding</t>
+        </is>
+      </c>
+      <c r="D213" s="18" t="n">
+        <v>-18971.72</v>
+      </c>
+      <c r="E213" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T03:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B214" s="10" t="n">
+        <v>792</v>
+      </c>
+      <c r="C214" s="11" t="inlineStr">
+        <is>
+          <t>add capacity</t>
+        </is>
+      </c>
+      <c r="D214" s="14" t="n">
+        <v>-1749840.87</v>
+      </c>
+      <c r="E214" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T03:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B215" s="15" t="n">
+        <v>792</v>
+      </c>
+      <c r="C215" s="16" t="inlineStr">
+        <is>
+          <t>Pipeline inventory holding</t>
+        </is>
+      </c>
+      <c r="D215" s="18" t="n">
+        <v>-27520.55</v>
+      </c>
+      <c r="E215" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T03:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B216" s="10" t="n">
+        <v>792</v>
+      </c>
+      <c r="C216" s="11" t="inlineStr">
+        <is>
+          <t>production</t>
+        </is>
+      </c>
+      <c r="D216" s="14" t="n">
+        <v>-14692500</v>
+      </c>
+      <c r="E216" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T03:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B217" s="15" t="n">
+        <v>792</v>
+      </c>
+      <c r="C217" s="16" t="inlineStr">
+        <is>
+          <t>Cash Balance</t>
+        </is>
+      </c>
+      <c r="D217" s="18" t="n">
+        <v>793180.9399999999</v>
+      </c>
+      <c r="E217" s="16" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E205"/>
+  <autoFilter ref="A1:E217"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update game data: day 829, cash 1232642.13, 3-day period 277
</commit_message>
<xml_diff>
--- a/data/supply_chain_game.xlsx
+++ b/data/supply_chain_game.xlsx
@@ -20,16 +20,16 @@
     <sheet name="排行榜" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$265</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$793</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$278</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$830</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'资金构成_旧版'!$A$1:$C$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'运营参数_旧版'!$A$9:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$40</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'排行榜_旧版'!$A$1:$C$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$217</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'运营参数'!$A$1:$J$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$487</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$229</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'运营参数'!$A$1:$J$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$514</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -590,7 +590,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-06T03:11:02+08:00</t>
+          <t>2026-09-06T11:41:02+08:00</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>792</v>
+        <v>829</v>
       </c>
     </row>
     <row r="7">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>668</v>
+        <v>631</v>
       </c>
     </row>
     <row r="8">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>793180.9399999999</v>
+        <v>1232642.13</v>
       </c>
     </row>
     <row r="11">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>2252128.45</v>
+        <v>2004506.73</v>
       </c>
     </row>
     <row r="15"/>
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="B18" s="6" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
     </row>
     <row r="19">
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>571</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>0</v>
+        <v>400</v>
       </c>
     </row>
     <row r="26">
@@ -827,7 +827,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>264</v>
+        <v>277</v>
       </c>
     </row>
     <row r="30">
@@ -838,7 +838,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>790–792</t>
+          <t>829–831</t>
         </is>
       </c>
     </row>
@@ -850,7 +850,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否（进行中）</t>
         </is>
       </c>
     </row>
@@ -861,7 +861,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>46</v>
+        <v>36</v>
       </c>
     </row>
     <row r="33">
@@ -871,7 +871,7 @@
         </is>
       </c>
       <c r="B33" s="7" t="n">
-        <v>0</v>
+        <v>34</v>
       </c>
     </row>
     <row r="34">
@@ -881,7 +881,7 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>46</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35">
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B35" s="8" t="n">
-        <v>1</v>
+        <v>0.05555555555555555</v>
       </c>
     </row>
     <row r="36">
@@ -901,7 +901,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>46</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37">
@@ -909,9 +909,6 @@
         <is>
           <t>周期现金变动</t>
         </is>
-      </c>
-      <c r="B37" s="4" t="n">
-        <v>30226.64187802165</v>
       </c>
     </row>
     <row r="38"/>
@@ -929,7 +926,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>264</v>
+        <v>276</v>
       </c>
     </row>
     <row r="41">
@@ -940,7 +937,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>790–792</t>
+          <t>826–828</t>
         </is>
       </c>
     </row>
@@ -952,7 +949,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>46.0 / 0.0 / 46.0</t>
+          <t>129.0 / 0.0 / 129.0</t>
         </is>
       </c>
     </row>
@@ -973,7 +970,7 @@
         </is>
       </c>
       <c r="B44" s="4" t="n">
-        <v>30226.64187802165</v>
+        <v>109781.8996437623</v>
       </c>
     </row>
     <row r="45"/>
@@ -1008,7 +1005,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1159,8 +1156,50 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="n">
+        <v>829</v>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="D4" s="21" t="n">
+        <v>40</v>
+      </c>
+      <c r="E4" s="21" t="n">
+        <v>55</v>
+      </c>
+      <c r="F4" s="11" t="inlineStr">
+        <is>
+          <t>truck</t>
+        </is>
+      </c>
+      <c r="G4" s="22" t="n">
+        <v>3600</v>
+      </c>
+      <c r="H4" s="22" t="n">
+        <v>200</v>
+      </c>
+      <c r="I4" s="11" t="inlineStr">
+        <is>
+          <t>truck</t>
+        </is>
+      </c>
+      <c r="J4" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J3"/>
+  <autoFilter ref="A1:J4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1171,7 +1210,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E487"/>
+  <dimension ref="A1:E514"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -11414,8 +11453,575 @@
         <v>793180.9399999999</v>
       </c>
     </row>
+    <row r="488">
+      <c r="A488" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B488" s="10" t="n">
+        <v>829</v>
+      </c>
+      <c r="C488" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D488" s="11" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="E488" s="14" t="n">
+        <v>3237148.86</v>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B489" s="15" t="n">
+        <v>829</v>
+      </c>
+      <c r="C489" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D489" s="16" t="inlineStr">
+        <is>
+          <t>nicetry</t>
+        </is>
+      </c>
+      <c r="E489" s="18" t="n">
+        <v>2438101.27</v>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B490" s="10" t="n">
+        <v>829</v>
+      </c>
+      <c r="C490" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D490" s="11" t="inlineStr">
+        <is>
+          <t>group9</t>
+        </is>
+      </c>
+      <c r="E490" s="14" t="n">
+        <v>2339305.27</v>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B491" s="15" t="n">
+        <v>829</v>
+      </c>
+      <c r="C491" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D491" s="16" t="inlineStr">
+        <is>
+          <t>group8</t>
+        </is>
+      </c>
+      <c r="E491" s="18" t="n">
+        <v>2327547.6</v>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B492" s="10" t="n">
+        <v>829</v>
+      </c>
+      <c r="C492" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="D492" s="11" t="inlineStr">
+        <is>
+          <t>montesquieu</t>
+        </is>
+      </c>
+      <c r="E492" s="14" t="n">
+        <v>2255370.89</v>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B493" s="15" t="n">
+        <v>829</v>
+      </c>
+      <c r="C493" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="D493" s="16" t="inlineStr">
+        <is>
+          <t>t24</t>
+        </is>
+      </c>
+      <c r="E493" s="18" t="n">
+        <v>2195538.85</v>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B494" s="10" t="n">
+        <v>829</v>
+      </c>
+      <c r="C494" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="D494" s="11" t="inlineStr">
+        <is>
+          <t>group14</t>
+        </is>
+      </c>
+      <c r="E494" s="14" t="n">
+        <v>2142938.76</v>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B495" s="15" t="n">
+        <v>829</v>
+      </c>
+      <c r="C495" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="D495" s="16" t="inlineStr">
+        <is>
+          <t>group15</t>
+        </is>
+      </c>
+      <c r="E495" s="18" t="n">
+        <v>2101735.66</v>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B496" s="10" t="n">
+        <v>829</v>
+      </c>
+      <c r="C496" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="D496" s="11" t="inlineStr">
+        <is>
+          <t>tigagroup20</t>
+        </is>
+      </c>
+      <c r="E496" s="14" t="n">
+        <v>2058771.76</v>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B497" s="15" t="n">
+        <v>829</v>
+      </c>
+      <c r="C497" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="D497" s="16" t="inlineStr">
+        <is>
+          <t>group7</t>
+        </is>
+      </c>
+      <c r="E497" s="18" t="n">
+        <v>2044581.42</v>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B498" s="10" t="n">
+        <v>829</v>
+      </c>
+      <c r="C498" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="D498" s="11" t="inlineStr">
+        <is>
+          <t>teamhlly</t>
+        </is>
+      </c>
+      <c r="E498" s="14" t="n">
+        <v>1999048.62</v>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B499" s="15" t="n">
+        <v>829</v>
+      </c>
+      <c r="C499" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="D499" s="16" t="inlineStr">
+        <is>
+          <t>group2</t>
+        </is>
+      </c>
+      <c r="E499" s="18" t="n">
+        <v>1998574.6</v>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B500" s="10" t="n">
+        <v>829</v>
+      </c>
+      <c r="C500" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="D500" s="11" t="inlineStr">
+        <is>
+          <t>group25</t>
+        </is>
+      </c>
+      <c r="E500" s="14" t="n">
+        <v>1998417.21</v>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B501" s="15" t="n">
+        <v>829</v>
+      </c>
+      <c r="C501" s="15" t="n">
+        <v>14</v>
+      </c>
+      <c r="D501" s="16" t="inlineStr">
+        <is>
+          <t>group11</t>
+        </is>
+      </c>
+      <c r="E501" s="18" t="n">
+        <v>1998404.96</v>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B502" s="10" t="n">
+        <v>829</v>
+      </c>
+      <c r="C502" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="D502" s="11" t="inlineStr">
+        <is>
+          <t>88888888</t>
+        </is>
+      </c>
+      <c r="E502" s="14" t="n">
+        <v>1998382.38</v>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B503" s="15" t="n">
+        <v>829</v>
+      </c>
+      <c r="C503" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="D503" s="16" t="inlineStr">
+        <is>
+          <t>deepsleep</t>
+        </is>
+      </c>
+      <c r="E503" s="18" t="n">
+        <v>1940331.67</v>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B504" s="10" t="n">
+        <v>829</v>
+      </c>
+      <c r="C504" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="D504" s="11" t="inlineStr">
+        <is>
+          <t>jit</t>
+        </is>
+      </c>
+      <c r="E504" s="14" t="n">
+        <v>1910478.84</v>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B505" s="15" t="n">
+        <v>829</v>
+      </c>
+      <c r="C505" s="15" t="n">
+        <v>18</v>
+      </c>
+      <c r="D505" s="16" t="inlineStr">
+        <is>
+          <t>666666</t>
+        </is>
+      </c>
+      <c r="E505" s="18" t="n">
+        <v>1844270.63</v>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B506" s="10" t="n">
+        <v>829</v>
+      </c>
+      <c r="C506" s="10" t="n">
+        <v>19</v>
+      </c>
+      <c r="D506" s="11" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E506" s="14" t="n">
+        <v>1817863.51</v>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B507" s="15" t="n">
+        <v>829</v>
+      </c>
+      <c r="C507" s="15" t="n">
+        <v>20</v>
+      </c>
+      <c r="D507" s="16" t="inlineStr">
+        <is>
+          <t>cleveregg</t>
+        </is>
+      </c>
+      <c r="E507" s="18" t="n">
+        <v>1690197.01</v>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B508" s="10" t="n">
+        <v>829</v>
+      </c>
+      <c r="C508" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="D508" s="11" t="inlineStr">
+        <is>
+          <t>aaachemicalseller</t>
+        </is>
+      </c>
+      <c r="E508" s="14" t="n">
+        <v>1630455.52</v>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B509" s="15" t="n">
+        <v>829</v>
+      </c>
+      <c r="C509" s="15" t="n">
+        <v>22</v>
+      </c>
+      <c r="D509" s="16" t="inlineStr">
+        <is>
+          <t>newgroup18</t>
+        </is>
+      </c>
+      <c r="E509" s="18" t="n">
+        <v>1555091.67</v>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B510" s="10" t="n">
+        <v>829</v>
+      </c>
+      <c r="C510" s="10" t="n">
+        <v>23</v>
+      </c>
+      <c r="D510" s="11" t="inlineStr">
+        <is>
+          <t>vivo50</t>
+        </is>
+      </c>
+      <c r="E510" s="14" t="n">
+        <v>1485981.25</v>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B511" s="15" t="n">
+        <v>829</v>
+      </c>
+      <c r="C511" s="15" t="n">
+        <v>24</v>
+      </c>
+      <c r="D511" s="16" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E511" s="18" t="n">
+        <v>1413988.51</v>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B512" s="10" t="n">
+        <v>829</v>
+      </c>
+      <c r="C512" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="D512" s="11" t="inlineStr">
+        <is>
+          <t>group12</t>
+        </is>
+      </c>
+      <c r="E512" s="14" t="n">
+        <v>1412218.62</v>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B513" s="15" t="n">
+        <v>829</v>
+      </c>
+      <c r="C513" s="15" t="n">
+        <v>26</v>
+      </c>
+      <c r="D513" s="16" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="E513" s="18" t="n">
+        <v>1258053.52</v>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B514" s="24" t="n">
+        <v>829</v>
+      </c>
+      <c r="C514" s="24" t="n">
+        <v>27</v>
+      </c>
+      <c r="D514" s="25" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="E514" s="26" t="n">
+        <v>1232642.13</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E487"/>
+  <autoFilter ref="A1:E514"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -11426,7 +12032,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S265"/>
+  <dimension ref="A1:S278"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -28179,8 +28785,825 @@
         <v>66700</v>
       </c>
     </row>
+    <row r="266">
+      <c r="A266" s="10" t="n">
+        <v>265</v>
+      </c>
+      <c r="B266" s="10" t="n">
+        <v>793</v>
+      </c>
+      <c r="C266" s="10" t="n">
+        <v>795</v>
+      </c>
+      <c r="D266" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E266" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="F266" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G266" s="12" t="n">
+        <v>90</v>
+      </c>
+      <c r="H266" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I266" s="12" t="n">
+        <v>90</v>
+      </c>
+      <c r="J266" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K266" s="12" t="n">
+        <v>90</v>
+      </c>
+      <c r="L266" s="14" t="n">
+        <v>819236.7618458089</v>
+      </c>
+      <c r="M266" s="14" t="n">
+        <v>687286.2674140512</v>
+      </c>
+      <c r="N266" s="14" t="n">
+        <v>-131950.4944317577</v>
+      </c>
+      <c r="O266" s="12" t="n">
+        <v>481</v>
+      </c>
+      <c r="P266" s="12" t="n">
+        <v>515.6666666666666</v>
+      </c>
+      <c r="Q266" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="R266" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="S266" s="14" t="n">
+        <v>130500</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="15" t="n">
+        <v>266</v>
+      </c>
+      <c r="B267" s="15" t="n">
+        <v>796</v>
+      </c>
+      <c r="C267" s="15" t="n">
+        <v>798</v>
+      </c>
+      <c r="D267" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E267" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="F267" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G267" s="17" t="n">
+        <v>102</v>
+      </c>
+      <c r="H267" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I267" s="17" t="n">
+        <v>102</v>
+      </c>
+      <c r="J267" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K267" s="17" t="n">
+        <v>102</v>
+      </c>
+      <c r="L267" s="18" t="n">
+        <v>723688.4451556315</v>
+      </c>
+      <c r="M267" s="18" t="n">
+        <v>819949.6593412205</v>
+      </c>
+      <c r="N267" s="18" t="n">
+        <v>96261.21418558899</v>
+      </c>
+      <c r="O267" s="17" t="n">
+        <v>379</v>
+      </c>
+      <c r="P267" s="17" t="n">
+        <v>418.6666666666667</v>
+      </c>
+      <c r="Q267" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="R267" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="S267" s="18" t="n">
+        <v>147900</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="10" t="n">
+        <v>267</v>
+      </c>
+      <c r="B268" s="10" t="n">
+        <v>799</v>
+      </c>
+      <c r="C268" s="10" t="n">
+        <v>801</v>
+      </c>
+      <c r="D268" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E268" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="F268" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G268" s="12" t="n">
+        <v>66</v>
+      </c>
+      <c r="H268" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I268" s="12" t="n">
+        <v>66</v>
+      </c>
+      <c r="J268" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K268" s="12" t="n">
+        <v>66</v>
+      </c>
+      <c r="L268" s="14" t="n">
+        <v>849910.6568799117</v>
+      </c>
+      <c r="M268" s="14" t="n">
+        <v>905978.3933006477</v>
+      </c>
+      <c r="N268" s="14" t="n">
+        <v>56067.73642073607</v>
+      </c>
+      <c r="O268" s="12" t="n">
+        <v>513</v>
+      </c>
+      <c r="P268" s="12" t="n">
+        <v>400</v>
+      </c>
+      <c r="Q268" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R268" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="S268" s="14" t="n">
+        <v>95700</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="15" t="n">
+        <v>268</v>
+      </c>
+      <c r="B269" s="15" t="n">
+        <v>802</v>
+      </c>
+      <c r="C269" s="15" t="n">
+        <v>804</v>
+      </c>
+      <c r="D269" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E269" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="F269" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G269" s="17" t="n">
+        <v>115</v>
+      </c>
+      <c r="H269" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I269" s="17" t="n">
+        <v>115</v>
+      </c>
+      <c r="J269" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K269" s="17" t="n">
+        <v>115</v>
+      </c>
+      <c r="L269" s="18" t="n">
+        <v>960687.6182285527</v>
+      </c>
+      <c r="M269" s="18" t="n">
+        <v>839376.8427660714</v>
+      </c>
+      <c r="N269" s="18" t="n">
+        <v>-121310.7754624813</v>
+      </c>
+      <c r="O269" s="17" t="n">
+        <v>398</v>
+      </c>
+      <c r="P269" s="17" t="n">
+        <v>436.6666666666667</v>
+      </c>
+      <c r="Q269" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="R269" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="S269" s="18" t="n">
+        <v>166750</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="10" t="n">
+        <v>269</v>
+      </c>
+      <c r="B270" s="10" t="n">
+        <v>805</v>
+      </c>
+      <c r="C270" s="10" t="n">
+        <v>807</v>
+      </c>
+      <c r="D270" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E270" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="F270" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G270" s="12" t="n">
+        <v>106</v>
+      </c>
+      <c r="H270" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I270" s="12" t="n">
+        <v>106</v>
+      </c>
+      <c r="J270" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K270" s="12" t="n">
+        <v>106</v>
+      </c>
+      <c r="L270" s="14" t="n">
+        <v>882342.9434852329</v>
+      </c>
+      <c r="M270" s="14" t="n">
+        <v>977451.7725586459</v>
+      </c>
+      <c r="N270" s="14" t="n">
+        <v>95108.82907341304</v>
+      </c>
+      <c r="O270" s="12" t="n">
+        <v>292</v>
+      </c>
+      <c r="P270" s="12" t="n">
+        <v>324.3333333333333</v>
+      </c>
+      <c r="Q270" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="R270" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="S270" s="14" t="n">
+        <v>153700</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="15" t="n">
+        <v>270</v>
+      </c>
+      <c r="B271" s="15" t="n">
+        <v>808</v>
+      </c>
+      <c r="C271" s="15" t="n">
+        <v>810</v>
+      </c>
+      <c r="D271" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E271" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="F271" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G271" s="17" t="n">
+        <v>90</v>
+      </c>
+      <c r="H271" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I271" s="17" t="n">
+        <v>90</v>
+      </c>
+      <c r="J271" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K271" s="17" t="n">
+        <v>90</v>
+      </c>
+      <c r="L271" s="18" t="n">
+        <v>1007477.926182033</v>
+      </c>
+      <c r="M271" s="18" t="n">
+        <v>1094899.648125981</v>
+      </c>
+      <c r="N271" s="18" t="n">
+        <v>87421.72194394749</v>
+      </c>
+      <c r="O271" s="17" t="n">
+        <v>202</v>
+      </c>
+      <c r="P271" s="17" t="n">
+        <v>232.6666666666667</v>
+      </c>
+      <c r="Q271" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="R271" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="S271" s="18" t="n">
+        <v>130500</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="10" t="n">
+        <v>271</v>
+      </c>
+      <c r="B272" s="10" t="n">
+        <v>811</v>
+      </c>
+      <c r="C272" s="10" t="n">
+        <v>813</v>
+      </c>
+      <c r="D272" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E272" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="F272" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G272" s="12" t="n">
+        <v>116</v>
+      </c>
+      <c r="H272" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I272" s="12" t="n">
+        <v>116</v>
+      </c>
+      <c r="J272" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K272" s="12" t="n">
+        <v>116</v>
+      </c>
+      <c r="L272" s="14" t="n">
+        <v>1128881.627269907</v>
+      </c>
+      <c r="M272" s="14" t="n">
+        <v>1246323.468159911</v>
+      </c>
+      <c r="N272" s="14" t="n">
+        <v>117441.8408900034</v>
+      </c>
+      <c r="O272" s="12" t="n">
+        <v>286</v>
+      </c>
+      <c r="P272" s="12" t="n">
+        <v>329.6666666666667</v>
+      </c>
+      <c r="Q272" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R272" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="S272" s="14" t="n">
+        <v>168200</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="15" t="n">
+        <v>272</v>
+      </c>
+      <c r="B273" s="15" t="n">
+        <v>814</v>
+      </c>
+      <c r="C273" s="15" t="n">
+        <v>816</v>
+      </c>
+      <c r="D273" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E273" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="F273" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G273" s="17" t="n">
+        <v>72</v>
+      </c>
+      <c r="H273" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I273" s="17" t="n">
+        <v>72</v>
+      </c>
+      <c r="J273" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K273" s="17" t="n">
+        <v>72</v>
+      </c>
+      <c r="L273" s="18" t="n">
+        <v>1049575.782540787</v>
+      </c>
+      <c r="M273" s="18" t="n">
+        <v>1123993.312617932</v>
+      </c>
+      <c r="N273" s="18" t="n">
+        <v>74417.53007714543</v>
+      </c>
+      <c r="O273" s="17" t="n">
+        <v>214</v>
+      </c>
+      <c r="P273" s="17" t="n">
+        <v>245</v>
+      </c>
+      <c r="Q273" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="R273" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="S273" s="18" t="n">
+        <v>104400</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="10" t="n">
+        <v>273</v>
+      </c>
+      <c r="B274" s="10" t="n">
+        <v>817</v>
+      </c>
+      <c r="C274" s="10" t="n">
+        <v>819</v>
+      </c>
+      <c r="D274" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E274" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="F274" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G274" s="12" t="n">
+        <v>92</v>
+      </c>
+      <c r="H274" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I274" s="12" t="n">
+        <v>92</v>
+      </c>
+      <c r="J274" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K274" s="12" t="n">
+        <v>92</v>
+      </c>
+      <c r="L274" s="14" t="n">
+        <v>1174884.256456956</v>
+      </c>
+      <c r="M274" s="14" t="n">
+        <v>1244216.781823416</v>
+      </c>
+      <c r="N274" s="14" t="n">
+        <v>69332.52536646067</v>
+      </c>
+      <c r="O274" s="12" t="n">
+        <v>122</v>
+      </c>
+      <c r="P274" s="12" t="n">
+        <v>153.6666666666667</v>
+      </c>
+      <c r="Q274" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="R274" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="S274" s="14" t="n">
+        <v>133400</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="15" t="n">
+        <v>274</v>
+      </c>
+      <c r="B275" s="15" t="n">
+        <v>820</v>
+      </c>
+      <c r="C275" s="15" t="n">
+        <v>822</v>
+      </c>
+      <c r="D275" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E275" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="F275" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G275" s="17" t="n">
+        <v>92</v>
+      </c>
+      <c r="H275" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I275" s="17" t="n">
+        <v>92</v>
+      </c>
+      <c r="J275" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K275" s="17" t="n">
+        <v>92</v>
+      </c>
+      <c r="L275" s="18" t="n">
+        <v>1296461.27694519</v>
+      </c>
+      <c r="M275" s="18" t="n">
+        <v>1364613.943219726</v>
+      </c>
+      <c r="N275" s="18" t="n">
+        <v>68152.66627453594</v>
+      </c>
+      <c r="O275" s="17" t="n">
+        <v>230</v>
+      </c>
+      <c r="P275" s="17" t="n">
+        <v>193.6666666666667</v>
+      </c>
+      <c r="Q275" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="R275" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="S275" s="18" t="n">
+        <v>133400</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="10" t="n">
+        <v>275</v>
+      </c>
+      <c r="B276" s="10" t="n">
+        <v>823</v>
+      </c>
+      <c r="C276" s="10" t="n">
+        <v>825</v>
+      </c>
+      <c r="D276" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E276" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="F276" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G276" s="12" t="n">
+        <v>99</v>
+      </c>
+      <c r="H276" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I276" s="12" t="n">
+        <v>99</v>
+      </c>
+      <c r="J276" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K276" s="12" t="n">
+        <v>99</v>
+      </c>
+      <c r="L276" s="14" t="n">
+        <v>1403917.095221187</v>
+      </c>
+      <c r="M276" s="14" t="n">
+        <v>1277670.034218953</v>
+      </c>
+      <c r="N276" s="14" t="n">
+        <v>-126247.0610022335</v>
+      </c>
+      <c r="O276" s="12" t="n">
+        <v>131</v>
+      </c>
+      <c r="P276" s="12" t="n">
+        <v>170</v>
+      </c>
+      <c r="Q276" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="R276" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="S276" s="14" t="n">
+        <v>143550</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="15" t="n">
+        <v>276</v>
+      </c>
+      <c r="B277" s="15" t="n">
+        <v>826</v>
+      </c>
+      <c r="C277" s="15" t="n">
+        <v>828</v>
+      </c>
+      <c r="D277" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E277" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="F277" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G277" s="17" t="n">
+        <v>129</v>
+      </c>
+      <c r="H277" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I277" s="17" t="n">
+        <v>129</v>
+      </c>
+      <c r="J277" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K277" s="17" t="n">
+        <v>129</v>
+      </c>
+      <c r="L277" s="18" t="n">
+        <v>1336436.661694922</v>
+      </c>
+      <c r="M277" s="18" t="n">
+        <v>1446218.561338685</v>
+      </c>
+      <c r="N277" s="18" t="n">
+        <v>109781.8996437623</v>
+      </c>
+      <c r="O277" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="P277" s="17" t="n">
+        <v>52.33333333333334</v>
+      </c>
+      <c r="Q277" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="R277" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="S277" s="18" t="n">
+        <v>187050</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="10" t="n">
+        <v>277</v>
+      </c>
+      <c r="B278" s="10" t="n">
+        <v>829</v>
+      </c>
+      <c r="C278" s="10" t="n">
+        <v>831</v>
+      </c>
+      <c r="D278" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E278" s="11" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="F278" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G278" s="12" t="n">
+        <v>36</v>
+      </c>
+      <c r="H278" s="12" t="n">
+        <v>34</v>
+      </c>
+      <c r="I278" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="J278" s="13" t="n">
+        <v>0.05555555555555555</v>
+      </c>
+      <c r="K278" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="L278" s="14" t="n">
+        <v>1232642.13</v>
+      </c>
+      <c r="M278" s="14" t="n">
+        <v>1232642.13</v>
+      </c>
+      <c r="N278" s="11" t="n"/>
+      <c r="O278" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="P278" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q278" s="12" t="n">
+        <v>400</v>
+      </c>
+      <c r="R278" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="S278" s="14" t="n">
+        <v>2900</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S265"/>
+  <autoFilter ref="A1:S278"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -28191,7 +29614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N793"/>
+  <dimension ref="A1:N830"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -64714,8 +66137,1710 @@
         <v>27550</v>
       </c>
     </row>
+    <row r="794">
+      <c r="A794" s="10" t="n">
+        <v>793</v>
+      </c>
+      <c r="B794" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C794" s="12" t="n">
+        <v>25</v>
+      </c>
+      <c r="D794" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E794" s="12" t="n">
+        <v>25</v>
+      </c>
+      <c r="F794" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G794" s="12" t="n">
+        <v>25</v>
+      </c>
+      <c r="H794" s="14" t="n">
+        <v>819236.7618458089</v>
+      </c>
+      <c r="I794" s="12" t="n">
+        <v>546</v>
+      </c>
+      <c r="J794" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K794" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L794" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M794" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N794" s="14" t="n">
+        <v>36250</v>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" s="15" t="n">
+        <v>794</v>
+      </c>
+      <c r="B795" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C795" s="17" t="n">
+        <v>26</v>
+      </c>
+      <c r="D795" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E795" s="17" t="n">
+        <v>26</v>
+      </c>
+      <c r="F795" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G795" s="17" t="n">
+        <v>26</v>
+      </c>
+      <c r="H795" s="18" t="n">
+        <v>636610.5777368078</v>
+      </c>
+      <c r="I795" s="17" t="n">
+        <v>520</v>
+      </c>
+      <c r="J795" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K795" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="L795" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="M795" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N795" s="18" t="n">
+        <v>37700</v>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" s="10" t="n">
+        <v>795</v>
+      </c>
+      <c r="B796" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C796" s="12" t="n">
+        <v>39</v>
+      </c>
+      <c r="D796" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E796" s="12" t="n">
+        <v>39</v>
+      </c>
+      <c r="F796" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G796" s="12" t="n">
+        <v>39</v>
+      </c>
+      <c r="H796" s="14" t="n">
+        <v>687286.2674140512</v>
+      </c>
+      <c r="I796" s="12" t="n">
+        <v>481</v>
+      </c>
+      <c r="J796" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K796" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="L796" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="M796" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N796" s="14" t="n">
+        <v>56550</v>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" s="15" t="n">
+        <v>796</v>
+      </c>
+      <c r="B797" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C797" s="17" t="n">
+        <v>28</v>
+      </c>
+      <c r="D797" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E797" s="17" t="n">
+        <v>28</v>
+      </c>
+      <c r="F797" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G797" s="17" t="n">
+        <v>28</v>
+      </c>
+      <c r="H797" s="18" t="n">
+        <v>723688.4451556315</v>
+      </c>
+      <c r="I797" s="17" t="n">
+        <v>453</v>
+      </c>
+      <c r="J797" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K797" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="L797" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="M797" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N797" s="18" t="n">
+        <v>40600</v>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" s="10" t="n">
+        <v>797</v>
+      </c>
+      <c r="B798" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C798" s="12" t="n">
+        <v>29</v>
+      </c>
+      <c r="D798" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E798" s="12" t="n">
+        <v>29</v>
+      </c>
+      <c r="F798" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G798" s="12" t="n">
+        <v>29</v>
+      </c>
+      <c r="H798" s="14" t="n">
+        <v>761404.4622225834</v>
+      </c>
+      <c r="I798" s="12" t="n">
+        <v>424</v>
+      </c>
+      <c r="J798" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K798" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="L798" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="M798" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N798" s="14" t="n">
+        <v>42050</v>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" s="15" t="n">
+        <v>798</v>
+      </c>
+      <c r="B799" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C799" s="17" t="n">
+        <v>45</v>
+      </c>
+      <c r="D799" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E799" s="17" t="n">
+        <v>45</v>
+      </c>
+      <c r="F799" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G799" s="17" t="n">
+        <v>45</v>
+      </c>
+      <c r="H799" s="18" t="n">
+        <v>819949.6593412205</v>
+      </c>
+      <c r="I799" s="17" t="n">
+        <v>379</v>
+      </c>
+      <c r="J799" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K799" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="L799" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="M799" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N799" s="18" t="n">
+        <v>65250</v>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" s="10" t="n">
+        <v>799</v>
+      </c>
+      <c r="B800" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C800" s="12" t="n">
+        <v>23</v>
+      </c>
+      <c r="D800" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E800" s="12" t="n">
+        <v>23</v>
+      </c>
+      <c r="F800" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G800" s="12" t="n">
+        <v>23</v>
+      </c>
+      <c r="H800" s="14" t="n">
+        <v>849910.6568799117</v>
+      </c>
+      <c r="I800" s="12" t="n">
+        <v>356</v>
+      </c>
+      <c r="J800" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K800" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="L800" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="M800" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N800" s="14" t="n">
+        <v>33350</v>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" s="15" t="n">
+        <v>800</v>
+      </c>
+      <c r="B801" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C801" s="17" t="n">
+        <v>25</v>
+      </c>
+      <c r="D801" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E801" s="17" t="n">
+        <v>25</v>
+      </c>
+      <c r="F801" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G801" s="17" t="n">
+        <v>25</v>
+      </c>
+      <c r="H801" s="18" t="n">
+        <v>882489.1923255296</v>
+      </c>
+      <c r="I801" s="17" t="n">
+        <v>331</v>
+      </c>
+      <c r="J801" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K801" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="L801" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="M801" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N801" s="18" t="n">
+        <v>36250</v>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" s="10" t="n">
+        <v>801</v>
+      </c>
+      <c r="B802" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C802" s="12" t="n">
+        <v>18</v>
+      </c>
+      <c r="D802" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E802" s="12" t="n">
+        <v>18</v>
+      </c>
+      <c r="F802" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G802" s="12" t="n">
+        <v>18</v>
+      </c>
+      <c r="H802" s="14" t="n">
+        <v>905978.3933006477</v>
+      </c>
+      <c r="I802" s="12" t="n">
+        <v>513</v>
+      </c>
+      <c r="J802" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K802" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L802" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M802" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N802" s="14" t="n">
+        <v>26100</v>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" s="15" t="n">
+        <v>802</v>
+      </c>
+      <c r="B803" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C803" s="17" t="n">
+        <v>42</v>
+      </c>
+      <c r="D803" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E803" s="17" t="n">
+        <v>42</v>
+      </c>
+      <c r="F803" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G803" s="17" t="n">
+        <v>42</v>
+      </c>
+      <c r="H803" s="18" t="n">
+        <v>960687.6182285527</v>
+      </c>
+      <c r="I803" s="17" t="n">
+        <v>471</v>
+      </c>
+      <c r="J803" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K803" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L803" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M803" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N803" s="18" t="n">
+        <v>60900</v>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" s="10" t="n">
+        <v>803</v>
+      </c>
+      <c r="B804" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C804" s="12" t="n">
+        <v>30</v>
+      </c>
+      <c r="D804" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E804" s="12" t="n">
+        <v>30</v>
+      </c>
+      <c r="F804" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G804" s="12" t="n">
+        <v>30</v>
+      </c>
+      <c r="H804" s="14" t="n">
+        <v>999818.5989640168</v>
+      </c>
+      <c r="I804" s="12" t="n">
+        <v>441</v>
+      </c>
+      <c r="J804" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K804" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L804" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M804" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N804" s="14" t="n">
+        <v>43500</v>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" s="15" t="n">
+        <v>804</v>
+      </c>
+      <c r="B805" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C805" s="17" t="n">
+        <v>43</v>
+      </c>
+      <c r="D805" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E805" s="17" t="n">
+        <v>43</v>
+      </c>
+      <c r="F805" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G805" s="17" t="n">
+        <v>43</v>
+      </c>
+      <c r="H805" s="18" t="n">
+        <v>839376.8427660714</v>
+      </c>
+      <c r="I805" s="17" t="n">
+        <v>398</v>
+      </c>
+      <c r="J805" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K805" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="L805" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="M805" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N805" s="18" t="n">
+        <v>62350</v>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" s="10" t="n">
+        <v>805</v>
+      </c>
+      <c r="B806" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C806" s="12" t="n">
+        <v>33</v>
+      </c>
+      <c r="D806" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E806" s="12" t="n">
+        <v>33</v>
+      </c>
+      <c r="F806" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G806" s="12" t="n">
+        <v>33</v>
+      </c>
+      <c r="H806" s="14" t="n">
+        <v>882342.9434852329</v>
+      </c>
+      <c r="I806" s="12" t="n">
+        <v>365</v>
+      </c>
+      <c r="J806" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K806" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="L806" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="M806" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N806" s="14" t="n">
+        <v>47850</v>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" s="15" t="n">
+        <v>806</v>
+      </c>
+      <c r="B807" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C807" s="17" t="n">
+        <v>49</v>
+      </c>
+      <c r="D807" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E807" s="17" t="n">
+        <v>49</v>
+      </c>
+      <c r="F807" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G807" s="17" t="n">
+        <v>49</v>
+      </c>
+      <c r="H807" s="18" t="n">
+        <v>946137.2196371516</v>
+      </c>
+      <c r="I807" s="17" t="n">
+        <v>316</v>
+      </c>
+      <c r="J807" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K807" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="L807" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="M807" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N807" s="18" t="n">
+        <v>71050</v>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" s="10" t="n">
+        <v>807</v>
+      </c>
+      <c r="B808" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C808" s="12" t="n">
+        <v>24</v>
+      </c>
+      <c r="D808" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E808" s="12" t="n">
+        <v>24</v>
+      </c>
+      <c r="F808" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G808" s="12" t="n">
+        <v>24</v>
+      </c>
+      <c r="H808" s="14" t="n">
+        <v>977451.7725586459</v>
+      </c>
+      <c r="I808" s="12" t="n">
+        <v>292</v>
+      </c>
+      <c r="J808" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K808" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="L808" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="M808" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N808" s="14" t="n">
+        <v>34800</v>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" s="15" t="n">
+        <v>808</v>
+      </c>
+      <c r="B809" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C809" s="17" t="n">
+        <v>23</v>
+      </c>
+      <c r="D809" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E809" s="17" t="n">
+        <v>23</v>
+      </c>
+      <c r="F809" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G809" s="17" t="n">
+        <v>23</v>
+      </c>
+      <c r="H809" s="18" t="n">
+        <v>1007477.926182033</v>
+      </c>
+      <c r="I809" s="17" t="n">
+        <v>269</v>
+      </c>
+      <c r="J809" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K809" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="L809" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="M809" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N809" s="18" t="n">
+        <v>33350</v>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" s="10" t="n">
+        <v>809</v>
+      </c>
+      <c r="B810" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C810" s="12" t="n">
+        <v>42</v>
+      </c>
+      <c r="D810" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E810" s="12" t="n">
+        <v>42</v>
+      </c>
+      <c r="F810" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G810" s="12" t="n">
+        <v>42</v>
+      </c>
+      <c r="H810" s="14" t="n">
+        <v>1062229.743607742</v>
+      </c>
+      <c r="I810" s="12" t="n">
+        <v>227</v>
+      </c>
+      <c r="J810" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K810" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="L810" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="M810" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N810" s="14" t="n">
+        <v>60900</v>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" s="15" t="n">
+        <v>810</v>
+      </c>
+      <c r="B811" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C811" s="17" t="n">
+        <v>25</v>
+      </c>
+      <c r="D811" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E811" s="17" t="n">
+        <v>25</v>
+      </c>
+      <c r="F811" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G811" s="17" t="n">
+        <v>25</v>
+      </c>
+      <c r="H811" s="18" t="n">
+        <v>1094899.648125981</v>
+      </c>
+      <c r="I811" s="17" t="n">
+        <v>202</v>
+      </c>
+      <c r="J811" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K811" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="L811" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="M811" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N811" s="18" t="n">
+        <v>36250</v>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" s="10" t="n">
+        <v>811</v>
+      </c>
+      <c r="B812" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C812" s="12" t="n">
+        <v>26</v>
+      </c>
+      <c r="D812" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E812" s="12" t="n">
+        <v>26</v>
+      </c>
+      <c r="F812" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G812" s="12" t="n">
+        <v>26</v>
+      </c>
+      <c r="H812" s="14" t="n">
+        <v>1128881.627269907</v>
+      </c>
+      <c r="I812" s="12" t="n">
+        <v>376</v>
+      </c>
+      <c r="J812" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K812" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L812" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M812" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N812" s="14" t="n">
+        <v>37700</v>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" s="15" t="n">
+        <v>812</v>
+      </c>
+      <c r="B813" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C813" s="17" t="n">
+        <v>49</v>
+      </c>
+      <c r="D813" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E813" s="17" t="n">
+        <v>49</v>
+      </c>
+      <c r="F813" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G813" s="17" t="n">
+        <v>49</v>
+      </c>
+      <c r="H813" s="18" t="n">
+        <v>1192789.73212802</v>
+      </c>
+      <c r="I813" s="17" t="n">
+        <v>327</v>
+      </c>
+      <c r="J813" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K813" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L813" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M813" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N813" s="18" t="n">
+        <v>71050</v>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" s="10" t="n">
+        <v>813</v>
+      </c>
+      <c r="B814" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C814" s="12" t="n">
+        <v>41</v>
+      </c>
+      <c r="D814" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E814" s="12" t="n">
+        <v>41</v>
+      </c>
+      <c r="F814" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G814" s="12" t="n">
+        <v>41</v>
+      </c>
+      <c r="H814" s="14" t="n">
+        <v>1246323.468159911</v>
+      </c>
+      <c r="I814" s="12" t="n">
+        <v>286</v>
+      </c>
+      <c r="J814" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K814" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L814" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M814" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N814" s="14" t="n">
+        <v>59450</v>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" s="15" t="n">
+        <v>814</v>
+      </c>
+      <c r="B815" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C815" s="17" t="n">
+        <v>15</v>
+      </c>
+      <c r="D815" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E815" s="17" t="n">
+        <v>15</v>
+      </c>
+      <c r="F815" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G815" s="17" t="n">
+        <v>15</v>
+      </c>
+      <c r="H815" s="18" t="n">
+        <v>1049575.782540787</v>
+      </c>
+      <c r="I815" s="17" t="n">
+        <v>271</v>
+      </c>
+      <c r="J815" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K815" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="L815" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="M815" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N815" s="18" t="n">
+        <v>21750</v>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" s="10" t="n">
+        <v>815</v>
+      </c>
+      <c r="B816" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C816" s="12" t="n">
+        <v>21</v>
+      </c>
+      <c r="D816" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E816" s="12" t="n">
+        <v>21</v>
+      </c>
+      <c r="F816" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G816" s="12" t="n">
+        <v>21</v>
+      </c>
+      <c r="H816" s="14" t="n">
+        <v>1077028.011926319</v>
+      </c>
+      <c r="I816" s="12" t="n">
+        <v>250</v>
+      </c>
+      <c r="J816" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K816" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="L816" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="M816" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N816" s="14" t="n">
+        <v>30450</v>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" s="15" t="n">
+        <v>816</v>
+      </c>
+      <c r="B817" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C817" s="17" t="n">
+        <v>36</v>
+      </c>
+      <c r="D817" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E817" s="17" t="n">
+        <v>36</v>
+      </c>
+      <c r="F817" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G817" s="17" t="n">
+        <v>36</v>
+      </c>
+      <c r="H817" s="18" t="n">
+        <v>1123993.312617932</v>
+      </c>
+      <c r="I817" s="17" t="n">
+        <v>214</v>
+      </c>
+      <c r="J817" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K817" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="L817" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="M817" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N817" s="18" t="n">
+        <v>52200</v>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" s="10" t="n">
+        <v>817</v>
+      </c>
+      <c r="B818" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C818" s="12" t="n">
+        <v>39</v>
+      </c>
+      <c r="D818" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E818" s="12" t="n">
+        <v>39</v>
+      </c>
+      <c r="F818" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G818" s="12" t="n">
+        <v>39</v>
+      </c>
+      <c r="H818" s="14" t="n">
+        <v>1174884.256456956</v>
+      </c>
+      <c r="I818" s="12" t="n">
+        <v>175</v>
+      </c>
+      <c r="J818" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K818" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="L818" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="M818" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N818" s="14" t="n">
+        <v>56550</v>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" s="15" t="n">
+        <v>818</v>
+      </c>
+      <c r="B819" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C819" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="D819" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E819" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="F819" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G819" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="H819" s="18" t="n">
+        <v>1189392.042563901</v>
+      </c>
+      <c r="I819" s="17" t="n">
+        <v>164</v>
+      </c>
+      <c r="J819" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K819" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="L819" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="M819" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N819" s="18" t="n">
+        <v>15950</v>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" s="10" t="n">
+        <v>819</v>
+      </c>
+      <c r="B820" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C820" s="12" t="n">
+        <v>42</v>
+      </c>
+      <c r="D820" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E820" s="12" t="n">
+        <v>42</v>
+      </c>
+      <c r="F820" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G820" s="12" t="n">
+        <v>42</v>
+      </c>
+      <c r="H820" s="14" t="n">
+        <v>1244216.781823416</v>
+      </c>
+      <c r="I820" s="12" t="n">
+        <v>122</v>
+      </c>
+      <c r="J820" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K820" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="L820" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="M820" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N820" s="14" t="n">
+        <v>60900</v>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" s="15" t="n">
+        <v>820</v>
+      </c>
+      <c r="B821" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C821" s="17" t="n">
+        <v>40</v>
+      </c>
+      <c r="D821" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E821" s="17" t="n">
+        <v>40</v>
+      </c>
+      <c r="F821" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G821" s="17" t="n">
+        <v>40</v>
+      </c>
+      <c r="H821" s="18" t="n">
+        <v>1296461.27694519</v>
+      </c>
+      <c r="I821" s="17" t="n">
+        <v>82</v>
+      </c>
+      <c r="J821" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K821" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="L821" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="M821" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N821" s="18" t="n">
+        <v>58000</v>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" s="10" t="n">
+        <v>821</v>
+      </c>
+      <c r="B822" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C822" s="12" t="n">
+        <v>13</v>
+      </c>
+      <c r="D822" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E822" s="12" t="n">
+        <v>13</v>
+      </c>
+      <c r="F822" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G822" s="12" t="n">
+        <v>13</v>
+      </c>
+      <c r="H822" s="14" t="n">
+        <v>1313627.327485397</v>
+      </c>
+      <c r="I822" s="12" t="n">
+        <v>269</v>
+      </c>
+      <c r="J822" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K822" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L822" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M822" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N822" s="14" t="n">
+        <v>18850</v>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" s="15" t="n">
+        <v>822</v>
+      </c>
+      <c r="B823" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C823" s="17" t="n">
+        <v>39</v>
+      </c>
+      <c r="D823" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E823" s="17" t="n">
+        <v>39</v>
+      </c>
+      <c r="F823" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G823" s="17" t="n">
+        <v>39</v>
+      </c>
+      <c r="H823" s="18" t="n">
+        <v>1364613.943219726</v>
+      </c>
+      <c r="I823" s="17" t="n">
+        <v>230</v>
+      </c>
+      <c r="J823" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K823" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L823" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M823" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N823" s="18" t="n">
+        <v>56550</v>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" s="10" t="n">
+        <v>823</v>
+      </c>
+      <c r="B824" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C824" s="12" t="n">
+        <v>30</v>
+      </c>
+      <c r="D824" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E824" s="12" t="n">
+        <v>30</v>
+      </c>
+      <c r="F824" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G824" s="12" t="n">
+        <v>30</v>
+      </c>
+      <c r="H824" s="14" t="n">
+        <v>1403917.095221187</v>
+      </c>
+      <c r="I824" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="J824" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K824" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L824" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M824" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N824" s="14" t="n">
+        <v>43500</v>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" s="15" t="n">
+        <v>824</v>
+      </c>
+      <c r="B825" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C825" s="17" t="n">
+        <v>21</v>
+      </c>
+      <c r="D825" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E825" s="17" t="n">
+        <v>21</v>
+      </c>
+      <c r="F825" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G825" s="17" t="n">
+        <v>21</v>
+      </c>
+      <c r="H825" s="18" t="n">
+        <v>1215035.44317431</v>
+      </c>
+      <c r="I825" s="17" t="n">
+        <v>179</v>
+      </c>
+      <c r="J825" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K825" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="L825" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="M825" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N825" s="18" t="n">
+        <v>30450</v>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" s="10" t="n">
+        <v>825</v>
+      </c>
+      <c r="B826" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C826" s="12" t="n">
+        <v>48</v>
+      </c>
+      <c r="D826" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E826" s="12" t="n">
+        <v>48</v>
+      </c>
+      <c r="F826" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G826" s="12" t="n">
+        <v>48</v>
+      </c>
+      <c r="H826" s="14" t="n">
+        <v>1277670.034218953</v>
+      </c>
+      <c r="I826" s="12" t="n">
+        <v>131</v>
+      </c>
+      <c r="J826" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K826" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="L826" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="M826" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N826" s="14" t="n">
+        <v>69600</v>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" s="15" t="n">
+        <v>826</v>
+      </c>
+      <c r="B827" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C827" s="17" t="n">
+        <v>45</v>
+      </c>
+      <c r="D827" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E827" s="17" t="n">
+        <v>45</v>
+      </c>
+      <c r="F827" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G827" s="17" t="n">
+        <v>45</v>
+      </c>
+      <c r="H827" s="18" t="n">
+        <v>1336436.661694922</v>
+      </c>
+      <c r="I827" s="17" t="n">
+        <v>86</v>
+      </c>
+      <c r="J827" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K827" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="L827" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="M827" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N827" s="18" t="n">
+        <v>65250</v>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" s="10" t="n">
+        <v>827</v>
+      </c>
+      <c r="B828" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C828" s="12" t="n">
+        <v>17</v>
+      </c>
+      <c r="D828" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E828" s="12" t="n">
+        <v>17</v>
+      </c>
+      <c r="F828" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G828" s="12" t="n">
+        <v>17</v>
+      </c>
+      <c r="H828" s="14" t="n">
+        <v>1358811.361060816</v>
+      </c>
+      <c r="I828" s="12" t="n">
+        <v>69</v>
+      </c>
+      <c r="J828" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K828" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="L828" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="M828" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N828" s="14" t="n">
+        <v>24650</v>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" s="15" t="n">
+        <v>828</v>
+      </c>
+      <c r="B829" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C829" s="17" t="n">
+        <v>67</v>
+      </c>
+      <c r="D829" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E829" s="17" t="n">
+        <v>67</v>
+      </c>
+      <c r="F829" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G829" s="17" t="n">
+        <v>67</v>
+      </c>
+      <c r="H829" s="18" t="n">
+        <v>1446218.561338685</v>
+      </c>
+      <c r="I829" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="J829" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K829" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="L829" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="M829" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N829" s="18" t="n">
+        <v>97150</v>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" s="10" t="n">
+        <v>829</v>
+      </c>
+      <c r="B830" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C830" s="12" t="n">
+        <v>36</v>
+      </c>
+      <c r="D830" s="12" t="n">
+        <v>34</v>
+      </c>
+      <c r="E830" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="F830" s="13" t="n">
+        <v>0.05555555555555555</v>
+      </c>
+      <c r="G830" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="H830" s="14" t="n">
+        <v>1232642.13</v>
+      </c>
+      <c r="I830" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J830" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K830" s="12" t="n">
+        <v>400</v>
+      </c>
+      <c r="L830" s="12" t="n">
+        <v>400</v>
+      </c>
+      <c r="M830" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N830" s="14" t="n">
+        <v>2900</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N793"/>
+  <autoFilter ref="A1:N830"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -65110,7 +68235,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -66049,8 +69174,56 @@
         <v>55</v>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" s="23" t="n">
+        <v>730.66</v>
+      </c>
+      <c r="B39" s="16" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C39" s="16" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D39" s="16" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E39" s="16" t="inlineStr"/>
+      <c r="F39" s="17" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="21" t="n">
+        <v>742.75</v>
+      </c>
+      <c r="B40" s="11" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C40" s="11" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D40" s="11" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E40" s="11" t="inlineStr"/>
+      <c r="F40" s="12" t="n">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F38"/>
+  <autoFilter ref="A1:F40"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -66449,7 +69622,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U19"/>
+  <dimension ref="A1:U20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -66471,7 +69644,7 @@
     <col width="12" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
-    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="21" customWidth="1" min="20" max="20"/>
     <col width="20" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
@@ -67846,8 +71019,77 @@
         <v>30226.64187802165</v>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="n">
+        <v>829</v>
+      </c>
+      <c r="C20" s="14" t="n">
+        <v>1232642.13</v>
+      </c>
+      <c r="D20" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="E20" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="G20" s="14" t="n">
+        <v>2004506.73</v>
+      </c>
+      <c r="H20" s="21" t="n">
+        <v>40</v>
+      </c>
+      <c r="I20" s="21" t="n">
+        <v>55</v>
+      </c>
+      <c r="J20" s="11" t="inlineStr">
+        <is>
+          <t>truck</t>
+        </is>
+      </c>
+      <c r="K20" s="22" t="n">
+        <v>3600</v>
+      </c>
+      <c r="L20" s="22" t="n">
+        <v>200</v>
+      </c>
+      <c r="M20" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" s="12" t="n">
+        <v>400</v>
+      </c>
+      <c r="O20" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="P20" s="10" t="n">
+        <v>277</v>
+      </c>
+      <c r="Q20" s="12" t="n">
+        <v>36</v>
+      </c>
+      <c r="R20" s="12" t="n">
+        <v>34</v>
+      </c>
+      <c r="S20" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="T20" s="13" t="n">
+        <v>0.05555555555555555</v>
+      </c>
+      <c r="U20" s="11" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U19"/>
+  <autoFilter ref="A1:U20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -67858,7 +71100,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E217"/>
+  <dimension ref="A1:E229"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -72791,8 +76033,280 @@
         </is>
       </c>
     </row>
+    <row r="218">
+      <c r="A218" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B218" s="10" t="n">
+        <v>829</v>
+      </c>
+      <c r="C218" s="11" t="inlineStr">
+        <is>
+          <t>Starting Cash</t>
+        </is>
+      </c>
+      <c r="D218" s="14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E218" s="11" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B219" s="15" t="n">
+        <v>829</v>
+      </c>
+      <c r="C219" s="16" t="inlineStr">
+        <is>
+          <t>Cash Sources</t>
+        </is>
+      </c>
+      <c r="D219" s="16" t="n"/>
+      <c r="E219" s="16" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B220" s="10" t="n">
+        <v>829</v>
+      </c>
+      <c r="C220" s="11" t="inlineStr">
+        <is>
+          <t>revenues</t>
+        </is>
+      </c>
+      <c r="D220" s="14" t="n">
+        <v>21677500</v>
+      </c>
+      <c r="E220" s="11" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B221" s="15" t="n">
+        <v>829</v>
+      </c>
+      <c r="C221" s="16" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D221" s="18" t="n">
+        <v>298236.49</v>
+      </c>
+      <c r="E221" s="16" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B222" s="10" t="n">
+        <v>829</v>
+      </c>
+      <c r="C222" s="11" t="inlineStr">
+        <is>
+          <t>Cash Uses</t>
+        </is>
+      </c>
+      <c r="D222" s="11" t="n"/>
+      <c r="E222" s="11" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B223" s="15" t="n">
+        <v>829</v>
+      </c>
+      <c r="C223" s="16" t="inlineStr">
+        <is>
+          <t>outbound shipping</t>
+        </is>
+      </c>
+      <c r="D223" s="18" t="n">
+        <v>-2242500</v>
+      </c>
+      <c r="E223" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B224" s="10" t="n">
+        <v>829</v>
+      </c>
+      <c r="C224" s="11" t="inlineStr">
+        <is>
+          <t>inbound shipping</t>
+        </is>
+      </c>
+      <c r="D224" s="14" t="n">
+        <v>-1500000</v>
+      </c>
+      <c r="E224" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B225" s="15" t="n">
+        <v>829</v>
+      </c>
+      <c r="C225" s="16" t="inlineStr">
+        <is>
+          <t>FGI holding</t>
+        </is>
+      </c>
+      <c r="D225" s="18" t="n">
+        <v>-21808.28</v>
+      </c>
+      <c r="E225" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B226" s="10" t="n">
+        <v>829</v>
+      </c>
+      <c r="C226" s="11" t="inlineStr">
+        <is>
+          <t>add capacity</t>
+        </is>
+      </c>
+      <c r="D226" s="14" t="n">
+        <v>-1749840.87</v>
+      </c>
+      <c r="E226" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B227" s="15" t="n">
+        <v>829</v>
+      </c>
+      <c r="C227" s="16" t="inlineStr">
+        <is>
+          <t>Pipeline inventory holding</t>
+        </is>
+      </c>
+      <c r="D227" s="18" t="n">
+        <v>-28945.21</v>
+      </c>
+      <c r="E227" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B228" s="10" t="n">
+        <v>829</v>
+      </c>
+      <c r="C228" s="11" t="inlineStr">
+        <is>
+          <t>production</t>
+        </is>
+      </c>
+      <c r="D228" s="14" t="n">
+        <v>-15700000</v>
+      </c>
+      <c r="E228" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B229" s="15" t="n">
+        <v>829</v>
+      </c>
+      <c r="C229" s="16" t="inlineStr">
+        <is>
+          <t>Cash Balance</t>
+        </is>
+      </c>
+      <c r="D229" s="18" t="n">
+        <v>1232642.13</v>
+      </c>
+      <c r="E229" s="16" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E217"/>
+  <autoFilter ref="A1:E229"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update game data: day 830, cash 1232854.46, 3-day period 277
</commit_message>
<xml_diff>
--- a/data/supply_chain_game.xlsx
+++ b/data/supply_chain_game.xlsx
@@ -21,15 +21,15 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$278</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$830</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$831</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'资金构成_旧版'!$A$1:$C$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'运营参数_旧版'!$A$9:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$45</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'排行榜_旧版'!$A$1:$C$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$241</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$253</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'运营参数'!$A$1:$J$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$541</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$568</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -590,7 +590,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-06T11:48:32+08:00</t>
+          <t>2026-09-06T11:56:02+08:00</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>829</v>
+        <v>830</v>
       </c>
     </row>
     <row r="7">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>631</v>
+        <v>630</v>
       </c>
     </row>
     <row r="8">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>1232642.13</v>
+        <v>1232854.46</v>
       </c>
     </row>
     <row r="11">
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>2004506.73</v>
+        <v>2005098.71</v>
       </c>
     </row>
     <row r="15"/>
@@ -861,7 +861,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>36</v>
+        <v>72</v>
       </c>
     </row>
     <row r="33">
@@ -871,7 +871,7 @@
         </is>
       </c>
       <c r="B33" s="7" t="n">
-        <v>34</v>
+        <v>70</v>
       </c>
     </row>
     <row r="34">
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B35" s="8" t="n">
-        <v>0.05555555555555555</v>
+        <v>0.02777777777777778</v>
       </c>
     </row>
     <row r="36">
@@ -909,6 +909,9 @@
         <is>
           <t>周期现金变动</t>
         </is>
+      </c>
+      <c r="B37" s="4" t="n">
+        <v>212.3251607038546</v>
       </c>
     </row>
     <row r="38"/>
@@ -970,7 +973,7 @@
         </is>
       </c>
       <c r="B44" s="4" t="n">
-        <v>109781.8996437623</v>
+        <v>109781.9000747609</v>
       </c>
     </row>
     <row r="45"/>
@@ -1252,7 +1255,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E541"/>
+  <dimension ref="A1:E568"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -12629,8 +12632,575 @@
         <v>1232642.13</v>
       </c>
     </row>
+    <row r="542">
+      <c r="A542" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B542" s="10" t="n">
+        <v>830</v>
+      </c>
+      <c r="C542" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D542" s="11" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="E542" s="14" t="n">
+        <v>3237953.17</v>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B543" s="15" t="n">
+        <v>830</v>
+      </c>
+      <c r="C543" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D543" s="16" t="inlineStr">
+        <is>
+          <t>nicetry</t>
+        </is>
+      </c>
+      <c r="E543" s="18" t="n">
+        <v>2438683.21</v>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B544" s="10" t="n">
+        <v>830</v>
+      </c>
+      <c r="C544" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D544" s="11" t="inlineStr">
+        <is>
+          <t>group8</t>
+        </is>
+      </c>
+      <c r="E544" s="14" t="n">
+        <v>2403545.28</v>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B545" s="15" t="n">
+        <v>830</v>
+      </c>
+      <c r="C545" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D545" s="16" t="inlineStr">
+        <is>
+          <t>montesquieu</t>
+        </is>
+      </c>
+      <c r="E545" s="18" t="n">
+        <v>2331250.31</v>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B546" s="10" t="n">
+        <v>830</v>
+      </c>
+      <c r="C546" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="D546" s="11" t="inlineStr">
+        <is>
+          <t>group9</t>
+        </is>
+      </c>
+      <c r="E546" s="14" t="n">
+        <v>2198732.28</v>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B547" s="15" t="n">
+        <v>830</v>
+      </c>
+      <c r="C547" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="D547" s="16" t="inlineStr">
+        <is>
+          <t>tigagroup20</t>
+        </is>
+      </c>
+      <c r="E547" s="18" t="n">
+        <v>2116510.21</v>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B548" s="10" t="n">
+        <v>830</v>
+      </c>
+      <c r="C548" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="D548" s="11" t="inlineStr">
+        <is>
+          <t>group2</t>
+        </is>
+      </c>
+      <c r="E548" s="14" t="n">
+        <v>2074386.95</v>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B549" s="15" t="n">
+        <v>830</v>
+      </c>
+      <c r="C549" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="D549" s="16" t="inlineStr">
+        <is>
+          <t>group25</t>
+        </is>
+      </c>
+      <c r="E549" s="18" t="n">
+        <v>2074229.53</v>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B550" s="10" t="n">
+        <v>830</v>
+      </c>
+      <c r="C550" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="D550" s="11" t="inlineStr">
+        <is>
+          <t>group11</t>
+        </is>
+      </c>
+      <c r="E550" s="14" t="n">
+        <v>2074217.27</v>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B551" s="15" t="n">
+        <v>830</v>
+      </c>
+      <c r="C551" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="D551" s="16" t="inlineStr">
+        <is>
+          <t>88888888</t>
+        </is>
+      </c>
+      <c r="E551" s="18" t="n">
+        <v>2074194.69</v>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B552" s="10" t="n">
+        <v>830</v>
+      </c>
+      <c r="C552" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="D552" s="11" t="inlineStr">
+        <is>
+          <t>group7</t>
+        </is>
+      </c>
+      <c r="E552" s="14" t="n">
+        <v>2045033.19</v>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B553" s="15" t="n">
+        <v>830</v>
+      </c>
+      <c r="C553" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="D553" s="16" t="inlineStr">
+        <is>
+          <t>t24</t>
+        </is>
+      </c>
+      <c r="E553" s="18" t="n">
+        <v>2039973.09</v>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B554" s="10" t="n">
+        <v>830</v>
+      </c>
+      <c r="C554" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="D554" s="11" t="inlineStr">
+        <is>
+          <t>teamhlly</t>
+        </is>
+      </c>
+      <c r="E554" s="14" t="n">
+        <v>1999461.1</v>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B555" s="15" t="n">
+        <v>830</v>
+      </c>
+      <c r="C555" s="15" t="n">
+        <v>14</v>
+      </c>
+      <c r="D555" s="16" t="inlineStr">
+        <is>
+          <t>jit</t>
+        </is>
+      </c>
+      <c r="E555" s="18" t="n">
+        <v>1968178.56</v>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B556" s="10" t="n">
+        <v>830</v>
+      </c>
+      <c r="C556" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="D556" s="11" t="inlineStr">
+        <is>
+          <t>deepsleep</t>
+        </is>
+      </c>
+      <c r="E556" s="14" t="n">
+        <v>1960291.88</v>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B557" s="15" t="n">
+        <v>830</v>
+      </c>
+      <c r="C557" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="D557" s="16" t="inlineStr">
+        <is>
+          <t>group14</t>
+        </is>
+      </c>
+      <c r="E557" s="18" t="n">
+        <v>1926932.37</v>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B558" s="10" t="n">
+        <v>830</v>
+      </c>
+      <c r="C558" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="D558" s="11" t="inlineStr">
+        <is>
+          <t>666666</t>
+        </is>
+      </c>
+      <c r="E558" s="14" t="n">
+        <v>1920042.68</v>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B559" s="15" t="n">
+        <v>830</v>
+      </c>
+      <c r="C559" s="15" t="n">
+        <v>18</v>
+      </c>
+      <c r="D559" s="16" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E559" s="18" t="n">
+        <v>1893728.09</v>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B560" s="10" t="n">
+        <v>830</v>
+      </c>
+      <c r="C560" s="10" t="n">
+        <v>19</v>
+      </c>
+      <c r="D560" s="11" t="inlineStr">
+        <is>
+          <t>group15</t>
+        </is>
+      </c>
+      <c r="E560" s="14" t="n">
+        <v>1885712.27</v>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B561" s="15" t="n">
+        <v>830</v>
+      </c>
+      <c r="C561" s="15" t="n">
+        <v>20</v>
+      </c>
+      <c r="D561" s="16" t="inlineStr">
+        <is>
+          <t>cleveregg</t>
+        </is>
+      </c>
+      <c r="E561" s="18" t="n">
+        <v>1765928.83</v>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B562" s="10" t="n">
+        <v>830</v>
+      </c>
+      <c r="C562" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="D562" s="11" t="inlineStr">
+        <is>
+          <t>vivo50</t>
+        </is>
+      </c>
+      <c r="E562" s="14" t="n">
+        <v>1486259.73</v>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B563" s="15" t="n">
+        <v>830</v>
+      </c>
+      <c r="C563" s="15" t="n">
+        <v>22</v>
+      </c>
+      <c r="D563" s="16" t="inlineStr">
+        <is>
+          <t>aaachemicalseller</t>
+        </is>
+      </c>
+      <c r="E563" s="18" t="n">
+        <v>1414326.53</v>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B564" s="10" t="n">
+        <v>830</v>
+      </c>
+      <c r="C564" s="10" t="n">
+        <v>23</v>
+      </c>
+      <c r="D564" s="11" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E564" s="14" t="n">
+        <v>1414248.19</v>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B565" s="15" t="n">
+        <v>830</v>
+      </c>
+      <c r="C565" s="15" t="n">
+        <v>24</v>
+      </c>
+      <c r="D565" s="16" t="inlineStr">
+        <is>
+          <t>group12</t>
+        </is>
+      </c>
+      <c r="E565" s="18" t="n">
+        <v>1412477.84</v>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B566" s="10" t="n">
+        <v>830</v>
+      </c>
+      <c r="C566" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="D566" s="11" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="E566" s="14" t="n">
+        <v>1275284.63</v>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B567" s="24" t="n">
+        <v>830</v>
+      </c>
+      <c r="C567" s="24" t="n">
+        <v>26</v>
+      </c>
+      <c r="D567" s="25" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="E567" s="26" t="n">
+        <v>1232854.46</v>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B568" s="10" t="n">
+        <v>830</v>
+      </c>
+      <c r="C568" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="D568" s="11" t="inlineStr">
+        <is>
+          <t>newgroup18</t>
+        </is>
+      </c>
+      <c r="E568" s="14" t="n">
+        <v>1199320.77</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E541"/>
+  <autoFilter ref="A1:E568"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -30161,7 +30731,7 @@
         <v>831</v>
       </c>
       <c r="D278" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E278" s="11" t="inlineStr">
         <is>
@@ -30174,27 +30744,29 @@
         </is>
       </c>
       <c r="G278" s="12" t="n">
-        <v>36</v>
+        <v>72</v>
       </c>
       <c r="H278" s="12" t="n">
-        <v>34</v>
+        <v>70</v>
       </c>
       <c r="I278" s="12" t="n">
         <v>2</v>
       </c>
       <c r="J278" s="13" t="n">
-        <v>0.05555555555555555</v>
+        <v>0.02777777777777778</v>
       </c>
       <c r="K278" s="12" t="n">
         <v>2</v>
       </c>
       <c r="L278" s="14" t="n">
-        <v>1232642.13</v>
+        <v>1232642.134839296</v>
       </c>
       <c r="M278" s="14" t="n">
-        <v>1232642.13</v>
-      </c>
-      <c r="N278" s="11" t="n"/>
+        <v>1232854.46</v>
+      </c>
+      <c r="N278" s="14" t="n">
+        <v>212.3251607038546</v>
+      </c>
       <c r="O278" s="12" t="n">
         <v>0</v>
       </c>
@@ -30223,7 +30795,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N830"/>
+  <dimension ref="A1:N831"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -68448,8 +69020,54 @@
         <v>2900</v>
       </c>
     </row>
+    <row r="831">
+      <c r="A831" s="15" t="n">
+        <v>830</v>
+      </c>
+      <c r="B831" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C831" s="17" t="n">
+        <v>36</v>
+      </c>
+      <c r="D831" s="17" t="n">
+        <v>36</v>
+      </c>
+      <c r="E831" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F831" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G831" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H831" s="18" t="n">
+        <v>1232854.46</v>
+      </c>
+      <c r="I831" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J831" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K831" s="17" t="n">
+        <v>400</v>
+      </c>
+      <c r="L831" s="17" t="n">
+        <v>400</v>
+      </c>
+      <c r="M831" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N831" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N830"/>
+  <autoFilter ref="A1:N831"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -68844,7 +69462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -69909,8 +70527,56 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" s="21" t="n">
+        <v>730.66</v>
+      </c>
+      <c r="B44" s="11" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C44" s="11" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D44" s="11" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E44" s="11" t="inlineStr"/>
+      <c r="F44" s="12" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="23" t="n">
+        <v>742.75</v>
+      </c>
+      <c r="B45" s="16" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C45" s="16" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D45" s="16" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E45" s="16" t="inlineStr"/>
+      <c r="F45" s="17" t="n">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F43"/>
+  <autoFilter ref="A1:F45"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -70309,7 +70975,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U20"/>
+  <dimension ref="A1:U21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -70331,7 +70997,7 @@
     <col width="12" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
-    <col width="21" customWidth="1" min="20" max="20"/>
+    <col width="22" customWidth="1" min="20" max="20"/>
     <col width="20" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
@@ -71775,8 +72441,79 @@
       </c>
       <c r="U20" s="11" t="n"/>
     </row>
+    <row r="21">
+      <c r="A21" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B21" s="15" t="n">
+        <v>830</v>
+      </c>
+      <c r="C21" s="18" t="n">
+        <v>1232854.46</v>
+      </c>
+      <c r="D21" s="15" t="n">
+        <v>26</v>
+      </c>
+      <c r="E21" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="F21" s="16" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="G21" s="18" t="n">
+        <v>2005098.71</v>
+      </c>
+      <c r="H21" s="23" t="n">
+        <v>40</v>
+      </c>
+      <c r="I21" s="23" t="n">
+        <v>55</v>
+      </c>
+      <c r="J21" s="16" t="inlineStr">
+        <is>
+          <t>mail</t>
+        </is>
+      </c>
+      <c r="K21" s="27" t="n">
+        <v>3600</v>
+      </c>
+      <c r="L21" s="27" t="n">
+        <v>200</v>
+      </c>
+      <c r="M21" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" s="17" t="n">
+        <v>400</v>
+      </c>
+      <c r="O21" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="P21" s="15" t="n">
+        <v>277</v>
+      </c>
+      <c r="Q21" s="17" t="n">
+        <v>72</v>
+      </c>
+      <c r="R21" s="17" t="n">
+        <v>70</v>
+      </c>
+      <c r="S21" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="T21" s="13" t="n">
+        <v>0.02777777777777778</v>
+      </c>
+      <c r="U21" s="18" t="n">
+        <v>212.3251607038546</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U20"/>
+  <autoFilter ref="A1:U21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -71787,7 +72524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E241"/>
+  <dimension ref="A1:E253"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -77264,8 +78001,280 @@
         </is>
       </c>
     </row>
+    <row r="242">
+      <c r="A242" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B242" s="10" t="n">
+        <v>830</v>
+      </c>
+      <c r="C242" s="11" t="inlineStr">
+        <is>
+          <t>Starting Cash</t>
+        </is>
+      </c>
+      <c r="D242" s="14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E242" s="11" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B243" s="15" t="n">
+        <v>830</v>
+      </c>
+      <c r="C243" s="16" t="inlineStr">
+        <is>
+          <t>Cash Sources</t>
+        </is>
+      </c>
+      <c r="D243" s="16" t="n"/>
+      <c r="E243" s="16" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B244" s="10" t="n">
+        <v>830</v>
+      </c>
+      <c r="C244" s="11" t="inlineStr">
+        <is>
+          <t>revenues</t>
+        </is>
+      </c>
+      <c r="D244" s="14" t="n">
+        <v>21677500</v>
+      </c>
+      <c r="E244" s="11" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B245" s="15" t="n">
+        <v>830</v>
+      </c>
+      <c r="C245" s="16" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D245" s="18" t="n">
+        <v>298558.4</v>
+      </c>
+      <c r="E245" s="16" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B246" s="10" t="n">
+        <v>830</v>
+      </c>
+      <c r="C246" s="11" t="inlineStr">
+        <is>
+          <t>Cash Uses</t>
+        </is>
+      </c>
+      <c r="D246" s="11" t="n"/>
+      <c r="E246" s="11" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B247" s="15" t="n">
+        <v>830</v>
+      </c>
+      <c r="C247" s="16" t="inlineStr">
+        <is>
+          <t>outbound shipping</t>
+        </is>
+      </c>
+      <c r="D247" s="18" t="n">
+        <v>-2242500</v>
+      </c>
+      <c r="E247" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B248" s="10" t="n">
+        <v>830</v>
+      </c>
+      <c r="C248" s="11" t="inlineStr">
+        <is>
+          <t>inbound shipping</t>
+        </is>
+      </c>
+      <c r="D248" s="14" t="n">
+        <v>-1500000</v>
+      </c>
+      <c r="E248" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B249" s="15" t="n">
+        <v>830</v>
+      </c>
+      <c r="C249" s="16" t="inlineStr">
+        <is>
+          <t>FGI holding</t>
+        </is>
+      </c>
+      <c r="D249" s="18" t="n">
+        <v>-21808.28</v>
+      </c>
+      <c r="E249" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B250" s="10" t="n">
+        <v>830</v>
+      </c>
+      <c r="C250" s="11" t="inlineStr">
+        <is>
+          <t>add capacity</t>
+        </is>
+      </c>
+      <c r="D250" s="14" t="n">
+        <v>-1749840.87</v>
+      </c>
+      <c r="E250" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B251" s="15" t="n">
+        <v>830</v>
+      </c>
+      <c r="C251" s="16" t="inlineStr">
+        <is>
+          <t>Pipeline inventory holding</t>
+        </is>
+      </c>
+      <c r="D251" s="18" t="n">
+        <v>-29054.79</v>
+      </c>
+      <c r="E251" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B252" s="10" t="n">
+        <v>830</v>
+      </c>
+      <c r="C252" s="11" t="inlineStr">
+        <is>
+          <t>production</t>
+        </is>
+      </c>
+      <c r="D252" s="14" t="n">
+        <v>-15700000</v>
+      </c>
+      <c r="E252" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T11:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B253" s="15" t="n">
+        <v>830</v>
+      </c>
+      <c r="C253" s="16" t="inlineStr">
+        <is>
+          <t>Cash Balance</t>
+        </is>
+      </c>
+      <c r="D253" s="18" t="n">
+        <v>1232854.46</v>
+      </c>
+      <c r="E253" s="16" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E241"/>
+  <autoFilter ref="A1:E253"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update game data: day 831, cash 1357866.84, 3-day period 277
</commit_message>
<xml_diff>
--- a/data/supply_chain_game.xlsx
+++ b/data/supply_chain_game.xlsx
@@ -21,15 +21,15 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$278</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$831</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$832</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'资金构成_旧版'!$A$1:$C$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'运营参数_旧版'!$A$9:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$47</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'排行榜_旧版'!$A$1:$C$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$253</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$265</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'运营参数'!$A$1:$J$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$568</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$595</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -590,7 +590,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-06T11:56:02+08:00</t>
+          <t>2026-09-06T12:11:03+08:00</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>830</v>
+        <v>831</v>
       </c>
     </row>
     <row r="7">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>630</v>
+        <v>629</v>
       </c>
     </row>
     <row r="8">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>1232854.46</v>
+        <v>1357866.84</v>
       </c>
     </row>
     <row r="11">
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>2005098.71</v>
+        <v>1880890.85</v>
       </c>
     </row>
     <row r="15"/>
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>0</v>
+        <v>119</v>
       </c>
     </row>
     <row r="25">
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>400</v>
+        <v>200</v>
       </c>
     </row>
     <row r="26">
@@ -850,7 +850,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>否（进行中）</t>
+          <t>是</t>
         </is>
       </c>
     </row>
@@ -861,7 +861,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>72</v>
+        <v>153</v>
       </c>
     </row>
     <row r="33">
@@ -881,7 +881,7 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>2</v>
+        <v>83</v>
       </c>
     </row>
     <row r="35">
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B35" s="8" t="n">
-        <v>0.02777777777777778</v>
+        <v>0.5424836601307189</v>
       </c>
     </row>
     <row r="36">
@@ -901,7 +901,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>2</v>
+        <v>83</v>
       </c>
     </row>
     <row r="37">
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="B37" s="4" t="n">
-        <v>212.3251607038546</v>
+        <v>107265.1143798644</v>
       </c>
     </row>
     <row r="38"/>
@@ -929,7 +929,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="41">
@@ -940,7 +940,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>826–828</t>
+          <t>829–831</t>
         </is>
       </c>
     </row>
@@ -952,7 +952,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>129.0 / 0.0 / 129.0</t>
+          <t>153.0 / 70.0 / 83.0</t>
         </is>
       </c>
     </row>
@@ -963,7 +963,7 @@
         </is>
       </c>
       <c r="B43" s="8" t="n">
-        <v>1</v>
+        <v>0.5424836601307189</v>
       </c>
     </row>
     <row r="44">
@@ -973,7 +973,7 @@
         </is>
       </c>
       <c r="B44" s="4" t="n">
-        <v>109781.9000747609</v>
+        <v>107265.1143798644</v>
       </c>
     </row>
     <row r="45"/>
@@ -1255,7 +1255,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E568"/>
+  <dimension ref="A1:E595"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -13199,8 +13199,575 @@
         <v>1199320.77</v>
       </c>
     </row>
+    <row r="569">
+      <c r="A569" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B569" s="15" t="n">
+        <v>831</v>
+      </c>
+      <c r="C569" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D569" s="16" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="E569" s="18" t="n">
+        <v>3238757.69</v>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B570" s="10" t="n">
+        <v>831</v>
+      </c>
+      <c r="C570" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D570" s="11" t="inlineStr">
+        <is>
+          <t>nicetry</t>
+        </is>
+      </c>
+      <c r="E570" s="14" t="n">
+        <v>2439265.29</v>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B571" s="15" t="n">
+        <v>831</v>
+      </c>
+      <c r="C571" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D571" s="16" t="inlineStr">
+        <is>
+          <t>montesquieu</t>
+        </is>
+      </c>
+      <c r="E571" s="18" t="n">
+        <v>2427977.68</v>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B572" s="10" t="n">
+        <v>831</v>
+      </c>
+      <c r="C572" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D572" s="11" t="inlineStr">
+        <is>
+          <t>group9</t>
+        </is>
+      </c>
+      <c r="E572" s="14" t="n">
+        <v>2220051.36</v>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B573" s="15" t="n">
+        <v>831</v>
+      </c>
+      <c r="C573" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="D573" s="16" t="inlineStr">
+        <is>
+          <t>group2</t>
+        </is>
+      </c>
+      <c r="E573" s="18" t="n">
+        <v>2171047.24</v>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B574" s="10" t="n">
+        <v>831</v>
+      </c>
+      <c r="C574" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="D574" s="11" t="inlineStr">
+        <is>
+          <t>group25</t>
+        </is>
+      </c>
+      <c r="E574" s="14" t="n">
+        <v>2170889.78</v>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B575" s="15" t="n">
+        <v>831</v>
+      </c>
+      <c r="C575" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="D575" s="16" t="inlineStr">
+        <is>
+          <t>group11</t>
+        </is>
+      </c>
+      <c r="E575" s="18" t="n">
+        <v>2170877.52</v>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B576" s="10" t="n">
+        <v>831</v>
+      </c>
+      <c r="C576" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="D576" s="11" t="inlineStr">
+        <is>
+          <t>88888888</t>
+        </is>
+      </c>
+      <c r="E576" s="14" t="n">
+        <v>2170854.93</v>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B577" s="15" t="n">
+        <v>831</v>
+      </c>
+      <c r="C577" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="D577" s="16" t="inlineStr">
+        <is>
+          <t>teamhlly</t>
+        </is>
+      </c>
+      <c r="E577" s="18" t="n">
+        <v>2124675.24</v>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B578" s="10" t="n">
+        <v>831</v>
+      </c>
+      <c r="C578" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="D578" s="11" t="inlineStr">
+        <is>
+          <t>tigagroup20</t>
+        </is>
+      </c>
+      <c r="E578" s="14" t="n">
+        <v>2117062.3</v>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B579" s="15" t="n">
+        <v>831</v>
+      </c>
+      <c r="C579" s="15" t="n">
+        <v>11</v>
+      </c>
+      <c r="D579" s="16" t="inlineStr">
+        <is>
+          <t>t24</t>
+        </is>
+      </c>
+      <c r="E579" s="18" t="n">
+        <v>2066450.8</v>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B580" s="10" t="n">
+        <v>831</v>
+      </c>
+      <c r="C580" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="D580" s="11" t="inlineStr">
+        <is>
+          <t>group7</t>
+        </is>
+      </c>
+      <c r="E580" s="14" t="n">
+        <v>2045485.07</v>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B581" s="15" t="n">
+        <v>831</v>
+      </c>
+      <c r="C581" s="15" t="n">
+        <v>13</v>
+      </c>
+      <c r="D581" s="16" t="inlineStr">
+        <is>
+          <t>666666</t>
+        </is>
+      </c>
+      <c r="E581" s="18" t="n">
+        <v>2016662.67</v>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B582" s="10" t="n">
+        <v>831</v>
+      </c>
+      <c r="C582" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="D582" s="11" t="inlineStr">
+        <is>
+          <t>group8</t>
+        </is>
+      </c>
+      <c r="E582" s="14" t="n">
+        <v>2006400.34</v>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B583" s="15" t="n">
+        <v>831</v>
+      </c>
+      <c r="C583" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="D583" s="16" t="inlineStr">
+        <is>
+          <t>jit</t>
+        </is>
+      </c>
+      <c r="E583" s="18" t="n">
+        <v>1968691.91</v>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B584" s="10" t="n">
+        <v>831</v>
+      </c>
+      <c r="C584" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="D584" s="11" t="inlineStr">
+        <is>
+          <t>deepsleep</t>
+        </is>
+      </c>
+      <c r="E584" s="14" t="n">
+        <v>1960754.51</v>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B585" s="15" t="n">
+        <v>831</v>
+      </c>
+      <c r="C585" s="15" t="n">
+        <v>17</v>
+      </c>
+      <c r="D585" s="16" t="inlineStr">
+        <is>
+          <t>group14</t>
+        </is>
+      </c>
+      <c r="E585" s="18" t="n">
+        <v>1927326.02</v>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B586" s="10" t="n">
+        <v>831</v>
+      </c>
+      <c r="C586" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="D586" s="11" t="inlineStr">
+        <is>
+          <t>group15</t>
+        </is>
+      </c>
+      <c r="E586" s="14" t="n">
+        <v>1886095.15</v>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B587" s="15" t="n">
+        <v>831</v>
+      </c>
+      <c r="C587" s="15" t="n">
+        <v>19</v>
+      </c>
+      <c r="D587" s="16" t="inlineStr">
+        <is>
+          <t>cleveregg</t>
+        </is>
+      </c>
+      <c r="E587" s="18" t="n">
+        <v>1862508.57</v>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B588" s="10" t="n">
+        <v>831</v>
+      </c>
+      <c r="C588" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="D588" s="11" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E588" s="14" t="n">
+        <v>1711474.32</v>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B589" s="15" t="n">
+        <v>831</v>
+      </c>
+      <c r="C589" s="15" t="n">
+        <v>21</v>
+      </c>
+      <c r="D589" s="16" t="inlineStr">
+        <is>
+          <t>vivo50</t>
+        </is>
+      </c>
+      <c r="E589" s="18" t="n">
+        <v>1611339.84</v>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B590" s="10" t="n">
+        <v>831</v>
+      </c>
+      <c r="C590" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="D590" s="11" t="inlineStr">
+        <is>
+          <t>group12</t>
+        </is>
+      </c>
+      <c r="E590" s="14" t="n">
+        <v>1537538.68</v>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B591" s="15" t="n">
+        <v>831</v>
+      </c>
+      <c r="C591" s="15" t="n">
+        <v>23</v>
+      </c>
+      <c r="D591" s="16" t="inlineStr">
+        <is>
+          <t>aaachemicalseller</t>
+        </is>
+      </c>
+      <c r="E591" s="18" t="n">
+        <v>1414592.05</v>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B592" s="10" t="n">
+        <v>831</v>
+      </c>
+      <c r="C592" s="10" t="n">
+        <v>24</v>
+      </c>
+      <c r="D592" s="11" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E592" s="14" t="n">
+        <v>1414507.95</v>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B593" s="24" t="n">
+        <v>831</v>
+      </c>
+      <c r="C593" s="24" t="n">
+        <v>25</v>
+      </c>
+      <c r="D593" s="25" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="E593" s="26" t="n">
+        <v>1357866.84</v>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B594" s="10" t="n">
+        <v>831</v>
+      </c>
+      <c r="C594" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="D594" s="11" t="inlineStr">
+        <is>
+          <t>newgroup18</t>
+        </is>
+      </c>
+      <c r="E594" s="14" t="n">
+        <v>1295695.57</v>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B595" s="15" t="n">
+        <v>831</v>
+      </c>
+      <c r="C595" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="D595" s="16" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="E595" s="18" t="n">
+        <v>1275617.69</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E568"/>
+  <autoFilter ref="A1:E595"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -30731,11 +31298,11 @@
         <v>831</v>
       </c>
       <c r="D278" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E278" s="11" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="F278" s="11" t="inlineStr">
@@ -30744,43 +31311,43 @@
         </is>
       </c>
       <c r="G278" s="12" t="n">
-        <v>72</v>
+        <v>153</v>
       </c>
       <c r="H278" s="12" t="n">
         <v>70</v>
       </c>
       <c r="I278" s="12" t="n">
-        <v>2</v>
+        <v>83</v>
       </c>
       <c r="J278" s="13" t="n">
-        <v>0.02777777777777778</v>
+        <v>0.5424836601307189</v>
       </c>
       <c r="K278" s="12" t="n">
-        <v>2</v>
+        <v>83</v>
       </c>
       <c r="L278" s="14" t="n">
-        <v>1232642.134839296</v>
+        <v>1250601.725620136</v>
       </c>
       <c r="M278" s="14" t="n">
-        <v>1232854.46</v>
+        <v>1357866.84</v>
       </c>
       <c r="N278" s="14" t="n">
-        <v>212.3251607038546</v>
+        <v>107265.1143798644</v>
       </c>
       <c r="O278" s="12" t="n">
-        <v>0</v>
+        <v>119</v>
       </c>
       <c r="P278" s="12" t="n">
-        <v>0</v>
+        <v>39.66666666666666</v>
       </c>
       <c r="Q278" s="12" t="n">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="R278" s="12" t="n">
         <v>200</v>
       </c>
       <c r="S278" s="14" t="n">
-        <v>2900</v>
+        <v>120350</v>
       </c>
     </row>
   </sheetData>
@@ -30795,7 +31362,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N831"/>
+  <dimension ref="A1:N832"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -69066,8 +69633,54 @@
         <v>0</v>
       </c>
     </row>
+    <row r="832">
+      <c r="A832" s="10" t="n">
+        <v>831</v>
+      </c>
+      <c r="B832" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C832" s="12" t="n">
+        <v>81</v>
+      </c>
+      <c r="D832" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E832" s="12" t="n">
+        <v>81</v>
+      </c>
+      <c r="F832" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G832" s="12" t="n">
+        <v>81</v>
+      </c>
+      <c r="H832" s="14" t="n">
+        <v>1357866.84</v>
+      </c>
+      <c r="I832" s="12" t="n">
+        <v>119</v>
+      </c>
+      <c r="J832" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K832" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="L832" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="M832" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N832" s="14" t="n">
+        <v>117450</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N831"/>
+  <autoFilter ref="A1:N832"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -69462,7 +70075,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -70575,8 +71188,56 @@
         <v>55</v>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" s="21" t="n">
+        <v>730.66</v>
+      </c>
+      <c r="B46" s="11" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C46" s="11" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D46" s="11" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E46" s="11" t="inlineStr"/>
+      <c r="F46" s="12" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="23" t="n">
+        <v>742.75</v>
+      </c>
+      <c r="B47" s="16" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C47" s="16" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D47" s="16" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E47" s="16" t="inlineStr"/>
+      <c r="F47" s="17" t="n">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F45"/>
+  <autoFilter ref="A1:F47"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -70975,7 +71636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U21"/>
+  <dimension ref="A1:U22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -70984,7 +71645,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
@@ -70997,7 +71658,7 @@
     <col width="12" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
-    <col width="22" customWidth="1" min="20" max="20"/>
+    <col width="21" customWidth="1" min="20" max="20"/>
     <col width="20" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
@@ -72512,8 +73173,79 @@
         <v>212.3251607038546</v>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="n">
+        <v>831</v>
+      </c>
+      <c r="C22" s="14" t="n">
+        <v>1357866.84</v>
+      </c>
+      <c r="D22" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="E22" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="F22" s="11" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="G22" s="14" t="n">
+        <v>1880890.85</v>
+      </c>
+      <c r="H22" s="21" t="n">
+        <v>40</v>
+      </c>
+      <c r="I22" s="21" t="n">
+        <v>55</v>
+      </c>
+      <c r="J22" s="11" t="inlineStr">
+        <is>
+          <t>mail</t>
+        </is>
+      </c>
+      <c r="K22" s="22" t="n">
+        <v>3600</v>
+      </c>
+      <c r="L22" s="22" t="n">
+        <v>200</v>
+      </c>
+      <c r="M22" s="12" t="n">
+        <v>119</v>
+      </c>
+      <c r="N22" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="O22" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="P22" s="10" t="n">
+        <v>277</v>
+      </c>
+      <c r="Q22" s="12" t="n">
+        <v>153</v>
+      </c>
+      <c r="R22" s="12" t="n">
+        <v>70</v>
+      </c>
+      <c r="S22" s="12" t="n">
+        <v>83</v>
+      </c>
+      <c r="T22" s="13" t="n">
+        <v>0.5424836601307189</v>
+      </c>
+      <c r="U22" s="14" t="n">
+        <v>107265.1143798644</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U21"/>
+  <autoFilter ref="A1:U22"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -72524,7 +73256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E253"/>
+  <dimension ref="A1:E265"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -78273,8 +79005,280 @@
         </is>
       </c>
     </row>
+    <row r="254">
+      <c r="A254" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B254" s="10" t="n">
+        <v>831</v>
+      </c>
+      <c r="C254" s="11" t="inlineStr">
+        <is>
+          <t>Starting Cash</t>
+        </is>
+      </c>
+      <c r="D254" s="14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E254" s="11" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B255" s="15" t="n">
+        <v>831</v>
+      </c>
+      <c r="C255" s="16" t="inlineStr">
+        <is>
+          <t>Cash Sources</t>
+        </is>
+      </c>
+      <c r="D255" s="16" t="n"/>
+      <c r="E255" s="16" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B256" s="10" t="n">
+        <v>831</v>
+      </c>
+      <c r="C256" s="11" t="inlineStr">
+        <is>
+          <t>revenues</t>
+        </is>
+      </c>
+      <c r="D256" s="14" t="n">
+        <v>21816700</v>
+      </c>
+      <c r="E256" s="11" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B257" s="15" t="n">
+        <v>831</v>
+      </c>
+      <c r="C257" s="16" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D257" s="18" t="n">
+        <v>298880.37</v>
+      </c>
+      <c r="E257" s="16" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B258" s="10" t="n">
+        <v>831</v>
+      </c>
+      <c r="C258" s="11" t="inlineStr">
+        <is>
+          <t>Cash Uses</t>
+        </is>
+      </c>
+      <c r="D258" s="11" t="n"/>
+      <c r="E258" s="11" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B259" s="15" t="n">
+        <v>831</v>
+      </c>
+      <c r="C259" s="16" t="inlineStr">
+        <is>
+          <t>outbound shipping</t>
+        </is>
+      </c>
+      <c r="D259" s="18" t="n">
+        <v>-2256900</v>
+      </c>
+      <c r="E259" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B260" s="10" t="n">
+        <v>831</v>
+      </c>
+      <c r="C260" s="11" t="inlineStr">
+        <is>
+          <t>inbound shipping</t>
+        </is>
+      </c>
+      <c r="D260" s="14" t="n">
+        <v>-1500000</v>
+      </c>
+      <c r="E260" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B261" s="15" t="n">
+        <v>831</v>
+      </c>
+      <c r="C261" s="16" t="inlineStr">
+        <is>
+          <t>FGI holding</t>
+        </is>
+      </c>
+      <c r="D261" s="18" t="n">
+        <v>-21808.28</v>
+      </c>
+      <c r="E261" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B262" s="10" t="n">
+        <v>831</v>
+      </c>
+      <c r="C262" s="11" t="inlineStr">
+        <is>
+          <t>add capacity</t>
+        </is>
+      </c>
+      <c r="D262" s="14" t="n">
+        <v>-1749840.87</v>
+      </c>
+      <c r="E262" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B263" s="15" t="n">
+        <v>831</v>
+      </c>
+      <c r="C263" s="16" t="inlineStr">
+        <is>
+          <t>Pipeline inventory holding</t>
+        </is>
+      </c>
+      <c r="D263" s="18" t="n">
+        <v>-29164.38</v>
+      </c>
+      <c r="E263" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B264" s="10" t="n">
+        <v>831</v>
+      </c>
+      <c r="C264" s="11" t="inlineStr">
+        <is>
+          <t>production</t>
+        </is>
+      </c>
+      <c r="D264" s="14" t="n">
+        <v>-15700000</v>
+      </c>
+      <c r="E264" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B265" s="15" t="n">
+        <v>831</v>
+      </c>
+      <c r="C265" s="16" t="inlineStr">
+        <is>
+          <t>Cash Balance</t>
+        </is>
+      </c>
+      <c r="D265" s="18" t="n">
+        <v>1357866.84</v>
+      </c>
+      <c r="E265" s="16" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E253"/>
+  <autoFilter ref="A1:E265"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update game data: day 832, cash 1412740.4, 3-day period 278
</commit_message>
<xml_diff>
--- a/data/supply_chain_game.xlsx
+++ b/data/supply_chain_game.xlsx
@@ -20,16 +20,16 @@
     <sheet name="排行榜" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$278</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$832</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$279</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$833</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'资金构成_旧版'!$A$1:$C$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'运营参数_旧版'!$A$9:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$49</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'排行榜_旧版'!$A$1:$C$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$265</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$277</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'运营参数'!$A$1:$J$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$595</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$622</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -590,7 +590,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-06T12:11:03+08:00</t>
+          <t>2026-09-06T12:26:02+08:00</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>831</v>
+        <v>832</v>
       </c>
     </row>
     <row r="7">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>629</v>
+        <v>628</v>
       </c>
     </row>
     <row r="8">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>1357866.84</v>
+        <v>1412740.4</v>
       </c>
     </row>
     <row r="11">
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>1880890.85</v>
+        <v>1811141.08</v>
       </c>
     </row>
     <row r="15"/>
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>119</v>
+        <v>87</v>
       </c>
     </row>
     <row r="25">
@@ -827,7 +827,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="30">
@@ -838,7 +838,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>829–831</t>
+          <t>832–834</t>
         </is>
       </c>
     </row>
@@ -850,7 +850,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否（进行中）</t>
         </is>
       </c>
     </row>
@@ -861,7 +861,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>153</v>
+        <v>32</v>
       </c>
     </row>
     <row r="33">
@@ -871,7 +871,7 @@
         </is>
       </c>
       <c r="B33" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -881,7 +881,7 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>83</v>
+        <v>32</v>
       </c>
     </row>
     <row r="35">
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B35" s="8" t="n">
-        <v>0.5424836601307189</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36">
@@ -901,7 +901,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>83</v>
+        <v>32</v>
       </c>
     </row>
     <row r="37">
@@ -909,9 +909,6 @@
         <is>
           <t>周期现金变动</t>
         </is>
-      </c>
-      <c r="B37" s="4" t="n">
-        <v>107265.1143798644</v>
       </c>
     </row>
     <row r="38"/>
@@ -973,7 +970,7 @@
         </is>
       </c>
       <c r="B44" s="4" t="n">
-        <v>107265.1143798644</v>
+        <v>108214.1651679503</v>
       </c>
     </row>
     <row r="45"/>
@@ -1255,7 +1252,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E595"/>
+  <dimension ref="A1:E622"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -13766,8 +13763,575 @@
         <v>1275617.69</v>
       </c>
     </row>
+    <row r="596">
+      <c r="A596" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B596" s="10" t="n">
+        <v>832</v>
+      </c>
+      <c r="C596" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D596" s="11" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="E596" s="14" t="n">
+        <v>3223881.48</v>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B597" s="15" t="n">
+        <v>832</v>
+      </c>
+      <c r="C597" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D597" s="16" t="inlineStr">
+        <is>
+          <t>montesquieu</t>
+        </is>
+      </c>
+      <c r="E597" s="18" t="n">
+        <v>2483140.58</v>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B598" s="10" t="n">
+        <v>832</v>
+      </c>
+      <c r="C598" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D598" s="11" t="inlineStr">
+        <is>
+          <t>nicetry</t>
+        </is>
+      </c>
+      <c r="E598" s="14" t="n">
+        <v>2439847.53</v>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B599" s="15" t="n">
+        <v>832</v>
+      </c>
+      <c r="C599" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D599" s="16" t="inlineStr">
+        <is>
+          <t>group2</t>
+        </is>
+      </c>
+      <c r="E599" s="18" t="n">
+        <v>2226143.04</v>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B600" s="10" t="n">
+        <v>832</v>
+      </c>
+      <c r="C600" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="D600" s="11" t="inlineStr">
+        <is>
+          <t>group25</t>
+        </is>
+      </c>
+      <c r="E600" s="14" t="n">
+        <v>2225985.54</v>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B601" s="15" t="n">
+        <v>832</v>
+      </c>
+      <c r="C601" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="D601" s="16" t="inlineStr">
+        <is>
+          <t>group11</t>
+        </is>
+      </c>
+      <c r="E601" s="18" t="n">
+        <v>2225973.27</v>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B602" s="10" t="n">
+        <v>832</v>
+      </c>
+      <c r="C602" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="D602" s="11" t="inlineStr">
+        <is>
+          <t>88888888</t>
+        </is>
+      </c>
+      <c r="E602" s="14" t="n">
+        <v>2225950.68</v>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B603" s="15" t="n">
+        <v>832</v>
+      </c>
+      <c r="C603" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="D603" s="16" t="inlineStr">
+        <is>
+          <t>group9</t>
+        </is>
+      </c>
+      <c r="E603" s="18" t="n">
+        <v>2220576.35</v>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B604" s="10" t="n">
+        <v>832</v>
+      </c>
+      <c r="C604" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="D604" s="11" t="inlineStr">
+        <is>
+          <t>teamhlly</t>
+        </is>
+      </c>
+      <c r="E604" s="14" t="n">
+        <v>2179749.06</v>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B605" s="15" t="n">
+        <v>832</v>
+      </c>
+      <c r="C605" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="D605" s="16" t="inlineStr">
+        <is>
+          <t>tigagroup20</t>
+        </is>
+      </c>
+      <c r="E605" s="18" t="n">
+        <v>2117615.19</v>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B606" s="10" t="n">
+        <v>832</v>
+      </c>
+      <c r="C606" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="D606" s="11" t="inlineStr">
+        <is>
+          <t>666666</t>
+        </is>
+      </c>
+      <c r="E606" s="14" t="n">
+        <v>2071718.15</v>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B607" s="15" t="n">
+        <v>832</v>
+      </c>
+      <c r="C607" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="D607" s="16" t="inlineStr">
+        <is>
+          <t>t24</t>
+        </is>
+      </c>
+      <c r="E607" s="18" t="n">
+        <v>2066935.67</v>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B608" s="10" t="n">
+        <v>832</v>
+      </c>
+      <c r="C608" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="D608" s="11" t="inlineStr">
+        <is>
+          <t>group8</t>
+        </is>
+      </c>
+      <c r="E608" s="14" t="n">
+        <v>2006869.53</v>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B609" s="15" t="n">
+        <v>832</v>
+      </c>
+      <c r="C609" s="15" t="n">
+        <v>14</v>
+      </c>
+      <c r="D609" s="16" t="inlineStr">
+        <is>
+          <t>group14</t>
+        </is>
+      </c>
+      <c r="E609" s="18" t="n">
+        <v>2001821.75</v>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B610" s="10" t="n">
+        <v>832</v>
+      </c>
+      <c r="C610" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="D610" s="11" t="inlineStr">
+        <is>
+          <t>jit</t>
+        </is>
+      </c>
+      <c r="E610" s="14" t="n">
+        <v>1969206.05</v>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B611" s="15" t="n">
+        <v>832</v>
+      </c>
+      <c r="C611" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="D611" s="16" t="inlineStr">
+        <is>
+          <t>group15</t>
+        </is>
+      </c>
+      <c r="E611" s="18" t="n">
+        <v>1968381.79</v>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B612" s="10" t="n">
+        <v>832</v>
+      </c>
+      <c r="C612" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="D612" s="11" t="inlineStr">
+        <is>
+          <t>group7</t>
+        </is>
+      </c>
+      <c r="E612" s="14" t="n">
+        <v>1765243.19</v>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B613" s="15" t="n">
+        <v>832</v>
+      </c>
+      <c r="C613" s="15" t="n">
+        <v>18</v>
+      </c>
+      <c r="D613" s="16" t="inlineStr">
+        <is>
+          <t>deepsleep</t>
+        </is>
+      </c>
+      <c r="E613" s="18" t="n">
+        <v>1764714.12</v>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B614" s="10" t="n">
+        <v>832</v>
+      </c>
+      <c r="C614" s="10" t="n">
+        <v>19</v>
+      </c>
+      <c r="D614" s="11" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E614" s="14" t="n">
+        <v>1711866.49</v>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B615" s="15" t="n">
+        <v>832</v>
+      </c>
+      <c r="C615" s="15" t="n">
+        <v>20</v>
+      </c>
+      <c r="D615" s="16" t="inlineStr">
+        <is>
+          <t>cleveregg</t>
+        </is>
+      </c>
+      <c r="E615" s="18" t="n">
+        <v>1701003.07</v>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B616" s="10" t="n">
+        <v>832</v>
+      </c>
+      <c r="C616" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="D616" s="11" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E616" s="14" t="n">
+        <v>1488867.77</v>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B617" s="15" t="n">
+        <v>832</v>
+      </c>
+      <c r="C617" s="15" t="n">
+        <v>22</v>
+      </c>
+      <c r="D617" s="16" t="inlineStr">
+        <is>
+          <t>vivo50</t>
+        </is>
+      </c>
+      <c r="E617" s="18" t="n">
+        <v>1449776.13</v>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B618" s="10" t="n">
+        <v>832</v>
+      </c>
+      <c r="C618" s="10" t="n">
+        <v>23</v>
+      </c>
+      <c r="D618" s="11" t="inlineStr">
+        <is>
+          <t>aaachemicalseller</t>
+        </is>
+      </c>
+      <c r="E618" s="14" t="n">
+        <v>1414851.89</v>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B619" s="24" t="n">
+        <v>832</v>
+      </c>
+      <c r="C619" s="24" t="n">
+        <v>24</v>
+      </c>
+      <c r="D619" s="25" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="E619" s="26" t="n">
+        <v>1412740.4</v>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B620" s="10" t="n">
+        <v>832</v>
+      </c>
+      <c r="C620" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="D620" s="11" t="inlineStr">
+        <is>
+          <t>group12</t>
+        </is>
+      </c>
+      <c r="E620" s="14" t="n">
+        <v>1375955.69</v>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B621" s="15" t="n">
+        <v>832</v>
+      </c>
+      <c r="C621" s="15" t="n">
+        <v>26</v>
+      </c>
+      <c r="D621" s="16" t="inlineStr">
+        <is>
+          <t>newgroup18</t>
+        </is>
+      </c>
+      <c r="E621" s="18" t="n">
+        <v>1350472.9</v>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B622" s="10" t="n">
+        <v>832</v>
+      </c>
+      <c r="C622" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="D622" s="11" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="E622" s="14" t="n">
+        <v>1275950.82</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E595"/>
+  <autoFilter ref="A1:E622"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -13778,7 +14342,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S278"/>
+  <dimension ref="A1:S279"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -31350,8 +31914,69 @@
         <v>120350</v>
       </c>
     </row>
+    <row r="279">
+      <c r="A279" s="15" t="n">
+        <v>278</v>
+      </c>
+      <c r="B279" s="15" t="n">
+        <v>832</v>
+      </c>
+      <c r="C279" s="15" t="n">
+        <v>834</v>
+      </c>
+      <c r="D279" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E279" s="16" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="F279" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G279" s="17" t="n">
+        <v>32</v>
+      </c>
+      <c r="H279" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I279" s="17" t="n">
+        <v>32</v>
+      </c>
+      <c r="J279" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K279" s="17" t="n">
+        <v>32</v>
+      </c>
+      <c r="L279" s="18" t="n">
+        <v>1412740.4</v>
+      </c>
+      <c r="M279" s="18" t="n">
+        <v>1412740.4</v>
+      </c>
+      <c r="N279" s="16" t="n"/>
+      <c r="O279" s="17" t="n">
+        <v>87</v>
+      </c>
+      <c r="P279" s="17" t="n">
+        <v>87</v>
+      </c>
+      <c r="Q279" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="R279" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="S279" s="18" t="n">
+        <v>46400</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S278"/>
+  <autoFilter ref="A1:S279"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -31362,7 +31987,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N832"/>
+  <dimension ref="A1:N833"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -69679,8 +70304,54 @@
         <v>117450</v>
       </c>
     </row>
+    <row r="833">
+      <c r="A833" s="15" t="n">
+        <v>832</v>
+      </c>
+      <c r="B833" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C833" s="17" t="n">
+        <v>32</v>
+      </c>
+      <c r="D833" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E833" s="17" t="n">
+        <v>32</v>
+      </c>
+      <c r="F833" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G833" s="17" t="n">
+        <v>32</v>
+      </c>
+      <c r="H833" s="18" t="n">
+        <v>1412740.4</v>
+      </c>
+      <c r="I833" s="17" t="n">
+        <v>87</v>
+      </c>
+      <c r="J833" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K833" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="L833" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="M833" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N833" s="18" t="n">
+        <v>46400</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N832"/>
+  <autoFilter ref="A1:N833"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -70075,7 +70746,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -71236,8 +71907,56 @@
         <v>55</v>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" s="21" t="n">
+        <v>730.66</v>
+      </c>
+      <c r="B48" s="11" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C48" s="11" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D48" s="11" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E48" s="11" t="inlineStr"/>
+      <c r="F48" s="12" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="23" t="n">
+        <v>742.75</v>
+      </c>
+      <c r="B49" s="16" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C49" s="16" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D49" s="16" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E49" s="16" t="inlineStr"/>
+      <c r="F49" s="17" t="n">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F47"/>
+  <autoFilter ref="A1:F49"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -71636,7 +72355,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U22"/>
+  <dimension ref="A1:U23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -71645,7 +72364,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
@@ -73244,8 +73963,77 @@
         <v>107265.1143798644</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B23" s="15" t="n">
+        <v>832</v>
+      </c>
+      <c r="C23" s="18" t="n">
+        <v>1412740.4</v>
+      </c>
+      <c r="D23" s="15" t="n">
+        <v>24</v>
+      </c>
+      <c r="E23" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="F23" s="16" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="G23" s="18" t="n">
+        <v>1811141.08</v>
+      </c>
+      <c r="H23" s="23" t="n">
+        <v>40</v>
+      </c>
+      <c r="I23" s="23" t="n">
+        <v>55</v>
+      </c>
+      <c r="J23" s="16" t="inlineStr">
+        <is>
+          <t>mail</t>
+        </is>
+      </c>
+      <c r="K23" s="27" t="n">
+        <v>3600</v>
+      </c>
+      <c r="L23" s="27" t="n">
+        <v>200</v>
+      </c>
+      <c r="M23" s="17" t="n">
+        <v>87</v>
+      </c>
+      <c r="N23" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="O23" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="P23" s="15" t="n">
+        <v>278</v>
+      </c>
+      <c r="Q23" s="17" t="n">
+        <v>32</v>
+      </c>
+      <c r="R23" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="S23" s="17" t="n">
+        <v>32</v>
+      </c>
+      <c r="T23" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="U23" s="16" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U22"/>
+  <autoFilter ref="A1:U23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -73256,7 +74044,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E265"/>
+  <dimension ref="A1:E277"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -79277,8 +80065,280 @@
         </is>
       </c>
     </row>
+    <row r="266">
+      <c r="A266" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B266" s="10" t="n">
+        <v>832</v>
+      </c>
+      <c r="C266" s="11" t="inlineStr">
+        <is>
+          <t>Starting Cash</t>
+        </is>
+      </c>
+      <c r="D266" s="14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E266" s="11" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B267" s="15" t="n">
+        <v>832</v>
+      </c>
+      <c r="C267" s="16" t="inlineStr">
+        <is>
+          <t>Cash Sources</t>
+        </is>
+      </c>
+      <c r="D267" s="16" t="n"/>
+      <c r="E267" s="16" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B268" s="10" t="n">
+        <v>832</v>
+      </c>
+      <c r="C268" s="11" t="inlineStr">
+        <is>
+          <t>revenues</t>
+        </is>
+      </c>
+      <c r="D268" s="14" t="n">
+        <v>21877600</v>
+      </c>
+      <c r="E268" s="11" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B269" s="15" t="n">
+        <v>832</v>
+      </c>
+      <c r="C269" s="16" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D269" s="18" t="n">
+        <v>299236.23</v>
+      </c>
+      <c r="E269" s="16" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B270" s="10" t="n">
+        <v>832</v>
+      </c>
+      <c r="C270" s="11" t="inlineStr">
+        <is>
+          <t>Cash Uses</t>
+        </is>
+      </c>
+      <c r="D270" s="11" t="n"/>
+      <c r="E270" s="11" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B271" s="15" t="n">
+        <v>832</v>
+      </c>
+      <c r="C271" s="16" t="inlineStr">
+        <is>
+          <t>outbound shipping</t>
+        </is>
+      </c>
+      <c r="D271" s="18" t="n">
+        <v>-2263200</v>
+      </c>
+      <c r="E271" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B272" s="10" t="n">
+        <v>832</v>
+      </c>
+      <c r="C272" s="11" t="inlineStr">
+        <is>
+          <t>inbound shipping</t>
+        </is>
+      </c>
+      <c r="D272" s="14" t="n">
+        <v>-1500000</v>
+      </c>
+      <c r="E272" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B273" s="15" t="n">
+        <v>832</v>
+      </c>
+      <c r="C273" s="16" t="inlineStr">
+        <is>
+          <t>FGI holding</t>
+        </is>
+      </c>
+      <c r="D273" s="18" t="n">
+        <v>-21835.78</v>
+      </c>
+      <c r="E273" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B274" s="10" t="n">
+        <v>832</v>
+      </c>
+      <c r="C274" s="11" t="inlineStr">
+        <is>
+          <t>add capacity</t>
+        </is>
+      </c>
+      <c r="D274" s="14" t="n">
+        <v>-1749840.87</v>
+      </c>
+      <c r="E274" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B275" s="15" t="n">
+        <v>832</v>
+      </c>
+      <c r="C275" s="16" t="inlineStr">
+        <is>
+          <t>Pipeline inventory holding</t>
+        </is>
+      </c>
+      <c r="D275" s="18" t="n">
+        <v>-29219.18</v>
+      </c>
+      <c r="E275" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B276" s="10" t="n">
+        <v>832</v>
+      </c>
+      <c r="C276" s="11" t="inlineStr">
+        <is>
+          <t>production</t>
+        </is>
+      </c>
+      <c r="D276" s="14" t="n">
+        <v>-15700000</v>
+      </c>
+      <c r="E276" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B277" s="15" t="n">
+        <v>832</v>
+      </c>
+      <c r="C277" s="16" t="inlineStr">
+        <is>
+          <t>Cash Balance</t>
+        </is>
+      </c>
+      <c r="D277" s="18" t="n">
+        <v>1412740.4</v>
+      </c>
+      <c r="E277" s="16" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E265"/>
+  <autoFilter ref="A1:E277"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update game data: day 833, cash 1493645.2, 3-day period 278
</commit_message>
<xml_diff>
--- a/data/supply_chain_game.xlsx
+++ b/data/supply_chain_game.xlsx
@@ -21,15 +21,15 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$279</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$833</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$834</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'资金构成_旧版'!$A$1:$C$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'运营参数_旧版'!$A$9:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'排行榜_旧版'!$A$1:$C$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$23</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$277</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'运营参数'!$A$1:$J$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$622</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$289</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'运营参数'!$A$1:$J$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$649</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -590,7 +590,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-06T12:26:02+08:00</t>
+          <t>2026-09-06T12:41:03+08:00</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>832</v>
+        <v>833</v>
       </c>
     </row>
     <row r="7">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="8">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>1412740.4</v>
+        <v>1493645.2</v>
       </c>
     </row>
     <row r="11">
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="12">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>1811141.08</v>
+        <v>1775234.97</v>
       </c>
     </row>
     <row r="15"/>
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="B18" s="6" t="n">
-        <v>40</v>
+        <v>55</v>
       </c>
     </row>
     <row r="19">
@@ -734,9 +734,6 @@
           <t>计划产能 (鼓/日)</t>
         </is>
       </c>
-      <c r="B19" s="6" t="n">
-        <v>55</v>
-      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -789,7 +786,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>87</v>
+        <v>24</v>
       </c>
     </row>
     <row r="25">
@@ -861,7 +858,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>32</v>
+        <v>95</v>
       </c>
     </row>
     <row r="33">
@@ -881,7 +878,7 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>32</v>
+        <v>95</v>
       </c>
     </row>
     <row r="35">
@@ -901,7 +898,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>32</v>
+        <v>95</v>
       </c>
     </row>
     <row r="37">
@@ -909,6 +906,9 @@
         <is>
           <t>周期现金变动</t>
         </is>
+      </c>
+      <c r="B37" s="4" t="n">
+        <v>83958.56230855989</v>
       </c>
     </row>
     <row r="38"/>
@@ -970,7 +970,7 @@
         </is>
       </c>
       <c r="B44" s="4" t="n">
-        <v>108214.1651679503</v>
+        <v>107980.250756752</v>
       </c>
     </row>
     <row r="45"/>
@@ -1005,7 +1005,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1240,8 +1240,48 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="n">
+        <v>833</v>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="D6" s="21" t="n">
+        <v>55</v>
+      </c>
+      <c r="E6" s="11" t="n"/>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>mail</t>
+        </is>
+      </c>
+      <c r="G6" s="22" t="n">
+        <v>3600</v>
+      </c>
+      <c r="H6" s="22" t="n">
+        <v>200</v>
+      </c>
+      <c r="I6" s="11" t="inlineStr">
+        <is>
+          <t>mail</t>
+        </is>
+      </c>
+      <c r="J6" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J5"/>
+  <autoFilter ref="A1:J6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1252,7 +1292,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E622"/>
+  <dimension ref="A1:E649"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -14330,8 +14370,575 @@
         <v>1275950.82</v>
       </c>
     </row>
+    <row r="623">
+      <c r="A623" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B623" s="15" t="n">
+        <v>833</v>
+      </c>
+      <c r="C623" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D623" s="16" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="E623" s="18" t="n">
+        <v>3268880.17</v>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B624" s="10" t="n">
+        <v>833</v>
+      </c>
+      <c r="C624" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D624" s="11" t="inlineStr">
+        <is>
+          <t>montesquieu</t>
+        </is>
+      </c>
+      <c r="E624" s="14" t="n">
+        <v>2517532.37</v>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B625" s="15" t="n">
+        <v>833</v>
+      </c>
+      <c r="C625" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D625" s="16" t="inlineStr">
+        <is>
+          <t>nicetry</t>
+        </is>
+      </c>
+      <c r="E625" s="18" t="n">
+        <v>2440429.92</v>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B626" s="10" t="n">
+        <v>833</v>
+      </c>
+      <c r="C626" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D626" s="11" t="inlineStr">
+        <is>
+          <t>teamhlly</t>
+        </is>
+      </c>
+      <c r="E626" s="14" t="n">
+        <v>2260854.17</v>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B627" s="15" t="n">
+        <v>833</v>
+      </c>
+      <c r="C627" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="D627" s="16" t="inlineStr">
+        <is>
+          <t>group9</t>
+        </is>
+      </c>
+      <c r="E627" s="18" t="n">
+        <v>2221101.47</v>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B628" s="10" t="n">
+        <v>833</v>
+      </c>
+      <c r="C628" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="D628" s="11" t="inlineStr">
+        <is>
+          <t>group14</t>
+        </is>
+      </c>
+      <c r="E628" s="14" t="n">
+        <v>2101058.19</v>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B629" s="15" t="n">
+        <v>833</v>
+      </c>
+      <c r="C629" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="D629" s="16" t="inlineStr">
+        <is>
+          <t>group15</t>
+        </is>
+      </c>
+      <c r="E629" s="18" t="n">
+        <v>2067611.15</v>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B630" s="10" t="n">
+        <v>833</v>
+      </c>
+      <c r="C630" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="D630" s="11" t="inlineStr">
+        <is>
+          <t>t24</t>
+        </is>
+      </c>
+      <c r="E630" s="14" t="n">
+        <v>2067420.67</v>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B631" s="15" t="n">
+        <v>833</v>
+      </c>
+      <c r="C631" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="D631" s="16" t="inlineStr">
+        <is>
+          <t>group2</t>
+        </is>
+      </c>
+      <c r="E631" s="18" t="n">
+        <v>2043967.72</v>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B632" s="10" t="n">
+        <v>833</v>
+      </c>
+      <c r="C632" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="D632" s="11" t="inlineStr">
+        <is>
+          <t>group25</t>
+        </is>
+      </c>
+      <c r="E632" s="14" t="n">
+        <v>2043810.17</v>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B633" s="15" t="n">
+        <v>833</v>
+      </c>
+      <c r="C633" s="15" t="n">
+        <v>11</v>
+      </c>
+      <c r="D633" s="16" t="inlineStr">
+        <is>
+          <t>group11</t>
+        </is>
+      </c>
+      <c r="E633" s="18" t="n">
+        <v>2043797.9</v>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B634" s="10" t="n">
+        <v>833</v>
+      </c>
+      <c r="C634" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="D634" s="11" t="inlineStr">
+        <is>
+          <t>88888888</t>
+        </is>
+      </c>
+      <c r="E634" s="14" t="n">
+        <v>2043775.3</v>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B635" s="15" t="n">
+        <v>833</v>
+      </c>
+      <c r="C635" s="15" t="n">
+        <v>13</v>
+      </c>
+      <c r="D635" s="16" t="inlineStr">
+        <is>
+          <t>group8</t>
+        </is>
+      </c>
+      <c r="E635" s="18" t="n">
+        <v>2007338.85</v>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B636" s="10" t="n">
+        <v>833</v>
+      </c>
+      <c r="C636" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="D636" s="11" t="inlineStr">
+        <is>
+          <t>666666</t>
+        </is>
+      </c>
+      <c r="E636" s="14" t="n">
+        <v>1889437.96</v>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B637" s="15" t="n">
+        <v>833</v>
+      </c>
+      <c r="C637" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="D637" s="16" t="inlineStr">
+        <is>
+          <t>tigagroup20</t>
+        </is>
+      </c>
+      <c r="E637" s="18" t="n">
+        <v>1886668.22</v>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B638" s="10" t="n">
+        <v>833</v>
+      </c>
+      <c r="C638" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="D638" s="11" t="inlineStr">
+        <is>
+          <t>group7</t>
+        </is>
+      </c>
+      <c r="E638" s="14" t="n">
+        <v>1809819.86</v>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B639" s="15" t="n">
+        <v>833</v>
+      </c>
+      <c r="C639" s="15" t="n">
+        <v>17</v>
+      </c>
+      <c r="D639" s="16" t="inlineStr">
+        <is>
+          <t>deepsleep</t>
+        </is>
+      </c>
+      <c r="E639" s="18" t="n">
+        <v>1765076.36</v>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B640" s="10" t="n">
+        <v>833</v>
+      </c>
+      <c r="C640" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="D640" s="11" t="inlineStr">
+        <is>
+          <t>jit</t>
+        </is>
+      </c>
+      <c r="E640" s="14" t="n">
+        <v>1753220.32</v>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B641" s="15" t="n">
+        <v>833</v>
+      </c>
+      <c r="C641" s="15" t="n">
+        <v>19</v>
+      </c>
+      <c r="D641" s="16" t="inlineStr">
+        <is>
+          <t>cleveregg</t>
+        </is>
+      </c>
+      <c r="E641" s="18" t="n">
+        <v>1735135.81</v>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B642" s="10" t="n">
+        <v>833</v>
+      </c>
+      <c r="C642" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="D642" s="11" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E642" s="14" t="n">
+        <v>1712258.76</v>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B643" s="15" t="n">
+        <v>833</v>
+      </c>
+      <c r="C643" s="15" t="n">
+        <v>21</v>
+      </c>
+      <c r="D643" s="16" t="inlineStr">
+        <is>
+          <t>aaachemicalseller</t>
+        </is>
+      </c>
+      <c r="E643" s="18" t="n">
+        <v>1536011.8</v>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B644" s="10" t="n">
+        <v>833</v>
+      </c>
+      <c r="C644" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="D644" s="11" t="inlineStr">
+        <is>
+          <t>vivo50</t>
+        </is>
+      </c>
+      <c r="E644" s="14" t="n">
+        <v>1530635.8</v>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B645" s="24" t="n">
+        <v>833</v>
+      </c>
+      <c r="C645" s="24" t="n">
+        <v>23</v>
+      </c>
+      <c r="D645" s="25" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="E645" s="26" t="n">
+        <v>1493645.2</v>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B646" s="10" t="n">
+        <v>833</v>
+      </c>
+      <c r="C646" s="10" t="n">
+        <v>24</v>
+      </c>
+      <c r="D646" s="11" t="inlineStr">
+        <is>
+          <t>group12</t>
+        </is>
+      </c>
+      <c r="E646" s="14" t="n">
+        <v>1456796.08</v>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B647" s="15" t="n">
+        <v>833</v>
+      </c>
+      <c r="C647" s="15" t="n">
+        <v>25</v>
+      </c>
+      <c r="D647" s="16" t="inlineStr">
+        <is>
+          <t>newgroup18</t>
+        </is>
+      </c>
+      <c r="E647" s="18" t="n">
+        <v>1449481.43</v>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B648" s="10" t="n">
+        <v>833</v>
+      </c>
+      <c r="C648" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="D648" s="11" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E648" s="14" t="n">
+        <v>1371470.25</v>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B649" s="15" t="n">
+        <v>833</v>
+      </c>
+      <c r="C649" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="D649" s="16" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="E649" s="18" t="n">
+        <v>1102244.3</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E622"/>
+  <autoFilter ref="A1:E649"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -31925,7 +32532,7 @@
         <v>834</v>
       </c>
       <c r="D279" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E279" s="16" t="inlineStr">
         <is>
@@ -31938,32 +32545,34 @@
         </is>
       </c>
       <c r="G279" s="17" t="n">
-        <v>32</v>
+        <v>95</v>
       </c>
       <c r="H279" s="17" t="n">
         <v>0</v>
       </c>
       <c r="I279" s="17" t="n">
-        <v>32</v>
+        <v>95</v>
       </c>
       <c r="J279" s="19" t="n">
         <v>1</v>
       </c>
       <c r="K279" s="17" t="n">
-        <v>32</v>
+        <v>95</v>
       </c>
       <c r="L279" s="18" t="n">
-        <v>1412740.4</v>
+        <v>1409686.63769144</v>
       </c>
       <c r="M279" s="18" t="n">
-        <v>1412740.4</v>
-      </c>
-      <c r="N279" s="16" t="n"/>
+        <v>1493645.2</v>
+      </c>
+      <c r="N279" s="18" t="n">
+        <v>83958.56230855989</v>
+      </c>
       <c r="O279" s="17" t="n">
-        <v>87</v>
+        <v>24</v>
       </c>
       <c r="P279" s="17" t="n">
-        <v>87</v>
+        <v>55.5</v>
       </c>
       <c r="Q279" s="17" t="n">
         <v>200</v>
@@ -31972,7 +32581,7 @@
         <v>200</v>
       </c>
       <c r="S279" s="18" t="n">
-        <v>46400</v>
+        <v>137750</v>
       </c>
     </row>
   </sheetData>
@@ -31987,7 +32596,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N833"/>
+  <dimension ref="A1:N834"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -70350,8 +70959,54 @@
         <v>46400</v>
       </c>
     </row>
+    <row r="834">
+      <c r="A834" s="10" t="n">
+        <v>833</v>
+      </c>
+      <c r="B834" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C834" s="12" t="n">
+        <v>63</v>
+      </c>
+      <c r="D834" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E834" s="12" t="n">
+        <v>63</v>
+      </c>
+      <c r="F834" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G834" s="12" t="n">
+        <v>63</v>
+      </c>
+      <c r="H834" s="14" t="n">
+        <v>1493645.2</v>
+      </c>
+      <c r="I834" s="12" t="n">
+        <v>24</v>
+      </c>
+      <c r="J834" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K834" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="L834" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="M834" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N834" s="14" t="n">
+        <v>91350</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N833"/>
+  <autoFilter ref="A1:N834"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -70746,7 +71401,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -71955,8 +72610,56 @@
         <v>55</v>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" s="21" t="n">
+        <v>730.66</v>
+      </c>
+      <c r="B50" s="11" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C50" s="11" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D50" s="11" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E50" s="11" t="inlineStr"/>
+      <c r="F50" s="12" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="23" t="n">
+        <v>742.75</v>
+      </c>
+      <c r="B51" s="16" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C51" s="16" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D51" s="16" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E51" s="16" t="inlineStr"/>
+      <c r="F51" s="17" t="n">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F49"/>
+  <autoFilter ref="A1:F51"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -72355,7 +73058,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U23"/>
+  <dimension ref="A1:U24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -74032,8 +74735,77 @@
       </c>
       <c r="U23" s="16" t="n"/>
     </row>
+    <row r="24">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="n">
+        <v>833</v>
+      </c>
+      <c r="C24" s="14" t="n">
+        <v>1493645.2</v>
+      </c>
+      <c r="D24" s="10" t="n">
+        <v>23</v>
+      </c>
+      <c r="E24" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="G24" s="14" t="n">
+        <v>1775234.97</v>
+      </c>
+      <c r="H24" s="21" t="n">
+        <v>55</v>
+      </c>
+      <c r="I24" s="11" t="n"/>
+      <c r="J24" s="11" t="inlineStr">
+        <is>
+          <t>mail</t>
+        </is>
+      </c>
+      <c r="K24" s="22" t="n">
+        <v>3600</v>
+      </c>
+      <c r="L24" s="22" t="n">
+        <v>200</v>
+      </c>
+      <c r="M24" s="12" t="n">
+        <v>24</v>
+      </c>
+      <c r="N24" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="O24" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="P24" s="10" t="n">
+        <v>278</v>
+      </c>
+      <c r="Q24" s="12" t="n">
+        <v>95</v>
+      </c>
+      <c r="R24" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S24" s="12" t="n">
+        <v>95</v>
+      </c>
+      <c r="T24" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="U24" s="14" t="n">
+        <v>83958.56230855989</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U23"/>
+  <autoFilter ref="A1:U24"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -74044,7 +74816,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E277"/>
+  <dimension ref="A1:E289"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -80337,8 +81109,280 @@
         </is>
       </c>
     </row>
+    <row r="278">
+      <c r="A278" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B278" s="10" t="n">
+        <v>833</v>
+      </c>
+      <c r="C278" s="11" t="inlineStr">
+        <is>
+          <t>Starting Cash</t>
+        </is>
+      </c>
+      <c r="D278" s="14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E278" s="11" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B279" s="15" t="n">
+        <v>833</v>
+      </c>
+      <c r="C279" s="16" t="inlineStr">
+        <is>
+          <t>Cash Sources</t>
+        </is>
+      </c>
+      <c r="D279" s="16" t="n"/>
+      <c r="E279" s="16" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B280" s="10" t="n">
+        <v>833</v>
+      </c>
+      <c r="C280" s="11" t="inlineStr">
+        <is>
+          <t>revenues</t>
+        </is>
+      </c>
+      <c r="D280" s="14" t="n">
+        <v>21967500</v>
+      </c>
+      <c r="E280" s="11" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B281" s="15" t="n">
+        <v>833</v>
+      </c>
+      <c r="C281" s="16" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D281" s="18" t="n">
+        <v>299609.39</v>
+      </c>
+      <c r="E281" s="16" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B282" s="10" t="n">
+        <v>833</v>
+      </c>
+      <c r="C282" s="11" t="inlineStr">
+        <is>
+          <t>Cash Uses</t>
+        </is>
+      </c>
+      <c r="D282" s="11" t="n"/>
+      <c r="E282" s="11" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B283" s="15" t="n">
+        <v>833</v>
+      </c>
+      <c r="C283" s="16" t="inlineStr">
+        <is>
+          <t>outbound shipping</t>
+        </is>
+      </c>
+      <c r="D283" s="18" t="n">
+        <v>-2272500</v>
+      </c>
+      <c r="E283" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B284" s="10" t="n">
+        <v>833</v>
+      </c>
+      <c r="C284" s="11" t="inlineStr">
+        <is>
+          <t>inbound shipping</t>
+        </is>
+      </c>
+      <c r="D284" s="14" t="n">
+        <v>-1500000</v>
+      </c>
+      <c r="E284" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B285" s="15" t="n">
+        <v>833</v>
+      </c>
+      <c r="C285" s="16" t="inlineStr">
+        <is>
+          <t>FGI holding</t>
+        </is>
+      </c>
+      <c r="D285" s="18" t="n">
+        <v>-21849.36</v>
+      </c>
+      <c r="E285" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B286" s="10" t="n">
+        <v>833</v>
+      </c>
+      <c r="C286" s="11" t="inlineStr">
+        <is>
+          <t>add capacity</t>
+        </is>
+      </c>
+      <c r="D286" s="14" t="n">
+        <v>-1749840.87</v>
+      </c>
+      <c r="E286" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B287" s="15" t="n">
+        <v>833</v>
+      </c>
+      <c r="C287" s="16" t="inlineStr">
+        <is>
+          <t>Pipeline inventory holding</t>
+        </is>
+      </c>
+      <c r="D287" s="18" t="n">
+        <v>-29273.97</v>
+      </c>
+      <c r="E287" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B288" s="10" t="n">
+        <v>833</v>
+      </c>
+      <c r="C288" s="11" t="inlineStr">
+        <is>
+          <t>production</t>
+        </is>
+      </c>
+      <c r="D288" s="14" t="n">
+        <v>-15700000</v>
+      </c>
+      <c r="E288" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B289" s="15" t="n">
+        <v>833</v>
+      </c>
+      <c r="C289" s="16" t="inlineStr">
+        <is>
+          <t>Cash Balance</t>
+        </is>
+      </c>
+      <c r="D289" s="18" t="n">
+        <v>1493645.2</v>
+      </c>
+      <c r="E289" s="16" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E277"/>
+  <autoFilter ref="A1:E289"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update game data: day 834, cash 1262477.47, 3-day period 278
</commit_message>
<xml_diff>
--- a/data/supply_chain_game.xlsx
+++ b/data/supply_chain_game.xlsx
@@ -21,15 +21,15 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$279</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$834</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$835</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'资金构成_旧版'!$A$1:$C$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'运营参数_旧版'!$A$9:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$53</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'排行榜_旧版'!$A$1:$C$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$289</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$301</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'运营参数'!$A$1:$J$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$649</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$676</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -590,7 +590,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-06T12:41:03+08:00</t>
+          <t>2026-09-06T12:56:02+08:00</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>833</v>
+        <v>834</v>
       </c>
     </row>
     <row r="7">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>627</v>
+        <v>626</v>
       </c>
     </row>
     <row r="8">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>1493645.2</v>
+        <v>1262477.47</v>
       </c>
     </row>
     <row r="11">
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>1775234.97</v>
+        <v>2007215.3</v>
       </c>
     </row>
     <row r="15"/>
@@ -786,7 +786,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -796,7 +796,7 @@
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>200</v>
+        <v>400</v>
       </c>
     </row>
     <row r="26">
@@ -847,7 +847,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>否（进行中）</t>
+          <t>是</t>
         </is>
       </c>
     </row>
@@ -858,7 +858,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>95</v>
+        <v>150</v>
       </c>
     </row>
     <row r="33">
@@ -868,7 +868,7 @@
         </is>
       </c>
       <c r="B33" s="7" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
     </row>
     <row r="34">
@@ -878,7 +878,7 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>95</v>
+        <v>119</v>
       </c>
     </row>
     <row r="35">
@@ -888,7 +888,7 @@
         </is>
       </c>
       <c r="B35" s="8" t="n">
-        <v>1</v>
+        <v>0.7933333333333333</v>
       </c>
     </row>
     <row r="36">
@@ -898,7 +898,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>95</v>
+        <v>119</v>
       </c>
     </row>
     <row r="37">
@@ -908,7 +908,7 @@
         </is>
       </c>
       <c r="B37" s="4" t="n">
-        <v>83958.56230855989</v>
+        <v>-117762.9396656046</v>
       </c>
     </row>
     <row r="38"/>
@@ -926,7 +926,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="41">
@@ -937,7 +937,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>829–831</t>
+          <t>832–834</t>
         </is>
       </c>
     </row>
@@ -949,7 +949,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>153.0 / 70.0 / 83.0</t>
+          <t>150.0 / 31.0 / 119.0</t>
         </is>
       </c>
     </row>
@@ -960,7 +960,7 @@
         </is>
       </c>
       <c r="B43" s="8" t="n">
-        <v>0.5424836601307189</v>
+        <v>0.7933333333333333</v>
       </c>
     </row>
     <row r="44">
@@ -970,7 +970,7 @@
         </is>
       </c>
       <c r="B44" s="4" t="n">
-        <v>107980.250756752</v>
+        <v>-117762.9396656046</v>
       </c>
     </row>
     <row r="45"/>
@@ -1292,7 +1292,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E649"/>
+  <dimension ref="A1:E676"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -14937,8 +14937,575 @@
         <v>1102244.3</v>
       </c>
     </row>
+    <row r="650">
+      <c r="A650" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B650" s="10" t="n">
+        <v>834</v>
+      </c>
+      <c r="C650" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D650" s="11" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="E650" s="14" t="n">
+        <v>3269692.77</v>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B651" s="15" t="n">
+        <v>834</v>
+      </c>
+      <c r="C651" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D651" s="16" t="inlineStr">
+        <is>
+          <t>montesquieu</t>
+        </is>
+      </c>
+      <c r="E651" s="18" t="n">
+        <v>2301635.05</v>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B652" s="10" t="n">
+        <v>834</v>
+      </c>
+      <c r="C652" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D652" s="11" t="inlineStr">
+        <is>
+          <t>nicetry</t>
+        </is>
+      </c>
+      <c r="E652" s="14" t="n">
+        <v>2224483.9</v>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B653" s="15" t="n">
+        <v>834</v>
+      </c>
+      <c r="C653" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D653" s="16" t="inlineStr">
+        <is>
+          <t>group14</t>
+        </is>
+      </c>
+      <c r="E653" s="18" t="n">
+        <v>2165230.34</v>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B654" s="10" t="n">
+        <v>834</v>
+      </c>
+      <c r="C654" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="D654" s="11" t="inlineStr">
+        <is>
+          <t>group15</t>
+        </is>
+      </c>
+      <c r="E654" s="14" t="n">
+        <v>2131776.21</v>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B655" s="15" t="n">
+        <v>834</v>
+      </c>
+      <c r="C655" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="D655" s="16" t="inlineStr">
+        <is>
+          <t>teamhlly</t>
+        </is>
+      </c>
+      <c r="E655" s="18" t="n">
+        <v>2044883.31</v>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B656" s="10" t="n">
+        <v>834</v>
+      </c>
+      <c r="C656" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="D656" s="11" t="inlineStr">
+        <is>
+          <t>group2</t>
+        </is>
+      </c>
+      <c r="E656" s="14" t="n">
+        <v>2044405.23</v>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B657" s="15" t="n">
+        <v>834</v>
+      </c>
+      <c r="C657" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="D657" s="16" t="inlineStr">
+        <is>
+          <t>group25</t>
+        </is>
+      </c>
+      <c r="E657" s="18" t="n">
+        <v>2044247.64</v>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B658" s="10" t="n">
+        <v>834</v>
+      </c>
+      <c r="C658" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="D658" s="11" t="inlineStr">
+        <is>
+          <t>group11</t>
+        </is>
+      </c>
+      <c r="E658" s="14" t="n">
+        <v>2044235.37</v>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B659" s="15" t="n">
+        <v>834</v>
+      </c>
+      <c r="C659" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="D659" s="16" t="inlineStr">
+        <is>
+          <t>88888888</t>
+        </is>
+      </c>
+      <c r="E659" s="18" t="n">
+        <v>2044212.76</v>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B660" s="10" t="n">
+        <v>834</v>
+      </c>
+      <c r="C660" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="D660" s="11" t="inlineStr">
+        <is>
+          <t>group8</t>
+        </is>
+      </c>
+      <c r="E660" s="14" t="n">
+        <v>2007808.28</v>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B661" s="15" t="n">
+        <v>834</v>
+      </c>
+      <c r="C661" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="D661" s="16" t="inlineStr">
+        <is>
+          <t>group9</t>
+        </is>
+      </c>
+      <c r="E661" s="18" t="n">
+        <v>2005126.74</v>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B662" s="10" t="n">
+        <v>834</v>
+      </c>
+      <c r="C662" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="D662" s="11" t="inlineStr">
+        <is>
+          <t>666666</t>
+        </is>
+      </c>
+      <c r="E662" s="14" t="n">
+        <v>1889821.82</v>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B663" s="15" t="n">
+        <v>834</v>
+      </c>
+      <c r="C663" s="15" t="n">
+        <v>14</v>
+      </c>
+      <c r="D663" s="16" t="inlineStr">
+        <is>
+          <t>tigagroup20</t>
+        </is>
+      </c>
+      <c r="E663" s="18" t="n">
+        <v>1887071.66</v>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B664" s="10" t="n">
+        <v>834</v>
+      </c>
+      <c r="C664" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="D664" s="11" t="inlineStr">
+        <is>
+          <t>t24</t>
+        </is>
+      </c>
+      <c r="E664" s="14" t="n">
+        <v>1836405.8</v>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B665" s="15" t="n">
+        <v>834</v>
+      </c>
+      <c r="C665" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="D665" s="16" t="inlineStr">
+        <is>
+          <t>group7</t>
+        </is>
+      </c>
+      <c r="E665" s="18" t="n">
+        <v>1810210.32</v>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B666" s="10" t="n">
+        <v>834</v>
+      </c>
+      <c r="C666" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="D666" s="11" t="inlineStr">
+        <is>
+          <t>cleveregg</t>
+        </is>
+      </c>
+      <c r="E666" s="14" t="n">
+        <v>1799179.36</v>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B667" s="15" t="n">
+        <v>834</v>
+      </c>
+      <c r="C667" s="15" t="n">
+        <v>18</v>
+      </c>
+      <c r="D667" s="16" t="inlineStr">
+        <is>
+          <t>deepsleep</t>
+        </is>
+      </c>
+      <c r="E667" s="18" t="n">
+        <v>1765438.69</v>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B668" s="10" t="n">
+        <v>834</v>
+      </c>
+      <c r="C668" s="10" t="n">
+        <v>19</v>
+      </c>
+      <c r="D668" s="11" t="inlineStr">
+        <is>
+          <t>jit</t>
+        </is>
+      </c>
+      <c r="E668" s="14" t="n">
+        <v>1753588.44</v>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B669" s="15" t="n">
+        <v>834</v>
+      </c>
+      <c r="C669" s="15" t="n">
+        <v>20</v>
+      </c>
+      <c r="D669" s="16" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E669" s="18" t="n">
+        <v>1712651.14</v>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B670" s="10" t="n">
+        <v>834</v>
+      </c>
+      <c r="C670" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="D670" s="11" t="inlineStr">
+        <is>
+          <t>vivo50</t>
+        </is>
+      </c>
+      <c r="E670" s="14" t="n">
+        <v>1530922.93</v>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B671" s="15" t="n">
+        <v>834</v>
+      </c>
+      <c r="C671" s="15" t="n">
+        <v>22</v>
+      </c>
+      <c r="D671" s="16" t="inlineStr">
+        <is>
+          <t>newgroup18</t>
+        </is>
+      </c>
+      <c r="E671" s="18" t="n">
+        <v>1513425.61</v>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B672" s="10" t="n">
+        <v>834</v>
+      </c>
+      <c r="C672" s="10" t="n">
+        <v>23</v>
+      </c>
+      <c r="D672" s="11" t="inlineStr">
+        <is>
+          <t>group12</t>
+        </is>
+      </c>
+      <c r="E672" s="14" t="n">
+        <v>1457063.93</v>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B673" s="15" t="n">
+        <v>834</v>
+      </c>
+      <c r="C673" s="15" t="n">
+        <v>24</v>
+      </c>
+      <c r="D673" s="16" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E673" s="18" t="n">
+        <v>1435397.07</v>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B674" s="10" t="n">
+        <v>834</v>
+      </c>
+      <c r="C674" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="D674" s="11" t="inlineStr">
+        <is>
+          <t>aaachemicalseller</t>
+        </is>
+      </c>
+      <c r="E674" s="14" t="n">
+        <v>1383523.68</v>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B675" s="24" t="n">
+        <v>834</v>
+      </c>
+      <c r="C675" s="24" t="n">
+        <v>26</v>
+      </c>
+      <c r="D675" s="25" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="E675" s="26" t="n">
+        <v>1262477.47</v>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B676" s="10" t="n">
+        <v>834</v>
+      </c>
+      <c r="C676" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="D676" s="11" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="E676" s="14" t="n">
+        <v>1255912.8</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E649"/>
+  <autoFilter ref="A1:E676"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -32532,11 +33099,11 @@
         <v>834</v>
       </c>
       <c r="D279" s="15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E279" s="16" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="F279" s="16" t="inlineStr">
@@ -32545,43 +33112,43 @@
         </is>
       </c>
       <c r="G279" s="17" t="n">
-        <v>95</v>
+        <v>150</v>
       </c>
       <c r="H279" s="17" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="I279" s="17" t="n">
-        <v>95</v>
-      </c>
-      <c r="J279" s="19" t="n">
-        <v>1</v>
+        <v>119</v>
+      </c>
+      <c r="J279" s="13" t="n">
+        <v>0.7933333333333333</v>
       </c>
       <c r="K279" s="17" t="n">
-        <v>95</v>
+        <v>119</v>
       </c>
       <c r="L279" s="18" t="n">
-        <v>1409686.63769144</v>
+        <v>1380240.409665605</v>
       </c>
       <c r="M279" s="18" t="n">
-        <v>1493645.2</v>
+        <v>1262477.47</v>
       </c>
       <c r="N279" s="18" t="n">
-        <v>83958.56230855989</v>
+        <v>-117762.9396656046</v>
       </c>
       <c r="O279" s="17" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="P279" s="17" t="n">
-        <v>55.5</v>
+        <v>37</v>
       </c>
       <c r="Q279" s="17" t="n">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="R279" s="17" t="n">
         <v>200</v>
       </c>
       <c r="S279" s="18" t="n">
-        <v>137750</v>
+        <v>172550</v>
       </c>
     </row>
   </sheetData>
@@ -32596,7 +33163,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N834"/>
+  <dimension ref="A1:N835"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -71005,8 +71572,54 @@
         <v>91350</v>
       </c>
     </row>
+    <row r="835">
+      <c r="A835" s="15" t="n">
+        <v>834</v>
+      </c>
+      <c r="B835" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C835" s="17" t="n">
+        <v>55</v>
+      </c>
+      <c r="D835" s="17" t="n">
+        <v>31</v>
+      </c>
+      <c r="E835" s="17" t="n">
+        <v>24</v>
+      </c>
+      <c r="F835" s="13" t="n">
+        <v>0.4363636363636363</v>
+      </c>
+      <c r="G835" s="17" t="n">
+        <v>24</v>
+      </c>
+      <c r="H835" s="18" t="n">
+        <v>1262477.47</v>
+      </c>
+      <c r="I835" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J835" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K835" s="17" t="n">
+        <v>400</v>
+      </c>
+      <c r="L835" s="17" t="n">
+        <v>400</v>
+      </c>
+      <c r="M835" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N835" s="18" t="n">
+        <v>34800</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N834"/>
+  <autoFilter ref="A1:N835"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -71401,7 +72014,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -72658,8 +73271,56 @@
         <v>55</v>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" s="21" t="n">
+        <v>730.66</v>
+      </c>
+      <c r="B52" s="11" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C52" s="11" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D52" s="11" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E52" s="11" t="inlineStr"/>
+      <c r="F52" s="12" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="23" t="n">
+        <v>742.75</v>
+      </c>
+      <c r="B53" s="16" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C53" s="16" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D53" s="16" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E53" s="16" t="inlineStr"/>
+      <c r="F53" s="17" t="n">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F51"/>
+  <autoFilter ref="A1:F53"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -73058,7 +73719,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U24"/>
+  <dimension ref="A1:U25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -73081,7 +73742,7 @@
     <col width="12" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
-    <col width="20" customWidth="1" min="21" max="21"/>
+    <col width="21" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -74804,8 +75465,77 @@
         <v>83958.56230855989</v>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B25" s="15" t="n">
+        <v>834</v>
+      </c>
+      <c r="C25" s="18" t="n">
+        <v>1262477.47</v>
+      </c>
+      <c r="D25" s="15" t="n">
+        <v>26</v>
+      </c>
+      <c r="E25" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="F25" s="16" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="G25" s="18" t="n">
+        <v>2007215.3</v>
+      </c>
+      <c r="H25" s="23" t="n">
+        <v>55</v>
+      </c>
+      <c r="I25" s="16" t="n"/>
+      <c r="J25" s="16" t="inlineStr">
+        <is>
+          <t>mail</t>
+        </is>
+      </c>
+      <c r="K25" s="27" t="n">
+        <v>3600</v>
+      </c>
+      <c r="L25" s="27" t="n">
+        <v>200</v>
+      </c>
+      <c r="M25" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N25" s="17" t="n">
+        <v>400</v>
+      </c>
+      <c r="O25" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="P25" s="15" t="n">
+        <v>278</v>
+      </c>
+      <c r="Q25" s="17" t="n">
+        <v>150</v>
+      </c>
+      <c r="R25" s="17" t="n">
+        <v>31</v>
+      </c>
+      <c r="S25" s="17" t="n">
+        <v>119</v>
+      </c>
+      <c r="T25" s="13" t="n">
+        <v>0.7933333333333333</v>
+      </c>
+      <c r="U25" s="18" t="n">
+        <v>-117762.9396656046</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U24"/>
+  <autoFilter ref="A1:U25"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -74816,7 +75546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E289"/>
+  <dimension ref="A1:E301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -81381,8 +82111,280 @@
         </is>
       </c>
     </row>
+    <row r="290">
+      <c r="A290" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B290" s="10" t="n">
+        <v>834</v>
+      </c>
+      <c r="C290" s="11" t="inlineStr">
+        <is>
+          <t>Starting Cash</t>
+        </is>
+      </c>
+      <c r="D290" s="14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E290" s="11" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B291" s="15" t="n">
+        <v>834</v>
+      </c>
+      <c r="C291" s="16" t="inlineStr">
+        <is>
+          <t>Cash Sources</t>
+        </is>
+      </c>
+      <c r="D291" s="16" t="n"/>
+      <c r="E291" s="16" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B292" s="10" t="n">
+        <v>834</v>
+      </c>
+      <c r="C292" s="11" t="inlineStr">
+        <is>
+          <t>revenues</t>
+        </is>
+      </c>
+      <c r="D292" s="14" t="n">
+        <v>21967500</v>
+      </c>
+      <c r="E292" s="11" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B293" s="15" t="n">
+        <v>834</v>
+      </c>
+      <c r="C293" s="16" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D293" s="18" t="n">
+        <v>299997.8</v>
+      </c>
+      <c r="E293" s="16" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B294" s="10" t="n">
+        <v>834</v>
+      </c>
+      <c r="C294" s="11" t="inlineStr">
+        <is>
+          <t>Cash Uses</t>
+        </is>
+      </c>
+      <c r="D294" s="11" t="n"/>
+      <c r="E294" s="11" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B295" s="15" t="n">
+        <v>834</v>
+      </c>
+      <c r="C295" s="16" t="inlineStr">
+        <is>
+          <t>outbound shipping</t>
+        </is>
+      </c>
+      <c r="D295" s="18" t="n">
+        <v>-2272500</v>
+      </c>
+      <c r="E295" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B296" s="10" t="n">
+        <v>834</v>
+      </c>
+      <c r="C296" s="11" t="inlineStr">
+        <is>
+          <t>inbound shipping</t>
+        </is>
+      </c>
+      <c r="D296" s="14" t="n">
+        <v>-1530000</v>
+      </c>
+      <c r="E296" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B297" s="15" t="n">
+        <v>834</v>
+      </c>
+      <c r="C297" s="16" t="inlineStr">
+        <is>
+          <t>FGI holding</t>
+        </is>
+      </c>
+      <c r="D297" s="18" t="n">
+        <v>-21850.7</v>
+      </c>
+      <c r="E297" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B298" s="10" t="n">
+        <v>834</v>
+      </c>
+      <c r="C298" s="11" t="inlineStr">
+        <is>
+          <t>add capacity</t>
+        </is>
+      </c>
+      <c r="D298" s="14" t="n">
+        <v>-1749840.87</v>
+      </c>
+      <c r="E298" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B299" s="15" t="n">
+        <v>834</v>
+      </c>
+      <c r="C299" s="16" t="inlineStr">
+        <is>
+          <t>Pipeline inventory holding</t>
+        </is>
+      </c>
+      <c r="D299" s="18" t="n">
+        <v>-29328.77</v>
+      </c>
+      <c r="E299" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B300" s="10" t="n">
+        <v>834</v>
+      </c>
+      <c r="C300" s="11" t="inlineStr">
+        <is>
+          <t>production</t>
+        </is>
+      </c>
+      <c r="D300" s="14" t="n">
+        <v>-15901500</v>
+      </c>
+      <c r="E300" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T12:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B301" s="15" t="n">
+        <v>834</v>
+      </c>
+      <c r="C301" s="16" t="inlineStr">
+        <is>
+          <t>Cash Balance</t>
+        </is>
+      </c>
+      <c r="D301" s="18" t="n">
+        <v>1262477.47</v>
+      </c>
+      <c r="E301" s="16" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E289"/>
+  <autoFilter ref="A1:E301"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update game data: day 835, cash 1262697.58, 3-day period 279
</commit_message>
<xml_diff>
--- a/data/supply_chain_game.xlsx
+++ b/data/supply_chain_game.xlsx
@@ -20,16 +20,16 @@
     <sheet name="排行榜" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$279</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$835</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$280</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$836</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'资金构成_旧版'!$A$1:$C$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'运营参数_旧版'!$A$9:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$55</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'排行榜_旧版'!$A$1:$C$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$301</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$313</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'运营参数'!$A$1:$J$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$676</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$703</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -590,7 +590,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-06T12:56:02+08:00</t>
+          <t>2026-09-06T13:11:01+08:00</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>834</v>
+        <v>835</v>
       </c>
     </row>
     <row r="7">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>626</v>
+        <v>625</v>
       </c>
     </row>
     <row r="8">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>1262477.47</v>
+        <v>1262697.58</v>
       </c>
     </row>
     <row r="11">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>2007215.3</v>
+        <v>2007808</v>
       </c>
     </row>
     <row r="15"/>
@@ -824,7 +824,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>278</v>
+        <v>279</v>
       </c>
     </row>
     <row r="30">
@@ -835,7 +835,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>832–834</t>
+          <t>835–837</t>
         </is>
       </c>
     </row>
@@ -847,7 +847,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否（进行中）</t>
         </is>
       </c>
     </row>
@@ -858,7 +858,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>150</v>
+        <v>58</v>
       </c>
     </row>
     <row r="33">
@@ -868,7 +868,7 @@
         </is>
       </c>
       <c r="B33" s="7" t="n">
-        <v>31</v>
+        <v>58</v>
       </c>
     </row>
     <row r="34">
@@ -878,7 +878,7 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>119</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
@@ -888,7 +888,7 @@
         </is>
       </c>
       <c r="B35" s="8" t="n">
-        <v>0.7933333333333333</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -898,7 +898,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>119</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -906,9 +906,6 @@
         <is>
           <t>周期现金变动</t>
         </is>
-      </c>
-      <c r="B37" s="4" t="n">
-        <v>-117762.9396656046</v>
       </c>
     </row>
     <row r="38"/>
@@ -970,7 +967,7 @@
         </is>
       </c>
       <c r="B44" s="4" t="n">
-        <v>-117762.9396656046</v>
+        <v>-117762.9390227285</v>
       </c>
     </row>
     <row r="45"/>
@@ -1292,7 +1289,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E676"/>
+  <dimension ref="A1:E703"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -15504,8 +15501,575 @@
         <v>1255912.8</v>
       </c>
     </row>
+    <row r="677">
+      <c r="A677" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:11:01+08:00</t>
+        </is>
+      </c>
+      <c r="B677" s="15" t="n">
+        <v>835</v>
+      </c>
+      <c r="C677" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D677" s="16" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="E677" s="18" t="n">
+        <v>3270505.58</v>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:11:01+08:00</t>
+        </is>
+      </c>
+      <c r="B678" s="10" t="n">
+        <v>835</v>
+      </c>
+      <c r="C678" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D678" s="11" t="inlineStr">
+        <is>
+          <t>nicetry</t>
+        </is>
+      </c>
+      <c r="E678" s="14" t="n">
+        <v>2349755.25</v>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:11:01+08:00</t>
+        </is>
+      </c>
+      <c r="B679" s="15" t="n">
+        <v>835</v>
+      </c>
+      <c r="C679" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D679" s="16" t="inlineStr">
+        <is>
+          <t>montesquieu</t>
+        </is>
+      </c>
+      <c r="E679" s="18" t="n">
+        <v>2302187.79</v>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:11:01+08:00</t>
+        </is>
+      </c>
+      <c r="B680" s="10" t="n">
+        <v>835</v>
+      </c>
+      <c r="C680" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D680" s="11" t="inlineStr">
+        <is>
+          <t>group2</t>
+        </is>
+      </c>
+      <c r="E680" s="14" t="n">
+        <v>2138429.55</v>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:11:01+08:00</t>
+        </is>
+      </c>
+      <c r="B681" s="15" t="n">
+        <v>835</v>
+      </c>
+      <c r="C681" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="D681" s="16" t="inlineStr">
+        <is>
+          <t>group25</t>
+        </is>
+      </c>
+      <c r="E681" s="18" t="n">
+        <v>2138271.92</v>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:11:01+08:00</t>
+        </is>
+      </c>
+      <c r="B682" s="10" t="n">
+        <v>835</v>
+      </c>
+      <c r="C682" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="D682" s="11" t="inlineStr">
+        <is>
+          <t>group11</t>
+        </is>
+      </c>
+      <c r="E682" s="14" t="n">
+        <v>2138259.65</v>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:11:01+08:00</t>
+        </is>
+      </c>
+      <c r="B683" s="15" t="n">
+        <v>835</v>
+      </c>
+      <c r="C683" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="D683" s="16" t="inlineStr">
+        <is>
+          <t>88888888</t>
+        </is>
+      </c>
+      <c r="E683" s="18" t="n">
+        <v>2138237.03</v>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:11:01+08:00</t>
+        </is>
+      </c>
+      <c r="B684" s="10" t="n">
+        <v>835</v>
+      </c>
+      <c r="C684" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="D684" s="11" t="inlineStr">
+        <is>
+          <t>teamhlly</t>
+        </is>
+      </c>
+      <c r="E684" s="14" t="n">
+        <v>2045307.76</v>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:11:01+08:00</t>
+        </is>
+      </c>
+      <c r="B685" s="15" t="n">
+        <v>835</v>
+      </c>
+      <c r="C685" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="D685" s="16" t="inlineStr">
+        <is>
+          <t>666666</t>
+        </is>
+      </c>
+      <c r="E685" s="18" t="n">
+        <v>2029314.18</v>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:11:01+08:00</t>
+        </is>
+      </c>
+      <c r="B686" s="10" t="n">
+        <v>835</v>
+      </c>
+      <c r="C686" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="D686" s="11" t="inlineStr">
+        <is>
+          <t>group8</t>
+        </is>
+      </c>
+      <c r="E686" s="14" t="n">
+        <v>2008277.85</v>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:11:01+08:00</t>
+        </is>
+      </c>
+      <c r="B687" s="15" t="n">
+        <v>835</v>
+      </c>
+      <c r="C687" s="15" t="n">
+        <v>11</v>
+      </c>
+      <c r="D687" s="16" t="inlineStr">
+        <is>
+          <t>group9</t>
+        </is>
+      </c>
+      <c r="E687" s="18" t="n">
+        <v>2005575.66</v>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:11:01+08:00</t>
+        </is>
+      </c>
+      <c r="B688" s="10" t="n">
+        <v>835</v>
+      </c>
+      <c r="C688" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="D688" s="11" t="inlineStr">
+        <is>
+          <t>group14</t>
+        </is>
+      </c>
+      <c r="E688" s="14" t="n">
+        <v>1972625.74</v>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:11:01+08:00</t>
+        </is>
+      </c>
+      <c r="B689" s="15" t="n">
+        <v>835</v>
+      </c>
+      <c r="C689" s="15" t="n">
+        <v>13</v>
+      </c>
+      <c r="D689" s="16" t="inlineStr">
+        <is>
+          <t>group15</t>
+        </is>
+      </c>
+      <c r="E689" s="18" t="n">
+        <v>1931357.8</v>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:11:01+08:00</t>
+        </is>
+      </c>
+      <c r="B690" s="10" t="n">
+        <v>835</v>
+      </c>
+      <c r="C690" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="D690" s="11" t="inlineStr">
+        <is>
+          <t>t24</t>
+        </is>
+      </c>
+      <c r="E690" s="14" t="n">
+        <v>1920032.96</v>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:11:01+08:00</t>
+        </is>
+      </c>
+      <c r="B691" s="15" t="n">
+        <v>835</v>
+      </c>
+      <c r="C691" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="D691" s="16" t="inlineStr">
+        <is>
+          <t>group7</t>
+        </is>
+      </c>
+      <c r="E691" s="18" t="n">
+        <v>1904200.88</v>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:11:01+08:00</t>
+        </is>
+      </c>
+      <c r="B692" s="10" t="n">
+        <v>835</v>
+      </c>
+      <c r="C692" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="D692" s="11" t="inlineStr">
+        <is>
+          <t>deepsleep</t>
+        </is>
+      </c>
+      <c r="E692" s="14" t="n">
+        <v>1890602.23</v>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:11:01+08:00</t>
+        </is>
+      </c>
+      <c r="B693" s="15" t="n">
+        <v>835</v>
+      </c>
+      <c r="C693" s="15" t="n">
+        <v>17</v>
+      </c>
+      <c r="D693" s="16" t="inlineStr">
+        <is>
+          <t>tigagroup20</t>
+        </is>
+      </c>
+      <c r="E693" s="18" t="n">
+        <v>1887454.9</v>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:11:01+08:00</t>
+        </is>
+      </c>
+      <c r="B694" s="10" t="n">
+        <v>835</v>
+      </c>
+      <c r="C694" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="D694" s="11" t="inlineStr">
+        <is>
+          <t>cleveregg</t>
+        </is>
+      </c>
+      <c r="E694" s="14" t="n">
+        <v>1882742.63</v>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:11:01+08:00</t>
+        </is>
+      </c>
+      <c r="B695" s="15" t="n">
+        <v>835</v>
+      </c>
+      <c r="C695" s="15" t="n">
+        <v>19</v>
+      </c>
+      <c r="D695" s="16" t="inlineStr">
+        <is>
+          <t>jit</t>
+        </is>
+      </c>
+      <c r="E695" s="18" t="n">
+        <v>1753936.82</v>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:11:01+08:00</t>
+        </is>
+      </c>
+      <c r="B696" s="10" t="n">
+        <v>835</v>
+      </c>
+      <c r="C696" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="D696" s="11" t="inlineStr">
+        <is>
+          <t>vivo50</t>
+        </is>
+      </c>
+      <c r="E696" s="14" t="n">
+        <v>1656014.27</v>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:11:01+08:00</t>
+        </is>
+      </c>
+      <c r="B697" s="15" t="n">
+        <v>835</v>
+      </c>
+      <c r="C697" s="15" t="n">
+        <v>21</v>
+      </c>
+      <c r="D697" s="16" t="inlineStr">
+        <is>
+          <t>group12</t>
+        </is>
+      </c>
+      <c r="E697" s="18" t="n">
+        <v>1582135.98</v>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:11:01+08:00</t>
+        </is>
+      </c>
+      <c r="B698" s="10" t="n">
+        <v>835</v>
+      </c>
+      <c r="C698" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="D698" s="11" t="inlineStr">
+        <is>
+          <t>newgroup18</t>
+        </is>
+      </c>
+      <c r="E698" s="14" t="n">
+        <v>1551404.39</v>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:11:01+08:00</t>
+        </is>
+      </c>
+      <c r="B699" s="15" t="n">
+        <v>835</v>
+      </c>
+      <c r="C699" s="15" t="n">
+        <v>23</v>
+      </c>
+      <c r="D699" s="16" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E699" s="18" t="n">
+        <v>1496495.39</v>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:11:01+08:00</t>
+        </is>
+      </c>
+      <c r="B700" s="10" t="n">
+        <v>835</v>
+      </c>
+      <c r="C700" s="10" t="n">
+        <v>24</v>
+      </c>
+      <c r="D700" s="11" t="inlineStr">
+        <is>
+          <t>aaachemicalseller</t>
+        </is>
+      </c>
+      <c r="E700" s="14" t="n">
+        <v>1459166.34</v>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:11:01+08:00</t>
+        </is>
+      </c>
+      <c r="B701" s="15" t="n">
+        <v>835</v>
+      </c>
+      <c r="C701" s="15" t="n">
+        <v>25</v>
+      </c>
+      <c r="D701" s="16" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E701" s="18" t="n">
+        <v>1459058.31</v>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:11:01+08:00</t>
+        </is>
+      </c>
+      <c r="B702" s="24" t="n">
+        <v>835</v>
+      </c>
+      <c r="C702" s="24" t="n">
+        <v>26</v>
+      </c>
+      <c r="D702" s="25" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="E702" s="26" t="n">
+        <v>1262697.58</v>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:11:01+08:00</t>
+        </is>
+      </c>
+      <c r="B703" s="15" t="n">
+        <v>835</v>
+      </c>
+      <c r="C703" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="D703" s="16" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="E703" s="18" t="n">
+        <v>1123833.09</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E676"/>
+  <autoFilter ref="A1:E703"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -15516,7 +16080,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S279"/>
+  <dimension ref="A1:S280"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -33151,8 +33715,69 @@
         <v>172550</v>
       </c>
     </row>
+    <row r="280">
+      <c r="A280" s="10" t="n">
+        <v>279</v>
+      </c>
+      <c r="B280" s="10" t="n">
+        <v>835</v>
+      </c>
+      <c r="C280" s="10" t="n">
+        <v>837</v>
+      </c>
+      <c r="D280" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E280" s="11" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="F280" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G280" s="12" t="n">
+        <v>58</v>
+      </c>
+      <c r="H280" s="12" t="n">
+        <v>58</v>
+      </c>
+      <c r="I280" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J280" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K280" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L280" s="14" t="n">
+        <v>1262697.58</v>
+      </c>
+      <c r="M280" s="14" t="n">
+        <v>1262697.58</v>
+      </c>
+      <c r="N280" s="11" t="n"/>
+      <c r="O280" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="P280" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q280" s="12" t="n">
+        <v>400</v>
+      </c>
+      <c r="R280" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="S280" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S279"/>
+  <autoFilter ref="A1:S280"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -33163,7 +33788,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N835"/>
+  <dimension ref="A1:N836"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -71618,8 +72243,54 @@
         <v>34800</v>
       </c>
     </row>
+    <row r="836">
+      <c r="A836" s="10" t="n">
+        <v>835</v>
+      </c>
+      <c r="B836" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C836" s="12" t="n">
+        <v>58</v>
+      </c>
+      <c r="D836" s="12" t="n">
+        <v>58</v>
+      </c>
+      <c r="E836" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F836" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G836" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H836" s="14" t="n">
+        <v>1262697.58</v>
+      </c>
+      <c r="I836" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J836" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K836" s="12" t="n">
+        <v>400</v>
+      </c>
+      <c r="L836" s="12" t="n">
+        <v>400</v>
+      </c>
+      <c r="M836" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N836" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N835"/>
+  <autoFilter ref="A1:N836"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -72014,7 +72685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:F55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -73319,8 +73990,56 @@
         <v>55</v>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" s="21" t="n">
+        <v>730.66</v>
+      </c>
+      <c r="B54" s="11" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C54" s="11" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D54" s="11" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E54" s="11" t="inlineStr"/>
+      <c r="F54" s="12" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="23" t="n">
+        <v>742.75</v>
+      </c>
+      <c r="B55" s="16" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C55" s="16" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D55" s="16" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E55" s="16" t="inlineStr"/>
+      <c r="F55" s="17" t="n">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F53"/>
+  <autoFilter ref="A1:F55"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -73719,7 +74438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U25"/>
+  <dimension ref="A1:U26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -73742,7 +74461,7 @@
     <col width="12" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
-    <col width="21" customWidth="1" min="21" max="21"/>
+    <col width="20" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -75534,8 +76253,75 @@
         <v>-117762.9396656046</v>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:11:01+08:00</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="n">
+        <v>835</v>
+      </c>
+      <c r="C26" s="14" t="n">
+        <v>1262697.58</v>
+      </c>
+      <c r="D26" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="E26" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="F26" s="11" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="G26" s="14" t="n">
+        <v>2007808</v>
+      </c>
+      <c r="H26" s="21" t="n">
+        <v>55</v>
+      </c>
+      <c r="I26" s="11" t="n"/>
+      <c r="J26" s="11" t="inlineStr">
+        <is>
+          <t>mail</t>
+        </is>
+      </c>
+      <c r="K26" s="22" t="n">
+        <v>3600</v>
+      </c>
+      <c r="L26" s="22" t="n">
+        <v>200</v>
+      </c>
+      <c r="M26" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N26" s="12" t="n">
+        <v>400</v>
+      </c>
+      <c r="O26" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="P26" s="10" t="n">
+        <v>279</v>
+      </c>
+      <c r="Q26" s="12" t="n">
+        <v>58</v>
+      </c>
+      <c r="R26" s="12" t="n">
+        <v>58</v>
+      </c>
+      <c r="S26" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="T26" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="U26" s="11" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U25"/>
+  <autoFilter ref="A1:U26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -75546,7 +76332,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E301"/>
+  <dimension ref="A1:E313"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -82383,8 +83169,280 @@
         </is>
       </c>
     </row>
+    <row r="302">
+      <c r="A302" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:11:01+08:00</t>
+        </is>
+      </c>
+      <c r="B302" s="10" t="n">
+        <v>835</v>
+      </c>
+      <c r="C302" s="11" t="inlineStr">
+        <is>
+          <t>Starting Cash</t>
+        </is>
+      </c>
+      <c r="D302" s="14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E302" s="11" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:11:01+08:00</t>
+        </is>
+      </c>
+      <c r="B303" s="15" t="n">
+        <v>835</v>
+      </c>
+      <c r="C303" s="16" t="inlineStr">
+        <is>
+          <t>Cash Sources</t>
+        </is>
+      </c>
+      <c r="D303" s="16" t="n"/>
+      <c r="E303" s="16" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:11:01+08:00</t>
+        </is>
+      </c>
+      <c r="B304" s="10" t="n">
+        <v>835</v>
+      </c>
+      <c r="C304" s="11" t="inlineStr">
+        <is>
+          <t>revenues</t>
+        </is>
+      </c>
+      <c r="D304" s="14" t="n">
+        <v>21967500</v>
+      </c>
+      <c r="E304" s="11" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:11:01+08:00</t>
+        </is>
+      </c>
+      <c r="B305" s="15" t="n">
+        <v>835</v>
+      </c>
+      <c r="C305" s="16" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D305" s="18" t="n">
+        <v>300327.51</v>
+      </c>
+      <c r="E305" s="16" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:11:01+08:00</t>
+        </is>
+      </c>
+      <c r="B306" s="10" t="n">
+        <v>835</v>
+      </c>
+      <c r="C306" s="11" t="inlineStr">
+        <is>
+          <t>Cash Uses</t>
+        </is>
+      </c>
+      <c r="D306" s="11" t="n"/>
+      <c r="E306" s="11" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:11:01+08:00</t>
+        </is>
+      </c>
+      <c r="B307" s="15" t="n">
+        <v>835</v>
+      </c>
+      <c r="C307" s="16" t="inlineStr">
+        <is>
+          <t>outbound shipping</t>
+        </is>
+      </c>
+      <c r="D307" s="18" t="n">
+        <v>-2272500</v>
+      </c>
+      <c r="E307" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:11:01+08:00</t>
+        </is>
+      </c>
+      <c r="B308" s="10" t="n">
+        <v>835</v>
+      </c>
+      <c r="C308" s="11" t="inlineStr">
+        <is>
+          <t>inbound shipping</t>
+        </is>
+      </c>
+      <c r="D308" s="14" t="n">
+        <v>-1530000</v>
+      </c>
+      <c r="E308" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:11:01+08:00</t>
+        </is>
+      </c>
+      <c r="B309" s="15" t="n">
+        <v>835</v>
+      </c>
+      <c r="C309" s="16" t="inlineStr">
+        <is>
+          <t>FGI holding</t>
+        </is>
+      </c>
+      <c r="D309" s="18" t="n">
+        <v>-21850.7</v>
+      </c>
+      <c r="E309" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:11:01+08:00</t>
+        </is>
+      </c>
+      <c r="B310" s="10" t="n">
+        <v>835</v>
+      </c>
+      <c r="C310" s="11" t="inlineStr">
+        <is>
+          <t>add capacity</t>
+        </is>
+      </c>
+      <c r="D310" s="14" t="n">
+        <v>-1749840.87</v>
+      </c>
+      <c r="E310" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:11:01+08:00</t>
+        </is>
+      </c>
+      <c r="B311" s="15" t="n">
+        <v>835</v>
+      </c>
+      <c r="C311" s="16" t="inlineStr">
+        <is>
+          <t>Pipeline inventory holding</t>
+        </is>
+      </c>
+      <c r="D311" s="18" t="n">
+        <v>-29438.36</v>
+      </c>
+      <c r="E311" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:11:01+08:00</t>
+        </is>
+      </c>
+      <c r="B312" s="10" t="n">
+        <v>835</v>
+      </c>
+      <c r="C312" s="11" t="inlineStr">
+        <is>
+          <t>production</t>
+        </is>
+      </c>
+      <c r="D312" s="14" t="n">
+        <v>-15901500</v>
+      </c>
+      <c r="E312" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:11:01+08:00</t>
+        </is>
+      </c>
+      <c r="B313" s="15" t="n">
+        <v>835</v>
+      </c>
+      <c r="C313" s="16" t="inlineStr">
+        <is>
+          <t>Cash Balance</t>
+        </is>
+      </c>
+      <c r="D313" s="18" t="n">
+        <v>1262697.58</v>
+      </c>
+      <c r="E313" s="16" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E301"/>
+  <autoFilter ref="A1:E313"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update game data: day 836, cash 1386417.76, 3-day period 279
</commit_message>
<xml_diff>
--- a/data/supply_chain_game.xlsx
+++ b/data/supply_chain_game.xlsx
@@ -21,15 +21,15 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$280</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$836</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$837</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'资金构成_旧版'!$A$1:$C$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'运营参数_旧版'!$A$9:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$57</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'排行榜_旧版'!$A$1:$C$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$26</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$313</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$325</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'运营参数'!$A$1:$J$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$703</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$730</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -590,7 +590,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-06T13:11:01+08:00</t>
+          <t>2026-09-06T13:26:02+08:00</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>835</v>
+        <v>836</v>
       </c>
     </row>
     <row r="7">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>625</v>
+        <v>624</v>
       </c>
     </row>
     <row r="8">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>1262697.58</v>
+        <v>1386417.76</v>
       </c>
     </row>
     <row r="11">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>2007808</v>
+        <v>1884900.84</v>
       </c>
     </row>
     <row r="15"/>
@@ -786,7 +786,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>0</v>
+        <v>151</v>
       </c>
     </row>
     <row r="25">
@@ -796,7 +796,7 @@
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>400</v>
+        <v>200</v>
       </c>
     </row>
     <row r="26">
@@ -858,7 +858,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>58</v>
+        <v>107</v>
       </c>
     </row>
     <row r="33">
@@ -878,7 +878,7 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
     </row>
     <row r="35">
@@ -888,7 +888,7 @@
         </is>
       </c>
       <c r="B35" s="8" t="n">
-        <v>0</v>
+        <v>0.4579439252336449</v>
       </c>
     </row>
     <row r="36">
@@ -898,7 +898,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
     </row>
     <row r="37">
@@ -906,6 +906,9 @@
         <is>
           <t>周期现金变动</t>
         </is>
+      </c>
+      <c r="B37" s="4" t="n">
+        <v>66801.5067131212</v>
       </c>
     </row>
     <row r="38"/>
@@ -967,7 +970,7 @@
         </is>
       </c>
       <c r="B44" s="4" t="n">
-        <v>-117762.9390227285</v>
+        <v>-123071.3441053906</v>
       </c>
     </row>
     <row r="45"/>
@@ -1289,7 +1292,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E703"/>
+  <dimension ref="A1:E730"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -16068,8 +16071,575 @@
         <v>1123833.09</v>
       </c>
     </row>
+    <row r="704">
+      <c r="A704" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B704" s="10" t="n">
+        <v>836</v>
+      </c>
+      <c r="C704" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D704" s="11" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="E704" s="14" t="n">
+        <v>3271318.6</v>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B705" s="15" t="n">
+        <v>836</v>
+      </c>
+      <c r="C705" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D705" s="16" t="inlineStr">
+        <is>
+          <t>montesquieu</t>
+        </is>
+      </c>
+      <c r="E705" s="18" t="n">
+        <v>2440485.48</v>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B706" s="10" t="n">
+        <v>836</v>
+      </c>
+      <c r="C706" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D706" s="11" t="inlineStr">
+        <is>
+          <t>nicetry</t>
+        </is>
+      </c>
+      <c r="E706" s="14" t="n">
+        <v>2424377.2</v>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B707" s="15" t="n">
+        <v>836</v>
+      </c>
+      <c r="C707" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D707" s="16" t="inlineStr">
+        <is>
+          <t>group2</t>
+        </is>
+      </c>
+      <c r="E707" s="18" t="n">
+        <v>2212988.24</v>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B708" s="10" t="n">
+        <v>836</v>
+      </c>
+      <c r="C708" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="D708" s="11" t="inlineStr">
+        <is>
+          <t>group25</t>
+        </is>
+      </c>
+      <c r="E708" s="14" t="n">
+        <v>2212830.57</v>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B709" s="15" t="n">
+        <v>836</v>
+      </c>
+      <c r="C709" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="D709" s="16" t="inlineStr">
+        <is>
+          <t>group11</t>
+        </is>
+      </c>
+      <c r="E709" s="18" t="n">
+        <v>2212818.29</v>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B710" s="10" t="n">
+        <v>836</v>
+      </c>
+      <c r="C710" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="D710" s="11" t="inlineStr">
+        <is>
+          <t>88888888</t>
+        </is>
+      </c>
+      <c r="E710" s="14" t="n">
+        <v>2212795.68</v>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B711" s="15" t="n">
+        <v>836</v>
+      </c>
+      <c r="C711" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="D711" s="16" t="inlineStr">
+        <is>
+          <t>teamhlly</t>
+        </is>
+      </c>
+      <c r="E711" s="18" t="n">
+        <v>2169233.26</v>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B712" s="10" t="n">
+        <v>836</v>
+      </c>
+      <c r="C712" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="D712" s="11" t="inlineStr">
+        <is>
+          <t>group9</t>
+        </is>
+      </c>
+      <c r="E712" s="14" t="n">
+        <v>2119089.84</v>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B713" s="15" t="n">
+        <v>836</v>
+      </c>
+      <c r="C713" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="D713" s="16" t="inlineStr">
+        <is>
+          <t>666666</t>
+        </is>
+      </c>
+      <c r="E713" s="18" t="n">
+        <v>2103856.46</v>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B714" s="10" t="n">
+        <v>836</v>
+      </c>
+      <c r="C714" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="D714" s="11" t="inlineStr">
+        <is>
+          <t>group8</t>
+        </is>
+      </c>
+      <c r="E714" s="14" t="n">
+        <v>2008747.53</v>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B715" s="15" t="n">
+        <v>836</v>
+      </c>
+      <c r="C715" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="D715" s="16" t="inlineStr">
+        <is>
+          <t>t24</t>
+        </is>
+      </c>
+      <c r="E715" s="18" t="n">
+        <v>1994524.65</v>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B716" s="10" t="n">
+        <v>836</v>
+      </c>
+      <c r="C716" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="D716" s="11" t="inlineStr">
+        <is>
+          <t>group7</t>
+        </is>
+      </c>
+      <c r="E716" s="14" t="n">
+        <v>1978726.97</v>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B717" s="15" t="n">
+        <v>836</v>
+      </c>
+      <c r="C717" s="15" t="n">
+        <v>14</v>
+      </c>
+      <c r="D717" s="16" t="inlineStr">
+        <is>
+          <t>group14</t>
+        </is>
+      </c>
+      <c r="E717" s="18" t="n">
+        <v>1973031.31</v>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B718" s="10" t="n">
+        <v>836</v>
+      </c>
+      <c r="C718" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="D718" s="11" t="inlineStr">
+        <is>
+          <t>group15</t>
+        </is>
+      </c>
+      <c r="E718" s="14" t="n">
+        <v>1931752.6</v>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B719" s="15" t="n">
+        <v>836</v>
+      </c>
+      <c r="C719" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="D719" s="16" t="inlineStr">
+        <is>
+          <t>tigagroup20</t>
+        </is>
+      </c>
+      <c r="E719" s="18" t="n">
+        <v>1887838.23</v>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B720" s="10" t="n">
+        <v>836</v>
+      </c>
+      <c r="C720" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="D720" s="11" t="inlineStr">
+        <is>
+          <t>deepsleep</t>
+        </is>
+      </c>
+      <c r="E720" s="14" t="n">
+        <v>1768613.08</v>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B721" s="15" t="n">
+        <v>836</v>
+      </c>
+      <c r="C721" s="15" t="n">
+        <v>18</v>
+      </c>
+      <c r="D721" s="16" t="inlineStr">
+        <is>
+          <t>jit</t>
+        </is>
+      </c>
+      <c r="E721" s="18" t="n">
+        <v>1754285.28</v>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B722" s="10" t="n">
+        <v>836</v>
+      </c>
+      <c r="C722" s="10" t="n">
+        <v>19</v>
+      </c>
+      <c r="D722" s="11" t="inlineStr">
+        <is>
+          <t>cleveregg</t>
+        </is>
+      </c>
+      <c r="E722" s="14" t="n">
+        <v>1740748.27</v>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B723" s="15" t="n">
+        <v>836</v>
+      </c>
+      <c r="C723" s="15" t="n">
+        <v>20</v>
+      </c>
+      <c r="D723" s="16" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E723" s="18" t="n">
+        <v>1582829.76</v>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B724" s="10" t="n">
+        <v>836</v>
+      </c>
+      <c r="C724" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="D724" s="11" t="inlineStr">
+        <is>
+          <t>newgroup18</t>
+        </is>
+      </c>
+      <c r="E724" s="14" t="n">
+        <v>1551699.7</v>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B725" s="15" t="n">
+        <v>836</v>
+      </c>
+      <c r="C725" s="15" t="n">
+        <v>22</v>
+      </c>
+      <c r="D725" s="16" t="inlineStr">
+        <is>
+          <t>vivo50</t>
+        </is>
+      </c>
+      <c r="E725" s="18" t="n">
+        <v>1513952.56</v>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B726" s="10" t="n">
+        <v>836</v>
+      </c>
+      <c r="C726" s="10" t="n">
+        <v>23</v>
+      </c>
+      <c r="D726" s="11" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E726" s="14" t="n">
+        <v>1496776.62</v>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B727" s="15" t="n">
+        <v>836</v>
+      </c>
+      <c r="C727" s="15" t="n">
+        <v>24</v>
+      </c>
+      <c r="D727" s="16" t="inlineStr">
+        <is>
+          <t>aaachemicalseller</t>
+        </is>
+      </c>
+      <c r="E727" s="18" t="n">
+        <v>1459430.35</v>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B728" s="10" t="n">
+        <v>836</v>
+      </c>
+      <c r="C728" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="D728" s="11" t="inlineStr">
+        <is>
+          <t>group12</t>
+        </is>
+      </c>
+      <c r="E728" s="14" t="n">
+        <v>1440054.98</v>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B729" s="24" t="n">
+        <v>836</v>
+      </c>
+      <c r="C729" s="24" t="n">
+        <v>26</v>
+      </c>
+      <c r="D729" s="25" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="E729" s="26" t="n">
+        <v>1386417.76</v>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B730" s="10" t="n">
+        <v>836</v>
+      </c>
+      <c r="C730" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="D730" s="11" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="E730" s="14" t="n">
+        <v>1239788.49</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E703"/>
+  <autoFilter ref="A1:E730"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -33726,7 +34296,7 @@
         <v>837</v>
       </c>
       <c r="D280" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E280" s="11" t="inlineStr">
         <is>
@@ -33739,41 +34309,43 @@
         </is>
       </c>
       <c r="G280" s="12" t="n">
-        <v>58</v>
+        <v>107</v>
       </c>
       <c r="H280" s="12" t="n">
         <v>58</v>
       </c>
       <c r="I280" s="12" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="J280" s="13" t="n">
-        <v>0</v>
+        <v>0.4579439252336449</v>
       </c>
       <c r="K280" s="12" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="L280" s="14" t="n">
-        <v>1262697.58</v>
+        <v>1319616.253286879</v>
       </c>
       <c r="M280" s="14" t="n">
-        <v>1262697.58</v>
-      </c>
-      <c r="N280" s="11" t="n"/>
+        <v>1386417.76</v>
+      </c>
+      <c r="N280" s="14" t="n">
+        <v>66801.5067131212</v>
+      </c>
       <c r="O280" s="12" t="n">
-        <v>0</v>
+        <v>151</v>
       </c>
       <c r="P280" s="12" t="n">
-        <v>0</v>
+        <v>75.5</v>
       </c>
       <c r="Q280" s="12" t="n">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="R280" s="12" t="n">
         <v>200</v>
       </c>
       <c r="S280" s="14" t="n">
-        <v>0</v>
+        <v>71050</v>
       </c>
     </row>
   </sheetData>
@@ -33788,7 +34360,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N836"/>
+  <dimension ref="A1:N837"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -72289,8 +72861,54 @@
         <v>0</v>
       </c>
     </row>
+    <row r="837">
+      <c r="A837" s="15" t="n">
+        <v>836</v>
+      </c>
+      <c r="B837" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C837" s="17" t="n">
+        <v>49</v>
+      </c>
+      <c r="D837" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E837" s="17" t="n">
+        <v>49</v>
+      </c>
+      <c r="F837" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G837" s="17" t="n">
+        <v>49</v>
+      </c>
+      <c r="H837" s="18" t="n">
+        <v>1386417.76</v>
+      </c>
+      <c r="I837" s="17" t="n">
+        <v>151</v>
+      </c>
+      <c r="J837" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K837" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="L837" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="M837" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N837" s="18" t="n">
+        <v>71050</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N836"/>
+  <autoFilter ref="A1:N837"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -72685,7 +73303,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -74038,8 +74656,56 @@
         <v>55</v>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" s="21" t="n">
+        <v>730.66</v>
+      </c>
+      <c r="B56" s="11" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C56" s="11" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D56" s="11" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E56" s="11" t="inlineStr"/>
+      <c r="F56" s="12" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="23" t="n">
+        <v>742.75</v>
+      </c>
+      <c r="B57" s="16" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C57" s="16" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D57" s="16" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E57" s="16" t="inlineStr"/>
+      <c r="F57" s="17" t="n">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F55"/>
+  <autoFilter ref="A1:F57"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -74438,7 +75104,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U26"/>
+  <dimension ref="A1:U27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -76320,8 +76986,77 @@
       </c>
       <c r="U26" s="11" t="n"/>
     </row>
+    <row r="27">
+      <c r="A27" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B27" s="15" t="n">
+        <v>836</v>
+      </c>
+      <c r="C27" s="18" t="n">
+        <v>1386417.76</v>
+      </c>
+      <c r="D27" s="15" t="n">
+        <v>26</v>
+      </c>
+      <c r="E27" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="F27" s="16" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="G27" s="18" t="n">
+        <v>1884900.84</v>
+      </c>
+      <c r="H27" s="23" t="n">
+        <v>55</v>
+      </c>
+      <c r="I27" s="16" t="n"/>
+      <c r="J27" s="16" t="inlineStr">
+        <is>
+          <t>mail</t>
+        </is>
+      </c>
+      <c r="K27" s="27" t="n">
+        <v>3600</v>
+      </c>
+      <c r="L27" s="27" t="n">
+        <v>200</v>
+      </c>
+      <c r="M27" s="17" t="n">
+        <v>151</v>
+      </c>
+      <c r="N27" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="O27" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="P27" s="15" t="n">
+        <v>279</v>
+      </c>
+      <c r="Q27" s="17" t="n">
+        <v>107</v>
+      </c>
+      <c r="R27" s="17" t="n">
+        <v>58</v>
+      </c>
+      <c r="S27" s="17" t="n">
+        <v>49</v>
+      </c>
+      <c r="T27" s="13" t="n">
+        <v>0.4579439252336449</v>
+      </c>
+      <c r="U27" s="18" t="n">
+        <v>66801.5067131212</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U26"/>
+  <autoFilter ref="A1:U27"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -76332,7 +77067,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E313"/>
+  <dimension ref="A1:E325"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -83441,8 +84176,280 @@
         </is>
       </c>
     </row>
+    <row r="314">
+      <c r="A314" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B314" s="10" t="n">
+        <v>836</v>
+      </c>
+      <c r="C314" s="11" t="inlineStr">
+        <is>
+          <t>Starting Cash</t>
+        </is>
+      </c>
+      <c r="D314" s="14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E314" s="11" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B315" s="15" t="n">
+        <v>836</v>
+      </c>
+      <c r="C315" s="16" t="inlineStr">
+        <is>
+          <t>Cash Sources</t>
+        </is>
+      </c>
+      <c r="D315" s="16" t="n"/>
+      <c r="E315" s="16" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B316" s="10" t="n">
+        <v>836</v>
+      </c>
+      <c r="C316" s="11" t="inlineStr">
+        <is>
+          <t>revenues</t>
+        </is>
+      </c>
+      <c r="D316" s="14" t="n">
+        <v>22105250</v>
+      </c>
+      <c r="E316" s="11" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B317" s="15" t="n">
+        <v>836</v>
+      </c>
+      <c r="C317" s="16" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D317" s="18" t="n">
+        <v>300657.27</v>
+      </c>
+      <c r="E317" s="16" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B318" s="10" t="n">
+        <v>836</v>
+      </c>
+      <c r="C318" s="11" t="inlineStr">
+        <is>
+          <t>Cash Uses</t>
+        </is>
+      </c>
+      <c r="D318" s="11" t="n"/>
+      <c r="E318" s="11" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B319" s="15" t="n">
+        <v>836</v>
+      </c>
+      <c r="C319" s="16" t="inlineStr">
+        <is>
+          <t>outbound shipping</t>
+        </is>
+      </c>
+      <c r="D319" s="18" t="n">
+        <v>-2286750</v>
+      </c>
+      <c r="E319" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B320" s="10" t="n">
+        <v>836</v>
+      </c>
+      <c r="C320" s="11" t="inlineStr">
+        <is>
+          <t>inbound shipping</t>
+        </is>
+      </c>
+      <c r="D320" s="14" t="n">
+        <v>-1530000</v>
+      </c>
+      <c r="E320" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B321" s="15" t="n">
+        <v>836</v>
+      </c>
+      <c r="C321" s="16" t="inlineStr">
+        <is>
+          <t>FGI holding</t>
+        </is>
+      </c>
+      <c r="D321" s="18" t="n">
+        <v>-21850.7</v>
+      </c>
+      <c r="E321" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B322" s="10" t="n">
+        <v>836</v>
+      </c>
+      <c r="C322" s="11" t="inlineStr">
+        <is>
+          <t>add capacity</t>
+        </is>
+      </c>
+      <c r="D322" s="14" t="n">
+        <v>-1749840.87</v>
+      </c>
+      <c r="E322" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B323" s="15" t="n">
+        <v>836</v>
+      </c>
+      <c r="C323" s="16" t="inlineStr">
+        <is>
+          <t>Pipeline inventory holding</t>
+        </is>
+      </c>
+      <c r="D323" s="18" t="n">
+        <v>-29547.95</v>
+      </c>
+      <c r="E323" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B324" s="10" t="n">
+        <v>836</v>
+      </c>
+      <c r="C324" s="11" t="inlineStr">
+        <is>
+          <t>production</t>
+        </is>
+      </c>
+      <c r="D324" s="14" t="n">
+        <v>-15901500</v>
+      </c>
+      <c r="E324" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B325" s="15" t="n">
+        <v>836</v>
+      </c>
+      <c r="C325" s="16" t="inlineStr">
+        <is>
+          <t>Cash Balance</t>
+        </is>
+      </c>
+      <c r="D325" s="18" t="n">
+        <v>1386417.76</v>
+      </c>
+      <c r="E325" s="16" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E313"/>
+  <autoFilter ref="A1:E325"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update game data: day 837, cash 1256589.79, 3-day period 279
</commit_message>
<xml_diff>
--- a/data/supply_chain_game.xlsx
+++ b/data/supply_chain_game.xlsx
@@ -21,15 +21,15 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$280</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$837</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$838</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'资金构成_旧版'!$A$1:$C$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'运营参数_旧版'!$A$9:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$59</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'排行榜_旧版'!$A$1:$C$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$27</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$325</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$337</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'运营参数'!$A$1:$J$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$730</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$757</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -590,7 +590,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-06T13:26:02+08:00</t>
+          <t>2026-09-06T13:41:02+08:00</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>836</v>
+        <v>837</v>
       </c>
     </row>
     <row r="7">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>624</v>
+        <v>623</v>
       </c>
     </row>
     <row r="8">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>1386417.76</v>
+        <v>1256589.79</v>
       </c>
     </row>
     <row r="11">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>1884900.84</v>
+        <v>2015542.05</v>
       </c>
     </row>
     <row r="15"/>
@@ -786,7 +786,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>151</v>
+        <v>89</v>
       </c>
     </row>
     <row r="25">
@@ -847,7 +847,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>否（进行中）</t>
+          <t>是</t>
         </is>
       </c>
     </row>
@@ -858,7 +858,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>107</v>
+        <v>169</v>
       </c>
     </row>
     <row r="33">
@@ -878,7 +878,7 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>49</v>
+        <v>111</v>
       </c>
     </row>
     <row r="35">
@@ -888,7 +888,7 @@
         </is>
       </c>
       <c r="B35" s="8" t="n">
-        <v>0.4579439252336449</v>
+        <v>0.6568047337278107</v>
       </c>
     </row>
     <row r="36">
@@ -898,7 +898,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>49</v>
+        <v>111</v>
       </c>
     </row>
     <row r="37">
@@ -908,7 +908,7 @@
         </is>
       </c>
       <c r="B37" s="4" t="n">
-        <v>66801.5067131212</v>
+        <v>129268.7262096691</v>
       </c>
     </row>
     <row r="38"/>
@@ -926,7 +926,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>278</v>
+        <v>279</v>
       </c>
     </row>
     <row r="41">
@@ -937,7 +937,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>832–834</t>
+          <t>835–837</t>
         </is>
       </c>
     </row>
@@ -949,7 +949,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>150.0 / 31.0 / 119.0</t>
+          <t>169.0 / 58.0 / 111.0</t>
         </is>
       </c>
     </row>
@@ -960,7 +960,7 @@
         </is>
       </c>
       <c r="B43" s="8" t="n">
-        <v>0.7933333333333333</v>
+        <v>0.6568047337278107</v>
       </c>
     </row>
     <row r="44">
@@ -970,7 +970,7 @@
         </is>
       </c>
       <c r="B44" s="4" t="n">
-        <v>-123071.3441053906</v>
+        <v>129268.7262096691</v>
       </c>
     </row>
     <row r="45"/>
@@ -1292,7 +1292,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E730"/>
+  <dimension ref="A1:E757"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -16638,8 +16638,575 @@
         <v>1239788.49</v>
       </c>
     </row>
+    <row r="731">
+      <c r="A731" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B731" s="15" t="n">
+        <v>837</v>
+      </c>
+      <c r="C731" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D731" s="16" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="E731" s="18" t="n">
+        <v>3272131.84</v>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B732" s="10" t="n">
+        <v>837</v>
+      </c>
+      <c r="C732" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D732" s="11" t="inlineStr">
+        <is>
+          <t>montesquieu</t>
+        </is>
+      </c>
+      <c r="E732" s="14" t="n">
+        <v>2542435.81</v>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B733" s="15" t="n">
+        <v>837</v>
+      </c>
+      <c r="C733" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D733" s="16" t="inlineStr">
+        <is>
+          <t>nicetry</t>
+        </is>
+      </c>
+      <c r="E733" s="18" t="n">
+        <v>2486036.2</v>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B734" s="10" t="n">
+        <v>837</v>
+      </c>
+      <c r="C734" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D734" s="11" t="inlineStr">
+        <is>
+          <t>group2</t>
+        </is>
+      </c>
+      <c r="E734" s="14" t="n">
+        <v>2305785.46</v>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B735" s="15" t="n">
+        <v>837</v>
+      </c>
+      <c r="C735" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="D735" s="16" t="inlineStr">
+        <is>
+          <t>group25</t>
+        </is>
+      </c>
+      <c r="E735" s="18" t="n">
+        <v>2305627.75</v>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B736" s="10" t="n">
+        <v>837</v>
+      </c>
+      <c r="C736" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="D736" s="11" t="inlineStr">
+        <is>
+          <t>group11</t>
+        </is>
+      </c>
+      <c r="E736" s="14" t="n">
+        <v>2305615.47</v>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B737" s="15" t="n">
+        <v>837</v>
+      </c>
+      <c r="C737" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="D737" s="16" t="inlineStr">
+        <is>
+          <t>88888888</t>
+        </is>
+      </c>
+      <c r="E737" s="18" t="n">
+        <v>2305592.84</v>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B738" s="10" t="n">
+        <v>837</v>
+      </c>
+      <c r="C738" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="D738" s="11" t="inlineStr">
+        <is>
+          <t>teamhlly</t>
+        </is>
+      </c>
+      <c r="E738" s="14" t="n">
+        <v>2271109.74</v>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B739" s="15" t="n">
+        <v>837</v>
+      </c>
+      <c r="C739" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="D739" s="16" t="inlineStr">
+        <is>
+          <t>group9</t>
+        </is>
+      </c>
+      <c r="E739" s="18" t="n">
+        <v>2220941.21</v>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B740" s="10" t="n">
+        <v>837</v>
+      </c>
+      <c r="C740" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="D740" s="11" t="inlineStr">
+        <is>
+          <t>group14</t>
+        </is>
+      </c>
+      <c r="E740" s="14" t="n">
+        <v>2134640.78</v>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B741" s="15" t="n">
+        <v>837</v>
+      </c>
+      <c r="C741" s="15" t="n">
+        <v>11</v>
+      </c>
+      <c r="D741" s="16" t="inlineStr">
+        <is>
+          <t>group8</t>
+        </is>
+      </c>
+      <c r="E741" s="18" t="n">
+        <v>2113217.33</v>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B742" s="10" t="n">
+        <v>837</v>
+      </c>
+      <c r="C742" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="D742" s="11" t="inlineStr">
+        <is>
+          <t>t24</t>
+        </is>
+      </c>
+      <c r="E742" s="14" t="n">
+        <v>2096362.62</v>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B743" s="15" t="n">
+        <v>837</v>
+      </c>
+      <c r="C743" s="15" t="n">
+        <v>13</v>
+      </c>
+      <c r="D743" s="16" t="inlineStr">
+        <is>
+          <t>group15</t>
+        </is>
+      </c>
+      <c r="E743" s="18" t="n">
+        <v>2095953.5</v>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B744" s="10" t="n">
+        <v>837</v>
+      </c>
+      <c r="C744" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="D744" s="11" t="inlineStr">
+        <is>
+          <t>group7</t>
+        </is>
+      </c>
+      <c r="E744" s="14" t="n">
+        <v>2006490.41</v>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B745" s="15" t="n">
+        <v>837</v>
+      </c>
+      <c r="C745" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="D745" s="16" t="inlineStr">
+        <is>
+          <t>666666</t>
+        </is>
+      </c>
+      <c r="E745" s="18" t="n">
+        <v>1934634.76</v>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B746" s="10" t="n">
+        <v>837</v>
+      </c>
+      <c r="C746" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="D746" s="11" t="inlineStr">
+        <is>
+          <t>tigagroup20</t>
+        </is>
+      </c>
+      <c r="E746" s="14" t="n">
+        <v>1888221.67</v>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B747" s="15" t="n">
+        <v>837</v>
+      </c>
+      <c r="C747" s="15" t="n">
+        <v>17</v>
+      </c>
+      <c r="D747" s="16" t="inlineStr">
+        <is>
+          <t>deepsleep</t>
+        </is>
+      </c>
+      <c r="E747" s="18" t="n">
+        <v>1804062.47</v>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B748" s="10" t="n">
+        <v>837</v>
+      </c>
+      <c r="C748" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="D748" s="11" t="inlineStr">
+        <is>
+          <t>cleveregg</t>
+        </is>
+      </c>
+      <c r="E748" s="14" t="n">
+        <v>1780096.54</v>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B749" s="15" t="n">
+        <v>837</v>
+      </c>
+      <c r="C749" s="15" t="n">
+        <v>19</v>
+      </c>
+      <c r="D749" s="16" t="inlineStr">
+        <is>
+          <t>jit</t>
+        </is>
+      </c>
+      <c r="E749" s="18" t="n">
+        <v>1754633.84</v>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B750" s="10" t="n">
+        <v>837</v>
+      </c>
+      <c r="C750" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="D750" s="11" t="inlineStr">
+        <is>
+          <t>newgroup18</t>
+        </is>
+      </c>
+      <c r="E750" s="14" t="n">
+        <v>1702795.35</v>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B751" s="15" t="n">
+        <v>837</v>
+      </c>
+      <c r="C751" s="15" t="n">
+        <v>21</v>
+      </c>
+      <c r="D751" s="16" t="inlineStr">
+        <is>
+          <t>aaachemicalseller</t>
+        </is>
+      </c>
+      <c r="E751" s="18" t="n">
+        <v>1610501.9</v>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B752" s="10" t="n">
+        <v>837</v>
+      </c>
+      <c r="C752" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="D752" s="11" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E752" s="14" t="n">
+        <v>1601057.93</v>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B753" s="15" t="n">
+        <v>837</v>
+      </c>
+      <c r="C753" s="15" t="n">
+        <v>23</v>
+      </c>
+      <c r="D753" s="16" t="inlineStr">
+        <is>
+          <t>vivo50</t>
+        </is>
+      </c>
+      <c r="E753" s="18" t="n">
+        <v>1575319</v>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B754" s="10" t="n">
+        <v>837</v>
+      </c>
+      <c r="C754" s="10" t="n">
+        <v>24</v>
+      </c>
+      <c r="D754" s="11" t="inlineStr">
+        <is>
+          <t>group12</t>
+        </is>
+      </c>
+      <c r="E754" s="14" t="n">
+        <v>1501402.12</v>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B755" s="15" t="n">
+        <v>837</v>
+      </c>
+      <c r="C755" s="15" t="n">
+        <v>25</v>
+      </c>
+      <c r="D755" s="16" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E755" s="18" t="n">
+        <v>1468053.09</v>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B756" s="24" t="n">
+        <v>837</v>
+      </c>
+      <c r="C756" s="24" t="n">
+        <v>26</v>
+      </c>
+      <c r="D756" s="25" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="E756" s="26" t="n">
+        <v>1256589.79</v>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B757" s="15" t="n">
+        <v>837</v>
+      </c>
+      <c r="C757" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="D757" s="16" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="E757" s="18" t="n">
+        <v>1145388.01</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E730"/>
+  <autoFilter ref="A1:E757"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -34296,11 +34863,11 @@
         <v>837</v>
       </c>
       <c r="D280" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E280" s="11" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="F280" s="11" t="inlineStr">
@@ -34309,34 +34876,34 @@
         </is>
       </c>
       <c r="G280" s="12" t="n">
-        <v>107</v>
+        <v>169</v>
       </c>
       <c r="H280" s="12" t="n">
         <v>58</v>
       </c>
       <c r="I280" s="12" t="n">
-        <v>49</v>
+        <v>111</v>
       </c>
       <c r="J280" s="13" t="n">
-        <v>0.4579439252336449</v>
+        <v>0.6568047337278107</v>
       </c>
       <c r="K280" s="12" t="n">
-        <v>49</v>
+        <v>111</v>
       </c>
       <c r="L280" s="14" t="n">
-        <v>1319616.253286879</v>
+        <v>1127321.063790331</v>
       </c>
       <c r="M280" s="14" t="n">
-        <v>1386417.76</v>
+        <v>1256589.79</v>
       </c>
       <c r="N280" s="14" t="n">
-        <v>66801.5067131212</v>
+        <v>129268.7262096691</v>
       </c>
       <c r="O280" s="12" t="n">
-        <v>151</v>
+        <v>89</v>
       </c>
       <c r="P280" s="12" t="n">
-        <v>75.5</v>
+        <v>80</v>
       </c>
       <c r="Q280" s="12" t="n">
         <v>200</v>
@@ -34345,7 +34912,7 @@
         <v>200</v>
       </c>
       <c r="S280" s="14" t="n">
-        <v>71050</v>
+        <v>160950</v>
       </c>
     </row>
   </sheetData>
@@ -34360,7 +34927,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N837"/>
+  <dimension ref="A1:N838"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -72907,8 +73474,54 @@
         <v>71050</v>
       </c>
     </row>
+    <row r="838">
+      <c r="A838" s="10" t="n">
+        <v>837</v>
+      </c>
+      <c r="B838" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C838" s="12" t="n">
+        <v>62</v>
+      </c>
+      <c r="D838" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E838" s="12" t="n">
+        <v>62</v>
+      </c>
+      <c r="F838" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G838" s="12" t="n">
+        <v>62</v>
+      </c>
+      <c r="H838" s="14" t="n">
+        <v>1256589.79</v>
+      </c>
+      <c r="I838" s="12" t="n">
+        <v>89</v>
+      </c>
+      <c r="J838" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K838" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="L838" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="M838" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N838" s="14" t="n">
+        <v>89900</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N837"/>
+  <autoFilter ref="A1:N838"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -73303,7 +73916,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F57"/>
+  <dimension ref="A1:F59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -74704,8 +75317,56 @@
         <v>55</v>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" s="21" t="n">
+        <v>730.66</v>
+      </c>
+      <c r="B58" s="11" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C58" s="11" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D58" s="11" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E58" s="11" t="inlineStr"/>
+      <c r="F58" s="12" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="23" t="n">
+        <v>742.75</v>
+      </c>
+      <c r="B59" s="16" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C59" s="16" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D59" s="16" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E59" s="16" t="inlineStr"/>
+      <c r="F59" s="17" t="n">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F57"/>
+  <autoFilter ref="A1:F59"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -75104,7 +75765,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U27"/>
+  <dimension ref="A1:U28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -75113,7 +75774,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
@@ -77055,8 +77716,77 @@
         <v>66801.5067131212</v>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="n">
+        <v>837</v>
+      </c>
+      <c r="C28" s="14" t="n">
+        <v>1256589.79</v>
+      </c>
+      <c r="D28" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="E28" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="F28" s="11" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="G28" s="14" t="n">
+        <v>2015542.05</v>
+      </c>
+      <c r="H28" s="21" t="n">
+        <v>55</v>
+      </c>
+      <c r="I28" s="11" t="n"/>
+      <c r="J28" s="11" t="inlineStr">
+        <is>
+          <t>mail</t>
+        </is>
+      </c>
+      <c r="K28" s="22" t="n">
+        <v>3600</v>
+      </c>
+      <c r="L28" s="22" t="n">
+        <v>200</v>
+      </c>
+      <c r="M28" s="12" t="n">
+        <v>89</v>
+      </c>
+      <c r="N28" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="O28" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="P28" s="10" t="n">
+        <v>279</v>
+      </c>
+      <c r="Q28" s="12" t="n">
+        <v>169</v>
+      </c>
+      <c r="R28" s="12" t="n">
+        <v>58</v>
+      </c>
+      <c r="S28" s="12" t="n">
+        <v>111</v>
+      </c>
+      <c r="T28" s="13" t="n">
+        <v>0.6568047337278107</v>
+      </c>
+      <c r="U28" s="14" t="n">
+        <v>129268.7262096691</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U27"/>
+  <autoFilter ref="A1:U28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -77067,7 +77797,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E325"/>
+  <dimension ref="A1:E337"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -84448,8 +85178,280 @@
         </is>
       </c>
     </row>
+    <row r="326">
+      <c r="A326" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B326" s="10" t="n">
+        <v>837</v>
+      </c>
+      <c r="C326" s="11" t="inlineStr">
+        <is>
+          <t>Starting Cash</t>
+        </is>
+      </c>
+      <c r="D326" s="14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E326" s="11" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B327" s="15" t="n">
+        <v>837</v>
+      </c>
+      <c r="C327" s="16" t="inlineStr">
+        <is>
+          <t>Cash Sources</t>
+        </is>
+      </c>
+      <c r="D327" s="16" t="n"/>
+      <c r="E327" s="16" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B328" s="10" t="n">
+        <v>837</v>
+      </c>
+      <c r="C328" s="11" t="inlineStr">
+        <is>
+          <t>revenues</t>
+        </is>
+      </c>
+      <c r="D328" s="14" t="n">
+        <v>22218350</v>
+      </c>
+      <c r="E328" s="11" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B329" s="15" t="n">
+        <v>837</v>
+      </c>
+      <c r="C329" s="16" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D329" s="18" t="n">
+        <v>301015.76</v>
+      </c>
+      <c r="E329" s="16" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B330" s="10" t="n">
+        <v>837</v>
+      </c>
+      <c r="C330" s="11" t="inlineStr">
+        <is>
+          <t>Cash Uses</t>
+        </is>
+      </c>
+      <c r="D330" s="11" t="n"/>
+      <c r="E330" s="11" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B331" s="15" t="n">
+        <v>837</v>
+      </c>
+      <c r="C331" s="16" t="inlineStr">
+        <is>
+          <t>outbound shipping</t>
+        </is>
+      </c>
+      <c r="D331" s="18" t="n">
+        <v>-2298450</v>
+      </c>
+      <c r="E331" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B332" s="10" t="n">
+        <v>837</v>
+      </c>
+      <c r="C332" s="11" t="inlineStr">
+        <is>
+          <t>inbound shipping</t>
+        </is>
+      </c>
+      <c r="D332" s="14" t="n">
+        <v>-1560000</v>
+      </c>
+      <c r="E332" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B333" s="15" t="n">
+        <v>837</v>
+      </c>
+      <c r="C333" s="16" t="inlineStr">
+        <is>
+          <t>FGI holding</t>
+        </is>
+      </c>
+      <c r="D333" s="18" t="n">
+        <v>-21882.36</v>
+      </c>
+      <c r="E333" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B334" s="10" t="n">
+        <v>837</v>
+      </c>
+      <c r="C334" s="11" t="inlineStr">
+        <is>
+          <t>add capacity</t>
+        </is>
+      </c>
+      <c r="D334" s="14" t="n">
+        <v>-1749840.87</v>
+      </c>
+      <c r="E334" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B335" s="15" t="n">
+        <v>837</v>
+      </c>
+      <c r="C335" s="16" t="inlineStr">
+        <is>
+          <t>Pipeline inventory holding</t>
+        </is>
+      </c>
+      <c r="D335" s="18" t="n">
+        <v>-29602.74</v>
+      </c>
+      <c r="E335" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B336" s="10" t="n">
+        <v>837</v>
+      </c>
+      <c r="C336" s="11" t="inlineStr">
+        <is>
+          <t>production</t>
+        </is>
+      </c>
+      <c r="D336" s="14" t="n">
+        <v>-16103000</v>
+      </c>
+      <c r="E336" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B337" s="15" t="n">
+        <v>837</v>
+      </c>
+      <c r="C337" s="16" t="inlineStr">
+        <is>
+          <t>Cash Balance</t>
+        </is>
+      </c>
+      <c r="D337" s="18" t="n">
+        <v>1256589.79</v>
+      </c>
+      <c r="E337" s="16" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E325"/>
+  <autoFilter ref="A1:E337"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update game data: day 838, cash 1371261.61, 3-day period 280
</commit_message>
<xml_diff>
--- a/data/supply_chain_game.xlsx
+++ b/data/supply_chain_game.xlsx
@@ -20,16 +20,16 @@
     <sheet name="排行榜" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$280</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$838</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$281</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$839</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'资金构成_旧版'!$A$1:$C$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'运营参数_旧版'!$A$9:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$59</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$61</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'排行榜_旧版'!$A$1:$C$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$337</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$349</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'运营参数'!$A$1:$J$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$757</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$784</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -590,7 +590,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-06T13:41:02+08:00</t>
+          <t>2026-09-06T13:56:02+08:00</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>837</v>
+        <v>838</v>
       </c>
     </row>
     <row r="7">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>623</v>
+        <v>622</v>
       </c>
     </row>
     <row r="8">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>1256589.79</v>
+        <v>1371261.61</v>
       </c>
     </row>
     <row r="11">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>2015542.05</v>
+        <v>2016083.68</v>
       </c>
     </row>
     <row r="15"/>
@@ -786,7 +786,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>89</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25">
@@ -796,7 +796,7 @@
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>200</v>
+        <v>400</v>
       </c>
     </row>
     <row r="26">
@@ -824,7 +824,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>279</v>
+        <v>280</v>
       </c>
     </row>
     <row r="30">
@@ -835,7 +835,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>835–837</t>
+          <t>838–840</t>
         </is>
       </c>
     </row>
@@ -847,7 +847,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否（进行中）</t>
         </is>
       </c>
     </row>
@@ -858,7 +858,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>169</v>
+        <v>86</v>
       </c>
     </row>
     <row r="33">
@@ -868,7 +868,7 @@
         </is>
       </c>
       <c r="B33" s="7" t="n">
-        <v>58</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -878,7 +878,7 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>111</v>
+        <v>86</v>
       </c>
     </row>
     <row r="35">
@@ -888,7 +888,7 @@
         </is>
       </c>
       <c r="B35" s="8" t="n">
-        <v>0.6568047337278107</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36">
@@ -898,7 +898,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>111</v>
+        <v>86</v>
       </c>
     </row>
     <row r="37">
@@ -906,9 +906,6 @@
         <is>
           <t>周期现金变动</t>
         </is>
-      </c>
-      <c r="B37" s="4" t="n">
-        <v>129268.7262096691</v>
       </c>
     </row>
     <row r="38"/>
@@ -970,7 +967,7 @@
         </is>
       </c>
       <c r="B44" s="4" t="n">
-        <v>129268.7262096691</v>
+        <v>154144.7997774337</v>
       </c>
     </row>
     <row r="45"/>
@@ -1292,7 +1289,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E757"/>
+  <dimension ref="A1:E784"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -17205,8 +17202,575 @@
         <v>1145388.01</v>
       </c>
     </row>
+    <row r="758">
+      <c r="A758" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B758" s="10" t="n">
+        <v>838</v>
+      </c>
+      <c r="C758" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D758" s="11" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="E758" s="14" t="n">
+        <v>3387345.29</v>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B759" s="15" t="n">
+        <v>838</v>
+      </c>
+      <c r="C759" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D759" s="16" t="inlineStr">
+        <is>
+          <t>montesquieu</t>
+        </is>
+      </c>
+      <c r="E759" s="18" t="n">
+        <v>2563827.83</v>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B760" s="10" t="n">
+        <v>838</v>
+      </c>
+      <c r="C760" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D760" s="11" t="inlineStr">
+        <is>
+          <t>nicetry</t>
+        </is>
+      </c>
+      <c r="E760" s="14" t="n">
+        <v>2486625.41</v>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B761" s="15" t="n">
+        <v>838</v>
+      </c>
+      <c r="C761" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D761" s="16" t="inlineStr">
+        <is>
+          <t>teamhlly</t>
+        </is>
+      </c>
+      <c r="E761" s="18" t="n">
+        <v>2306727.93</v>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B762" s="10" t="n">
+        <v>838</v>
+      </c>
+      <c r="C762" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="D762" s="11" t="inlineStr">
+        <is>
+          <t>group9</t>
+        </is>
+      </c>
+      <c r="E762" s="14" t="n">
+        <v>2266944.11</v>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B763" s="15" t="n">
+        <v>838</v>
+      </c>
+      <c r="C763" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="D763" s="16" t="inlineStr">
+        <is>
+          <t>group14</t>
+        </is>
+      </c>
+      <c r="E763" s="18" t="n">
+        <v>2233909.91</v>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B764" s="10" t="n">
+        <v>838</v>
+      </c>
+      <c r="C764" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="D764" s="11" t="inlineStr">
+        <is>
+          <t>group8</t>
+        </is>
+      </c>
+      <c r="E764" s="14" t="n">
+        <v>2228109.42</v>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B765" s="15" t="n">
+        <v>838</v>
+      </c>
+      <c r="C765" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="D765" s="16" t="inlineStr">
+        <is>
+          <t>t24</t>
+        </is>
+      </c>
+      <c r="E765" s="18" t="n">
+        <v>2211242.3</v>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B766" s="10" t="n">
+        <v>838</v>
+      </c>
+      <c r="C766" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="D766" s="11" t="inlineStr">
+        <is>
+          <t>group15</t>
+        </is>
+      </c>
+      <c r="E766" s="14" t="n">
+        <v>2192613.07</v>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B767" s="15" t="n">
+        <v>838</v>
+      </c>
+      <c r="C767" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="D767" s="16" t="inlineStr">
+        <is>
+          <t>group7</t>
+        </is>
+      </c>
+      <c r="E767" s="18" t="n">
+        <v>2121372.66</v>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B768" s="10" t="n">
+        <v>838</v>
+      </c>
+      <c r="C768" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="D768" s="11" t="inlineStr">
+        <is>
+          <t>group2</t>
+        </is>
+      </c>
+      <c r="E768" s="14" t="n">
+        <v>2089821.64</v>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B769" s="15" t="n">
+        <v>838</v>
+      </c>
+      <c r="C769" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="D769" s="16" t="inlineStr">
+        <is>
+          <t>group25</t>
+        </is>
+      </c>
+      <c r="E769" s="18" t="n">
+        <v>2089663.89</v>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B770" s="10" t="n">
+        <v>838</v>
+      </c>
+      <c r="C770" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="D770" s="11" t="inlineStr">
+        <is>
+          <t>group11</t>
+        </is>
+      </c>
+      <c r="E770" s="14" t="n">
+        <v>2089651.6</v>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B771" s="15" t="n">
+        <v>838</v>
+      </c>
+      <c r="C771" s="15" t="n">
+        <v>14</v>
+      </c>
+      <c r="D771" s="16" t="inlineStr">
+        <is>
+          <t>88888888</t>
+        </is>
+      </c>
+      <c r="E771" s="18" t="n">
+        <v>2089628.97</v>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B772" s="10" t="n">
+        <v>838</v>
+      </c>
+      <c r="C772" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="D772" s="11" t="inlineStr">
+        <is>
+          <t>666666</t>
+        </is>
+      </c>
+      <c r="E772" s="14" t="n">
+        <v>1935035</v>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B773" s="15" t="n">
+        <v>838</v>
+      </c>
+      <c r="C773" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="D773" s="16" t="inlineStr">
+        <is>
+          <t>cleveregg</t>
+        </is>
+      </c>
+      <c r="E773" s="18" t="n">
+        <v>1894849.58</v>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B774" s="10" t="n">
+        <v>838</v>
+      </c>
+      <c r="C774" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="D774" s="11" t="inlineStr">
+        <is>
+          <t>newgroup18</t>
+        </is>
+      </c>
+      <c r="E774" s="14" t="n">
+        <v>1817544.97</v>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B775" s="15" t="n">
+        <v>838</v>
+      </c>
+      <c r="C775" s="15" t="n">
+        <v>18</v>
+      </c>
+      <c r="D775" s="16" t="inlineStr">
+        <is>
+          <t>deepsleep</t>
+        </is>
+      </c>
+      <c r="E775" s="18" t="n">
+        <v>1804433.26</v>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B776" s="10" t="n">
+        <v>838</v>
+      </c>
+      <c r="C776" s="10" t="n">
+        <v>19</v>
+      </c>
+      <c r="D776" s="11" t="inlineStr">
+        <is>
+          <t>tigagroup20</t>
+        </is>
+      </c>
+      <c r="E776" s="14" t="n">
+        <v>1758491.49</v>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B777" s="15" t="n">
+        <v>838</v>
+      </c>
+      <c r="C777" s="15" t="n">
+        <v>20</v>
+      </c>
+      <c r="D777" s="16" t="inlineStr">
+        <is>
+          <t>vivo50</t>
+        </is>
+      </c>
+      <c r="E777" s="18" t="n">
+        <v>1575615.57</v>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B778" s="10" t="n">
+        <v>838</v>
+      </c>
+      <c r="C778" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="D778" s="11" t="inlineStr">
+        <is>
+          <t>jit</t>
+        </is>
+      </c>
+      <c r="E778" s="14" t="n">
+        <v>1538482.49</v>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B779" s="15" t="n">
+        <v>838</v>
+      </c>
+      <c r="C779" s="15" t="n">
+        <v>22</v>
+      </c>
+      <c r="D779" s="16" t="inlineStr">
+        <is>
+          <t>aaachemicalseller</t>
+        </is>
+      </c>
+      <c r="E779" s="18" t="n">
+        <v>1503530.25</v>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B780" s="10" t="n">
+        <v>838</v>
+      </c>
+      <c r="C780" s="10" t="n">
+        <v>23</v>
+      </c>
+      <c r="D780" s="11" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E780" s="14" t="n">
+        <v>1503406.77</v>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B781" s="15" t="n">
+        <v>838</v>
+      </c>
+      <c r="C781" s="15" t="n">
+        <v>24</v>
+      </c>
+      <c r="D781" s="16" t="inlineStr">
+        <is>
+          <t>group12</t>
+        </is>
+      </c>
+      <c r="E781" s="18" t="n">
+        <v>1501679.39</v>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B782" s="10" t="n">
+        <v>838</v>
+      </c>
+      <c r="C782" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="D782" s="11" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E782" s="14" t="n">
+        <v>1499261.47</v>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B783" s="24" t="n">
+        <v>838</v>
+      </c>
+      <c r="C783" s="24" t="n">
+        <v>26</v>
+      </c>
+      <c r="D783" s="25" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="E783" s="26" t="n">
+        <v>1371261.61</v>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B784" s="10" t="n">
+        <v>838</v>
+      </c>
+      <c r="C784" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="D784" s="11" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="E784" s="14" t="n">
+        <v>1269184.47</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E757"/>
+  <autoFilter ref="A1:E784"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17217,7 +17781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S280"/>
+  <dimension ref="A1:S281"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -34915,8 +35479,69 @@
         <v>160950</v>
       </c>
     </row>
+    <row r="281">
+      <c r="A281" s="15" t="n">
+        <v>280</v>
+      </c>
+      <c r="B281" s="15" t="n">
+        <v>838</v>
+      </c>
+      <c r="C281" s="15" t="n">
+        <v>840</v>
+      </c>
+      <c r="D281" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E281" s="16" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="F281" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G281" s="17" t="n">
+        <v>86</v>
+      </c>
+      <c r="H281" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I281" s="17" t="n">
+        <v>86</v>
+      </c>
+      <c r="J281" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K281" s="17" t="n">
+        <v>86</v>
+      </c>
+      <c r="L281" s="18" t="n">
+        <v>1371261.61</v>
+      </c>
+      <c r="M281" s="18" t="n">
+        <v>1371261.61</v>
+      </c>
+      <c r="N281" s="16" t="n"/>
+      <c r="O281" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="P281" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q281" s="17" t="n">
+        <v>400</v>
+      </c>
+      <c r="R281" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="S281" s="18" t="n">
+        <v>124700</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S280"/>
+  <autoFilter ref="A1:S281"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -34927,7 +35552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N838"/>
+  <dimension ref="A1:N839"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -73520,8 +74145,54 @@
         <v>89900</v>
       </c>
     </row>
+    <row r="839">
+      <c r="A839" s="15" t="n">
+        <v>838</v>
+      </c>
+      <c r="B839" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C839" s="17" t="n">
+        <v>86</v>
+      </c>
+      <c r="D839" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E839" s="17" t="n">
+        <v>86</v>
+      </c>
+      <c r="F839" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G839" s="17" t="n">
+        <v>86</v>
+      </c>
+      <c r="H839" s="18" t="n">
+        <v>1371261.61</v>
+      </c>
+      <c r="I839" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="J839" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="K839" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="L839" s="17" t="n">
+        <v>400</v>
+      </c>
+      <c r="M839" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N839" s="18" t="n">
+        <v>124700</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N838"/>
+  <autoFilter ref="A1:N839"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -73916,7 +74587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F59"/>
+  <dimension ref="A1:F61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -75365,8 +76036,56 @@
         <v>55</v>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" s="21" t="n">
+        <v>730.66</v>
+      </c>
+      <c r="B60" s="11" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C60" s="11" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D60" s="11" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E60" s="11" t="inlineStr"/>
+      <c r="F60" s="12" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="23" t="n">
+        <v>742.75</v>
+      </c>
+      <c r="B61" s="16" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C61" s="16" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D61" s="16" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E61" s="16" t="inlineStr"/>
+      <c r="F61" s="17" t="n">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F59"/>
+  <autoFilter ref="A1:F61"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -75765,7 +76484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U28"/>
+  <dimension ref="A1:U29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -75774,7 +76493,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
@@ -77785,8 +78504,75 @@
         <v>129268.7262096691</v>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B29" s="15" t="n">
+        <v>838</v>
+      </c>
+      <c r="C29" s="18" t="n">
+        <v>1371261.61</v>
+      </c>
+      <c r="D29" s="15" t="n">
+        <v>26</v>
+      </c>
+      <c r="E29" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="F29" s="16" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="G29" s="18" t="n">
+        <v>2016083.68</v>
+      </c>
+      <c r="H29" s="23" t="n">
+        <v>55</v>
+      </c>
+      <c r="I29" s="16" t="n"/>
+      <c r="J29" s="16" t="inlineStr">
+        <is>
+          <t>mail</t>
+        </is>
+      </c>
+      <c r="K29" s="27" t="n">
+        <v>3600</v>
+      </c>
+      <c r="L29" s="27" t="n">
+        <v>200</v>
+      </c>
+      <c r="M29" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="N29" s="17" t="n">
+        <v>400</v>
+      </c>
+      <c r="O29" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="P29" s="15" t="n">
+        <v>280</v>
+      </c>
+      <c r="Q29" s="17" t="n">
+        <v>86</v>
+      </c>
+      <c r="R29" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="S29" s="17" t="n">
+        <v>86</v>
+      </c>
+      <c r="T29" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="U29" s="16" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U28"/>
+  <autoFilter ref="A1:U29"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -77797,7 +78583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E337"/>
+  <dimension ref="A1:E349"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -85450,8 +86236,280 @@
         </is>
       </c>
     </row>
+    <row r="338">
+      <c r="A338" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B338" s="10" t="n">
+        <v>838</v>
+      </c>
+      <c r="C338" s="11" t="inlineStr">
+        <is>
+          <t>Starting Cash</t>
+        </is>
+      </c>
+      <c r="D338" s="14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E338" s="11" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B339" s="15" t="n">
+        <v>838</v>
+      </c>
+      <c r="C339" s="16" t="inlineStr">
+        <is>
+          <t>Cash Sources</t>
+        </is>
+      </c>
+      <c r="D339" s="16" t="n"/>
+      <c r="E339" s="16" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B340" s="10" t="n">
+        <v>838</v>
+      </c>
+      <c r="C340" s="11" t="inlineStr">
+        <is>
+          <t>revenues</t>
+        </is>
+      </c>
+      <c r="D340" s="14" t="n">
+        <v>22345950</v>
+      </c>
+      <c r="E340" s="11" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B341" s="15" t="n">
+        <v>838</v>
+      </c>
+      <c r="C341" s="16" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D341" s="18" t="n">
+        <v>301375.37</v>
+      </c>
+      <c r="E341" s="16" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B342" s="10" t="n">
+        <v>838</v>
+      </c>
+      <c r="C342" s="11" t="inlineStr">
+        <is>
+          <t>Cash Uses</t>
+        </is>
+      </c>
+      <c r="D342" s="11" t="n"/>
+      <c r="E342" s="11" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B343" s="15" t="n">
+        <v>838</v>
+      </c>
+      <c r="C343" s="16" t="inlineStr">
+        <is>
+          <t>outbound shipping</t>
+        </is>
+      </c>
+      <c r="D343" s="18" t="n">
+        <v>-2311650</v>
+      </c>
+      <c r="E343" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B344" s="10" t="n">
+        <v>838</v>
+      </c>
+      <c r="C344" s="11" t="inlineStr">
+        <is>
+          <t>inbound shipping</t>
+        </is>
+      </c>
+      <c r="D344" s="14" t="n">
+        <v>-1560000</v>
+      </c>
+      <c r="E344" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B345" s="15" t="n">
+        <v>838</v>
+      </c>
+      <c r="C345" s="16" t="inlineStr">
+        <is>
+          <t>FGI holding</t>
+        </is>
+      </c>
+      <c r="D345" s="18" t="n">
+        <v>-21895.45</v>
+      </c>
+      <c r="E345" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B346" s="10" t="n">
+        <v>838</v>
+      </c>
+      <c r="C346" s="11" t="inlineStr">
+        <is>
+          <t>add capacity</t>
+        </is>
+      </c>
+      <c r="D346" s="14" t="n">
+        <v>-1749840.87</v>
+      </c>
+      <c r="E346" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B347" s="15" t="n">
+        <v>838</v>
+      </c>
+      <c r="C347" s="16" t="inlineStr">
+        <is>
+          <t>Pipeline inventory holding</t>
+        </is>
+      </c>
+      <c r="D347" s="18" t="n">
+        <v>-29677.45</v>
+      </c>
+      <c r="E347" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B348" s="10" t="n">
+        <v>838</v>
+      </c>
+      <c r="C348" s="11" t="inlineStr">
+        <is>
+          <t>production</t>
+        </is>
+      </c>
+      <c r="D348" s="14" t="n">
+        <v>-16103000</v>
+      </c>
+      <c r="E348" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T13:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B349" s="15" t="n">
+        <v>838</v>
+      </c>
+      <c r="C349" s="16" t="inlineStr">
+        <is>
+          <t>Cash Balance</t>
+        </is>
+      </c>
+      <c r="D349" s="18" t="n">
+        <v>1371261.61</v>
+      </c>
+      <c r="E349" s="16" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E337"/>
+  <autoFilter ref="A1:E349"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update game data: day 839, cash 1483299.49, 3-day period 280
</commit_message>
<xml_diff>
--- a/data/supply_chain_game.xlsx
+++ b/data/supply_chain_game.xlsx
@@ -21,15 +21,15 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$281</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$839</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$840</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'资金构成_旧版'!$A$1:$C$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'运营参数_旧版'!$A$9:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$63</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'排行榜_旧版'!$A$1:$C$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$29</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$349</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$361</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'运营参数'!$A$1:$J$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$784</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$811</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -590,7 +590,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-06T13:56:02+08:00</t>
+          <t>2026-09-06T14:11:15+08:00</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>838</v>
+        <v>839</v>
       </c>
     </row>
     <row r="7">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>622</v>
+        <v>621</v>
       </c>
     </row>
     <row r="8">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>1371261.61</v>
+        <v>1483299.49</v>
       </c>
     </row>
     <row r="11">
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>2016083.68</v>
+        <v>1818968.87</v>
       </c>
     </row>
     <row r="15"/>
@@ -786,7 +786,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>3</v>
+        <v>139</v>
       </c>
     </row>
     <row r="25">
@@ -796,7 +796,7 @@
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>400</v>
+        <v>200</v>
       </c>
     </row>
     <row r="26">
@@ -858,7 +858,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>86</v>
+        <v>150</v>
       </c>
     </row>
     <row r="33">
@@ -878,7 +878,7 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>86</v>
+        <v>150</v>
       </c>
     </row>
     <row r="35">
@@ -898,7 +898,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>86</v>
+        <v>150</v>
       </c>
     </row>
     <row r="37">
@@ -906,6 +906,9 @@
         <is>
           <t>周期现金变动</t>
         </is>
+      </c>
+      <c r="B37" s="4" t="n">
+        <v>90239.45053751022</v>
       </c>
     </row>
     <row r="38"/>
@@ -967,7 +970,7 @@
         </is>
       </c>
       <c r="B44" s="4" t="n">
-        <v>154144.7997774337</v>
+        <v>156595.1816159203</v>
       </c>
     </row>
     <row r="45"/>
@@ -1289,7 +1292,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E784"/>
+  <dimension ref="A1:E811"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -17769,8 +17772,575 @@
         <v>1269184.47</v>
       </c>
     </row>
+    <row r="785">
+      <c r="A785" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:11:15+08:00</t>
+        </is>
+      </c>
+      <c r="B785" s="15" t="n">
+        <v>839</v>
+      </c>
+      <c r="C785" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D785" s="16" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="E785" s="18" t="n">
+        <v>3302268.36</v>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:11:15+08:00</t>
+        </is>
+      </c>
+      <c r="B786" s="10" t="n">
+        <v>839</v>
+      </c>
+      <c r="C786" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D786" s="11" t="inlineStr">
+        <is>
+          <t>montesquieu</t>
+        </is>
+      </c>
+      <c r="E786" s="14" t="n">
+        <v>2564442.6</v>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:11:15+08:00</t>
+        </is>
+      </c>
+      <c r="B787" s="15" t="n">
+        <v>839</v>
+      </c>
+      <c r="C787" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D787" s="16" t="inlineStr">
+        <is>
+          <t>nicetry</t>
+        </is>
+      </c>
+      <c r="E787" s="18" t="n">
+        <v>2270720.02</v>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:11:15+08:00</t>
+        </is>
+      </c>
+      <c r="B788" s="10" t="n">
+        <v>839</v>
+      </c>
+      <c r="C788" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D788" s="11" t="inlineStr">
+        <is>
+          <t>group8</t>
+        </is>
+      </c>
+      <c r="E788" s="14" t="n">
+        <v>2270261.14</v>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:11:15+08:00</t>
+        </is>
+      </c>
+      <c r="B789" s="15" t="n">
+        <v>839</v>
+      </c>
+      <c r="C789" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="D789" s="16" t="inlineStr">
+        <is>
+          <t>group7</t>
+        </is>
+      </c>
+      <c r="E789" s="18" t="n">
+        <v>2202465.11</v>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:11:15+08:00</t>
+        </is>
+      </c>
+      <c r="B790" s="10" t="n">
+        <v>839</v>
+      </c>
+      <c r="C790" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="D790" s="11" t="inlineStr">
+        <is>
+          <t>t24</t>
+        </is>
+      </c>
+      <c r="E790" s="14" t="n">
+        <v>2092067.43</v>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:11:15+08:00</t>
+        </is>
+      </c>
+      <c r="B791" s="15" t="n">
+        <v>839</v>
+      </c>
+      <c r="C791" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="D791" s="16" t="inlineStr">
+        <is>
+          <t>teamhlly</t>
+        </is>
+      </c>
+      <c r="E791" s="18" t="n">
+        <v>2090771.66</v>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:11:15+08:00</t>
+        </is>
+      </c>
+      <c r="B792" s="10" t="n">
+        <v>839</v>
+      </c>
+      <c r="C792" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="D792" s="11" t="inlineStr">
+        <is>
+          <t>group2</t>
+        </is>
+      </c>
+      <c r="E792" s="14" t="n">
+        <v>2090271.12</v>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:11:15+08:00</t>
+        </is>
+      </c>
+      <c r="B793" s="15" t="n">
+        <v>839</v>
+      </c>
+      <c r="C793" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="D793" s="16" t="inlineStr">
+        <is>
+          <t>group25</t>
+        </is>
+      </c>
+      <c r="E793" s="18" t="n">
+        <v>2090113.33</v>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:11:15+08:00</t>
+        </is>
+      </c>
+      <c r="B794" s="10" t="n">
+        <v>839</v>
+      </c>
+      <c r="C794" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="D794" s="11" t="inlineStr">
+        <is>
+          <t>group11</t>
+        </is>
+      </c>
+      <c r="E794" s="14" t="n">
+        <v>2090101.04</v>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:11:15+08:00</t>
+        </is>
+      </c>
+      <c r="B795" s="15" t="n">
+        <v>839</v>
+      </c>
+      <c r="C795" s="15" t="n">
+        <v>11</v>
+      </c>
+      <c r="D795" s="16" t="inlineStr">
+        <is>
+          <t>88888888</t>
+        </is>
+      </c>
+      <c r="E795" s="18" t="n">
+        <v>2090078.41</v>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:11:15+08:00</t>
+        </is>
+      </c>
+      <c r="B796" s="10" t="n">
+        <v>839</v>
+      </c>
+      <c r="C796" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="D796" s="11" t="inlineStr">
+        <is>
+          <t>666666</t>
+        </is>
+      </c>
+      <c r="E796" s="14" t="n">
+        <v>2087530.76</v>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:11:15+08:00</t>
+        </is>
+      </c>
+      <c r="B797" s="15" t="n">
+        <v>839</v>
+      </c>
+      <c r="C797" s="15" t="n">
+        <v>13</v>
+      </c>
+      <c r="D797" s="16" t="inlineStr">
+        <is>
+          <t>group9</t>
+        </is>
+      </c>
+      <c r="E797" s="18" t="n">
+        <v>2050979.26</v>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:11:15+08:00</t>
+        </is>
+      </c>
+      <c r="B798" s="10" t="n">
+        <v>839</v>
+      </c>
+      <c r="C798" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="D798" s="11" t="inlineStr">
+        <is>
+          <t>group14</t>
+        </is>
+      </c>
+      <c r="E798" s="14" t="n">
+        <v>2017923.47</v>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:11:15+08:00</t>
+        </is>
+      </c>
+      <c r="B799" s="15" t="n">
+        <v>839</v>
+      </c>
+      <c r="C799" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="D799" s="16" t="inlineStr">
+        <is>
+          <t>cleveregg</t>
+        </is>
+      </c>
+      <c r="E799" s="18" t="n">
+        <v>2007014.35</v>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:11:15+08:00</t>
+        </is>
+      </c>
+      <c r="B800" s="10" t="n">
+        <v>839</v>
+      </c>
+      <c r="C800" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="D800" s="11" t="inlineStr">
+        <is>
+          <t>group15</t>
+        </is>
+      </c>
+      <c r="E800" s="14" t="n">
+        <v>1976616.92</v>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:11:15+08:00</t>
+        </is>
+      </c>
+      <c r="B801" s="15" t="n">
+        <v>839</v>
+      </c>
+      <c r="C801" s="15" t="n">
+        <v>17</v>
+      </c>
+      <c r="D801" s="16" t="inlineStr">
+        <is>
+          <t>tigagroup20</t>
+        </is>
+      </c>
+      <c r="E801" s="18" t="n">
+        <v>1870565.56</v>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:11:15+08:00</t>
+        </is>
+      </c>
+      <c r="B802" s="10" t="n">
+        <v>839</v>
+      </c>
+      <c r="C802" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="D802" s="11" t="inlineStr">
+        <is>
+          <t>deepsleep</t>
+        </is>
+      </c>
+      <c r="E802" s="14" t="n">
+        <v>1821507.37</v>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:11:15+08:00</t>
+        </is>
+      </c>
+      <c r="B803" s="15" t="n">
+        <v>839</v>
+      </c>
+      <c r="C803" s="15" t="n">
+        <v>19</v>
+      </c>
+      <c r="D803" s="16" t="inlineStr">
+        <is>
+          <t>vivo50</t>
+        </is>
+      </c>
+      <c r="E803" s="18" t="n">
+        <v>1572618.97</v>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:11:15+08:00</t>
+        </is>
+      </c>
+      <c r="B804" s="10" t="n">
+        <v>839</v>
+      </c>
+      <c r="C804" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="D804" s="11" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E804" s="14" t="n">
+        <v>1541176.37</v>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:11:15+08:00</t>
+        </is>
+      </c>
+      <c r="B805" s="15" t="n">
+        <v>839</v>
+      </c>
+      <c r="C805" s="15" t="n">
+        <v>21</v>
+      </c>
+      <c r="D805" s="16" t="inlineStr">
+        <is>
+          <t>jit</t>
+        </is>
+      </c>
+      <c r="E805" s="18" t="n">
+        <v>1538733.19</v>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:11:15+08:00</t>
+        </is>
+      </c>
+      <c r="B806" s="10" t="n">
+        <v>839</v>
+      </c>
+      <c r="C806" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="D806" s="11" t="inlineStr">
+        <is>
+          <t>aaachemicalseller</t>
+        </is>
+      </c>
+      <c r="E806" s="14" t="n">
+        <v>1503799.78</v>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:11:15+08:00</t>
+        </is>
+      </c>
+      <c r="B807" s="15" t="n">
+        <v>839</v>
+      </c>
+      <c r="C807" s="15" t="n">
+        <v>23</v>
+      </c>
+      <c r="D807" s="16" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E807" s="18" t="n">
+        <v>1503689.39</v>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:11:15+08:00</t>
+        </is>
+      </c>
+      <c r="B808" s="10" t="n">
+        <v>839</v>
+      </c>
+      <c r="C808" s="10" t="n">
+        <v>24</v>
+      </c>
+      <c r="D808" s="11" t="inlineStr">
+        <is>
+          <t>group12</t>
+        </is>
+      </c>
+      <c r="E808" s="14" t="n">
+        <v>1498663.47</v>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:11:15+08:00</t>
+        </is>
+      </c>
+      <c r="B809" s="24" t="n">
+        <v>839</v>
+      </c>
+      <c r="C809" s="24" t="n">
+        <v>25</v>
+      </c>
+      <c r="D809" s="25" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="E809" s="26" t="n">
+        <v>1483299.49</v>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:11:15+08:00</t>
+        </is>
+      </c>
+      <c r="B810" s="10" t="n">
+        <v>839</v>
+      </c>
+      <c r="C810" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="D810" s="11" t="inlineStr">
+        <is>
+          <t>newgroup18</t>
+        </is>
+      </c>
+      <c r="E810" s="14" t="n">
+        <v>1468244.54</v>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:11:15+08:00</t>
+        </is>
+      </c>
+      <c r="B811" s="15" t="n">
+        <v>839</v>
+      </c>
+      <c r="C811" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="D811" s="16" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="E811" s="18" t="n">
+        <v>1340964.81</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E784"/>
+  <autoFilter ref="A1:E811"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -35490,7 +36060,7 @@
         <v>840</v>
       </c>
       <c r="D281" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E281" s="16" t="inlineStr">
         <is>
@@ -35503,41 +36073,43 @@
         </is>
       </c>
       <c r="G281" s="17" t="n">
-        <v>86</v>
+        <v>150</v>
       </c>
       <c r="H281" s="17" t="n">
         <v>0</v>
       </c>
       <c r="I281" s="17" t="n">
-        <v>86</v>
+        <v>150</v>
       </c>
       <c r="J281" s="19" t="n">
         <v>1</v>
       </c>
       <c r="K281" s="17" t="n">
-        <v>86</v>
+        <v>150</v>
       </c>
       <c r="L281" s="18" t="n">
-        <v>1371261.61</v>
+        <v>1393060.03946249</v>
       </c>
       <c r="M281" s="18" t="n">
-        <v>1371261.61</v>
-      </c>
-      <c r="N281" s="16" t="n"/>
+        <v>1483299.49</v>
+      </c>
+      <c r="N281" s="18" t="n">
+        <v>90239.45053751022</v>
+      </c>
       <c r="O281" s="17" t="n">
-        <v>3</v>
+        <v>139</v>
       </c>
       <c r="P281" s="17" t="n">
-        <v>3</v>
+        <v>71</v>
       </c>
       <c r="Q281" s="17" t="n">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="R281" s="17" t="n">
         <v>200</v>
       </c>
       <c r="S281" s="18" t="n">
-        <v>124700</v>
+        <v>217500</v>
       </c>
     </row>
   </sheetData>
@@ -35552,7 +36124,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N839"/>
+  <dimension ref="A1:N840"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -74191,8 +74763,54 @@
         <v>124700</v>
       </c>
     </row>
+    <row r="840">
+      <c r="A840" s="10" t="n">
+        <v>839</v>
+      </c>
+      <c r="B840" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C840" s="12" t="n">
+        <v>64</v>
+      </c>
+      <c r="D840" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E840" s="12" t="n">
+        <v>64</v>
+      </c>
+      <c r="F840" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G840" s="12" t="n">
+        <v>64</v>
+      </c>
+      <c r="H840" s="14" t="n">
+        <v>1483299.49</v>
+      </c>
+      <c r="I840" s="12" t="n">
+        <v>139</v>
+      </c>
+      <c r="J840" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K840" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="L840" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="M840" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N840" s="14" t="n">
+        <v>92800</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N839"/>
+  <autoFilter ref="A1:N840"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -74587,7 +75205,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F61"/>
+  <dimension ref="A1:F63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -76084,8 +76702,56 @@
         <v>55</v>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" s="21" t="n">
+        <v>730.66</v>
+      </c>
+      <c r="B62" s="11" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C62" s="11" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D62" s="11" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E62" s="11" t="inlineStr"/>
+      <c r="F62" s="12" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="23" t="n">
+        <v>742.75</v>
+      </c>
+      <c r="B63" s="16" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C63" s="16" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D63" s="16" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E63" s="16" t="inlineStr"/>
+      <c r="F63" s="17" t="n">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F61"/>
+  <autoFilter ref="A1:F63"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -76484,7 +77150,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U29"/>
+  <dimension ref="A1:U30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -76493,7 +77159,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
@@ -78571,8 +79237,77 @@
       </c>
       <c r="U29" s="16" t="n"/>
     </row>
+    <row r="30">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:11:15+08:00</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="n">
+        <v>839</v>
+      </c>
+      <c r="C30" s="14" t="n">
+        <v>1483299.49</v>
+      </c>
+      <c r="D30" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="E30" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="F30" s="11" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="G30" s="14" t="n">
+        <v>1818968.87</v>
+      </c>
+      <c r="H30" s="21" t="n">
+        <v>55</v>
+      </c>
+      <c r="I30" s="11" t="n"/>
+      <c r="J30" s="11" t="inlineStr">
+        <is>
+          <t>mail</t>
+        </is>
+      </c>
+      <c r="K30" s="22" t="n">
+        <v>3600</v>
+      </c>
+      <c r="L30" s="22" t="n">
+        <v>200</v>
+      </c>
+      <c r="M30" s="12" t="n">
+        <v>139</v>
+      </c>
+      <c r="N30" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="O30" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="P30" s="10" t="n">
+        <v>280</v>
+      </c>
+      <c r="Q30" s="12" t="n">
+        <v>150</v>
+      </c>
+      <c r="R30" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S30" s="12" t="n">
+        <v>150</v>
+      </c>
+      <c r="T30" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="U30" s="14" t="n">
+        <v>90239.45053751022</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U29"/>
+  <autoFilter ref="A1:U30"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -78583,7 +79318,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E349"/>
+  <dimension ref="A1:E361"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -86508,8 +87243,280 @@
         </is>
       </c>
     </row>
+    <row r="350">
+      <c r="A350" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:11:15+08:00</t>
+        </is>
+      </c>
+      <c r="B350" s="10" t="n">
+        <v>839</v>
+      </c>
+      <c r="C350" s="11" t="inlineStr">
+        <is>
+          <t>Starting Cash</t>
+        </is>
+      </c>
+      <c r="D350" s="14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E350" s="11" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:11:15+08:00</t>
+        </is>
+      </c>
+      <c r="B351" s="15" t="n">
+        <v>839</v>
+      </c>
+      <c r="C351" s="16" t="inlineStr">
+        <is>
+          <t>Cash Sources</t>
+        </is>
+      </c>
+      <c r="D351" s="16" t="n"/>
+      <c r="E351" s="16" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:11:15+08:00</t>
+        </is>
+      </c>
+      <c r="B352" s="10" t="n">
+        <v>839</v>
+      </c>
+      <c r="C352" s="11" t="inlineStr">
+        <is>
+          <t>revenues</t>
+        </is>
+      </c>
+      <c r="D352" s="14" t="n">
+        <v>22470650</v>
+      </c>
+      <c r="E352" s="11" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:11:15+08:00</t>
+        </is>
+      </c>
+      <c r="B353" s="15" t="n">
+        <v>839</v>
+      </c>
+      <c r="C353" s="16" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D353" s="18" t="n">
+        <v>301718.34</v>
+      </c>
+      <c r="E353" s="16" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:11:15+08:00</t>
+        </is>
+      </c>
+      <c r="B354" s="10" t="n">
+        <v>839</v>
+      </c>
+      <c r="C354" s="11" t="inlineStr">
+        <is>
+          <t>Cash Uses</t>
+        </is>
+      </c>
+      <c r="D354" s="11" t="n"/>
+      <c r="E354" s="11" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:11:15+08:00</t>
+        </is>
+      </c>
+      <c r="B355" s="15" t="n">
+        <v>839</v>
+      </c>
+      <c r="C355" s="16" t="inlineStr">
+        <is>
+          <t>outbound shipping</t>
+        </is>
+      </c>
+      <c r="D355" s="18" t="n">
+        <v>-2324550</v>
+      </c>
+      <c r="E355" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:11:15+08:00</t>
+        </is>
+      </c>
+      <c r="B356" s="10" t="n">
+        <v>839</v>
+      </c>
+      <c r="C356" s="11" t="inlineStr">
+        <is>
+          <t>inbound shipping</t>
+        </is>
+      </c>
+      <c r="D356" s="14" t="n">
+        <v>-1560000</v>
+      </c>
+      <c r="E356" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:11:15+08:00</t>
+        </is>
+      </c>
+      <c r="B357" s="15" t="n">
+        <v>839</v>
+      </c>
+      <c r="C357" s="16" t="inlineStr">
+        <is>
+          <t>FGI holding</t>
+        </is>
+      </c>
+      <c r="D357" s="18" t="n">
+        <v>-21910.87</v>
+      </c>
+      <c r="E357" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:11:15+08:00</t>
+        </is>
+      </c>
+      <c r="B358" s="10" t="n">
+        <v>839</v>
+      </c>
+      <c r="C358" s="11" t="inlineStr">
+        <is>
+          <t>add capacity</t>
+        </is>
+      </c>
+      <c r="D358" s="14" t="n">
+        <v>-1749840.87</v>
+      </c>
+      <c r="E358" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:11:15+08:00</t>
+        </is>
+      </c>
+      <c r="B359" s="15" t="n">
+        <v>839</v>
+      </c>
+      <c r="C359" s="16" t="inlineStr">
+        <is>
+          <t>Pipeline inventory holding</t>
+        </is>
+      </c>
+      <c r="D359" s="18" t="n">
+        <v>-29767.12</v>
+      </c>
+      <c r="E359" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:11:15+08:00</t>
+        </is>
+      </c>
+      <c r="B360" s="10" t="n">
+        <v>839</v>
+      </c>
+      <c r="C360" s="11" t="inlineStr">
+        <is>
+          <t>production</t>
+        </is>
+      </c>
+      <c r="D360" s="14" t="n">
+        <v>-16103000</v>
+      </c>
+      <c r="E360" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:11:15+08:00</t>
+        </is>
+      </c>
+      <c r="B361" s="15" t="n">
+        <v>839</v>
+      </c>
+      <c r="C361" s="16" t="inlineStr">
+        <is>
+          <t>Cash Balance</t>
+        </is>
+      </c>
+      <c r="D361" s="18" t="n">
+        <v>1483299.49</v>
+      </c>
+      <c r="E361" s="16" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E349"/>
+  <autoFilter ref="A1:E361"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update game data: day 841, cash 1552834.52, 3-day period 281
</commit_message>
<xml_diff>
--- a/data/supply_chain_game.xlsx
+++ b/data/supply_chain_game.xlsx
@@ -20,16 +20,16 @@
     <sheet name="排行榜" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$281</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$840</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$282</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$842</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'资金构成_旧版'!$A$1:$C$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'运营参数_旧版'!$A$9:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$65</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'排行榜_旧版'!$A$1:$C$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$30</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$361</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$373</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'运营参数'!$A$1:$J$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$811</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$838</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -590,7 +590,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-06T14:11:15+08:00</t>
+          <t>2026-09-06T14:26:02+08:00</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>839</v>
+        <v>841</v>
       </c>
     </row>
     <row r="7">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>621</v>
+        <v>619</v>
       </c>
     </row>
     <row r="8">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>1483299.49</v>
+        <v>1552834.52</v>
       </c>
     </row>
     <row r="11">
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>1818968.87</v>
+        <v>1751096.24</v>
       </c>
     </row>
     <row r="15"/>
@@ -786,7 +786,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>139</v>
+        <v>200</v>
       </c>
     </row>
     <row r="25">
@@ -796,7 +796,7 @@
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -824,7 +824,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>280</v>
+        <v>281</v>
       </c>
     </row>
     <row r="30">
@@ -835,7 +835,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>838–840</t>
+          <t>841–843</t>
         </is>
       </c>
     </row>
@@ -858,7 +858,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>150</v>
+        <v>53</v>
       </c>
     </row>
     <row r="33">
@@ -878,7 +878,7 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>150</v>
+        <v>53</v>
       </c>
     </row>
     <row r="35">
@@ -898,7 +898,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>150</v>
+        <v>53</v>
       </c>
     </row>
     <row r="37">
@@ -906,9 +906,6 @@
         <is>
           <t>周期现金变动</t>
         </is>
-      </c>
-      <c r="B37" s="4" t="n">
-        <v>90239.45053751022</v>
       </c>
     </row>
     <row r="38"/>
@@ -926,7 +923,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>279</v>
+        <v>280</v>
       </c>
     </row>
     <row r="41">
@@ -937,7 +934,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>835–837</t>
+          <t>838–840</t>
         </is>
       </c>
     </row>
@@ -949,7 +946,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>169.0 / 58.0 / 111.0</t>
+          <t>236.0 / 0.0 / 236.0</t>
         </is>
       </c>
     </row>
@@ -960,7 +957,7 @@
         </is>
       </c>
       <c r="B43" s="8" t="n">
-        <v>0.6568047337278107</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44">
@@ -970,7 +967,7 @@
         </is>
       </c>
       <c r="B44" s="4" t="n">
-        <v>156595.1816159203</v>
+        <v>195537.1141997681</v>
       </c>
     </row>
     <row r="45"/>
@@ -1292,7 +1289,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E811"/>
+  <dimension ref="A1:E838"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -18339,8 +18336,575 @@
         <v>1340964.81</v>
       </c>
     </row>
+    <row r="812">
+      <c r="A812" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B812" s="10" t="n">
+        <v>841</v>
+      </c>
+      <c r="C812" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D812" s="11" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="E812" s="14" t="n">
+        <v>3303930.76</v>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B813" s="15" t="n">
+        <v>841</v>
+      </c>
+      <c r="C813" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D813" s="16" t="inlineStr">
+        <is>
+          <t>nicetry</t>
+        </is>
+      </c>
+      <c r="E813" s="18" t="n">
+        <v>2354947.19</v>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B814" s="10" t="n">
+        <v>841</v>
+      </c>
+      <c r="C814" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D814" s="11" t="inlineStr">
+        <is>
+          <t>montesquieu</t>
+        </is>
+      </c>
+      <c r="E814" s="14" t="n">
+        <v>2349090.82</v>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B815" s="15" t="n">
+        <v>841</v>
+      </c>
+      <c r="C815" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D815" s="16" t="inlineStr">
+        <is>
+          <t>group2</t>
+        </is>
+      </c>
+      <c r="E815" s="18" t="n">
+        <v>2221186.6</v>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B816" s="10" t="n">
+        <v>841</v>
+      </c>
+      <c r="C816" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="D816" s="11" t="inlineStr">
+        <is>
+          <t>group25</t>
+        </is>
+      </c>
+      <c r="E816" s="14" t="n">
+        <v>2221028.73</v>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B817" s="15" t="n">
+        <v>841</v>
+      </c>
+      <c r="C817" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="D817" s="16" t="inlineStr">
+        <is>
+          <t>group11</t>
+        </is>
+      </c>
+      <c r="E817" s="18" t="n">
+        <v>2221016.43</v>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B818" s="10" t="n">
+        <v>841</v>
+      </c>
+      <c r="C818" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="D818" s="11" t="inlineStr">
+        <is>
+          <t>88888888</t>
+        </is>
+      </c>
+      <c r="E818" s="14" t="n">
+        <v>2220993.79</v>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B819" s="15" t="n">
+        <v>841</v>
+      </c>
+      <c r="C819" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="D819" s="16" t="inlineStr">
+        <is>
+          <t>group7</t>
+        </is>
+      </c>
+      <c r="E819" s="18" t="n">
+        <v>2203608.71</v>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B820" s="10" t="n">
+        <v>841</v>
+      </c>
+      <c r="C820" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="D820" s="11" t="inlineStr">
+        <is>
+          <t>t24</t>
+        </is>
+      </c>
+      <c r="E820" s="14" t="n">
+        <v>2161964.41</v>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B821" s="15" t="n">
+        <v>841</v>
+      </c>
+      <c r="C821" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="D821" s="16" t="inlineStr">
+        <is>
+          <t>teamhlly</t>
+        </is>
+      </c>
+      <c r="E821" s="18" t="n">
+        <v>2160545.66</v>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B822" s="10" t="n">
+        <v>841</v>
+      </c>
+      <c r="C822" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="D822" s="11" t="inlineStr">
+        <is>
+          <t>666666</t>
+        </is>
+      </c>
+      <c r="E822" s="14" t="n">
+        <v>2157347.11</v>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B823" s="15" t="n">
+        <v>841</v>
+      </c>
+      <c r="C823" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="D823" s="16" t="inlineStr">
+        <is>
+          <t>group8</t>
+        </is>
+      </c>
+      <c r="E823" s="18" t="n">
+        <v>2054874.4</v>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B824" s="10" t="n">
+        <v>841</v>
+      </c>
+      <c r="C824" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="D824" s="11" t="inlineStr">
+        <is>
+          <t>group9</t>
+        </is>
+      </c>
+      <c r="E824" s="14" t="n">
+        <v>2051866.31</v>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B825" s="15" t="n">
+        <v>841</v>
+      </c>
+      <c r="C825" s="15" t="n">
+        <v>14</v>
+      </c>
+      <c r="D825" s="16" t="inlineStr">
+        <is>
+          <t>group14</t>
+        </is>
+      </c>
+      <c r="E825" s="18" t="n">
+        <v>2018858.52</v>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B826" s="10" t="n">
+        <v>841</v>
+      </c>
+      <c r="C826" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="D826" s="11" t="inlineStr">
+        <is>
+          <t>group15</t>
+        </is>
+      </c>
+      <c r="E826" s="14" t="n">
+        <v>1977524.14</v>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B827" s="15" t="n">
+        <v>841</v>
+      </c>
+      <c r="C827" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="D827" s="16" t="inlineStr">
+        <is>
+          <t>tigagroup20</t>
+        </is>
+      </c>
+      <c r="E827" s="18" t="n">
+        <v>1940202.61</v>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B828" s="10" t="n">
+        <v>841</v>
+      </c>
+      <c r="C828" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="D828" s="11" t="inlineStr">
+        <is>
+          <t>deepsleep</t>
+        </is>
+      </c>
+      <c r="E828" s="14" t="n">
+        <v>1843140</v>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B829" s="15" t="n">
+        <v>841</v>
+      </c>
+      <c r="C829" s="15" t="n">
+        <v>18</v>
+      </c>
+      <c r="D829" s="16" t="inlineStr">
+        <is>
+          <t>cleveregg</t>
+        </is>
+      </c>
+      <c r="E829" s="18" t="n">
+        <v>1825178.47</v>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B830" s="10" t="n">
+        <v>841</v>
+      </c>
+      <c r="C830" s="10" t="n">
+        <v>19</v>
+      </c>
+      <c r="D830" s="11" t="inlineStr">
+        <is>
+          <t>jit</t>
+        </is>
+      </c>
+      <c r="E830" s="14" t="n">
+        <v>1669250.95</v>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B831" s="15" t="n">
+        <v>841</v>
+      </c>
+      <c r="C831" s="15" t="n">
+        <v>20</v>
+      </c>
+      <c r="D831" s="16" t="inlineStr">
+        <is>
+          <t>vivo50</t>
+        </is>
+      </c>
+      <c r="E831" s="18" t="n">
+        <v>1620106.35</v>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B832" s="24" t="n">
+        <v>841</v>
+      </c>
+      <c r="C832" s="24" t="n">
+        <v>21</v>
+      </c>
+      <c r="D832" s="25" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="E832" s="26" t="n">
+        <v>1552834.52</v>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B833" s="15" t="n">
+        <v>841</v>
+      </c>
+      <c r="C833" s="15" t="n">
+        <v>22</v>
+      </c>
+      <c r="D833" s="16" t="inlineStr">
+        <is>
+          <t>group12</t>
+        </is>
+      </c>
+      <c r="E833" s="18" t="n">
+        <v>1546112.22</v>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B834" s="10" t="n">
+        <v>841</v>
+      </c>
+      <c r="C834" s="10" t="n">
+        <v>23</v>
+      </c>
+      <c r="D834" s="11" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E834" s="14" t="n">
+        <v>1541761.52</v>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B835" s="15" t="n">
+        <v>841</v>
+      </c>
+      <c r="C835" s="15" t="n">
+        <v>24</v>
+      </c>
+      <c r="D835" s="16" t="inlineStr">
+        <is>
+          <t>newgroup18</t>
+        </is>
+      </c>
+      <c r="E835" s="18" t="n">
+        <v>1537636.63</v>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B836" s="10" t="n">
+        <v>841</v>
+      </c>
+      <c r="C836" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="D836" s="11" t="inlineStr">
+        <is>
+          <t>aaachemicalseller</t>
+        </is>
+      </c>
+      <c r="E836" s="14" t="n">
+        <v>1504366.14</v>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B837" s="15" t="n">
+        <v>841</v>
+      </c>
+      <c r="C837" s="15" t="n">
+        <v>26</v>
+      </c>
+      <c r="D837" s="16" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E837" s="18" t="n">
+        <v>1468526.11</v>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B838" s="10" t="n">
+        <v>841</v>
+      </c>
+      <c r="C838" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="D838" s="11" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="E838" s="14" t="n">
+        <v>1236477.74</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E811"/>
+  <autoFilter ref="A1:E838"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -18351,7 +18915,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S281"/>
+  <dimension ref="A1:S282"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -36060,11 +36624,11 @@
         <v>840</v>
       </c>
       <c r="D281" s="15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E281" s="16" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="F281" s="16" t="inlineStr">
@@ -36073,34 +36637,34 @@
         </is>
       </c>
       <c r="G281" s="17" t="n">
-        <v>150</v>
+        <v>236</v>
       </c>
       <c r="H281" s="17" t="n">
         <v>0</v>
       </c>
       <c r="I281" s="17" t="n">
-        <v>150</v>
+        <v>236</v>
       </c>
       <c r="J281" s="19" t="n">
         <v>1</v>
       </c>
       <c r="K281" s="17" t="n">
-        <v>150</v>
+        <v>236</v>
       </c>
       <c r="L281" s="18" t="n">
-        <v>1393060.03946249</v>
+        <v>1288061.607380919</v>
       </c>
       <c r="M281" s="18" t="n">
-        <v>1483299.49</v>
+        <v>1483598.721580687</v>
       </c>
       <c r="N281" s="18" t="n">
-        <v>90239.45053751022</v>
+        <v>195537.1141997681</v>
       </c>
       <c r="O281" s="17" t="n">
-        <v>139</v>
+        <v>53</v>
       </c>
       <c r="P281" s="17" t="n">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="Q281" s="17" t="n">
         <v>200</v>
@@ -36109,11 +36673,72 @@
         <v>200</v>
       </c>
       <c r="S281" s="18" t="n">
-        <v>217500</v>
+        <v>342200</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="10" t="n">
+        <v>281</v>
+      </c>
+      <c r="B282" s="10" t="n">
+        <v>841</v>
+      </c>
+      <c r="C282" s="10" t="n">
+        <v>843</v>
+      </c>
+      <c r="D282" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E282" s="11" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="F282" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G282" s="12" t="n">
+        <v>53</v>
+      </c>
+      <c r="H282" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I282" s="12" t="n">
+        <v>53</v>
+      </c>
+      <c r="J282" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K282" s="12" t="n">
+        <v>53</v>
+      </c>
+      <c r="L282" s="14" t="n">
+        <v>1552834.52</v>
+      </c>
+      <c r="M282" s="14" t="n">
+        <v>1552834.52</v>
+      </c>
+      <c r="N282" s="11" t="n"/>
+      <c r="O282" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="P282" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="Q282" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R282" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="S282" s="14" t="n">
+        <v>76850</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S281"/>
+  <autoFilter ref="A1:S282"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -36124,7 +36749,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N840"/>
+  <dimension ref="A1:N842"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -74809,8 +75434,100 @@
         <v>92800</v>
       </c>
     </row>
+    <row r="841">
+      <c r="A841" s="15" t="n">
+        <v>840</v>
+      </c>
+      <c r="B841" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C841" s="17" t="n">
+        <v>86</v>
+      </c>
+      <c r="D841" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E841" s="17" t="n">
+        <v>86</v>
+      </c>
+      <c r="F841" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G841" s="17" t="n">
+        <v>86</v>
+      </c>
+      <c r="H841" s="18" t="n">
+        <v>1483598.721580687</v>
+      </c>
+      <c r="I841" s="17" t="n">
+        <v>53</v>
+      </c>
+      <c r="J841" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K841" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="L841" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="M841" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N841" s="18" t="n">
+        <v>124700</v>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" s="10" t="n">
+        <v>841</v>
+      </c>
+      <c r="B842" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C842" s="12" t="n">
+        <v>53</v>
+      </c>
+      <c r="D842" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E842" s="12" t="n">
+        <v>53</v>
+      </c>
+      <c r="F842" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G842" s="12" t="n">
+        <v>53</v>
+      </c>
+      <c r="H842" s="14" t="n">
+        <v>1552834.52</v>
+      </c>
+      <c r="I842" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="J842" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K842" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L842" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M842" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N842" s="14" t="n">
+        <v>76850</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N840"/>
+  <autoFilter ref="A1:N842"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -75205,7 +75922,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F63"/>
+  <dimension ref="A1:F65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -76750,8 +77467,56 @@
         <v>55</v>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" s="21" t="n">
+        <v>730.66</v>
+      </c>
+      <c r="B64" s="11" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C64" s="11" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D64" s="11" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E64" s="11" t="inlineStr"/>
+      <c r="F64" s="12" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="23" t="n">
+        <v>742.75</v>
+      </c>
+      <c r="B65" s="16" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C65" s="16" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D65" s="16" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E65" s="16" t="inlineStr"/>
+      <c r="F65" s="17" t="n">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F63"/>
+  <autoFilter ref="A1:F65"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -77150,7 +77915,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U30"/>
+  <dimension ref="A1:U31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -79306,8 +80071,75 @@
         <v>90239.45053751022</v>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B31" s="15" t="n">
+        <v>841</v>
+      </c>
+      <c r="C31" s="18" t="n">
+        <v>1552834.52</v>
+      </c>
+      <c r="D31" s="15" t="n">
+        <v>21</v>
+      </c>
+      <c r="E31" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="F31" s="16" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="G31" s="18" t="n">
+        <v>1751096.24</v>
+      </c>
+      <c r="H31" s="23" t="n">
+        <v>55</v>
+      </c>
+      <c r="I31" s="16" t="n"/>
+      <c r="J31" s="16" t="inlineStr">
+        <is>
+          <t>mail</t>
+        </is>
+      </c>
+      <c r="K31" s="27" t="n">
+        <v>3600</v>
+      </c>
+      <c r="L31" s="27" t="n">
+        <v>200</v>
+      </c>
+      <c r="M31" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N31" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="P31" s="15" t="n">
+        <v>281</v>
+      </c>
+      <c r="Q31" s="17" t="n">
+        <v>53</v>
+      </c>
+      <c r="R31" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="S31" s="17" t="n">
+        <v>53</v>
+      </c>
+      <c r="T31" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="U31" s="16" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U30"/>
+  <autoFilter ref="A1:U31"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -79318,7 +80150,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E361"/>
+  <dimension ref="A1:E373"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -87515,8 +88347,280 @@
         </is>
       </c>
     </row>
+    <row r="362">
+      <c r="A362" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B362" s="10" t="n">
+        <v>841</v>
+      </c>
+      <c r="C362" s="11" t="inlineStr">
+        <is>
+          <t>Starting Cash</t>
+        </is>
+      </c>
+      <c r="D362" s="14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E362" s="11" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B363" s="15" t="n">
+        <v>841</v>
+      </c>
+      <c r="C363" s="16" t="inlineStr">
+        <is>
+          <t>Cash Sources</t>
+        </is>
+      </c>
+      <c r="D363" s="16" t="n"/>
+      <c r="E363" s="16" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B364" s="10" t="n">
+        <v>841</v>
+      </c>
+      <c r="C364" s="11" t="inlineStr">
+        <is>
+          <t>revenues</t>
+        </is>
+      </c>
+      <c r="D364" s="14" t="n">
+        <v>22547500</v>
+      </c>
+      <c r="E364" s="11" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B365" s="15" t="n">
+        <v>841</v>
+      </c>
+      <c r="C365" s="16" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D365" s="18" t="n">
+        <v>302492.53</v>
+      </c>
+      <c r="E365" s="16" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B366" s="10" t="n">
+        <v>841</v>
+      </c>
+      <c r="C366" s="11" t="inlineStr">
+        <is>
+          <t>Cash Uses</t>
+        </is>
+      </c>
+      <c r="D366" s="11" t="n"/>
+      <c r="E366" s="11" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B367" s="15" t="n">
+        <v>841</v>
+      </c>
+      <c r="C367" s="16" t="inlineStr">
+        <is>
+          <t>outbound shipping</t>
+        </is>
+      </c>
+      <c r="D367" s="18" t="n">
+        <v>-2332500</v>
+      </c>
+      <c r="E367" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B368" s="10" t="n">
+        <v>841</v>
+      </c>
+      <c r="C368" s="11" t="inlineStr">
+        <is>
+          <t>inbound shipping</t>
+        </is>
+      </c>
+      <c r="D368" s="14" t="n">
+        <v>-1560000</v>
+      </c>
+      <c r="E368" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B369" s="15" t="n">
+        <v>841</v>
+      </c>
+      <c r="C369" s="16" t="inlineStr">
+        <is>
+          <t>FGI holding</t>
+        </is>
+      </c>
+      <c r="D369" s="18" t="n">
+        <v>-21940.43</v>
+      </c>
+      <c r="E369" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B370" s="10" t="n">
+        <v>841</v>
+      </c>
+      <c r="C370" s="11" t="inlineStr">
+        <is>
+          <t>add capacity</t>
+        </is>
+      </c>
+      <c r="D370" s="14" t="n">
+        <v>-1749840.87</v>
+      </c>
+      <c r="E370" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B371" s="15" t="n">
+        <v>841</v>
+      </c>
+      <c r="C371" s="16" t="inlineStr">
+        <is>
+          <t>Pipeline inventory holding</t>
+        </is>
+      </c>
+      <c r="D371" s="18" t="n">
+        <v>-29876.71</v>
+      </c>
+      <c r="E371" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B372" s="10" t="n">
+        <v>841</v>
+      </c>
+      <c r="C372" s="11" t="inlineStr">
+        <is>
+          <t>production</t>
+        </is>
+      </c>
+      <c r="D372" s="14" t="n">
+        <v>-16103000</v>
+      </c>
+      <c r="E372" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:26:02+08:00</t>
+        </is>
+      </c>
+      <c r="B373" s="15" t="n">
+        <v>841</v>
+      </c>
+      <c r="C373" s="16" t="inlineStr">
+        <is>
+          <t>Cash Balance</t>
+        </is>
+      </c>
+      <c r="D373" s="18" t="n">
+        <v>1552834.52</v>
+      </c>
+      <c r="E373" s="16" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E361"/>
+  <autoFilter ref="A1:E373"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update game data: day 842, cash 1410022.51, 3-day period 281
</commit_message>
<xml_diff>
--- a/data/supply_chain_game.xlsx
+++ b/data/supply_chain_game.xlsx
@@ -21,15 +21,15 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$282</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$842</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$843</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'资金构成_旧版'!$A$1:$C$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'运营参数_旧版'!$A$9:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$65</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$67</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'排行榜_旧版'!$A$1:$C$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$31</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$373</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$385</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'运营参数'!$A$1:$J$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$838</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$865</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -590,7 +590,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-06T14:26:02+08:00</t>
+          <t>2026-09-06T14:41:02+08:00</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>841</v>
+        <v>842</v>
       </c>
     </row>
     <row r="7">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>619</v>
+        <v>618</v>
       </c>
     </row>
     <row r="8">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>1552834.52</v>
+        <v>1410022.51</v>
       </c>
     </row>
     <row r="11">
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>1751096.24</v>
+        <v>1894730</v>
       </c>
     </row>
     <row r="15"/>
@@ -786,7 +786,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>200</v>
+        <v>135</v>
       </c>
     </row>
     <row r="25">
@@ -796,7 +796,7 @@
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
     </row>
     <row r="26">
@@ -858,7 +858,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>53</v>
+        <v>118</v>
       </c>
     </row>
     <row r="33">
@@ -878,7 +878,7 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>53</v>
+        <v>118</v>
       </c>
     </row>
     <row r="35">
@@ -898,7 +898,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>53</v>
+        <v>118</v>
       </c>
     </row>
     <row r="37">
@@ -906,6 +906,9 @@
         <is>
           <t>周期现金变动</t>
         </is>
+      </c>
+      <c r="B37" s="4" t="n">
+        <v>-147118.9301720145</v>
       </c>
     </row>
     <row r="38"/>
@@ -967,7 +970,7 @@
         </is>
       </c>
       <c r="B44" s="4" t="n">
-        <v>195537.1141997681</v>
+        <v>196079.4532131515</v>
       </c>
     </row>
     <row r="45"/>
@@ -1289,7 +1292,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E838"/>
+  <dimension ref="A1:E865"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -18903,8 +18906,575 @@
         <v>1236477.74</v>
       </c>
     </row>
+    <row r="839">
+      <c r="A839" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B839" s="15" t="n">
+        <v>842</v>
+      </c>
+      <c r="C839" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D839" s="16" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="E839" s="18" t="n">
+        <v>3304752.51</v>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B840" s="10" t="n">
+        <v>842</v>
+      </c>
+      <c r="C840" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D840" s="11" t="inlineStr">
+        <is>
+          <t>montesquieu</t>
+        </is>
+      </c>
+      <c r="E840" s="14" t="n">
+        <v>2471816.04</v>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B841" s="15" t="n">
+        <v>842</v>
+      </c>
+      <c r="C841" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D841" s="16" t="inlineStr">
+        <is>
+          <t>nicetry</t>
+        </is>
+      </c>
+      <c r="E841" s="18" t="n">
+        <v>2443891.17</v>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B842" s="10" t="n">
+        <v>842</v>
+      </c>
+      <c r="C842" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D842" s="11" t="inlineStr">
+        <is>
+          <t>group2</t>
+        </is>
+      </c>
+      <c r="E842" s="14" t="n">
+        <v>2310105.51</v>
+      </c>
+    </row>
+    <row r="843">
+      <c r="A843" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B843" s="15" t="n">
+        <v>842</v>
+      </c>
+      <c r="C843" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="D843" s="16" t="inlineStr">
+        <is>
+          <t>group25</t>
+        </is>
+      </c>
+      <c r="E843" s="18" t="n">
+        <v>2309947.59</v>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B844" s="10" t="n">
+        <v>842</v>
+      </c>
+      <c r="C844" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="D844" s="11" t="inlineStr">
+        <is>
+          <t>group11</t>
+        </is>
+      </c>
+      <c r="E844" s="14" t="n">
+        <v>2309935.29</v>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B845" s="15" t="n">
+        <v>842</v>
+      </c>
+      <c r="C845" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="D845" s="16" t="inlineStr">
+        <is>
+          <t>88888888</t>
+        </is>
+      </c>
+      <c r="E845" s="18" t="n">
+        <v>2309912.64</v>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B846" s="10" t="n">
+        <v>842</v>
+      </c>
+      <c r="C846" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="D846" s="11" t="inlineStr">
+        <is>
+          <t>t24</t>
+        </is>
+      </c>
+      <c r="E846" s="14" t="n">
+        <v>2250902.37</v>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B847" s="15" t="n">
+        <v>842</v>
+      </c>
+      <c r="C847" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="D847" s="16" t="inlineStr">
+        <is>
+          <t>teamhlly</t>
+        </is>
+      </c>
+      <c r="E847" s="18" t="n">
+        <v>2249435.85</v>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B848" s="10" t="n">
+        <v>842</v>
+      </c>
+      <c r="C848" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="D848" s="11" t="inlineStr">
+        <is>
+          <t>group9</t>
+        </is>
+      </c>
+      <c r="E848" s="14" t="n">
+        <v>2175822.41</v>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B849" s="15" t="n">
+        <v>842</v>
+      </c>
+      <c r="C849" s="15" t="n">
+        <v>11</v>
+      </c>
+      <c r="D849" s="16" t="inlineStr">
+        <is>
+          <t>group14</t>
+        </is>
+      </c>
+      <c r="E849" s="18" t="n">
+        <v>2118080.44</v>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B850" s="10" t="n">
+        <v>842</v>
+      </c>
+      <c r="C850" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="D850" s="11" t="inlineStr">
+        <is>
+          <t>group15</t>
+        </is>
+      </c>
+      <c r="E850" s="14" t="n">
+        <v>2076737.47</v>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B851" s="15" t="n">
+        <v>842</v>
+      </c>
+      <c r="C851" s="15" t="n">
+        <v>13</v>
+      </c>
+      <c r="D851" s="16" t="inlineStr">
+        <is>
+          <t>group8</t>
+        </is>
+      </c>
+      <c r="E851" s="18" t="n">
+        <v>2055301.46</v>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B852" s="10" t="n">
+        <v>842</v>
+      </c>
+      <c r="C852" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="D852" s="11" t="inlineStr">
+        <is>
+          <t>tigagroup20</t>
+        </is>
+      </c>
+      <c r="E852" s="14" t="n">
+        <v>2029025.4</v>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B853" s="15" t="n">
+        <v>842</v>
+      </c>
+      <c r="C853" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="D853" s="16" t="inlineStr">
+        <is>
+          <t>666666</t>
+        </is>
+      </c>
+      <c r="E853" s="18" t="n">
+        <v>1980331</v>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B854" s="10" t="n">
+        <v>842</v>
+      </c>
+      <c r="C854" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="D854" s="11" t="inlineStr">
+        <is>
+          <t>deepsleep</t>
+        </is>
+      </c>
+      <c r="E854" s="14" t="n">
+        <v>1843522.72</v>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B855" s="15" t="n">
+        <v>842</v>
+      </c>
+      <c r="C855" s="15" t="n">
+        <v>17</v>
+      </c>
+      <c r="D855" s="16" t="inlineStr">
+        <is>
+          <t>cleveregg</t>
+        </is>
+      </c>
+      <c r="E855" s="18" t="n">
+        <v>1825545.55</v>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B856" s="10" t="n">
+        <v>842</v>
+      </c>
+      <c r="C856" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="D856" s="11" t="inlineStr">
+        <is>
+          <t>group7</t>
+        </is>
+      </c>
+      <c r="E856" s="14" t="n">
+        <v>1772642.64</v>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B857" s="15" t="n">
+        <v>842</v>
+      </c>
+      <c r="C857" s="15" t="n">
+        <v>19</v>
+      </c>
+      <c r="D857" s="16" t="inlineStr">
+        <is>
+          <t>jit</t>
+        </is>
+      </c>
+      <c r="E857" s="18" t="n">
+        <v>1757970.92</v>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B858" s="10" t="n">
+        <v>842</v>
+      </c>
+      <c r="C858" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="D858" s="11" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E858" s="14" t="n">
+        <v>1664275.23</v>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B859" s="15" t="n">
+        <v>842</v>
+      </c>
+      <c r="C859" s="15" t="n">
+        <v>21</v>
+      </c>
+      <c r="D859" s="16" t="inlineStr">
+        <is>
+          <t>vivo50</t>
+        </is>
+      </c>
+      <c r="E859" s="18" t="n">
+        <v>1620419.86</v>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B860" s="10" t="n">
+        <v>842</v>
+      </c>
+      <c r="C860" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="D860" s="11" t="inlineStr">
+        <is>
+          <t>newgroup18</t>
+        </is>
+      </c>
+      <c r="E860" s="14" t="n">
+        <v>1612033.73</v>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B861" s="15" t="n">
+        <v>842</v>
+      </c>
+      <c r="C861" s="15" t="n">
+        <v>23</v>
+      </c>
+      <c r="D861" s="16" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E861" s="18" t="n">
+        <v>1548104.2</v>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B862" s="10" t="n">
+        <v>842</v>
+      </c>
+      <c r="C862" s="10" t="n">
+        <v>24</v>
+      </c>
+      <c r="D862" s="11" t="inlineStr">
+        <is>
+          <t>group12</t>
+        </is>
+      </c>
+      <c r="E862" s="14" t="n">
+        <v>1546406.41</v>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B863" s="15" t="n">
+        <v>842</v>
+      </c>
+      <c r="C863" s="15" t="n">
+        <v>25</v>
+      </c>
+      <c r="D863" s="16" t="inlineStr">
+        <is>
+          <t>aaachemicalseller</t>
+        </is>
+      </c>
+      <c r="E863" s="18" t="n">
+        <v>1445501.28</v>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B864" s="24" t="n">
+        <v>842</v>
+      </c>
+      <c r="C864" s="24" t="n">
+        <v>26</v>
+      </c>
+      <c r="D864" s="25" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="E864" s="26" t="n">
+        <v>1410022.51</v>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B865" s="15" t="n">
+        <v>842</v>
+      </c>
+      <c r="C865" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="D865" s="16" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="E865" s="18" t="n">
+        <v>1325193.78</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E838"/>
+  <autoFilter ref="A1:E865"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -36687,7 +37257,7 @@
         <v>843</v>
       </c>
       <c r="D282" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E282" s="11" t="inlineStr">
         <is>
@@ -36700,41 +37270,43 @@
         </is>
       </c>
       <c r="G282" s="12" t="n">
-        <v>53</v>
+        <v>118</v>
       </c>
       <c r="H282" s="12" t="n">
         <v>0</v>
       </c>
       <c r="I282" s="12" t="n">
-        <v>53</v>
+        <v>118</v>
       </c>
       <c r="J282" s="19" t="n">
         <v>1</v>
       </c>
       <c r="K282" s="12" t="n">
-        <v>53</v>
+        <v>118</v>
       </c>
       <c r="L282" s="14" t="n">
-        <v>1552834.52</v>
+        <v>1557141.440172015</v>
       </c>
       <c r="M282" s="14" t="n">
-        <v>1552834.52</v>
-      </c>
-      <c r="N282" s="11" t="n"/>
+        <v>1410022.51</v>
+      </c>
+      <c r="N282" s="14" t="n">
+        <v>-147118.9301720145</v>
+      </c>
       <c r="O282" s="12" t="n">
+        <v>135</v>
+      </c>
+      <c r="P282" s="12" t="n">
+        <v>167.5</v>
+      </c>
+      <c r="Q282" s="12" t="n">
         <v>200</v>
-      </c>
-      <c r="P282" s="12" t="n">
-        <v>200</v>
-      </c>
-      <c r="Q282" s="12" t="n">
-        <v>0</v>
       </c>
       <c r="R282" s="12" t="n">
         <v>200</v>
       </c>
       <c r="S282" s="14" t="n">
-        <v>76850</v>
+        <v>171100</v>
       </c>
     </row>
   </sheetData>
@@ -36749,7 +37321,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N842"/>
+  <dimension ref="A1:N843"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -75526,8 +76098,54 @@
         <v>76850</v>
       </c>
     </row>
+    <row r="843">
+      <c r="A843" s="15" t="n">
+        <v>842</v>
+      </c>
+      <c r="B843" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C843" s="17" t="n">
+        <v>65</v>
+      </c>
+      <c r="D843" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E843" s="17" t="n">
+        <v>65</v>
+      </c>
+      <c r="F843" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G843" s="17" t="n">
+        <v>65</v>
+      </c>
+      <c r="H843" s="18" t="n">
+        <v>1410022.51</v>
+      </c>
+      <c r="I843" s="17" t="n">
+        <v>135</v>
+      </c>
+      <c r="J843" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="K843" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L843" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="M843" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N843" s="18" t="n">
+        <v>94250</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N842"/>
+  <autoFilter ref="A1:N843"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -75922,7 +76540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F65"/>
+  <dimension ref="A1:F67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -77515,8 +78133,56 @@
         <v>55</v>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" s="21" t="n">
+        <v>730.66</v>
+      </c>
+      <c r="B66" s="11" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C66" s="11" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D66" s="11" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E66" s="11" t="inlineStr"/>
+      <c r="F66" s="12" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="23" t="n">
+        <v>742.75</v>
+      </c>
+      <c r="B67" s="16" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C67" s="16" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D67" s="16" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E67" s="16" t="inlineStr"/>
+      <c r="F67" s="17" t="n">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F65"/>
+  <autoFilter ref="A1:F67"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -77915,7 +78581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U31"/>
+  <dimension ref="A1:U32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -77938,7 +78604,7 @@
     <col width="12" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
-    <col width="20" customWidth="1" min="21" max="21"/>
+    <col width="21" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -80138,8 +80804,77 @@
       </c>
       <c r="U31" s="16" t="n"/>
     </row>
+    <row r="32">
+      <c r="A32" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B32" s="10" t="n">
+        <v>842</v>
+      </c>
+      <c r="C32" s="14" t="n">
+        <v>1410022.51</v>
+      </c>
+      <c r="D32" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="E32" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="F32" s="11" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="G32" s="14" t="n">
+        <v>1894730</v>
+      </c>
+      <c r="H32" s="21" t="n">
+        <v>55</v>
+      </c>
+      <c r="I32" s="11" t="n"/>
+      <c r="J32" s="11" t="inlineStr">
+        <is>
+          <t>mail</t>
+        </is>
+      </c>
+      <c r="K32" s="22" t="n">
+        <v>3600</v>
+      </c>
+      <c r="L32" s="22" t="n">
+        <v>200</v>
+      </c>
+      <c r="M32" s="12" t="n">
+        <v>135</v>
+      </c>
+      <c r="N32" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="O32" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="P32" s="10" t="n">
+        <v>281</v>
+      </c>
+      <c r="Q32" s="12" t="n">
+        <v>118</v>
+      </c>
+      <c r="R32" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S32" s="12" t="n">
+        <v>118</v>
+      </c>
+      <c r="T32" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="U32" s="14" t="n">
+        <v>-147118.9301720145</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U31"/>
+  <autoFilter ref="A1:U32"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -80150,7 +80885,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E373"/>
+  <dimension ref="A1:E385"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -88619,8 +89354,280 @@
         </is>
       </c>
     </row>
+    <row r="374">
+      <c r="A374" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B374" s="10" t="n">
+        <v>842</v>
+      </c>
+      <c r="C374" s="11" t="inlineStr">
+        <is>
+          <t>Starting Cash</t>
+        </is>
+      </c>
+      <c r="D374" s="14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E374" s="11" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B375" s="15" t="n">
+        <v>842</v>
+      </c>
+      <c r="C375" s="16" t="inlineStr">
+        <is>
+          <t>Cash Sources</t>
+        </is>
+      </c>
+      <c r="D375" s="16" t="n"/>
+      <c r="E375" s="16" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B376" s="10" t="n">
+        <v>842</v>
+      </c>
+      <c r="C376" s="11" t="inlineStr">
+        <is>
+          <t>revenues</t>
+        </is>
+      </c>
+      <c r="D376" s="14" t="n">
+        <v>22646100</v>
+      </c>
+      <c r="E376" s="11" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B377" s="15" t="n">
+        <v>842</v>
+      </c>
+      <c r="C377" s="16" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D377" s="18" t="n">
+        <v>302865.75</v>
+      </c>
+      <c r="E377" s="16" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B378" s="10" t="n">
+        <v>842</v>
+      </c>
+      <c r="C378" s="11" t="inlineStr">
+        <is>
+          <t>Cash Uses</t>
+        </is>
+      </c>
+      <c r="D378" s="11" t="n"/>
+      <c r="E378" s="11" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B379" s="15" t="n">
+        <v>842</v>
+      </c>
+      <c r="C379" s="16" t="inlineStr">
+        <is>
+          <t>outbound shipping</t>
+        </is>
+      </c>
+      <c r="D379" s="18" t="n">
+        <v>-2342700</v>
+      </c>
+      <c r="E379" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B380" s="10" t="n">
+        <v>842</v>
+      </c>
+      <c r="C380" s="11" t="inlineStr">
+        <is>
+          <t>inbound shipping</t>
+        </is>
+      </c>
+      <c r="D380" s="14" t="n">
+        <v>-1590000</v>
+      </c>
+      <c r="E380" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B381" s="15" t="n">
+        <v>842</v>
+      </c>
+      <c r="C381" s="16" t="inlineStr">
+        <is>
+          <t>FGI holding</t>
+        </is>
+      </c>
+      <c r="D381" s="18" t="n">
+        <v>-21985.84</v>
+      </c>
+      <c r="E381" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B382" s="10" t="n">
+        <v>842</v>
+      </c>
+      <c r="C382" s="11" t="inlineStr">
+        <is>
+          <t>add capacity</t>
+        </is>
+      </c>
+      <c r="D382" s="14" t="n">
+        <v>-1749840.87</v>
+      </c>
+      <c r="E382" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B383" s="15" t="n">
+        <v>842</v>
+      </c>
+      <c r="C383" s="16" t="inlineStr">
+        <is>
+          <t>Pipeline inventory holding</t>
+        </is>
+      </c>
+      <c r="D383" s="18" t="n">
+        <v>-29916.54</v>
+      </c>
+      <c r="E383" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B384" s="10" t="n">
+        <v>842</v>
+      </c>
+      <c r="C384" s="11" t="inlineStr">
+        <is>
+          <t>production</t>
+        </is>
+      </c>
+      <c r="D384" s="14" t="n">
+        <v>-16304500</v>
+      </c>
+      <c r="E384" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:41:02+08:00</t>
+        </is>
+      </c>
+      <c r="B385" s="15" t="n">
+        <v>842</v>
+      </c>
+      <c r="C385" s="16" t="inlineStr">
+        <is>
+          <t>Cash Balance</t>
+        </is>
+      </c>
+      <c r="D385" s="18" t="n">
+        <v>1410022.51</v>
+      </c>
+      <c r="E385" s="16" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E373"/>
+  <autoFilter ref="A1:E385"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update game data: day 843, cash 1479208.02, 3-day period 281
</commit_message>
<xml_diff>
--- a/data/supply_chain_game.xlsx
+++ b/data/supply_chain_game.xlsx
@@ -21,15 +21,15 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$282</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$843</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$844</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'资金构成_旧版'!$A$1:$C$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'运营参数_旧版'!$A$9:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$67</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$69</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'排行榜_旧版'!$A$1:$C$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$32</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$385</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$397</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'运营参数'!$A$1:$J$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$865</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$892</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -590,7 +590,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-06T14:41:02+08:00</t>
+          <t>2026-09-06T14:56:02+08:00</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>842</v>
+        <v>843</v>
       </c>
     </row>
     <row r="7">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>618</v>
+        <v>617</v>
       </c>
     </row>
     <row r="8">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>1410022.51</v>
+        <v>1479208.02</v>
       </c>
     </row>
     <row r="11">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>1894730</v>
+        <v>1826366.45</v>
       </c>
     </row>
     <row r="15"/>
@@ -786,7 +786,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>135</v>
+        <v>284</v>
       </c>
     </row>
     <row r="25">
@@ -796,7 +796,7 @@
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -847,7 +847,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>否（进行中）</t>
+          <t>是</t>
         </is>
       </c>
     </row>
@@ -858,7 +858,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>118</v>
+        <v>169</v>
       </c>
     </row>
     <row r="33">
@@ -878,7 +878,7 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>118</v>
+        <v>169</v>
       </c>
     </row>
     <row r="35">
@@ -898,7 +898,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>118</v>
+        <v>169</v>
       </c>
     </row>
     <row r="37">
@@ -908,7 +908,7 @@
         </is>
       </c>
       <c r="B37" s="4" t="n">
-        <v>-147118.9301720145</v>
+        <v>-80480.14942186116</v>
       </c>
     </row>
     <row r="38"/>
@@ -926,7 +926,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>280</v>
+        <v>281</v>
       </c>
     </row>
     <row r="41">
@@ -937,7 +937,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>838–840</t>
+          <t>841–843</t>
         </is>
       </c>
     </row>
@@ -949,7 +949,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>236.0 / 0.0 / 236.0</t>
+          <t>169.0 / 0.0 / 169.0</t>
         </is>
       </c>
     </row>
@@ -970,7 +970,7 @@
         </is>
       </c>
       <c r="B44" s="4" t="n">
-        <v>196079.4532131515</v>
+        <v>-80480.14942186116</v>
       </c>
     </row>
     <row r="45"/>
@@ -1292,7 +1292,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E865"/>
+  <dimension ref="A1:E892"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -19473,8 +19473,575 @@
         <v>1325193.78</v>
       </c>
     </row>
+    <row r="866">
+      <c r="A866" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B866" s="10" t="n">
+        <v>843</v>
+      </c>
+      <c r="C866" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D866" s="11" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="E866" s="14" t="n">
+        <v>3305574.47</v>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B867" s="15" t="n">
+        <v>843</v>
+      </c>
+      <c r="C867" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D867" s="16" t="inlineStr">
+        <is>
+          <t>montesquieu</t>
+        </is>
+      </c>
+      <c r="E867" s="18" t="n">
+        <v>2541285.97</v>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B868" s="10" t="n">
+        <v>843</v>
+      </c>
+      <c r="C868" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D868" s="11" t="inlineStr">
+        <is>
+          <t>nicetry</t>
+        </is>
+      </c>
+      <c r="E868" s="14" t="n">
+        <v>2513364.22</v>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B869" s="15" t="n">
+        <v>843</v>
+      </c>
+      <c r="C869" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D869" s="16" t="inlineStr">
+        <is>
+          <t>t24</t>
+        </is>
+      </c>
+      <c r="E869" s="18" t="n">
+        <v>2320369.4</v>
+      </c>
+    </row>
+    <row r="870">
+      <c r="A870" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B870" s="10" t="n">
+        <v>843</v>
+      </c>
+      <c r="C870" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="D870" s="11" t="inlineStr">
+        <is>
+          <t>teamhlly</t>
+        </is>
+      </c>
+      <c r="E870" s="14" t="n">
+        <v>2318855.1</v>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B871" s="15" t="n">
+        <v>843</v>
+      </c>
+      <c r="C871" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="D871" s="16" t="inlineStr">
+        <is>
+          <t>group9</t>
+        </is>
+      </c>
+      <c r="E871" s="18" t="n">
+        <v>2245215.32</v>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B872" s="10" t="n">
+        <v>843</v>
+      </c>
+      <c r="C872" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="D872" s="11" t="inlineStr">
+        <is>
+          <t>group14</t>
+        </is>
+      </c>
+      <c r="E872" s="14" t="n">
+        <v>2187453.06</v>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B873" s="15" t="n">
+        <v>843</v>
+      </c>
+      <c r="C873" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="D873" s="16" t="inlineStr">
+        <is>
+          <t>group15</t>
+        </is>
+      </c>
+      <c r="E873" s="18" t="n">
+        <v>2146099.3</v>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B874" s="10" t="n">
+        <v>843</v>
+      </c>
+      <c r="C874" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="D874" s="11" t="inlineStr">
+        <is>
+          <t>group2</t>
+        </is>
+      </c>
+      <c r="E874" s="14" t="n">
+        <v>2135752.48</v>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B875" s="15" t="n">
+        <v>843</v>
+      </c>
+      <c r="C875" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="D875" s="16" t="inlineStr">
+        <is>
+          <t>group25</t>
+        </is>
+      </c>
+      <c r="E875" s="18" t="n">
+        <v>2135594.52</v>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B876" s="10" t="n">
+        <v>843</v>
+      </c>
+      <c r="C876" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="D876" s="11" t="inlineStr">
+        <is>
+          <t>group11</t>
+        </is>
+      </c>
+      <c r="E876" s="14" t="n">
+        <v>2135582.22</v>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B877" s="15" t="n">
+        <v>843</v>
+      </c>
+      <c r="C877" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="D877" s="16" t="inlineStr">
+        <is>
+          <t>88888888</t>
+        </is>
+      </c>
+      <c r="E877" s="18" t="n">
+        <v>2135559.57</v>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B878" s="10" t="n">
+        <v>843</v>
+      </c>
+      <c r="C878" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="D878" s="11" t="inlineStr">
+        <is>
+          <t>group8</t>
+        </is>
+      </c>
+      <c r="E878" s="14" t="n">
+        <v>2055728.63</v>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B879" s="15" t="n">
+        <v>843</v>
+      </c>
+      <c r="C879" s="15" t="n">
+        <v>14</v>
+      </c>
+      <c r="D879" s="16" t="inlineStr">
+        <is>
+          <t>666666</t>
+        </is>
+      </c>
+      <c r="E879" s="18" t="n">
+        <v>1980738.59</v>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B880" s="10" t="n">
+        <v>843</v>
+      </c>
+      <c r="C880" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="D880" s="11" t="inlineStr">
+        <is>
+          <t>deepsleep</t>
+        </is>
+      </c>
+      <c r="E880" s="14" t="n">
+        <v>1916706.52</v>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B881" s="15" t="n">
+        <v>843</v>
+      </c>
+      <c r="C881" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="D881" s="16" t="inlineStr">
+        <is>
+          <t>cleveregg</t>
+        </is>
+      </c>
+      <c r="E881" s="18" t="n">
+        <v>1894812.71</v>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B882" s="10" t="n">
+        <v>843</v>
+      </c>
+      <c r="C882" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="D882" s="11" t="inlineStr">
+        <is>
+          <t>tigagroup20</t>
+        </is>
+      </c>
+      <c r="E882" s="14" t="n">
+        <v>1866836.03</v>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B883" s="15" t="n">
+        <v>843</v>
+      </c>
+      <c r="C883" s="15" t="n">
+        <v>18</v>
+      </c>
+      <c r="D883" s="16" t="inlineStr">
+        <is>
+          <t>jit</t>
+        </is>
+      </c>
+      <c r="E883" s="18" t="n">
+        <v>1779719.91</v>
+      </c>
+    </row>
+    <row r="884">
+      <c r="A884" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B884" s="10" t="n">
+        <v>843</v>
+      </c>
+      <c r="C884" s="10" t="n">
+        <v>19</v>
+      </c>
+      <c r="D884" s="11" t="inlineStr">
+        <is>
+          <t>group7</t>
+        </is>
+      </c>
+      <c r="E884" s="14" t="n">
+        <v>1772995.99</v>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B885" s="15" t="n">
+        <v>843</v>
+      </c>
+      <c r="C885" s="15" t="n">
+        <v>20</v>
+      </c>
+      <c r="D885" s="16" t="inlineStr">
+        <is>
+          <t>vivo50</t>
+        </is>
+      </c>
+      <c r="E885" s="18" t="n">
+        <v>1693534.44</v>
+      </c>
+    </row>
+    <row r="886">
+      <c r="A886" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B886" s="10" t="n">
+        <v>843</v>
+      </c>
+      <c r="C886" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="D886" s="11" t="inlineStr">
+        <is>
+          <t>group12</t>
+        </is>
+      </c>
+      <c r="E886" s="14" t="n">
+        <v>1619501.66</v>
+      </c>
+    </row>
+    <row r="887">
+      <c r="A887" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B887" s="15" t="n">
+        <v>843</v>
+      </c>
+      <c r="C887" s="15" t="n">
+        <v>22</v>
+      </c>
+      <c r="D887" s="16" t="inlineStr">
+        <is>
+          <t>newgroup18</t>
+        </is>
+      </c>
+      <c r="E887" s="18" t="n">
+        <v>1612345.14</v>
+      </c>
+    </row>
+    <row r="888">
+      <c r="A888" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B888" s="10" t="n">
+        <v>843</v>
+      </c>
+      <c r="C888" s="10" t="n">
+        <v>23</v>
+      </c>
+      <c r="D888" s="11" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E888" s="14" t="n">
+        <v>1548398.92</v>
+      </c>
+    </row>
+    <row r="889">
+      <c r="A889" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B889" s="15" t="n">
+        <v>843</v>
+      </c>
+      <c r="C889" s="15" t="n">
+        <v>24</v>
+      </c>
+      <c r="D889" s="16" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E889" s="18" t="n">
+        <v>1516986.04</v>
+      </c>
+    </row>
+    <row r="890">
+      <c r="A890" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B890" s="10" t="n">
+        <v>843</v>
+      </c>
+      <c r="C890" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="D890" s="11" t="inlineStr">
+        <is>
+          <t>aaachemicalseller</t>
+        </is>
+      </c>
+      <c r="E890" s="14" t="n">
+        <v>1514661.53</v>
+      </c>
+    </row>
+    <row r="891">
+      <c r="A891" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B891" s="24" t="n">
+        <v>843</v>
+      </c>
+      <c r="C891" s="24" t="n">
+        <v>26</v>
+      </c>
+      <c r="D891" s="25" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="E891" s="26" t="n">
+        <v>1479208.02</v>
+      </c>
+    </row>
+    <row r="892">
+      <c r="A892" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B892" s="10" t="n">
+        <v>843</v>
+      </c>
+      <c r="C892" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="D892" s="11" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="E892" s="14" t="n">
+        <v>1189199.01</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E865"/>
+  <autoFilter ref="A1:E892"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -37257,11 +37824,11 @@
         <v>843</v>
       </c>
       <c r="D282" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E282" s="11" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="F282" s="11" t="inlineStr">
@@ -37270,43 +37837,43 @@
         </is>
       </c>
       <c r="G282" s="12" t="n">
-        <v>118</v>
+        <v>169</v>
       </c>
       <c r="H282" s="12" t="n">
         <v>0</v>
       </c>
       <c r="I282" s="12" t="n">
-        <v>118</v>
+        <v>169</v>
       </c>
       <c r="J282" s="19" t="n">
         <v>1</v>
       </c>
       <c r="K282" s="12" t="n">
-        <v>118</v>
+        <v>169</v>
       </c>
       <c r="L282" s="14" t="n">
-        <v>1557141.440172015</v>
+        <v>1559688.169421861</v>
       </c>
       <c r="M282" s="14" t="n">
-        <v>1410022.51</v>
+        <v>1479208.02</v>
       </c>
       <c r="N282" s="14" t="n">
-        <v>-147118.9301720145</v>
+        <v>-80480.14942186116</v>
       </c>
       <c r="O282" s="12" t="n">
-        <v>135</v>
+        <v>284</v>
       </c>
       <c r="P282" s="12" t="n">
-        <v>167.5</v>
+        <v>206.3333333333333</v>
       </c>
       <c r="Q282" s="12" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="R282" s="12" t="n">
         <v>200</v>
       </c>
       <c r="S282" s="14" t="n">
-        <v>171100</v>
+        <v>245050</v>
       </c>
     </row>
   </sheetData>
@@ -37321,7 +37888,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N843"/>
+  <dimension ref="A1:N844"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -76144,8 +76711,54 @@
         <v>94250</v>
       </c>
     </row>
+    <row r="844">
+      <c r="A844" s="10" t="n">
+        <v>843</v>
+      </c>
+      <c r="B844" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C844" s="12" t="n">
+        <v>51</v>
+      </c>
+      <c r="D844" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E844" s="12" t="n">
+        <v>51</v>
+      </c>
+      <c r="F844" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G844" s="12" t="n">
+        <v>51</v>
+      </c>
+      <c r="H844" s="14" t="n">
+        <v>1479208.02</v>
+      </c>
+      <c r="I844" s="12" t="n">
+        <v>284</v>
+      </c>
+      <c r="J844" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K844" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L844" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M844" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N844" s="14" t="n">
+        <v>73950</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N843"/>
+  <autoFilter ref="A1:N844"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -76540,7 +77153,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F67"/>
+  <dimension ref="A1:F69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -78181,8 +78794,56 @@
         <v>55</v>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" s="21" t="n">
+        <v>730.66</v>
+      </c>
+      <c r="B68" s="11" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C68" s="11" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D68" s="11" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E68" s="11" t="inlineStr"/>
+      <c r="F68" s="12" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="23" t="n">
+        <v>742.75</v>
+      </c>
+      <c r="B69" s="16" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C69" s="16" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D69" s="16" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E69" s="16" t="inlineStr"/>
+      <c r="F69" s="17" t="n">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F67"/>
+  <autoFilter ref="A1:F69"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -78581,7 +79242,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U32"/>
+  <dimension ref="A1:U33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -78604,7 +79265,7 @@
     <col width="12" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
-    <col width="21" customWidth="1" min="21" max="21"/>
+    <col width="20" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -80873,8 +81534,77 @@
         <v>-147118.9301720145</v>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B33" s="15" t="n">
+        <v>843</v>
+      </c>
+      <c r="C33" s="18" t="n">
+        <v>1479208.02</v>
+      </c>
+      <c r="D33" s="15" t="n">
+        <v>26</v>
+      </c>
+      <c r="E33" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="F33" s="16" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="G33" s="18" t="n">
+        <v>1826366.45</v>
+      </c>
+      <c r="H33" s="23" t="n">
+        <v>55</v>
+      </c>
+      <c r="I33" s="16" t="n"/>
+      <c r="J33" s="16" t="inlineStr">
+        <is>
+          <t>mail</t>
+        </is>
+      </c>
+      <c r="K33" s="27" t="n">
+        <v>3600</v>
+      </c>
+      <c r="L33" s="27" t="n">
+        <v>200</v>
+      </c>
+      <c r="M33" s="17" t="n">
+        <v>284</v>
+      </c>
+      <c r="N33" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O33" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="P33" s="15" t="n">
+        <v>281</v>
+      </c>
+      <c r="Q33" s="17" t="n">
+        <v>169</v>
+      </c>
+      <c r="R33" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="S33" s="17" t="n">
+        <v>169</v>
+      </c>
+      <c r="T33" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="U33" s="18" t="n">
+        <v>-80480.14942186116</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U32"/>
+  <autoFilter ref="A1:U33"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -80885,7 +81615,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E385"/>
+  <dimension ref="A1:E397"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -89626,8 +90356,280 @@
         </is>
       </c>
     </row>
+    <row r="386">
+      <c r="A386" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B386" s="10" t="n">
+        <v>843</v>
+      </c>
+      <c r="C386" s="11" t="inlineStr">
+        <is>
+          <t>Starting Cash</t>
+        </is>
+      </c>
+      <c r="D386" s="14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E386" s="11" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B387" s="15" t="n">
+        <v>843</v>
+      </c>
+      <c r="C387" s="16" t="inlineStr">
+        <is>
+          <t>Cash Sources</t>
+        </is>
+      </c>
+      <c r="D387" s="16" t="n"/>
+      <c r="E387" s="16" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B388" s="10" t="n">
+        <v>843</v>
+      </c>
+      <c r="C388" s="11" t="inlineStr">
+        <is>
+          <t>revenues</t>
+        </is>
+      </c>
+      <c r="D388" s="14" t="n">
+        <v>22722950</v>
+      </c>
+      <c r="E388" s="11" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B389" s="15" t="n">
+        <v>843</v>
+      </c>
+      <c r="C389" s="16" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D389" s="18" t="n">
+        <v>303238.55</v>
+      </c>
+      <c r="E389" s="16" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B390" s="10" t="n">
+        <v>843</v>
+      </c>
+      <c r="C390" s="11" t="inlineStr">
+        <is>
+          <t>Cash Uses</t>
+        </is>
+      </c>
+      <c r="D390" s="11" t="n"/>
+      <c r="E390" s="11" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B391" s="15" t="n">
+        <v>843</v>
+      </c>
+      <c r="C391" s="16" t="inlineStr">
+        <is>
+          <t>outbound shipping</t>
+        </is>
+      </c>
+      <c r="D391" s="18" t="n">
+        <v>-2350650</v>
+      </c>
+      <c r="E391" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B392" s="10" t="n">
+        <v>843</v>
+      </c>
+      <c r="C392" s="11" t="inlineStr">
+        <is>
+          <t>inbound shipping</t>
+        </is>
+      </c>
+      <c r="D392" s="14" t="n">
+        <v>-1590000</v>
+      </c>
+      <c r="E392" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B393" s="15" t="n">
+        <v>843</v>
+      </c>
+      <c r="C393" s="16" t="inlineStr">
+        <is>
+          <t>FGI holding</t>
+        </is>
+      </c>
+      <c r="D393" s="18" t="n">
+        <v>-22058.15</v>
+      </c>
+      <c r="E393" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B394" s="10" t="n">
+        <v>843</v>
+      </c>
+      <c r="C394" s="11" t="inlineStr">
+        <is>
+          <t>add capacity</t>
+        </is>
+      </c>
+      <c r="D394" s="14" t="n">
+        <v>-1749840.87</v>
+      </c>
+      <c r="E394" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B395" s="15" t="n">
+        <v>843</v>
+      </c>
+      <c r="C395" s="16" t="inlineStr">
+        <is>
+          <t>Pipeline inventory holding</t>
+        </is>
+      </c>
+      <c r="D395" s="18" t="n">
+        <v>-29931.51</v>
+      </c>
+      <c r="E395" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B396" s="10" t="n">
+        <v>843</v>
+      </c>
+      <c r="C396" s="11" t="inlineStr">
+        <is>
+          <t>production</t>
+        </is>
+      </c>
+      <c r="D396" s="14" t="n">
+        <v>-16304500</v>
+      </c>
+      <c r="E396" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T14:56:02+08:00</t>
+        </is>
+      </c>
+      <c r="B397" s="15" t="n">
+        <v>843</v>
+      </c>
+      <c r="C397" s="16" t="inlineStr">
+        <is>
+          <t>Cash Balance</t>
+        </is>
+      </c>
+      <c r="D397" s="18" t="n">
+        <v>1479208.02</v>
+      </c>
+      <c r="E397" s="16" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E385"/>
+  <autoFilter ref="A1:E397"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update game data: day 844, cash 1512021.31, 3-day period 282
</commit_message>
<xml_diff>
--- a/data/supply_chain_game.xlsx
+++ b/data/supply_chain_game.xlsx
@@ -20,16 +20,16 @@
     <sheet name="排行榜" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$282</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$844</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$283</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$845</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'资金构成_旧版'!$A$1:$C$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'运营参数_旧版'!$A$9:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$71</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'排行榜_旧版'!$A$1:$C$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$397</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$409</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'运营参数'!$A$1:$J$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$892</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$919</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -590,7 +590,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-06T14:56:02+08:00</t>
+          <t>2026-09-06T15:11:02+08:00</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>843</v>
+        <v>844</v>
       </c>
     </row>
     <row r="7">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>617</v>
+        <v>616</v>
       </c>
     </row>
     <row r="8">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>1479208.02</v>
+        <v>1512021.31</v>
       </c>
     </row>
     <row r="11">
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>1826366.45</v>
+        <v>1794375.34</v>
       </c>
     </row>
     <row r="15"/>
@@ -786,7 +786,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>284</v>
+        <v>266</v>
       </c>
     </row>
     <row r="25">
@@ -824,7 +824,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="30">
@@ -835,7 +835,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>841–843</t>
+          <t>844–846</t>
         </is>
       </c>
     </row>
@@ -847,7 +847,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否（进行中）</t>
         </is>
       </c>
     </row>
@@ -858,7 +858,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>169</v>
+        <v>18</v>
       </c>
     </row>
     <row r="33">
@@ -878,7 +878,7 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>169</v>
+        <v>18</v>
       </c>
     </row>
     <row r="35">
@@ -898,7 +898,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>169</v>
+        <v>18</v>
       </c>
     </row>
     <row r="37">
@@ -906,9 +906,6 @@
         <is>
           <t>周期现金变动</t>
         </is>
-      </c>
-      <c r="B37" s="4" t="n">
-        <v>-80480.14942186116</v>
       </c>
     </row>
     <row r="38"/>
@@ -970,7 +967,7 @@
         </is>
       </c>
       <c r="B44" s="4" t="n">
-        <v>-80480.14942186116</v>
+        <v>-80961.80881520314</v>
       </c>
     </row>
     <row r="45"/>
@@ -1292,7 +1289,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E892"/>
+  <dimension ref="A1:E919"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -20040,8 +20037,575 @@
         <v>1189199.01</v>
       </c>
     </row>
+    <row r="893">
+      <c r="A893" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B893" s="15" t="n">
+        <v>844</v>
+      </c>
+      <c r="C893" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D893" s="16" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="E893" s="18" t="n">
+        <v>3306396.65</v>
+      </c>
+    </row>
+    <row r="894">
+      <c r="A894" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B894" s="10" t="n">
+        <v>844</v>
+      </c>
+      <c r="C894" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D894" s="11" t="inlineStr">
+        <is>
+          <t>montesquieu</t>
+        </is>
+      </c>
+      <c r="E894" s="14" t="n">
+        <v>2574383.75</v>
+      </c>
+    </row>
+    <row r="895">
+      <c r="A895" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B895" s="15" t="n">
+        <v>844</v>
+      </c>
+      <c r="C895" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D895" s="16" t="inlineStr">
+        <is>
+          <t>nicetry</t>
+        </is>
+      </c>
+      <c r="E895" s="18" t="n">
+        <v>2533465.12</v>
+      </c>
+    </row>
+    <row r="896">
+      <c r="A896" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B896" s="10" t="n">
+        <v>844</v>
+      </c>
+      <c r="C896" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D896" s="11" t="inlineStr">
+        <is>
+          <t>group9</t>
+        </is>
+      </c>
+      <c r="E896" s="14" t="n">
+        <v>2278236.05</v>
+      </c>
+    </row>
+    <row r="897">
+      <c r="A897" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B897" s="15" t="n">
+        <v>844</v>
+      </c>
+      <c r="C897" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="D897" s="16" t="inlineStr">
+        <is>
+          <t>group14</t>
+        </is>
+      </c>
+      <c r="E897" s="18" t="n">
+        <v>2220453.5</v>
+      </c>
+    </row>
+    <row r="898">
+      <c r="A898" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B898" s="10" t="n">
+        <v>844</v>
+      </c>
+      <c r="C898" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="D898" s="11" t="inlineStr">
+        <is>
+          <t>group15</t>
+        </is>
+      </c>
+      <c r="E898" s="14" t="n">
+        <v>2179088.94</v>
+      </c>
+    </row>
+    <row r="899">
+      <c r="A899" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B899" s="15" t="n">
+        <v>844</v>
+      </c>
+      <c r="C899" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="D899" s="16" t="inlineStr">
+        <is>
+          <t>group2</t>
+        </is>
+      </c>
+      <c r="E899" s="18" t="n">
+        <v>2136213.96</v>
+      </c>
+    </row>
+    <row r="900">
+      <c r="A900" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B900" s="10" t="n">
+        <v>844</v>
+      </c>
+      <c r="C900" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="D900" s="11" t="inlineStr">
+        <is>
+          <t>group25</t>
+        </is>
+      </c>
+      <c r="E900" s="14" t="n">
+        <v>2136055.96</v>
+      </c>
+    </row>
+    <row r="901">
+      <c r="A901" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B901" s="15" t="n">
+        <v>844</v>
+      </c>
+      <c r="C901" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="D901" s="16" t="inlineStr">
+        <is>
+          <t>group11</t>
+        </is>
+      </c>
+      <c r="E901" s="18" t="n">
+        <v>2136043.66</v>
+      </c>
+    </row>
+    <row r="902">
+      <c r="A902" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B902" s="10" t="n">
+        <v>844</v>
+      </c>
+      <c r="C902" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="D902" s="11" t="inlineStr">
+        <is>
+          <t>88888888</t>
+        </is>
+      </c>
+      <c r="E902" s="14" t="n">
+        <v>2136020.99</v>
+      </c>
+    </row>
+    <row r="903">
+      <c r="A903" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B903" s="15" t="n">
+        <v>844</v>
+      </c>
+      <c r="C903" s="15" t="n">
+        <v>11</v>
+      </c>
+      <c r="D903" s="16" t="inlineStr">
+        <is>
+          <t>teamhlly</t>
+        </is>
+      </c>
+      <c r="E903" s="18" t="n">
+        <v>2135398.71</v>
+      </c>
+    </row>
+    <row r="904">
+      <c r="A904" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B904" s="10" t="n">
+        <v>844</v>
+      </c>
+      <c r="C904" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="D904" s="11" t="inlineStr">
+        <is>
+          <t>t24</t>
+        </is>
+      </c>
+      <c r="E904" s="14" t="n">
+        <v>2121964.28</v>
+      </c>
+    </row>
+    <row r="905">
+      <c r="A905" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B905" s="15" t="n">
+        <v>844</v>
+      </c>
+      <c r="C905" s="15" t="n">
+        <v>13</v>
+      </c>
+      <c r="D905" s="16" t="inlineStr">
+        <is>
+          <t>group8</t>
+        </is>
+      </c>
+      <c r="E905" s="18" t="n">
+        <v>2056155.91</v>
+      </c>
+    </row>
+    <row r="906">
+      <c r="A906" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B906" s="10" t="n">
+        <v>844</v>
+      </c>
+      <c r="C906" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="D906" s="11" t="inlineStr">
+        <is>
+          <t>666666</t>
+        </is>
+      </c>
+      <c r="E906" s="14" t="n">
+        <v>2020146.29</v>
+      </c>
+    </row>
+    <row r="907">
+      <c r="A907" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B907" s="15" t="n">
+        <v>844</v>
+      </c>
+      <c r="C907" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="D907" s="16" t="inlineStr">
+        <is>
+          <t>cleveregg</t>
+        </is>
+      </c>
+      <c r="E907" s="18" t="n">
+        <v>1927711.03</v>
+      </c>
+    </row>
+    <row r="908">
+      <c r="A908" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B908" s="10" t="n">
+        <v>844</v>
+      </c>
+      <c r="C908" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="D908" s="11" t="inlineStr">
+        <is>
+          <t>tigagroup20</t>
+        </is>
+      </c>
+      <c r="E908" s="14" t="n">
+        <v>1899700.41</v>
+      </c>
+    </row>
+    <row r="909">
+      <c r="A909" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B909" s="15" t="n">
+        <v>844</v>
+      </c>
+      <c r="C909" s="15" t="n">
+        <v>17</v>
+      </c>
+      <c r="D909" s="16" t="inlineStr">
+        <is>
+          <t>group7</t>
+        </is>
+      </c>
+      <c r="E909" s="18" t="n">
+        <v>1773349.43</v>
+      </c>
+    </row>
+    <row r="910">
+      <c r="A910" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B910" s="10" t="n">
+        <v>844</v>
+      </c>
+      <c r="C910" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="D910" s="11" t="inlineStr">
+        <is>
+          <t>jit</t>
+        </is>
+      </c>
+      <c r="E910" s="14" t="n">
+        <v>1765037.51</v>
+      </c>
+    </row>
+    <row r="911">
+      <c r="A911" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B911" s="15" t="n">
+        <v>844</v>
+      </c>
+      <c r="C911" s="15" t="n">
+        <v>19</v>
+      </c>
+      <c r="D911" s="16" t="inlineStr">
+        <is>
+          <t>deepsleep</t>
+        </is>
+      </c>
+      <c r="E911" s="18" t="n">
+        <v>1753124.06</v>
+      </c>
+    </row>
+    <row r="912">
+      <c r="A912" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B912" s="10" t="n">
+        <v>844</v>
+      </c>
+      <c r="C912" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="D912" s="11" t="inlineStr">
+        <is>
+          <t>newgroup18</t>
+        </is>
+      </c>
+      <c r="E912" s="14" t="n">
+        <v>1612656.62</v>
+      </c>
+    </row>
+    <row r="913">
+      <c r="A913" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B913" s="15" t="n">
+        <v>844</v>
+      </c>
+      <c r="C913" s="15" t="n">
+        <v>21</v>
+      </c>
+      <c r="D913" s="16" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E913" s="18" t="n">
+        <v>1587693.7</v>
+      </c>
+    </row>
+    <row r="914">
+      <c r="A914" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B914" s="10" t="n">
+        <v>844</v>
+      </c>
+      <c r="C914" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="D914" s="11" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E914" s="14" t="n">
+        <v>1549761.51</v>
+      </c>
+    </row>
+    <row r="915">
+      <c r="A915" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B915" s="15" t="n">
+        <v>844</v>
+      </c>
+      <c r="C915" s="15" t="n">
+        <v>23</v>
+      </c>
+      <c r="D915" s="16" t="inlineStr">
+        <is>
+          <t>aaachemicalseller</t>
+        </is>
+      </c>
+      <c r="E915" s="18" t="n">
+        <v>1547443.8</v>
+      </c>
+    </row>
+    <row r="916">
+      <c r="A916" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B916" s="24" t="n">
+        <v>844</v>
+      </c>
+      <c r="C916" s="24" t="n">
+        <v>24</v>
+      </c>
+      <c r="D916" s="25" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="E916" s="26" t="n">
+        <v>1512021.31</v>
+      </c>
+    </row>
+    <row r="917">
+      <c r="A917" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B917" s="15" t="n">
+        <v>844</v>
+      </c>
+      <c r="C917" s="15" t="n">
+        <v>25</v>
+      </c>
+      <c r="D917" s="16" t="inlineStr">
+        <is>
+          <t>vivo50</t>
+        </is>
+      </c>
+      <c r="E917" s="18" t="n">
+        <v>1509882.41</v>
+      </c>
+    </row>
+    <row r="918">
+      <c r="A918" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B918" s="10" t="n">
+        <v>844</v>
+      </c>
+      <c r="C918" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="D918" s="11" t="inlineStr">
+        <is>
+          <t>group12</t>
+        </is>
+      </c>
+      <c r="E918" s="14" t="n">
+        <v>1435830.29</v>
+      </c>
+    </row>
+    <row r="919">
+      <c r="A919" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B919" s="15" t="n">
+        <v>844</v>
+      </c>
+      <c r="C919" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="D919" s="16" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="E919" s="18" t="n">
+        <v>1253178.02</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E892"/>
+  <autoFilter ref="A1:E919"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -20052,7 +20616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S282"/>
+  <dimension ref="A1:S283"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -37876,8 +38440,69 @@
         <v>245050</v>
       </c>
     </row>
+    <row r="283">
+      <c r="A283" s="15" t="n">
+        <v>282</v>
+      </c>
+      <c r="B283" s="15" t="n">
+        <v>844</v>
+      </c>
+      <c r="C283" s="15" t="n">
+        <v>846</v>
+      </c>
+      <c r="D283" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E283" s="16" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="F283" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G283" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="H283" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I283" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="J283" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K283" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="L283" s="18" t="n">
+        <v>1512021.31</v>
+      </c>
+      <c r="M283" s="18" t="n">
+        <v>1512021.31</v>
+      </c>
+      <c r="N283" s="16" t="n"/>
+      <c r="O283" s="17" t="n">
+        <v>266</v>
+      </c>
+      <c r="P283" s="17" t="n">
+        <v>266</v>
+      </c>
+      <c r="Q283" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="R283" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="S283" s="18" t="n">
+        <v>26100</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S282"/>
+  <autoFilter ref="A1:S283"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -37888,7 +38513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N844"/>
+  <dimension ref="A1:N845"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -76757,8 +77382,54 @@
         <v>73950</v>
       </c>
     </row>
+    <row r="845">
+      <c r="A845" s="15" t="n">
+        <v>844</v>
+      </c>
+      <c r="B845" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C845" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="D845" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E845" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="F845" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G845" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="H845" s="18" t="n">
+        <v>1512021.31</v>
+      </c>
+      <c r="I845" s="17" t="n">
+        <v>266</v>
+      </c>
+      <c r="J845" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K845" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L845" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M845" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N845" s="18" t="n">
+        <v>26100</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N844"/>
+  <autoFilter ref="A1:N845"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -77153,7 +77824,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F69"/>
+  <dimension ref="A1:F71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -78842,8 +79513,56 @@
         <v>55</v>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" s="21" t="n">
+        <v>730.66</v>
+      </c>
+      <c r="B70" s="11" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C70" s="11" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D70" s="11" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E70" s="11" t="inlineStr"/>
+      <c r="F70" s="12" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="23" t="n">
+        <v>742.75</v>
+      </c>
+      <c r="B71" s="16" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C71" s="16" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D71" s="16" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E71" s="16" t="inlineStr"/>
+      <c r="F71" s="17" t="n">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F69"/>
+  <autoFilter ref="A1:F71"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -79242,7 +79961,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U33"/>
+  <dimension ref="A1:U34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -81603,8 +82322,75 @@
         <v>-80480.14942186116</v>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B34" s="10" t="n">
+        <v>844</v>
+      </c>
+      <c r="C34" s="14" t="n">
+        <v>1512021.31</v>
+      </c>
+      <c r="D34" s="10" t="n">
+        <v>24</v>
+      </c>
+      <c r="E34" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="F34" s="11" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="G34" s="14" t="n">
+        <v>1794375.34</v>
+      </c>
+      <c r="H34" s="21" t="n">
+        <v>55</v>
+      </c>
+      <c r="I34" s="11" t="n"/>
+      <c r="J34" s="11" t="inlineStr">
+        <is>
+          <t>mail</t>
+        </is>
+      </c>
+      <c r="K34" s="22" t="n">
+        <v>3600</v>
+      </c>
+      <c r="L34" s="22" t="n">
+        <v>200</v>
+      </c>
+      <c r="M34" s="12" t="n">
+        <v>266</v>
+      </c>
+      <c r="N34" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="O34" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="P34" s="10" t="n">
+        <v>282</v>
+      </c>
+      <c r="Q34" s="12" t="n">
+        <v>18</v>
+      </c>
+      <c r="R34" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S34" s="12" t="n">
+        <v>18</v>
+      </c>
+      <c r="T34" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="U34" s="11" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U33"/>
+  <autoFilter ref="A1:U34"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -81615,7 +82401,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E397"/>
+  <dimension ref="A1:E409"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -90628,8 +91414,280 @@
         </is>
       </c>
     </row>
+    <row r="398">
+      <c r="A398" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B398" s="10" t="n">
+        <v>844</v>
+      </c>
+      <c r="C398" s="11" t="inlineStr">
+        <is>
+          <t>Starting Cash</t>
+        </is>
+      </c>
+      <c r="D398" s="14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E398" s="11" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B399" s="15" t="n">
+        <v>844</v>
+      </c>
+      <c r="C399" s="16" t="inlineStr">
+        <is>
+          <t>Cash Sources</t>
+        </is>
+      </c>
+      <c r="D399" s="16" t="n"/>
+      <c r="E399" s="16" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B400" s="10" t="n">
+        <v>844</v>
+      </c>
+      <c r="C400" s="11" t="inlineStr">
+        <is>
+          <t>revenues</t>
+        </is>
+      </c>
+      <c r="D400" s="14" t="n">
+        <v>22759200</v>
+      </c>
+      <c r="E400" s="11" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B401" s="15" t="n">
+        <v>844</v>
+      </c>
+      <c r="C401" s="16" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D401" s="18" t="n">
+        <v>303626.74</v>
+      </c>
+      <c r="E401" s="16" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B402" s="10" t="n">
+        <v>844</v>
+      </c>
+      <c r="C402" s="11" t="inlineStr">
+        <is>
+          <t>Cash Uses</t>
+        </is>
+      </c>
+      <c r="D402" s="11" t="n"/>
+      <c r="E402" s="11" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B403" s="15" t="n">
+        <v>844</v>
+      </c>
+      <c r="C403" s="16" t="inlineStr">
+        <is>
+          <t>outbound shipping</t>
+        </is>
+      </c>
+      <c r="D403" s="18" t="n">
+        <v>-2354400</v>
+      </c>
+      <c r="E403" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B404" s="10" t="n">
+        <v>844</v>
+      </c>
+      <c r="C404" s="11" t="inlineStr">
+        <is>
+          <t>inbound shipping</t>
+        </is>
+      </c>
+      <c r="D404" s="14" t="n">
+        <v>-1590000</v>
+      </c>
+      <c r="E404" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B405" s="15" t="n">
+        <v>844</v>
+      </c>
+      <c r="C405" s="16" t="inlineStr">
+        <is>
+          <t>FGI holding</t>
+        </is>
+      </c>
+      <c r="D405" s="18" t="n">
+        <v>-22133.06</v>
+      </c>
+      <c r="E405" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B406" s="10" t="n">
+        <v>844</v>
+      </c>
+      <c r="C406" s="11" t="inlineStr">
+        <is>
+          <t>add capacity</t>
+        </is>
+      </c>
+      <c r="D406" s="14" t="n">
+        <v>-1749840.87</v>
+      </c>
+      <c r="E406" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B407" s="15" t="n">
+        <v>844</v>
+      </c>
+      <c r="C407" s="16" t="inlineStr">
+        <is>
+          <t>Pipeline inventory holding</t>
+        </is>
+      </c>
+      <c r="D407" s="18" t="n">
+        <v>-29931.51</v>
+      </c>
+      <c r="E407" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B408" s="10" t="n">
+        <v>844</v>
+      </c>
+      <c r="C408" s="11" t="inlineStr">
+        <is>
+          <t>production</t>
+        </is>
+      </c>
+      <c r="D408" s="14" t="n">
+        <v>-16304500</v>
+      </c>
+      <c r="E408" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:11:02+08:00</t>
+        </is>
+      </c>
+      <c r="B409" s="15" t="n">
+        <v>844</v>
+      </c>
+      <c r="C409" s="16" t="inlineStr">
+        <is>
+          <t>Cash Balance</t>
+        </is>
+      </c>
+      <c r="D409" s="18" t="n">
+        <v>1512021.31</v>
+      </c>
+      <c r="E409" s="16" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E397"/>
+  <autoFilter ref="A1:E409"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update game data: day 845, cash 1383547.43, 3-day period 282
</commit_message>
<xml_diff>
--- a/data/supply_chain_game.xlsx
+++ b/data/supply_chain_game.xlsx
@@ -21,15 +21,15 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$283</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$845</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$846</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'资金构成_旧版'!$A$1:$C$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'运营参数_旧版'!$A$9:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$71</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$73</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'排行榜_旧版'!$A$1:$C$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$409</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$421</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'运营参数'!$A$1:$J$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$919</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$946</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -590,7 +590,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-06T15:11:02+08:00</t>
+          <t>2026-09-06T15:26:09+08:00</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>844</v>
+        <v>845</v>
       </c>
     </row>
     <row r="7">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>616</v>
+        <v>615</v>
       </c>
     </row>
     <row r="8">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>1512021.31</v>
+        <v>1383547.43</v>
       </c>
     </row>
     <row r="11">
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>1794375.34</v>
+        <v>1923671.62</v>
       </c>
     </row>
     <row r="15"/>
@@ -786,7 +786,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>266</v>
+        <v>206</v>
       </c>
     </row>
     <row r="25">
@@ -796,7 +796,7 @@
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
     </row>
     <row r="26">
@@ -858,7 +858,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>18</v>
+        <v>78</v>
       </c>
     </row>
     <row r="33">
@@ -878,7 +878,7 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>18</v>
+        <v>78</v>
       </c>
     </row>
     <row r="35">
@@ -898,7 +898,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>18</v>
+        <v>78</v>
       </c>
     </row>
     <row r="37">
@@ -906,6 +906,9 @@
         <is>
           <t>周期现金变动</t>
         </is>
+      </c>
+      <c r="B37" s="4" t="n">
+        <v>-157769.3845113576</v>
       </c>
     </row>
     <row r="38"/>
@@ -967,7 +970,7 @@
         </is>
       </c>
       <c r="B44" s="4" t="n">
-        <v>-80961.80881520314</v>
+        <v>-82530.44876736961</v>
       </c>
     </row>
     <row r="45"/>
@@ -1289,7 +1292,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E919"/>
+  <dimension ref="A1:E946"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -20604,8 +20607,575 @@
         <v>1253178.02</v>
       </c>
     </row>
+    <row r="920">
+      <c r="A920" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:26:09+08:00</t>
+        </is>
+      </c>
+      <c r="B920" s="10" t="n">
+        <v>845</v>
+      </c>
+      <c r="C920" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D920" s="11" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="E920" s="14" t="n">
+        <v>3307219.05</v>
+      </c>
+    </row>
+    <row r="921">
+      <c r="A921" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:26:09+08:00</t>
+        </is>
+      </c>
+      <c r="B921" s="15" t="n">
+        <v>845</v>
+      </c>
+      <c r="C921" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D921" s="16" t="inlineStr">
+        <is>
+          <t>montesquieu</t>
+        </is>
+      </c>
+      <c r="E921" s="18" t="n">
+        <v>2611401.64</v>
+      </c>
+    </row>
+    <row r="922">
+      <c r="A922" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:26:09+08:00</t>
+        </is>
+      </c>
+      <c r="B922" s="10" t="n">
+        <v>845</v>
+      </c>
+      <c r="C922" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D922" s="11" t="inlineStr">
+        <is>
+          <t>nicetry</t>
+        </is>
+      </c>
+      <c r="E922" s="14" t="n">
+        <v>2317571.82</v>
+      </c>
+    </row>
+    <row r="923">
+      <c r="A923" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:26:09+08:00</t>
+        </is>
+      </c>
+      <c r="B923" s="15" t="n">
+        <v>845</v>
+      </c>
+      <c r="C923" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D923" s="16" t="inlineStr">
+        <is>
+          <t>group2</t>
+        </is>
+      </c>
+      <c r="E923" s="18" t="n">
+        <v>2244562.26</v>
+      </c>
+    </row>
+    <row r="924">
+      <c r="A924" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:26:09+08:00</t>
+        </is>
+      </c>
+      <c r="B924" s="10" t="n">
+        <v>845</v>
+      </c>
+      <c r="C924" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="D924" s="11" t="inlineStr">
+        <is>
+          <t>group25</t>
+        </is>
+      </c>
+      <c r="E924" s="14" t="n">
+        <v>2244404.22</v>
+      </c>
+    </row>
+    <row r="925">
+      <c r="A925" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:26:09+08:00</t>
+        </is>
+      </c>
+      <c r="B925" s="15" t="n">
+        <v>845</v>
+      </c>
+      <c r="C925" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="D925" s="16" t="inlineStr">
+        <is>
+          <t>group11</t>
+        </is>
+      </c>
+      <c r="E925" s="18" t="n">
+        <v>2244391.91</v>
+      </c>
+    </row>
+    <row r="926">
+      <c r="A926" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:26:09+08:00</t>
+        </is>
+      </c>
+      <c r="B926" s="10" t="n">
+        <v>845</v>
+      </c>
+      <c r="C926" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="D926" s="11" t="inlineStr">
+        <is>
+          <t>88888888</t>
+        </is>
+      </c>
+      <c r="E926" s="14" t="n">
+        <v>2244369.24</v>
+      </c>
+    </row>
+    <row r="927">
+      <c r="A927" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:26:09+08:00</t>
+        </is>
+      </c>
+      <c r="B927" s="15" t="n">
+        <v>845</v>
+      </c>
+      <c r="C927" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="D927" s="16" t="inlineStr">
+        <is>
+          <t>t24</t>
+        </is>
+      </c>
+      <c r="E927" s="18" t="n">
+        <v>2225166.21</v>
+      </c>
+    </row>
+    <row r="928">
+      <c r="A928" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:26:09+08:00</t>
+        </is>
+      </c>
+      <c r="B928" s="10" t="n">
+        <v>845</v>
+      </c>
+      <c r="C928" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="D928" s="11" t="inlineStr">
+        <is>
+          <t>teamhlly</t>
+        </is>
+      </c>
+      <c r="E928" s="14" t="n">
+        <v>2137145.63</v>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:26:09+08:00</t>
+        </is>
+      </c>
+      <c r="B929" s="15" t="n">
+        <v>845</v>
+      </c>
+      <c r="C929" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="D929" s="16" t="inlineStr">
+        <is>
+          <t>666666</t>
+        </is>
+      </c>
+      <c r="E929" s="18" t="n">
+        <v>2123282.96</v>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:26:09+08:00</t>
+        </is>
+      </c>
+      <c r="B930" s="10" t="n">
+        <v>845</v>
+      </c>
+      <c r="C930" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="D930" s="11" t="inlineStr">
+        <is>
+          <t>group9</t>
+        </is>
+      </c>
+      <c r="E930" s="14" t="n">
+        <v>2097300.15</v>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:26:09+08:00</t>
+        </is>
+      </c>
+      <c r="B931" s="15" t="n">
+        <v>845</v>
+      </c>
+      <c r="C931" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="D931" s="16" t="inlineStr">
+        <is>
+          <t>group14</t>
+        </is>
+      </c>
+      <c r="E931" s="18" t="n">
+        <v>2064265.92</v>
+      </c>
+    </row>
+    <row r="932">
+      <c r="A932" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:26:09+08:00</t>
+        </is>
+      </c>
+      <c r="B932" s="10" t="n">
+        <v>845</v>
+      </c>
+      <c r="C932" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="D932" s="11" t="inlineStr">
+        <is>
+          <t>group8</t>
+        </is>
+      </c>
+      <c r="E932" s="14" t="n">
+        <v>2056583.3</v>
+      </c>
+    </row>
+    <row r="933">
+      <c r="A933" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:26:09+08:00</t>
+        </is>
+      </c>
+      <c r="B933" s="15" t="n">
+        <v>845</v>
+      </c>
+      <c r="C933" s="15" t="n">
+        <v>14</v>
+      </c>
+      <c r="D933" s="16" t="inlineStr">
+        <is>
+          <t>group15</t>
+        </is>
+      </c>
+      <c r="E933" s="18" t="n">
+        <v>2022884.31</v>
+      </c>
+    </row>
+    <row r="934">
+      <c r="A934" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:26:09+08:00</t>
+        </is>
+      </c>
+      <c r="B934" s="10" t="n">
+        <v>845</v>
+      </c>
+      <c r="C934" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="D934" s="11" t="inlineStr">
+        <is>
+          <t>tigagroup20</t>
+        </is>
+      </c>
+      <c r="E934" s="14" t="n">
+        <v>2002788.05</v>
+      </c>
+    </row>
+    <row r="935">
+      <c r="A935" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:26:09+08:00</t>
+        </is>
+      </c>
+      <c r="B935" s="15" t="n">
+        <v>845</v>
+      </c>
+      <c r="C935" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="D935" s="16" t="inlineStr">
+        <is>
+          <t>deepsleep</t>
+        </is>
+      </c>
+      <c r="E935" s="18" t="n">
+        <v>1856167.39</v>
+      </c>
+    </row>
+    <row r="936">
+      <c r="A936" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:26:09+08:00</t>
+        </is>
+      </c>
+      <c r="B936" s="10" t="n">
+        <v>845</v>
+      </c>
+      <c r="C936" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="D936" s="11" t="inlineStr">
+        <is>
+          <t>jit</t>
+        </is>
+      </c>
+      <c r="E936" s="14" t="n">
+        <v>1820549.75</v>
+      </c>
+    </row>
+    <row r="937">
+      <c r="A937" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:26:09+08:00</t>
+        </is>
+      </c>
+      <c r="B937" s="15" t="n">
+        <v>845</v>
+      </c>
+      <c r="C937" s="15" t="n">
+        <v>18</v>
+      </c>
+      <c r="D937" s="16" t="inlineStr">
+        <is>
+          <t>cleveregg</t>
+        </is>
+      </c>
+      <c r="E937" s="18" t="n">
+        <v>1814321.41</v>
+      </c>
+    </row>
+    <row r="938">
+      <c r="A938" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:26:09+08:00</t>
+        </is>
+      </c>
+      <c r="B938" s="10" t="n">
+        <v>845</v>
+      </c>
+      <c r="C938" s="10" t="n">
+        <v>19</v>
+      </c>
+      <c r="D938" s="11" t="inlineStr">
+        <is>
+          <t>group7</t>
+        </is>
+      </c>
+      <c r="E938" s="14" t="n">
+        <v>1773702.97</v>
+      </c>
+    </row>
+    <row r="939">
+      <c r="A939" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:26:09+08:00</t>
+        </is>
+      </c>
+      <c r="B939" s="15" t="n">
+        <v>845</v>
+      </c>
+      <c r="C939" s="15" t="n">
+        <v>20</v>
+      </c>
+      <c r="D939" s="16" t="inlineStr">
+        <is>
+          <t>aaachemicalseller</t>
+        </is>
+      </c>
+      <c r="E939" s="18" t="n">
+        <v>1650437.17</v>
+      </c>
+    </row>
+    <row r="940">
+      <c r="A940" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:26:09+08:00</t>
+        </is>
+      </c>
+      <c r="B940" s="10" t="n">
+        <v>845</v>
+      </c>
+      <c r="C940" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="D940" s="11" t="inlineStr">
+        <is>
+          <t>newgroup18</t>
+        </is>
+      </c>
+      <c r="E940" s="14" t="n">
+        <v>1612968.19</v>
+      </c>
+    </row>
+    <row r="941">
+      <c r="A941" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:26:09+08:00</t>
+        </is>
+      </c>
+      <c r="B941" s="15" t="n">
+        <v>845</v>
+      </c>
+      <c r="C941" s="15" t="n">
+        <v>22</v>
+      </c>
+      <c r="D941" s="16" t="inlineStr">
+        <is>
+          <t>vivo50</t>
+        </is>
+      </c>
+      <c r="E941" s="18" t="n">
+        <v>1612845.78</v>
+      </c>
+    </row>
+    <row r="942">
+      <c r="A942" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:26:09+08:00</t>
+        </is>
+      </c>
+      <c r="B942" s="10" t="n">
+        <v>845</v>
+      </c>
+      <c r="C942" s="10" t="n">
+        <v>23</v>
+      </c>
+      <c r="D942" s="11" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E942" s="14" t="n">
+        <v>1586457.02</v>
+      </c>
+    </row>
+    <row r="943">
+      <c r="A943" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:26:09+08:00</t>
+        </is>
+      </c>
+      <c r="B943" s="15" t="n">
+        <v>845</v>
+      </c>
+      <c r="C943" s="15" t="n">
+        <v>24</v>
+      </c>
+      <c r="D943" s="16" t="inlineStr">
+        <is>
+          <t>group12</t>
+        </is>
+      </c>
+      <c r="E943" s="18" t="n">
+        <v>1538774.32</v>
+      </c>
+    </row>
+    <row r="944">
+      <c r="A944" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:26:09+08:00</t>
+        </is>
+      </c>
+      <c r="B944" s="10" t="n">
+        <v>845</v>
+      </c>
+      <c r="C944" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="D944" s="11" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E944" s="14" t="n">
+        <v>1474218.21</v>
+      </c>
+    </row>
+    <row r="945">
+      <c r="A945" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:26:09+08:00</t>
+        </is>
+      </c>
+      <c r="B945" s="24" t="n">
+        <v>845</v>
+      </c>
+      <c r="C945" s="24" t="n">
+        <v>26</v>
+      </c>
+      <c r="D945" s="25" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="E945" s="26" t="n">
+        <v>1383547.43</v>
+      </c>
+    </row>
+    <row r="946">
+      <c r="A946" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:26:09+08:00</t>
+        </is>
+      </c>
+      <c r="B946" s="10" t="n">
+        <v>845</v>
+      </c>
+      <c r="C946" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="D946" s="11" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="E946" s="14" t="n">
+        <v>1189688.87</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E919"/>
+  <autoFilter ref="A1:E946"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -38451,7 +39021,7 @@
         <v>846</v>
       </c>
       <c r="D283" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E283" s="16" t="inlineStr">
         <is>
@@ -38464,41 +39034,43 @@
         </is>
       </c>
       <c r="G283" s="17" t="n">
-        <v>18</v>
+        <v>78</v>
       </c>
       <c r="H283" s="17" t="n">
         <v>0</v>
       </c>
       <c r="I283" s="17" t="n">
-        <v>18</v>
+        <v>78</v>
       </c>
       <c r="J283" s="19" t="n">
         <v>1</v>
       </c>
       <c r="K283" s="17" t="n">
-        <v>18</v>
+        <v>78</v>
       </c>
       <c r="L283" s="18" t="n">
-        <v>1512021.31</v>
+        <v>1541316.814511358</v>
       </c>
       <c r="M283" s="18" t="n">
-        <v>1512021.31</v>
-      </c>
-      <c r="N283" s="16" t="n"/>
+        <v>1383547.43</v>
+      </c>
+      <c r="N283" s="18" t="n">
+        <v>-157769.3845113576</v>
+      </c>
       <c r="O283" s="17" t="n">
-        <v>266</v>
+        <v>206</v>
       </c>
       <c r="P283" s="17" t="n">
-        <v>266</v>
+        <v>236</v>
       </c>
       <c r="Q283" s="17" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="R283" s="17" t="n">
         <v>200</v>
       </c>
       <c r="S283" s="18" t="n">
-        <v>26100</v>
+        <v>113100</v>
       </c>
     </row>
   </sheetData>
@@ -38513,7 +39085,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N845"/>
+  <dimension ref="A1:N846"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -77428,8 +78000,54 @@
         <v>26100</v>
       </c>
     </row>
+    <row r="846">
+      <c r="A846" s="10" t="n">
+        <v>845</v>
+      </c>
+      <c r="B846" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C846" s="12" t="n">
+        <v>60</v>
+      </c>
+      <c r="D846" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E846" s="12" t="n">
+        <v>60</v>
+      </c>
+      <c r="F846" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G846" s="12" t="n">
+        <v>60</v>
+      </c>
+      <c r="H846" s="14" t="n">
+        <v>1383547.43</v>
+      </c>
+      <c r="I846" s="12" t="n">
+        <v>206</v>
+      </c>
+      <c r="J846" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="K846" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L846" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="M846" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N846" s="14" t="n">
+        <v>87000</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N845"/>
+  <autoFilter ref="A1:N846"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -77824,7 +78442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F71"/>
+  <dimension ref="A1:F73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -79561,8 +80179,56 @@
         <v>55</v>
       </c>
     </row>
+    <row r="72">
+      <c r="A72" s="21" t="n">
+        <v>730.66</v>
+      </c>
+      <c r="B72" s="11" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C72" s="11" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D72" s="11" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E72" s="11" t="inlineStr"/>
+      <c r="F72" s="12" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="23" t="n">
+        <v>742.75</v>
+      </c>
+      <c r="B73" s="16" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C73" s="16" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D73" s="16" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E73" s="16" t="inlineStr"/>
+      <c r="F73" s="17" t="n">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F71"/>
+  <autoFilter ref="A1:F73"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -79961,7 +80627,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U34"/>
+  <dimension ref="A1:U35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -79984,7 +80650,7 @@
     <col width="12" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
-    <col width="20" customWidth="1" min="21" max="21"/>
+    <col width="21" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -82389,8 +83055,77 @@
       </c>
       <c r="U34" s="11" t="n"/>
     </row>
+    <row r="35">
+      <c r="A35" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:26:09+08:00</t>
+        </is>
+      </c>
+      <c r="B35" s="15" t="n">
+        <v>845</v>
+      </c>
+      <c r="C35" s="18" t="n">
+        <v>1383547.43</v>
+      </c>
+      <c r="D35" s="15" t="n">
+        <v>26</v>
+      </c>
+      <c r="E35" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="F35" s="16" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="G35" s="18" t="n">
+        <v>1923671.62</v>
+      </c>
+      <c r="H35" s="23" t="n">
+        <v>55</v>
+      </c>
+      <c r="I35" s="16" t="n"/>
+      <c r="J35" s="16" t="inlineStr">
+        <is>
+          <t>mail</t>
+        </is>
+      </c>
+      <c r="K35" s="27" t="n">
+        <v>3600</v>
+      </c>
+      <c r="L35" s="27" t="n">
+        <v>200</v>
+      </c>
+      <c r="M35" s="17" t="n">
+        <v>206</v>
+      </c>
+      <c r="N35" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="O35" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="P35" s="15" t="n">
+        <v>282</v>
+      </c>
+      <c r="Q35" s="17" t="n">
+        <v>78</v>
+      </c>
+      <c r="R35" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="S35" s="17" t="n">
+        <v>78</v>
+      </c>
+      <c r="T35" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="U35" s="18" t="n">
+        <v>-157769.3845113576</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U34"/>
+  <autoFilter ref="A1:U35"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -82401,7 +83136,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E409"/>
+  <dimension ref="A1:E421"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -91686,8 +92421,280 @@
         </is>
       </c>
     </row>
+    <row r="410">
+      <c r="A410" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:26:09+08:00</t>
+        </is>
+      </c>
+      <c r="B410" s="10" t="n">
+        <v>845</v>
+      </c>
+      <c r="C410" s="11" t="inlineStr">
+        <is>
+          <t>Starting Cash</t>
+        </is>
+      </c>
+      <c r="D410" s="14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E410" s="11" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:26:09+08:00</t>
+        </is>
+      </c>
+      <c r="B411" s="15" t="n">
+        <v>845</v>
+      </c>
+      <c r="C411" s="16" t="inlineStr">
+        <is>
+          <t>Cash Sources</t>
+        </is>
+      </c>
+      <c r="D411" s="16" t="n"/>
+      <c r="E411" s="16" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:26:09+08:00</t>
+        </is>
+      </c>
+      <c r="B412" s="10" t="n">
+        <v>845</v>
+      </c>
+      <c r="C412" s="11" t="inlineStr">
+        <is>
+          <t>revenues</t>
+        </is>
+      </c>
+      <c r="D412" s="14" t="n">
+        <v>22873750</v>
+      </c>
+      <c r="E412" s="11" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:26:09+08:00</t>
+        </is>
+      </c>
+      <c r="B413" s="15" t="n">
+        <v>845</v>
+      </c>
+      <c r="C413" s="16" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D413" s="18" t="n">
+        <v>304022.38</v>
+      </c>
+      <c r="E413" s="16" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:26:09+08:00</t>
+        </is>
+      </c>
+      <c r="B414" s="10" t="n">
+        <v>845</v>
+      </c>
+      <c r="C414" s="11" t="inlineStr">
+        <is>
+          <t>Cash Uses</t>
+        </is>
+      </c>
+      <c r="D414" s="11" t="n"/>
+      <c r="E414" s="11" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:26:09+08:00</t>
+        </is>
+      </c>
+      <c r="B415" s="15" t="n">
+        <v>845</v>
+      </c>
+      <c r="C415" s="16" t="inlineStr">
+        <is>
+          <t>outbound shipping</t>
+        </is>
+      </c>
+      <c r="D415" s="18" t="n">
+        <v>-2366250</v>
+      </c>
+      <c r="E415" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:26:09+08:00</t>
+        </is>
+      </c>
+      <c r="B416" s="10" t="n">
+        <v>845</v>
+      </c>
+      <c r="C416" s="11" t="inlineStr">
+        <is>
+          <t>inbound shipping</t>
+        </is>
+      </c>
+      <c r="D416" s="14" t="n">
+        <v>-1620000</v>
+      </c>
+      <c r="E416" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:26:09+08:00</t>
+        </is>
+      </c>
+      <c r="B417" s="15" t="n">
+        <v>845</v>
+      </c>
+      <c r="C417" s="16" t="inlineStr">
+        <is>
+          <t>FGI holding</t>
+        </is>
+      </c>
+      <c r="D417" s="18" t="n">
+        <v>-22197.63</v>
+      </c>
+      <c r="E417" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:26:09+08:00</t>
+        </is>
+      </c>
+      <c r="B418" s="10" t="n">
+        <v>845</v>
+      </c>
+      <c r="C418" s="11" t="inlineStr">
+        <is>
+          <t>add capacity</t>
+        </is>
+      </c>
+      <c r="D418" s="14" t="n">
+        <v>-1749840.87</v>
+      </c>
+      <c r="E418" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:26:09+08:00</t>
+        </is>
+      </c>
+      <c r="B419" s="15" t="n">
+        <v>845</v>
+      </c>
+      <c r="C419" s="16" t="inlineStr">
+        <is>
+          <t>Pipeline inventory holding</t>
+        </is>
+      </c>
+      <c r="D419" s="18" t="n">
+        <v>-29936.45</v>
+      </c>
+      <c r="E419" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:26:09+08:00</t>
+        </is>
+      </c>
+      <c r="B420" s="10" t="n">
+        <v>845</v>
+      </c>
+      <c r="C420" s="11" t="inlineStr">
+        <is>
+          <t>production</t>
+        </is>
+      </c>
+      <c r="D420" s="14" t="n">
+        <v>-16506000</v>
+      </c>
+      <c r="E420" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:26:09+08:00</t>
+        </is>
+      </c>
+      <c r="B421" s="15" t="n">
+        <v>845</v>
+      </c>
+      <c r="C421" s="16" t="inlineStr">
+        <is>
+          <t>Cash Balance</t>
+        </is>
+      </c>
+      <c r="D421" s="18" t="n">
+        <v>1383547.43</v>
+      </c>
+      <c r="E421" s="16" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E409"/>
+  <autoFilter ref="A1:E421"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update game data: day 846, cash 1428006.31, 3-day period 282
</commit_message>
<xml_diff>
--- a/data/supply_chain_game.xlsx
+++ b/data/supply_chain_game.xlsx
@@ -21,15 +21,15 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$283</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$846</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$847</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'资金构成_旧版'!$A$1:$C$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'运营参数_旧版'!$A$9:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$75</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'排行榜_旧版'!$A$1:$C$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$35</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$421</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$433</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'运营参数'!$A$1:$J$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$946</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$973</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -590,7 +590,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-06T15:26:09+08:00</t>
+          <t>2026-09-06T15:41:03+08:00</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>845</v>
+        <v>846</v>
       </c>
     </row>
     <row r="7">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>615</v>
+        <v>614</v>
       </c>
     </row>
     <row r="8">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>1383547.43</v>
+        <v>1428006.31</v>
       </c>
     </row>
     <row r="11">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>1923671.62</v>
+        <v>1924235.35</v>
       </c>
     </row>
     <row r="15"/>
@@ -786,7 +786,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>206</v>
+        <v>354</v>
       </c>
     </row>
     <row r="25">
@@ -796,7 +796,7 @@
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -847,7 +847,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>否（进行中）</t>
+          <t>是</t>
         </is>
       </c>
     </row>
@@ -858,7 +858,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>78</v>
+        <v>130</v>
       </c>
     </row>
     <row r="33">
@@ -878,7 +878,7 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>78</v>
+        <v>130</v>
       </c>
     </row>
     <row r="35">
@@ -898,7 +898,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>78</v>
+        <v>130</v>
       </c>
     </row>
     <row r="37">
@@ -908,7 +908,7 @@
         </is>
       </c>
       <c r="B37" s="4" t="n">
-        <v>-157769.3845113576</v>
+        <v>-86336.76161287585</v>
       </c>
     </row>
     <row r="38"/>
@@ -926,7 +926,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="41">
@@ -937,7 +937,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>841–843</t>
+          <t>844–846</t>
         </is>
       </c>
     </row>
@@ -949,7 +949,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>169.0 / 0.0 / 169.0</t>
+          <t>130.0 / 0.0 / 130.0</t>
         </is>
       </c>
     </row>
@@ -970,7 +970,7 @@
         </is>
       </c>
       <c r="B44" s="4" t="n">
-        <v>-82530.44876736961</v>
+        <v>-86336.76161287585</v>
       </c>
     </row>
     <row r="45"/>
@@ -1292,7 +1292,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E946"/>
+  <dimension ref="A1:E973"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -21174,8 +21174,575 @@
         <v>1189688.87</v>
       </c>
     </row>
+    <row r="947">
+      <c r="A947" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B947" s="15" t="n">
+        <v>846</v>
+      </c>
+      <c r="C947" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D947" s="16" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="E947" s="18" t="n">
+        <v>3352241.66</v>
+      </c>
+    </row>
+    <row r="948">
+      <c r="A948" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B948" s="10" t="n">
+        <v>846</v>
+      </c>
+      <c r="C948" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D948" s="11" t="inlineStr">
+        <is>
+          <t>montesquieu</t>
+        </is>
+      </c>
+      <c r="E948" s="14" t="n">
+        <v>2395526.67</v>
+      </c>
+    </row>
+    <row r="949">
+      <c r="A949" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B949" s="15" t="n">
+        <v>846</v>
+      </c>
+      <c r="C949" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D949" s="16" t="inlineStr">
+        <is>
+          <t>nicetry</t>
+        </is>
+      </c>
+      <c r="E949" s="18" t="n">
+        <v>2354486.85</v>
+      </c>
+    </row>
+    <row r="950">
+      <c r="A950" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B950" s="10" t="n">
+        <v>846</v>
+      </c>
+      <c r="C950" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D950" s="11" t="inlineStr">
+        <is>
+          <t>group2</t>
+        </is>
+      </c>
+      <c r="E950" s="14" t="n">
+        <v>2289258.03</v>
+      </c>
+    </row>
+    <row r="951">
+      <c r="A951" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B951" s="15" t="n">
+        <v>846</v>
+      </c>
+      <c r="C951" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="D951" s="16" t="inlineStr">
+        <is>
+          <t>group25</t>
+        </is>
+      </c>
+      <c r="E951" s="18" t="n">
+        <v>2289099.95</v>
+      </c>
+    </row>
+    <row r="952">
+      <c r="A952" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B952" s="10" t="n">
+        <v>846</v>
+      </c>
+      <c r="C952" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="D952" s="11" t="inlineStr">
+        <is>
+          <t>group11</t>
+        </is>
+      </c>
+      <c r="E952" s="14" t="n">
+        <v>2289087.64</v>
+      </c>
+    </row>
+    <row r="953">
+      <c r="A953" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B953" s="15" t="n">
+        <v>846</v>
+      </c>
+      <c r="C953" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="D953" s="16" t="inlineStr">
+        <is>
+          <t>88888888</t>
+        </is>
+      </c>
+      <c r="E953" s="18" t="n">
+        <v>2289064.97</v>
+      </c>
+    </row>
+    <row r="954">
+      <c r="A954" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B954" s="10" t="n">
+        <v>846</v>
+      </c>
+      <c r="C954" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="D954" s="11" t="inlineStr">
+        <is>
+          <t>t24</t>
+        </is>
+      </c>
+      <c r="E954" s="14" t="n">
+        <v>2269906.57</v>
+      </c>
+    </row>
+    <row r="955">
+      <c r="A955" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B955" s="15" t="n">
+        <v>846</v>
+      </c>
+      <c r="C955" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="D955" s="16" t="inlineStr">
+        <is>
+          <t>teamhlly</t>
+        </is>
+      </c>
+      <c r="E955" s="18" t="n">
+        <v>2222095.17</v>
+      </c>
+    </row>
+    <row r="956">
+      <c r="A956" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B956" s="10" t="n">
+        <v>846</v>
+      </c>
+      <c r="C956" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="D956" s="11" t="inlineStr">
+        <is>
+          <t>group9</t>
+        </is>
+      </c>
+      <c r="E956" s="14" t="n">
+        <v>2141938.29</v>
+      </c>
+    </row>
+    <row r="957">
+      <c r="A957" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B957" s="15" t="n">
+        <v>846</v>
+      </c>
+      <c r="C957" s="15" t="n">
+        <v>11</v>
+      </c>
+      <c r="D957" s="16" t="inlineStr">
+        <is>
+          <t>group14</t>
+        </is>
+      </c>
+      <c r="E957" s="18" t="n">
+        <v>2064695.43</v>
+      </c>
+    </row>
+    <row r="958">
+      <c r="A958" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B958" s="10" t="n">
+        <v>846</v>
+      </c>
+      <c r="C958" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="D958" s="11" t="inlineStr">
+        <is>
+          <t>tigagroup20</t>
+        </is>
+      </c>
+      <c r="E958" s="14" t="n">
+        <v>2047413.31</v>
+      </c>
+    </row>
+    <row r="959">
+      <c r="A959" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B959" s="15" t="n">
+        <v>846</v>
+      </c>
+      <c r="C959" s="15" t="n">
+        <v>13</v>
+      </c>
+      <c r="D959" s="16" t="inlineStr">
+        <is>
+          <t>group15</t>
+        </is>
+      </c>
+      <c r="E959" s="18" t="n">
+        <v>2023303.01</v>
+      </c>
+    </row>
+    <row r="960">
+      <c r="A960" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B960" s="10" t="n">
+        <v>846</v>
+      </c>
+      <c r="C960" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="D960" s="11" t="inlineStr">
+        <is>
+          <t>666666</t>
+        </is>
+      </c>
+      <c r="E960" s="14" t="n">
+        <v>1951458.04</v>
+      </c>
+    </row>
+    <row r="961">
+      <c r="A961" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B961" s="15" t="n">
+        <v>846</v>
+      </c>
+      <c r="C961" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="D961" s="16" t="inlineStr">
+        <is>
+          <t>deepsleep</t>
+        </is>
+      </c>
+      <c r="E961" s="18" t="n">
+        <v>1882548.28</v>
+      </c>
+    </row>
+    <row r="962">
+      <c r="A962" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B962" s="10" t="n">
+        <v>846</v>
+      </c>
+      <c r="C962" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="D962" s="11" t="inlineStr">
+        <is>
+          <t>cleveregg</t>
+        </is>
+      </c>
+      <c r="E962" s="14" t="n">
+        <v>1858874.16</v>
+      </c>
+    </row>
+    <row r="963">
+      <c r="A963" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B963" s="15" t="n">
+        <v>846</v>
+      </c>
+      <c r="C963" s="15" t="n">
+        <v>17</v>
+      </c>
+      <c r="D963" s="16" t="inlineStr">
+        <is>
+          <t>group8</t>
+        </is>
+      </c>
+      <c r="E963" s="18" t="n">
+        <v>1840462.58</v>
+      </c>
+    </row>
+    <row r="964">
+      <c r="A964" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B964" s="10" t="n">
+        <v>846</v>
+      </c>
+      <c r="C964" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="D964" s="11" t="inlineStr">
+        <is>
+          <t>jit</t>
+        </is>
+      </c>
+      <c r="E964" s="14" t="n">
+        <v>1817576.24</v>
+      </c>
+    </row>
+    <row r="965">
+      <c r="A965" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B965" s="15" t="n">
+        <v>846</v>
+      </c>
+      <c r="C965" s="15" t="n">
+        <v>19</v>
+      </c>
+      <c r="D965" s="16" t="inlineStr">
+        <is>
+          <t>group7</t>
+        </is>
+      </c>
+      <c r="E965" s="18" t="n">
+        <v>1774056.6</v>
+      </c>
+    </row>
+    <row r="966">
+      <c r="A966" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B966" s="10" t="n">
+        <v>846</v>
+      </c>
+      <c r="C966" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="D966" s="11" t="inlineStr">
+        <is>
+          <t>newgroup18</t>
+        </is>
+      </c>
+      <c r="E966" s="14" t="n">
+        <v>1697779.84</v>
+      </c>
+    </row>
+    <row r="967">
+      <c r="A967" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B967" s="15" t="n">
+        <v>846</v>
+      </c>
+      <c r="C967" s="15" t="n">
+        <v>21</v>
+      </c>
+      <c r="D967" s="16" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E967" s="18" t="n">
+        <v>1697279.68</v>
+      </c>
+    </row>
+    <row r="968">
+      <c r="A968" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B968" s="10" t="n">
+        <v>846</v>
+      </c>
+      <c r="C968" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="D968" s="11" t="inlineStr">
+        <is>
+          <t>vivo50</t>
+        </is>
+      </c>
+      <c r="E968" s="14" t="n">
+        <v>1657346.73</v>
+      </c>
+    </row>
+    <row r="969">
+      <c r="A969" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B969" s="15" t="n">
+        <v>846</v>
+      </c>
+      <c r="C969" s="15" t="n">
+        <v>23</v>
+      </c>
+      <c r="D969" s="16" t="inlineStr">
+        <is>
+          <t>group12</t>
+        </is>
+      </c>
+      <c r="E969" s="18" t="n">
+        <v>1583255.93</v>
+      </c>
+    </row>
+    <row r="970">
+      <c r="A970" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B970" s="10" t="n">
+        <v>846</v>
+      </c>
+      <c r="C970" s="10" t="n">
+        <v>24</v>
+      </c>
+      <c r="D970" s="11" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E970" s="14" t="n">
+        <v>1518668.99</v>
+      </c>
+    </row>
+    <row r="971">
+      <c r="A971" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B971" s="15" t="n">
+        <v>846</v>
+      </c>
+      <c r="C971" s="15" t="n">
+        <v>25</v>
+      </c>
+      <c r="D971" s="16" t="inlineStr">
+        <is>
+          <t>aaachemicalseller</t>
+        </is>
+      </c>
+      <c r="E971" s="18" t="n">
+        <v>1478478.78</v>
+      </c>
+    </row>
+    <row r="972">
+      <c r="A972" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B972" s="24" t="n">
+        <v>846</v>
+      </c>
+      <c r="C972" s="24" t="n">
+        <v>26</v>
+      </c>
+      <c r="D972" s="25" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="E972" s="26" t="n">
+        <v>1428006.31</v>
+      </c>
+    </row>
+    <row r="973">
+      <c r="A973" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B973" s="15" t="n">
+        <v>846</v>
+      </c>
+      <c r="C973" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="D973" s="16" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="E973" s="18" t="n">
+        <v>1234156.18</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E946"/>
+  <autoFilter ref="A1:E973"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -39021,11 +39588,11 @@
         <v>846</v>
       </c>
       <c r="D283" s="15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E283" s="16" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="F283" s="16" t="inlineStr">
@@ -39034,43 +39601,43 @@
         </is>
       </c>
       <c r="G283" s="17" t="n">
-        <v>78</v>
+        <v>130</v>
       </c>
       <c r="H283" s="17" t="n">
         <v>0</v>
       </c>
       <c r="I283" s="17" t="n">
-        <v>78</v>
+        <v>130</v>
       </c>
       <c r="J283" s="19" t="n">
         <v>1</v>
       </c>
       <c r="K283" s="17" t="n">
-        <v>78</v>
+        <v>130</v>
       </c>
       <c r="L283" s="18" t="n">
-        <v>1541316.814511358</v>
+        <v>1514343.071612876</v>
       </c>
       <c r="M283" s="18" t="n">
-        <v>1383547.43</v>
+        <v>1428006.31</v>
       </c>
       <c r="N283" s="18" t="n">
-        <v>-157769.3845113576</v>
+        <v>-86336.76161287585</v>
       </c>
       <c r="O283" s="17" t="n">
-        <v>206</v>
+        <v>354</v>
       </c>
       <c r="P283" s="17" t="n">
-        <v>236</v>
+        <v>275.3333333333333</v>
       </c>
       <c r="Q283" s="17" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="R283" s="17" t="n">
         <v>200</v>
       </c>
       <c r="S283" s="18" t="n">
-        <v>113100</v>
+        <v>188500</v>
       </c>
     </row>
   </sheetData>
@@ -39085,7 +39652,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N846"/>
+  <dimension ref="A1:N847"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -78046,8 +78613,54 @@
         <v>87000</v>
       </c>
     </row>
+    <row r="847">
+      <c r="A847" s="15" t="n">
+        <v>846</v>
+      </c>
+      <c r="B847" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C847" s="17" t="n">
+        <v>52</v>
+      </c>
+      <c r="D847" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E847" s="17" t="n">
+        <v>52</v>
+      </c>
+      <c r="F847" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G847" s="17" t="n">
+        <v>52</v>
+      </c>
+      <c r="H847" s="18" t="n">
+        <v>1428006.31</v>
+      </c>
+      <c r="I847" s="17" t="n">
+        <v>354</v>
+      </c>
+      <c r="J847" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K847" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L847" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M847" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N847" s="18" t="n">
+        <v>75400</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N846"/>
+  <autoFilter ref="A1:N847"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -78442,7 +79055,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F73"/>
+  <dimension ref="A1:F75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -80227,8 +80840,56 @@
         <v>55</v>
       </c>
     </row>
+    <row r="74">
+      <c r="A74" s="21" t="n">
+        <v>730.66</v>
+      </c>
+      <c r="B74" s="11" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C74" s="11" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D74" s="11" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E74" s="11" t="inlineStr"/>
+      <c r="F74" s="12" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="23" t="n">
+        <v>742.75</v>
+      </c>
+      <c r="B75" s="16" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C75" s="16" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D75" s="16" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E75" s="16" t="inlineStr"/>
+      <c r="F75" s="17" t="n">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F73"/>
+  <autoFilter ref="A1:F75"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -80627,7 +81288,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U35"/>
+  <dimension ref="A1:U36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -80636,7 +81297,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
@@ -80650,7 +81311,7 @@
     <col width="12" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
-    <col width="21" customWidth="1" min="21" max="21"/>
+    <col width="20" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -83124,8 +83785,77 @@
         <v>-157769.3845113576</v>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B36" s="10" t="n">
+        <v>846</v>
+      </c>
+      <c r="C36" s="14" t="n">
+        <v>1428006.31</v>
+      </c>
+      <c r="D36" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="E36" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="F36" s="11" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="G36" s="14" t="n">
+        <v>1924235.35</v>
+      </c>
+      <c r="H36" s="21" t="n">
+        <v>55</v>
+      </c>
+      <c r="I36" s="11" t="n"/>
+      <c r="J36" s="11" t="inlineStr">
+        <is>
+          <t>mail</t>
+        </is>
+      </c>
+      <c r="K36" s="22" t="n">
+        <v>3600</v>
+      </c>
+      <c r="L36" s="22" t="n">
+        <v>200</v>
+      </c>
+      <c r="M36" s="12" t="n">
+        <v>354</v>
+      </c>
+      <c r="N36" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="O36" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="P36" s="10" t="n">
+        <v>282</v>
+      </c>
+      <c r="Q36" s="12" t="n">
+        <v>130</v>
+      </c>
+      <c r="R36" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S36" s="12" t="n">
+        <v>130</v>
+      </c>
+      <c r="T36" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="U36" s="14" t="n">
+        <v>-86336.76161287585</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U35"/>
+  <autoFilter ref="A1:U36"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -83136,7 +83866,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E421"/>
+  <dimension ref="A1:E433"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -92693,8 +93423,280 @@
         </is>
       </c>
     </row>
+    <row r="422">
+      <c r="A422" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B422" s="10" t="n">
+        <v>846</v>
+      </c>
+      <c r="C422" s="11" t="inlineStr">
+        <is>
+          <t>Starting Cash</t>
+        </is>
+      </c>
+      <c r="D422" s="14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E422" s="11" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B423" s="15" t="n">
+        <v>846</v>
+      </c>
+      <c r="C423" s="16" t="inlineStr">
+        <is>
+          <t>Cash Sources</t>
+        </is>
+      </c>
+      <c r="D423" s="16" t="n"/>
+      <c r="E423" s="16" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B424" s="10" t="n">
+        <v>846</v>
+      </c>
+      <c r="C424" s="11" t="inlineStr">
+        <is>
+          <t>revenues</t>
+        </is>
+      </c>
+      <c r="D424" s="14" t="n">
+        <v>22923050</v>
+      </c>
+      <c r="E424" s="11" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B425" s="15" t="n">
+        <v>846</v>
+      </c>
+      <c r="C425" s="16" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D425" s="18" t="n">
+        <v>304383.87</v>
+      </c>
+      <c r="E425" s="16" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B426" s="10" t="n">
+        <v>846</v>
+      </c>
+      <c r="C426" s="11" t="inlineStr">
+        <is>
+          <t>Cash Uses</t>
+        </is>
+      </c>
+      <c r="D426" s="11" t="n"/>
+      <c r="E426" s="11" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B427" s="15" t="n">
+        <v>846</v>
+      </c>
+      <c r="C427" s="16" t="inlineStr">
+        <is>
+          <t>outbound shipping</t>
+        </is>
+      </c>
+      <c r="D427" s="18" t="n">
+        <v>-2371350</v>
+      </c>
+      <c r="E427" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B428" s="10" t="n">
+        <v>846</v>
+      </c>
+      <c r="C428" s="11" t="inlineStr">
+        <is>
+          <t>inbound shipping</t>
+        </is>
+      </c>
+      <c r="D428" s="14" t="n">
+        <v>-1620000</v>
+      </c>
+      <c r="E428" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B429" s="15" t="n">
+        <v>846</v>
+      </c>
+      <c r="C429" s="16" t="inlineStr">
+        <is>
+          <t>FGI holding</t>
+        </is>
+      </c>
+      <c r="D429" s="18" t="n">
+        <v>-22250.39</v>
+      </c>
+      <c r="E429" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B430" s="10" t="n">
+        <v>846</v>
+      </c>
+      <c r="C430" s="11" t="inlineStr">
+        <is>
+          <t>add capacity</t>
+        </is>
+      </c>
+      <c r="D430" s="14" t="n">
+        <v>-1749840.87</v>
+      </c>
+      <c r="E430" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B431" s="15" t="n">
+        <v>846</v>
+      </c>
+      <c r="C431" s="16" t="inlineStr">
+        <is>
+          <t>Pipeline inventory holding</t>
+        </is>
+      </c>
+      <c r="D431" s="18" t="n">
+        <v>-29986.3</v>
+      </c>
+      <c r="E431" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B432" s="10" t="n">
+        <v>846</v>
+      </c>
+      <c r="C432" s="11" t="inlineStr">
+        <is>
+          <t>production</t>
+        </is>
+      </c>
+      <c r="D432" s="14" t="n">
+        <v>-16506000</v>
+      </c>
+      <c r="E432" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:41:03+08:00</t>
+        </is>
+      </c>
+      <c r="B433" s="15" t="n">
+        <v>846</v>
+      </c>
+      <c r="C433" s="16" t="inlineStr">
+        <is>
+          <t>Cash Balance</t>
+        </is>
+      </c>
+      <c r="D433" s="18" t="n">
+        <v>1428006.31</v>
+      </c>
+      <c r="E433" s="16" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E421"/>
+  <autoFilter ref="A1:E433"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update game data: day 847, cash 1495887.76, 3-day period 283
</commit_message>
<xml_diff>
--- a/data/supply_chain_game.xlsx
+++ b/data/supply_chain_game.xlsx
@@ -20,16 +20,16 @@
     <sheet name="排行榜" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$283</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$847</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$284</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$848</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'资金构成_旧版'!$A$1:$C$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'运营参数_旧版'!$A$9:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$75</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$77</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'排行榜_旧版'!$A$1:$C$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$36</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$433</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$445</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'运营参数'!$A$1:$J$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$973</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$1000</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -590,7 +590,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-06T15:41:03+08:00</t>
+          <t>2026-09-06T15:56:03+08:00</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>846</v>
+        <v>847</v>
       </c>
     </row>
     <row r="7">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>614</v>
+        <v>613</v>
       </c>
     </row>
     <row r="8">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>1428006.31</v>
+        <v>1495887.76</v>
       </c>
     </row>
     <row r="11">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>1924235.35</v>
+        <v>1758278.43</v>
       </c>
     </row>
     <row r="15"/>
@@ -786,7 +786,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>354</v>
+        <v>323</v>
       </c>
     </row>
     <row r="25">
@@ -824,7 +824,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>282</v>
+        <v>283</v>
       </c>
     </row>
     <row r="30">
@@ -835,7 +835,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>844–846</t>
+          <t>847–849</t>
         </is>
       </c>
     </row>
@@ -847,7 +847,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否（进行中）</t>
         </is>
       </c>
     </row>
@@ -858,7 +858,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>130</v>
+        <v>31</v>
       </c>
     </row>
     <row r="33">
@@ -878,7 +878,7 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>130</v>
+        <v>31</v>
       </c>
     </row>
     <row r="35">
@@ -898,7 +898,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>130</v>
+        <v>31</v>
       </c>
     </row>
     <row r="37">
@@ -906,9 +906,6 @@
         <is>
           <t>周期现金变动</t>
         </is>
-      </c>
-      <c r="B37" s="4" t="n">
-        <v>-86336.76161287585</v>
       </c>
     </row>
     <row r="38"/>
@@ -970,7 +967,7 @@
         </is>
       </c>
       <c r="B44" s="4" t="n">
-        <v>-86336.76161287585</v>
+        <v>-87912.60647675232</v>
       </c>
     </row>
     <row r="45"/>
@@ -1292,7 +1289,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E973"/>
+  <dimension ref="A1:E1000"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -21741,8 +21738,575 @@
         <v>1234156.18</v>
       </c>
     </row>
+    <row r="974">
+      <c r="A974" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B974" s="10" t="n">
+        <v>847</v>
+      </c>
+      <c r="C974" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D974" s="11" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="E974" s="14" t="n">
+        <v>3254166.19</v>
+      </c>
+    </row>
+    <row r="975">
+      <c r="A975" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B975" s="15" t="n">
+        <v>847</v>
+      </c>
+      <c r="C975" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D975" s="16" t="inlineStr">
+        <is>
+          <t>montesquieu</t>
+        </is>
+      </c>
+      <c r="E975" s="18" t="n">
+        <v>2464942.69</v>
+      </c>
+    </row>
+    <row r="976">
+      <c r="A976" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B976" s="10" t="n">
+        <v>847</v>
+      </c>
+      <c r="C976" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D976" s="11" t="inlineStr">
+        <is>
+          <t>nicetry</t>
+        </is>
+      </c>
+      <c r="E976" s="14" t="n">
+        <v>2422595.19</v>
+      </c>
+    </row>
+    <row r="977">
+      <c r="A977" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B977" s="15" t="n">
+        <v>847</v>
+      </c>
+      <c r="C977" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D977" s="16" t="inlineStr">
+        <is>
+          <t>group2</t>
+        </is>
+      </c>
+      <c r="E977" s="18" t="n">
+        <v>2357380.29</v>
+      </c>
+    </row>
+    <row r="978">
+      <c r="A978" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B978" s="10" t="n">
+        <v>847</v>
+      </c>
+      <c r="C978" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="D978" s="11" t="inlineStr">
+        <is>
+          <t>group25</t>
+        </is>
+      </c>
+      <c r="E978" s="14" t="n">
+        <v>2357222.17</v>
+      </c>
+    </row>
+    <row r="979">
+      <c r="A979" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B979" s="15" t="n">
+        <v>847</v>
+      </c>
+      <c r="C979" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="D979" s="16" t="inlineStr">
+        <is>
+          <t>group11</t>
+        </is>
+      </c>
+      <c r="E979" s="18" t="n">
+        <v>2357209.86</v>
+      </c>
+    </row>
+    <row r="980">
+      <c r="A980" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B980" s="10" t="n">
+        <v>847</v>
+      </c>
+      <c r="C980" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="D980" s="11" t="inlineStr">
+        <is>
+          <t>88888888</t>
+        </is>
+      </c>
+      <c r="E980" s="14" t="n">
+        <v>2357187.18</v>
+      </c>
+    </row>
+    <row r="981">
+      <c r="A981" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B981" s="15" t="n">
+        <v>847</v>
+      </c>
+      <c r="C981" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="D981" s="16" t="inlineStr">
+        <is>
+          <t>t24</t>
+        </is>
+      </c>
+      <c r="E981" s="18" t="n">
+        <v>2338069.81</v>
+      </c>
+    </row>
+    <row r="982">
+      <c r="A982" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B982" s="10" t="n">
+        <v>847</v>
+      </c>
+      <c r="C982" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="D982" s="11" t="inlineStr">
+        <is>
+          <t>teamhlly</t>
+        </is>
+      </c>
+      <c r="E982" s="14" t="n">
+        <v>2290185.64</v>
+      </c>
+    </row>
+    <row r="983">
+      <c r="A983" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B983" s="15" t="n">
+        <v>847</v>
+      </c>
+      <c r="C983" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="D983" s="16" t="inlineStr">
+        <is>
+          <t>group9</t>
+        </is>
+      </c>
+      <c r="E983" s="18" t="n">
+        <v>2209994.06</v>
+      </c>
+    </row>
+    <row r="984">
+      <c r="A984" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B984" s="10" t="n">
+        <v>847</v>
+      </c>
+      <c r="C984" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="D984" s="11" t="inlineStr">
+        <is>
+          <t>group14</t>
+        </is>
+      </c>
+      <c r="E984" s="14" t="n">
+        <v>2150927.03</v>
+      </c>
+    </row>
+    <row r="985">
+      <c r="A985" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B985" s="15" t="n">
+        <v>847</v>
+      </c>
+      <c r="C985" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="D985" s="16" t="inlineStr">
+        <is>
+          <t>group15</t>
+        </is>
+      </c>
+      <c r="E985" s="18" t="n">
+        <v>2109524.75</v>
+      </c>
+    </row>
+    <row r="986">
+      <c r="A986" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B986" s="10" t="n">
+        <v>847</v>
+      </c>
+      <c r="C986" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="D986" s="11" t="inlineStr">
+        <is>
+          <t>666666</t>
+        </is>
+      </c>
+      <c r="E986" s="14" t="n">
+        <v>2019485.8</v>
+      </c>
+    </row>
+    <row r="987">
+      <c r="A987" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B987" s="15" t="n">
+        <v>847</v>
+      </c>
+      <c r="C987" s="15" t="n">
+        <v>14</v>
+      </c>
+      <c r="D987" s="16" t="inlineStr">
+        <is>
+          <t>deepsleep</t>
+        </is>
+      </c>
+      <c r="E987" s="18" t="n">
+        <v>1967441.89</v>
+      </c>
+    </row>
+    <row r="988">
+      <c r="A988" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B988" s="10" t="n">
+        <v>847</v>
+      </c>
+      <c r="C988" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="D988" s="11" t="inlineStr">
+        <is>
+          <t>cleveregg</t>
+        </is>
+      </c>
+      <c r="E988" s="14" t="n">
+        <v>1926848.57</v>
+      </c>
+    </row>
+    <row r="989">
+      <c r="A989" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B989" s="15" t="n">
+        <v>847</v>
+      </c>
+      <c r="C989" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="D989" s="16" t="inlineStr">
+        <is>
+          <t>tigagroup20</t>
+        </is>
+      </c>
+      <c r="E989" s="18" t="n">
+        <v>1898961.18</v>
+      </c>
+    </row>
+    <row r="990">
+      <c r="A990" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B990" s="10" t="n">
+        <v>847</v>
+      </c>
+      <c r="C990" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="D990" s="11" t="inlineStr">
+        <is>
+          <t>group8</t>
+        </is>
+      </c>
+      <c r="E990" s="14" t="n">
+        <v>1840778.85</v>
+      </c>
+    </row>
+    <row r="991">
+      <c r="A991" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B991" s="15" t="n">
+        <v>847</v>
+      </c>
+      <c r="C991" s="15" t="n">
+        <v>18</v>
+      </c>
+      <c r="D991" s="16" t="inlineStr">
+        <is>
+          <t>jit</t>
+        </is>
+      </c>
+      <c r="E991" s="18" t="n">
+        <v>1838001.94</v>
+      </c>
+    </row>
+    <row r="992">
+      <c r="A992" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B992" s="10" t="n">
+        <v>847</v>
+      </c>
+      <c r="C992" s="10" t="n">
+        <v>19</v>
+      </c>
+      <c r="D992" s="11" t="inlineStr">
+        <is>
+          <t>group7</t>
+        </is>
+      </c>
+      <c r="E992" s="14" t="n">
+        <v>1774410.32</v>
+      </c>
+    </row>
+    <row r="993">
+      <c r="A993" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B993" s="15" t="n">
+        <v>847</v>
+      </c>
+      <c r="C993" s="15" t="n">
+        <v>20</v>
+      </c>
+      <c r="D993" s="16" t="inlineStr">
+        <is>
+          <t>newgroup18</t>
+        </is>
+      </c>
+      <c r="E993" s="18" t="n">
+        <v>1765732.59</v>
+      </c>
+    </row>
+    <row r="994">
+      <c r="A994" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B994" s="10" t="n">
+        <v>847</v>
+      </c>
+      <c r="C994" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="D994" s="11" t="inlineStr">
+        <is>
+          <t>vivo50</t>
+        </is>
+      </c>
+      <c r="E994" s="14" t="n">
+        <v>1725268.86</v>
+      </c>
+    </row>
+    <row r="995">
+      <c r="A995" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B995" s="15" t="n">
+        <v>847</v>
+      </c>
+      <c r="C995" s="15" t="n">
+        <v>22</v>
+      </c>
+      <c r="D995" s="16" t="inlineStr">
+        <is>
+          <t>group12</t>
+        </is>
+      </c>
+      <c r="E995" s="18" t="n">
+        <v>1651158.71</v>
+      </c>
+    </row>
+    <row r="996">
+      <c r="A996" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B996" s="10" t="n">
+        <v>847</v>
+      </c>
+      <c r="C996" s="10" t="n">
+        <v>23</v>
+      </c>
+      <c r="D996" s="11" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E996" s="14" t="n">
+        <v>1586542.34</v>
+      </c>
+    </row>
+    <row r="997">
+      <c r="A997" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B997" s="15" t="n">
+        <v>847</v>
+      </c>
+      <c r="C997" s="15" t="n">
+        <v>24</v>
+      </c>
+      <c r="D997" s="16" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E997" s="18" t="n">
+        <v>1548690.35</v>
+      </c>
+    </row>
+    <row r="998">
+      <c r="A998" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B998" s="10" t="n">
+        <v>847</v>
+      </c>
+      <c r="C998" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="D998" s="11" t="inlineStr">
+        <is>
+          <t>aaachemicalseller</t>
+        </is>
+      </c>
+      <c r="E998" s="14" t="n">
+        <v>1546340.32</v>
+      </c>
+    </row>
+    <row r="999">
+      <c r="A999" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B999" s="24" t="n">
+        <v>847</v>
+      </c>
+      <c r="C999" s="24" t="n">
+        <v>26</v>
+      </c>
+      <c r="D999" s="25" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="E999" s="26" t="n">
+        <v>1495887.76</v>
+      </c>
+    </row>
+    <row r="1000">
+      <c r="A1000" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B1000" s="10" t="n">
+        <v>847</v>
+      </c>
+      <c r="C1000" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="D1000" s="11" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="E1000" s="14" t="n">
+        <v>1085542.62</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E973"/>
+  <autoFilter ref="A1:E1000"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -21753,7 +22317,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S283"/>
+  <dimension ref="A1:S284"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -39640,8 +40204,69 @@
         <v>188500</v>
       </c>
     </row>
+    <row r="284">
+      <c r="A284" s="10" t="n">
+        <v>283</v>
+      </c>
+      <c r="B284" s="10" t="n">
+        <v>847</v>
+      </c>
+      <c r="C284" s="10" t="n">
+        <v>849</v>
+      </c>
+      <c r="D284" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E284" s="11" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="F284" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G284" s="12" t="n">
+        <v>31</v>
+      </c>
+      <c r="H284" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I284" s="12" t="n">
+        <v>31</v>
+      </c>
+      <c r="J284" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K284" s="12" t="n">
+        <v>31</v>
+      </c>
+      <c r="L284" s="14" t="n">
+        <v>1495887.76</v>
+      </c>
+      <c r="M284" s="14" t="n">
+        <v>1495887.76</v>
+      </c>
+      <c r="N284" s="11" t="n"/>
+      <c r="O284" s="12" t="n">
+        <v>323</v>
+      </c>
+      <c r="P284" s="12" t="n">
+        <v>323</v>
+      </c>
+      <c r="Q284" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R284" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="S284" s="14" t="n">
+        <v>44950</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S283"/>
+  <autoFilter ref="A1:S284"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -39652,7 +40277,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N847"/>
+  <dimension ref="A1:N848"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -78659,8 +79284,54 @@
         <v>75400</v>
       </c>
     </row>
+    <row r="848">
+      <c r="A848" s="10" t="n">
+        <v>847</v>
+      </c>
+      <c r="B848" s="11" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C848" s="12" t="n">
+        <v>31</v>
+      </c>
+      <c r="D848" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E848" s="12" t="n">
+        <v>31</v>
+      </c>
+      <c r="F848" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G848" s="12" t="n">
+        <v>31</v>
+      </c>
+      <c r="H848" s="14" t="n">
+        <v>1495887.76</v>
+      </c>
+      <c r="I848" s="12" t="n">
+        <v>323</v>
+      </c>
+      <c r="J848" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K848" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L848" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M848" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="N848" s="14" t="n">
+        <v>44950</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N847"/>
+  <autoFilter ref="A1:N848"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -79055,7 +79726,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F75"/>
+  <dimension ref="A1:F77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -80888,8 +81559,56 @@
         <v>55</v>
       </c>
     </row>
+    <row r="76">
+      <c r="A76" s="21" t="n">
+        <v>730.66</v>
+      </c>
+      <c r="B76" s="11" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C76" s="11" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D76" s="11" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E76" s="11" t="inlineStr"/>
+      <c r="F76" s="12" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="23" t="n">
+        <v>742.75</v>
+      </c>
+      <c r="B77" s="16" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C77" s="16" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D77" s="16" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E77" s="16" t="inlineStr"/>
+      <c r="F77" s="17" t="n">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F75"/>
+  <autoFilter ref="A1:F77"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -81288,7 +82007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U36"/>
+  <dimension ref="A1:U37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -83854,8 +84573,75 @@
         <v>-86336.76161287585</v>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B37" s="15" t="n">
+        <v>847</v>
+      </c>
+      <c r="C37" s="18" t="n">
+        <v>1495887.76</v>
+      </c>
+      <c r="D37" s="15" t="n">
+        <v>26</v>
+      </c>
+      <c r="E37" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="F37" s="16" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="G37" s="18" t="n">
+        <v>1758278.43</v>
+      </c>
+      <c r="H37" s="23" t="n">
+        <v>55</v>
+      </c>
+      <c r="I37" s="16" t="n"/>
+      <c r="J37" s="16" t="inlineStr">
+        <is>
+          <t>mail</t>
+        </is>
+      </c>
+      <c r="K37" s="27" t="n">
+        <v>3600</v>
+      </c>
+      <c r="L37" s="27" t="n">
+        <v>200</v>
+      </c>
+      <c r="M37" s="17" t="n">
+        <v>323</v>
+      </c>
+      <c r="N37" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O37" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="P37" s="15" t="n">
+        <v>283</v>
+      </c>
+      <c r="Q37" s="17" t="n">
+        <v>31</v>
+      </c>
+      <c r="R37" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="S37" s="17" t="n">
+        <v>31</v>
+      </c>
+      <c r="T37" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="U37" s="16" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U36"/>
+  <autoFilter ref="A1:U37"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -83866,7 +84652,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E433"/>
+  <dimension ref="A1:E445"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -93695,8 +94481,280 @@
         </is>
       </c>
     </row>
+    <row r="434">
+      <c r="A434" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B434" s="10" t="n">
+        <v>847</v>
+      </c>
+      <c r="C434" s="11" t="inlineStr">
+        <is>
+          <t>Starting Cash</t>
+        </is>
+      </c>
+      <c r="D434" s="14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E434" s="11" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B435" s="15" t="n">
+        <v>847</v>
+      </c>
+      <c r="C435" s="16" t="inlineStr">
+        <is>
+          <t>Cash Sources</t>
+        </is>
+      </c>
+      <c r="D435" s="16" t="n"/>
+      <c r="E435" s="16" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B436" s="10" t="n">
+        <v>847</v>
+      </c>
+      <c r="C436" s="11" t="inlineStr">
+        <is>
+          <t>revenues</t>
+        </is>
+      </c>
+      <c r="D436" s="14" t="n">
+        <v>22998450</v>
+      </c>
+      <c r="E436" s="11" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B437" s="15" t="n">
+        <v>847</v>
+      </c>
+      <c r="C437" s="16" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D437" s="18" t="n">
+        <v>304757.88</v>
+      </c>
+      <c r="E437" s="16" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B438" s="10" t="n">
+        <v>847</v>
+      </c>
+      <c r="C438" s="11" t="inlineStr">
+        <is>
+          <t>Cash Uses</t>
+        </is>
+      </c>
+      <c r="D438" s="11" t="n"/>
+      <c r="E438" s="11" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B439" s="15" t="n">
+        <v>847</v>
+      </c>
+      <c r="C439" s="16" t="inlineStr">
+        <is>
+          <t>outbound shipping</t>
+        </is>
+      </c>
+      <c r="D439" s="18" t="n">
+        <v>-2379150</v>
+      </c>
+      <c r="E439" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B440" s="10" t="n">
+        <v>847</v>
+      </c>
+      <c r="C440" s="11" t="inlineStr">
+        <is>
+          <t>inbound shipping</t>
+        </is>
+      </c>
+      <c r="D440" s="14" t="n">
+        <v>-1620000</v>
+      </c>
+      <c r="E440" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B441" s="15" t="n">
+        <v>847</v>
+      </c>
+      <c r="C441" s="16" t="inlineStr">
+        <is>
+          <t>FGI holding</t>
+        </is>
+      </c>
+      <c r="D441" s="18" t="n">
+        <v>-22342.95</v>
+      </c>
+      <c r="E441" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B442" s="10" t="n">
+        <v>847</v>
+      </c>
+      <c r="C442" s="11" t="inlineStr">
+        <is>
+          <t>add capacity</t>
+        </is>
+      </c>
+      <c r="D442" s="14" t="n">
+        <v>-1749840.87</v>
+      </c>
+      <c r="E442" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B443" s="15" t="n">
+        <v>847</v>
+      </c>
+      <c r="C443" s="16" t="inlineStr">
+        <is>
+          <t>Pipeline inventory holding</t>
+        </is>
+      </c>
+      <c r="D443" s="18" t="n">
+        <v>-29986.3</v>
+      </c>
+      <c r="E443" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B444" s="10" t="n">
+        <v>847</v>
+      </c>
+      <c r="C444" s="11" t="inlineStr">
+        <is>
+          <t>production</t>
+        </is>
+      </c>
+      <c r="D444" s="14" t="n">
+        <v>-16506000</v>
+      </c>
+      <c r="E444" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T15:56:03+08:00</t>
+        </is>
+      </c>
+      <c r="B445" s="15" t="n">
+        <v>847</v>
+      </c>
+      <c r="C445" s="16" t="inlineStr">
+        <is>
+          <t>Cash Balance</t>
+        </is>
+      </c>
+      <c r="D445" s="18" t="n">
+        <v>1495887.76</v>
+      </c>
+      <c r="E445" s="16" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E433"/>
+  <autoFilter ref="A1:E445"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update game data: day 848, cash 1289397.07, 3-day period 283
</commit_message>
<xml_diff>
--- a/data/supply_chain_game.xlsx
+++ b/data/supply_chain_game.xlsx
@@ -21,15 +21,15 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'三日周期'!$A$1:$S$284</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$848</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'每日数据'!$A$1:$N$849</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'资金构成_旧版'!$A$1:$C$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'运营参数_旧版'!$A$9:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$77</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'决策历史'!$A$1:$F$79</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'排行榜_旧版'!$A$1:$C$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$37</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$445</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'快照历史'!$A$1:$U$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'资金构成'!$A$1:$E$457</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'运营参数'!$A$1:$J$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$1000</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'排行榜'!$A$1:$E$1027</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -590,7 +590,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-06T15:56:03+08:00</t>
+          <t>2026-09-06T16:11:03+08:00</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>847</v>
+        <v>848</v>
       </c>
     </row>
     <row r="7">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>613</v>
+        <v>612</v>
       </c>
     </row>
     <row r="8">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>1495887.76</v>
+        <v>1289397.07</v>
       </c>
     </row>
     <row r="11">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>1758278.43</v>
+        <v>1990258.17</v>
       </c>
     </row>
     <row r="15"/>
@@ -786,7 +786,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>323</v>
+        <v>283</v>
       </c>
     </row>
     <row r="25">
@@ -858,7 +858,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>31</v>
+        <v>71</v>
       </c>
     </row>
     <row r="33">
@@ -878,7 +878,7 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>31</v>
+        <v>71</v>
       </c>
     </row>
     <row r="35">
@@ -898,7 +898,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>31</v>
+        <v>71</v>
       </c>
     </row>
     <row r="37">
@@ -906,6 +906,9 @@
         <is>
           <t>周期现金变动</t>
         </is>
+      </c>
+      <c r="B37" s="4" t="n">
+        <v>44845.47999748518</v>
       </c>
     </row>
     <row r="38"/>
@@ -967,7 +970,7 @@
         </is>
       </c>
       <c r="B44" s="4" t="n">
-        <v>-87912.60647675232</v>
+        <v>-73141.70026493655</v>
       </c>
     </row>
     <row r="45"/>
@@ -1289,7 +1292,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1000"/>
+  <dimension ref="A1:E1027"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -22305,8 +22308,575 @@
         <v>1085542.62</v>
       </c>
     </row>
+    <row r="1001">
+      <c r="A1001" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B1001" s="15" t="n">
+        <v>848</v>
+      </c>
+      <c r="C1001" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1001" s="16" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="E1001" s="18" t="n">
+        <v>3279655.24</v>
+      </c>
+    </row>
+    <row r="1002">
+      <c r="A1002" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B1002" s="10" t="n">
+        <v>848</v>
+      </c>
+      <c r="C1002" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D1002" s="11" t="inlineStr">
+        <is>
+          <t>montesquieu</t>
+        </is>
+      </c>
+      <c r="E1002" s="14" t="n">
+        <v>2490183.12</v>
+      </c>
+    </row>
+    <row r="1003">
+      <c r="A1003" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B1003" s="15" t="n">
+        <v>848</v>
+      </c>
+      <c r="C1003" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D1003" s="16" t="inlineStr">
+        <is>
+          <t>nicetry</t>
+        </is>
+      </c>
+      <c r="E1003" s="18" t="n">
+        <v>2447838.03</v>
+      </c>
+    </row>
+    <row r="1004">
+      <c r="A1004" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B1004" s="10" t="n">
+        <v>848</v>
+      </c>
+      <c r="C1004" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D1004" s="11" t="inlineStr">
+        <is>
+          <t>t24</t>
+        </is>
+      </c>
+      <c r="E1004" s="14" t="n">
+        <v>2363360.98</v>
+      </c>
+    </row>
+    <row r="1005">
+      <c r="A1005" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B1005" s="15" t="n">
+        <v>848</v>
+      </c>
+      <c r="C1005" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="D1005" s="16" t="inlineStr">
+        <is>
+          <t>teamhlly</t>
+        </is>
+      </c>
+      <c r="E1005" s="18" t="n">
+        <v>2315404.03</v>
+      </c>
+    </row>
+    <row r="1006">
+      <c r="A1006" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B1006" s="10" t="n">
+        <v>848</v>
+      </c>
+      <c r="C1006" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="D1006" s="11" t="inlineStr">
+        <is>
+          <t>group9</t>
+        </is>
+      </c>
+      <c r="E1006" s="14" t="n">
+        <v>2235183.01</v>
+      </c>
+    </row>
+    <row r="1007">
+      <c r="A1007" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B1007" s="15" t="n">
+        <v>848</v>
+      </c>
+      <c r="C1007" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1007" s="16" t="inlineStr">
+        <is>
+          <t>group14</t>
+        </is>
+      </c>
+      <c r="E1007" s="18" t="n">
+        <v>2176095.08</v>
+      </c>
+    </row>
+    <row r="1008">
+      <c r="A1008" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B1008" s="10" t="n">
+        <v>848</v>
+      </c>
+      <c r="C1008" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="D1008" s="11" t="inlineStr">
+        <is>
+          <t>group2</t>
+        </is>
+      </c>
+      <c r="E1008" s="14" t="n">
+        <v>2166130.48</v>
+      </c>
+    </row>
+    <row r="1009">
+      <c r="A1009" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B1009" s="15" t="n">
+        <v>848</v>
+      </c>
+      <c r="C1009" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="D1009" s="16" t="inlineStr">
+        <is>
+          <t>group25</t>
+        </is>
+      </c>
+      <c r="E1009" s="18" t="n">
+        <v>2165972.31</v>
+      </c>
+    </row>
+    <row r="1010">
+      <c r="A1010" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B1010" s="10" t="n">
+        <v>848</v>
+      </c>
+      <c r="C1010" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="D1010" s="11" t="inlineStr">
+        <is>
+          <t>group11</t>
+        </is>
+      </c>
+      <c r="E1010" s="14" t="n">
+        <v>2165960</v>
+      </c>
+    </row>
+    <row r="1011">
+      <c r="A1011" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B1011" s="15" t="n">
+        <v>848</v>
+      </c>
+      <c r="C1011" s="15" t="n">
+        <v>11</v>
+      </c>
+      <c r="D1011" s="16" t="inlineStr">
+        <is>
+          <t>88888888</t>
+        </is>
+      </c>
+      <c r="E1011" s="18" t="n">
+        <v>2165937.31</v>
+      </c>
+    </row>
+    <row r="1012">
+      <c r="A1012" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B1012" s="10" t="n">
+        <v>848</v>
+      </c>
+      <c r="C1012" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="D1012" s="11" t="inlineStr">
+        <is>
+          <t>group15</t>
+        </is>
+      </c>
+      <c r="E1012" s="14" t="n">
+        <v>2134681.99</v>
+      </c>
+    </row>
+    <row r="1013">
+      <c r="A1013" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B1013" s="15" t="n">
+        <v>848</v>
+      </c>
+      <c r="C1013" s="15" t="n">
+        <v>13</v>
+      </c>
+      <c r="D1013" s="16" t="inlineStr">
+        <is>
+          <t>666666</t>
+        </is>
+      </c>
+      <c r="E1013" s="18" t="n">
+        <v>2026399.98</v>
+      </c>
+    </row>
+    <row r="1014">
+      <c r="A1014" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B1014" s="10" t="n">
+        <v>848</v>
+      </c>
+      <c r="C1014" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="D1014" s="11" t="inlineStr">
+        <is>
+          <t>cleveregg</t>
+        </is>
+      </c>
+      <c r="E1014" s="14" t="n">
+        <v>1951941.49</v>
+      </c>
+    </row>
+    <row r="1015">
+      <c r="A1015" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B1015" s="15" t="n">
+        <v>848</v>
+      </c>
+      <c r="C1015" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="D1015" s="16" t="inlineStr">
+        <is>
+          <t>tigagroup20</t>
+        </is>
+      </c>
+      <c r="E1015" s="18" t="n">
+        <v>1924070.61</v>
+      </c>
+    </row>
+    <row r="1016">
+      <c r="A1016" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B1016" s="10" t="n">
+        <v>848</v>
+      </c>
+      <c r="C1016" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="D1016" s="11" t="inlineStr">
+        <is>
+          <t>group8</t>
+        </is>
+      </c>
+      <c r="E1016" s="14" t="n">
+        <v>1923007.84</v>
+      </c>
+    </row>
+    <row r="1017">
+      <c r="A1017" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B1017" s="15" t="n">
+        <v>848</v>
+      </c>
+      <c r="C1017" s="15" t="n">
+        <v>17</v>
+      </c>
+      <c r="D1017" s="16" t="inlineStr">
+        <is>
+          <t>jit</t>
+        </is>
+      </c>
+      <c r="E1017" s="18" t="n">
+        <v>1815532.15</v>
+      </c>
+    </row>
+    <row r="1018">
+      <c r="A1018" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B1018" s="10" t="n">
+        <v>848</v>
+      </c>
+      <c r="C1018" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="D1018" s="11" t="inlineStr">
+        <is>
+          <t>deepsleep</t>
+        </is>
+      </c>
+      <c r="E1018" s="14" t="n">
+        <v>1796069.56</v>
+      </c>
+    </row>
+    <row r="1019">
+      <c r="A1019" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B1019" s="15" t="n">
+        <v>848</v>
+      </c>
+      <c r="C1019" s="15" t="n">
+        <v>19</v>
+      </c>
+      <c r="D1019" s="16" t="inlineStr">
+        <is>
+          <t>group7</t>
+        </is>
+      </c>
+      <c r="E1019" s="18" t="n">
+        <v>1774764.13</v>
+      </c>
+    </row>
+    <row r="1020">
+      <c r="A1020" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B1020" s="10" t="n">
+        <v>848</v>
+      </c>
+      <c r="C1020" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="D1020" s="11" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E1020" s="14" t="n">
+        <v>1611543.45</v>
+      </c>
+    </row>
+    <row r="1021">
+      <c r="A1021" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B1021" s="15" t="n">
+        <v>848</v>
+      </c>
+      <c r="C1021" s="15" t="n">
+        <v>21</v>
+      </c>
+      <c r="D1021" s="16" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E1021" s="18" t="n">
+        <v>1573665.77</v>
+      </c>
+    </row>
+    <row r="1022">
+      <c r="A1022" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B1022" s="10" t="n">
+        <v>848</v>
+      </c>
+      <c r="C1022" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="D1022" s="11" t="inlineStr">
+        <is>
+          <t>aaachemicalseller</t>
+        </is>
+      </c>
+      <c r="E1022" s="14" t="n">
+        <v>1571322.53</v>
+      </c>
+    </row>
+    <row r="1023">
+      <c r="A1023" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B1023" s="15" t="n">
+        <v>848</v>
+      </c>
+      <c r="C1023" s="15" t="n">
+        <v>23</v>
+      </c>
+      <c r="D1023" s="16" t="inlineStr">
+        <is>
+          <t>vivo50</t>
+        </is>
+      </c>
+      <c r="E1023" s="18" t="n">
+        <v>1533816.78</v>
+      </c>
+    </row>
+    <row r="1024">
+      <c r="A1024" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B1024" s="10" t="n">
+        <v>848</v>
+      </c>
+      <c r="C1024" s="10" t="n">
+        <v>24</v>
+      </c>
+      <c r="D1024" s="11" t="inlineStr">
+        <is>
+          <t>group12</t>
+        </is>
+      </c>
+      <c r="E1024" s="14" t="n">
+        <v>1459687.28</v>
+      </c>
+    </row>
+    <row r="1025">
+      <c r="A1025" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B1025" s="15" t="n">
+        <v>848</v>
+      </c>
+      <c r="C1025" s="15" t="n">
+        <v>25</v>
+      </c>
+      <c r="D1025" s="16" t="inlineStr">
+        <is>
+          <t>newgroup18</t>
+        </is>
+      </c>
+      <c r="E1025" s="18" t="n">
+        <v>1329294.21</v>
+      </c>
+    </row>
+    <row r="1026">
+      <c r="A1026" s="25" t="inlineStr">
+        <is>
+          <t>2026-09-06T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B1026" s="24" t="n">
+        <v>848</v>
+      </c>
+      <c r="C1026" s="24" t="n">
+        <v>26</v>
+      </c>
+      <c r="D1026" s="25" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="E1026" s="26" t="n">
+        <v>1289397.07</v>
+      </c>
+    </row>
+    <row r="1027">
+      <c r="A1027" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B1027" s="15" t="n">
+        <v>848</v>
+      </c>
+      <c r="C1027" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="D1027" s="16" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="E1027" s="18" t="n">
+        <v>1110512.07</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E1000"/>
+  <autoFilter ref="A1:E1027"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -40215,7 +40785,7 @@
         <v>849</v>
       </c>
       <c r="D284" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E284" s="11" t="inlineStr">
         <is>
@@ -40228,32 +40798,34 @@
         </is>
       </c>
       <c r="G284" s="12" t="n">
-        <v>31</v>
+        <v>71</v>
       </c>
       <c r="H284" s="12" t="n">
         <v>0</v>
       </c>
       <c r="I284" s="12" t="n">
-        <v>31</v>
+        <v>71</v>
       </c>
       <c r="J284" s="19" t="n">
         <v>1</v>
       </c>
       <c r="K284" s="12" t="n">
-        <v>31</v>
+        <v>71</v>
       </c>
       <c r="L284" s="14" t="n">
-        <v>1495887.76</v>
+        <v>1244551.590002515</v>
       </c>
       <c r="M284" s="14" t="n">
-        <v>1495887.76</v>
-      </c>
-      <c r="N284" s="11" t="n"/>
+        <v>1289397.07</v>
+      </c>
+      <c r="N284" s="14" t="n">
+        <v>44845.47999748518</v>
+      </c>
       <c r="O284" s="12" t="n">
-        <v>323</v>
+        <v>283</v>
       </c>
       <c r="P284" s="12" t="n">
-        <v>323</v>
+        <v>303</v>
       </c>
       <c r="Q284" s="12" t="n">
         <v>0</v>
@@ -40262,7 +40834,7 @@
         <v>200</v>
       </c>
       <c r="S284" s="14" t="n">
-        <v>44950</v>
+        <v>102950</v>
       </c>
     </row>
   </sheetData>
@@ -40277,7 +40849,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N848"/>
+  <dimension ref="A1:N849"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -79330,8 +79902,54 @@
         <v>44950</v>
       </c>
     </row>
+    <row r="849">
+      <c r="A849" s="15" t="n">
+        <v>848</v>
+      </c>
+      <c r="B849" s="16" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C849" s="17" t="n">
+        <v>40</v>
+      </c>
+      <c r="D849" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E849" s="17" t="n">
+        <v>40</v>
+      </c>
+      <c r="F849" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G849" s="17" t="n">
+        <v>40</v>
+      </c>
+      <c r="H849" s="18" t="n">
+        <v>1289397.07</v>
+      </c>
+      <c r="I849" s="17" t="n">
+        <v>283</v>
+      </c>
+      <c r="J849" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K849" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L849" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M849" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="N849" s="18" t="n">
+        <v>58000</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N848"/>
+  <autoFilter ref="A1:N849"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -79726,7 +80344,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F77"/>
+  <dimension ref="A1:F79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -81607,8 +82225,56 @@
         <v>55</v>
       </c>
     </row>
+    <row r="78">
+      <c r="A78" s="21" t="n">
+        <v>730.66</v>
+      </c>
+      <c r="B78" s="11" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C78" s="11" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D78" s="11" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E78" s="11" t="inlineStr"/>
+      <c r="F78" s="12" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="23" t="n">
+        <v>742.75</v>
+      </c>
+      <c r="B79" s="16" t="inlineStr">
+        <is>
+          <t>Schedule factory capacity change in Calopeia</t>
+        </is>
+      </c>
+      <c r="C79" s="16" t="inlineStr">
+        <is>
+          <t>Schedule capacity change</t>
+        </is>
+      </c>
+      <c r="D79" s="16" t="inlineStr">
+        <is>
+          <t>Calopeia</t>
+        </is>
+      </c>
+      <c r="E79" s="16" t="inlineStr"/>
+      <c r="F79" s="17" t="n">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F77"/>
+  <autoFilter ref="A1:F79"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -82007,7 +82673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U37"/>
+  <dimension ref="A1:U38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -82016,7 +82682,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
@@ -84640,8 +85306,77 @@
       </c>
       <c r="U37" s="16" t="n"/>
     </row>
+    <row r="38">
+      <c r="A38" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B38" s="10" t="n">
+        <v>848</v>
+      </c>
+      <c r="C38" s="14" t="n">
+        <v>1289397.07</v>
+      </c>
+      <c r="D38" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="E38" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="F38" s="11" t="inlineStr">
+        <is>
+          <t>donothing</t>
+        </is>
+      </c>
+      <c r="G38" s="14" t="n">
+        <v>1990258.17</v>
+      </c>
+      <c r="H38" s="21" t="n">
+        <v>55</v>
+      </c>
+      <c r="I38" s="11" t="n"/>
+      <c r="J38" s="11" t="inlineStr">
+        <is>
+          <t>mail</t>
+        </is>
+      </c>
+      <c r="K38" s="22" t="n">
+        <v>3600</v>
+      </c>
+      <c r="L38" s="22" t="n">
+        <v>200</v>
+      </c>
+      <c r="M38" s="12" t="n">
+        <v>283</v>
+      </c>
+      <c r="N38" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="O38" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="P38" s="10" t="n">
+        <v>283</v>
+      </c>
+      <c r="Q38" s="12" t="n">
+        <v>71</v>
+      </c>
+      <c r="R38" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S38" s="12" t="n">
+        <v>71</v>
+      </c>
+      <c r="T38" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="U38" s="14" t="n">
+        <v>44845.47999748518</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U37"/>
+  <autoFilter ref="A1:U38"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -84652,7 +85387,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E445"/>
+  <dimension ref="A1:E457"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -94753,8 +95488,280 @@
         </is>
       </c>
     </row>
+    <row r="446">
+      <c r="A446" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B446" s="10" t="n">
+        <v>848</v>
+      </c>
+      <c r="C446" s="11" t="inlineStr">
+        <is>
+          <t>Starting Cash</t>
+        </is>
+      </c>
+      <c r="D446" s="14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E446" s="11" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B447" s="15" t="n">
+        <v>848</v>
+      </c>
+      <c r="C447" s="16" t="inlineStr">
+        <is>
+          <t>Cash Sources</t>
+        </is>
+      </c>
+      <c r="D447" s="16" t="n"/>
+      <c r="E447" s="16" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B448" s="10" t="n">
+        <v>848</v>
+      </c>
+      <c r="C448" s="11" t="inlineStr">
+        <is>
+          <t>revenues</t>
+        </is>
+      </c>
+      <c r="D448" s="14" t="n">
+        <v>23026000</v>
+      </c>
+      <c r="E448" s="11" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B449" s="15" t="n">
+        <v>848</v>
+      </c>
+      <c r="C449" s="16" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D449" s="18" t="n">
+        <v>305147.34</v>
+      </c>
+      <c r="E449" s="16" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B450" s="10" t="n">
+        <v>848</v>
+      </c>
+      <c r="C450" s="11" t="inlineStr">
+        <is>
+          <t>Cash Uses</t>
+        </is>
+      </c>
+      <c r="D450" s="11" t="n"/>
+      <c r="E450" s="11" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B451" s="15" t="n">
+        <v>848</v>
+      </c>
+      <c r="C451" s="16" t="inlineStr">
+        <is>
+          <t>outbound shipping</t>
+        </is>
+      </c>
+      <c r="D451" s="18" t="n">
+        <v>-2382000</v>
+      </c>
+      <c r="E451" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B452" s="10" t="n">
+        <v>848</v>
+      </c>
+      <c r="C452" s="11" t="inlineStr">
+        <is>
+          <t>inbound shipping</t>
+        </is>
+      </c>
+      <c r="D452" s="14" t="n">
+        <v>-1650000</v>
+      </c>
+      <c r="E452" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B453" s="15" t="n">
+        <v>848</v>
+      </c>
+      <c r="C453" s="16" t="inlineStr">
+        <is>
+          <t>FGI holding</t>
+        </is>
+      </c>
+      <c r="D453" s="18" t="n">
+        <v>-22423.1</v>
+      </c>
+      <c r="E453" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B454" s="10" t="n">
+        <v>848</v>
+      </c>
+      <c r="C454" s="11" t="inlineStr">
+        <is>
+          <t>add capacity</t>
+        </is>
+      </c>
+      <c r="D454" s="14" t="n">
+        <v>-1749840.87</v>
+      </c>
+      <c r="E454" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B455" s="15" t="n">
+        <v>848</v>
+      </c>
+      <c r="C455" s="16" t="inlineStr">
+        <is>
+          <t>Pipeline inventory holding</t>
+        </is>
+      </c>
+      <c r="D455" s="18" t="n">
+        <v>-29986.3</v>
+      </c>
+      <c r="E455" s="16" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B456" s="10" t="n">
+        <v>848</v>
+      </c>
+      <c r="C456" s="11" t="inlineStr">
+        <is>
+          <t>production</t>
+        </is>
+      </c>
+      <c r="D456" s="14" t="n">
+        <v>-16707500</v>
+      </c>
+      <c r="E456" s="11" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-06T16:11:03+08:00</t>
+        </is>
+      </c>
+      <c r="B457" s="15" t="n">
+        <v>848</v>
+      </c>
+      <c r="C457" s="16" t="inlineStr">
+        <is>
+          <t>Cash Balance</t>
+        </is>
+      </c>
+      <c r="D457" s="18" t="n">
+        <v>1289397.07</v>
+      </c>
+      <c r="E457" s="16" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E445"/>
+  <autoFilter ref="A1:E457"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>